<commit_message>
Resolve highlight header at sds-v2
</commit_message>
<xml_diff>
--- a/apps/ENG-Backend/api/engineer/mtc/templates/sds_template.xlsx
+++ b/apps/ENG-Backend/api/engineer/mtc/templates/sds_template.xlsx
@@ -736,7 +736,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="183">
+  <cellXfs count="185">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1009,9 +1009,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="190" fontId="3" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="190" fontId="3" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1113,14 +1110,170 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="190" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="190" fontId="3" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="190" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="190" fontId="16" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="1" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="189" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1128,160 +1281,13 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="189" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="188" fontId="1" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="190" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="190" fontId="26" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="190" fontId="3" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="190" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="190" fontId="16" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1779,29 +1785,29 @@
       <c r="AE3" s="11"/>
       <c r="AF3" s="11"/>
       <c r="AG3" s="16"/>
-      <c r="AH3" s="151" t="s">
+      <c r="AH3" s="150" t="s">
         <v>6</v>
       </c>
-      <c r="AI3" s="152"/>
-      <c r="AJ3" s="152"/>
-      <c r="AK3" s="152"/>
-      <c r="AL3" s="152"/>
-      <c r="AM3" s="153"/>
-      <c r="AN3" s="151" t="s">
+      <c r="AI3" s="151"/>
+      <c r="AJ3" s="151"/>
+      <c r="AK3" s="151"/>
+      <c r="AL3" s="151"/>
+      <c r="AM3" s="152"/>
+      <c r="AN3" s="150" t="s">
         <v>7</v>
       </c>
-      <c r="AO3" s="152"/>
-      <c r="AP3" s="153"/>
-      <c r="AQ3" s="151" t="s">
+      <c r="AO3" s="151"/>
+      <c r="AP3" s="152"/>
+      <c r="AQ3" s="150" t="s">
         <v>8</v>
       </c>
-      <c r="AR3" s="152"/>
-      <c r="AS3" s="153"/>
-      <c r="AT3" s="151" t="s">
+      <c r="AR3" s="151"/>
+      <c r="AS3" s="152"/>
+      <c r="AT3" s="150" t="s">
         <v>9</v>
       </c>
-      <c r="AU3" s="152"/>
-      <c r="AV3" s="153"/>
+      <c r="AU3" s="151"/>
+      <c r="AV3" s="152"/>
     </row>
     <row r="4" spans="1:48" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
@@ -1837,7 +1843,7 @@
       </c>
       <c r="X4" s="12"/>
       <c r="Y4" s="11"/>
-      <c r="Z4" s="108"/>
+      <c r="Z4" s="107"/>
       <c r="AA4" s="11"/>
       <c r="AB4" s="11"/>
       <c r="AC4" s="11"/>
@@ -1845,27 +1851,27 @@
       <c r="AE4" s="11"/>
       <c r="AF4" s="11"/>
       <c r="AG4" s="11"/>
-      <c r="AH4" s="139"/>
-      <c r="AI4" s="140"/>
-      <c r="AJ4" s="140"/>
-      <c r="AK4" s="140"/>
-      <c r="AL4" s="140"/>
-      <c r="AM4" s="142"/>
-      <c r="AN4" s="154"/>
-      <c r="AO4" s="155"/>
-      <c r="AP4" s="155"/>
-      <c r="AQ4" s="154"/>
-      <c r="AR4" s="155"/>
-      <c r="AS4" s="160"/>
-      <c r="AT4" s="154"/>
-      <c r="AU4" s="155"/>
-      <c r="AV4" s="160"/>
+      <c r="AH4" s="153"/>
+      <c r="AI4" s="154"/>
+      <c r="AJ4" s="154"/>
+      <c r="AK4" s="154"/>
+      <c r="AL4" s="154"/>
+      <c r="AM4" s="155"/>
+      <c r="AN4" s="156"/>
+      <c r="AO4" s="157"/>
+      <c r="AP4" s="157"/>
+      <c r="AQ4" s="156"/>
+      <c r="AR4" s="157"/>
+      <c r="AS4" s="162"/>
+      <c r="AT4" s="156"/>
+      <c r="AU4" s="157"/>
+      <c r="AV4" s="162"/>
     </row>
     <row r="5" spans="1:48" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="107"/>
+      <c r="B5" s="106"/>
       <c r="C5" s="19"/>
       <c r="D5" s="20"/>
       <c r="E5" s="21"/>
@@ -1893,7 +1899,7 @@
       </c>
       <c r="X5" s="12"/>
       <c r="Y5" s="12"/>
-      <c r="Z5" s="108"/>
+      <c r="Z5" s="107"/>
       <c r="AA5" s="11"/>
       <c r="AB5" s="11"/>
       <c r="AC5" s="11"/>
@@ -1907,15 +1913,15 @@
       <c r="AK5" s="3"/>
       <c r="AL5" s="3"/>
       <c r="AM5" s="27"/>
-      <c r="AN5" s="156"/>
-      <c r="AO5" s="157"/>
-      <c r="AP5" s="157"/>
-      <c r="AQ5" s="156"/>
-      <c r="AR5" s="157"/>
-      <c r="AS5" s="161"/>
-      <c r="AT5" s="156"/>
-      <c r="AU5" s="157"/>
-      <c r="AV5" s="161"/>
+      <c r="AN5" s="158"/>
+      <c r="AO5" s="159"/>
+      <c r="AP5" s="159"/>
+      <c r="AQ5" s="158"/>
+      <c r="AR5" s="159"/>
+      <c r="AS5" s="163"/>
+      <c r="AT5" s="158"/>
+      <c r="AU5" s="159"/>
+      <c r="AV5" s="163"/>
     </row>
     <row r="6" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
@@ -1959,15 +1965,15 @@
       <c r="AK6" s="1"/>
       <c r="AL6" s="1"/>
       <c r="AM6" s="30"/>
-      <c r="AN6" s="156"/>
-      <c r="AO6" s="157"/>
-      <c r="AP6" s="157"/>
-      <c r="AQ6" s="156"/>
-      <c r="AR6" s="157"/>
-      <c r="AS6" s="161"/>
-      <c r="AT6" s="156"/>
-      <c r="AU6" s="157"/>
-      <c r="AV6" s="161"/>
+      <c r="AN6" s="158"/>
+      <c r="AO6" s="159"/>
+      <c r="AP6" s="159"/>
+      <c r="AQ6" s="158"/>
+      <c r="AR6" s="159"/>
+      <c r="AS6" s="163"/>
+      <c r="AT6" s="158"/>
+      <c r="AU6" s="159"/>
+      <c r="AV6" s="163"/>
     </row>
     <row r="7" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="31"/>
@@ -2009,66 +2015,66 @@
       <c r="AK7" s="32"/>
       <c r="AL7" s="32"/>
       <c r="AM7" s="33"/>
-      <c r="AN7" s="158"/>
-      <c r="AO7" s="159"/>
-      <c r="AP7" s="159"/>
-      <c r="AQ7" s="158"/>
-      <c r="AR7" s="159"/>
-      <c r="AS7" s="162"/>
-      <c r="AT7" s="158"/>
-      <c r="AU7" s="159"/>
-      <c r="AV7" s="162"/>
+      <c r="AN7" s="160"/>
+      <c r="AO7" s="161"/>
+      <c r="AP7" s="161"/>
+      <c r="AQ7" s="160"/>
+      <c r="AR7" s="161"/>
+      <c r="AS7" s="164"/>
+      <c r="AT7" s="160"/>
+      <c r="AU7" s="161"/>
+      <c r="AV7" s="164"/>
     </row>
     <row r="8" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="163" t="s">
+      <c r="B8" s="165" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="149"/>
-      <c r="D8" s="149"/>
-      <c r="E8" s="149"/>
-      <c r="F8" s="149"/>
-      <c r="G8" s="164" t="s">
+      <c r="C8" s="166"/>
+      <c r="D8" s="166"/>
+      <c r="E8" s="166"/>
+      <c r="F8" s="166"/>
+      <c r="G8" s="167" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="149"/>
-      <c r="I8" s="165"/>
-      <c r="J8" s="151" t="s">
+      <c r="H8" s="166"/>
+      <c r="I8" s="168"/>
+      <c r="J8" s="150" t="s">
         <v>21</v>
       </c>
-      <c r="K8" s="152"/>
-      <c r="L8" s="152"/>
-      <c r="M8" s="152"/>
-      <c r="N8" s="152"/>
-      <c r="O8" s="152"/>
-      <c r="P8" s="152"/>
-      <c r="Q8" s="152"/>
-      <c r="R8" s="152"/>
-      <c r="S8" s="152"/>
-      <c r="T8" s="152"/>
-      <c r="U8" s="152"/>
-      <c r="V8" s="152"/>
-      <c r="W8" s="152"/>
-      <c r="X8" s="152"/>
-      <c r="Y8" s="152"/>
-      <c r="Z8" s="152"/>
-      <c r="AA8" s="152"/>
-      <c r="AB8" s="152"/>
-      <c r="AC8" s="152"/>
-      <c r="AD8" s="152"/>
-      <c r="AE8" s="152"/>
-      <c r="AF8" s="152"/>
-      <c r="AG8" s="153"/>
-      <c r="AH8" s="151" t="s">
+      <c r="K8" s="151"/>
+      <c r="L8" s="151"/>
+      <c r="M8" s="151"/>
+      <c r="N8" s="151"/>
+      <c r="O8" s="151"/>
+      <c r="P8" s="151"/>
+      <c r="Q8" s="151"/>
+      <c r="R8" s="151"/>
+      <c r="S8" s="151"/>
+      <c r="T8" s="151"/>
+      <c r="U8" s="151"/>
+      <c r="V8" s="151"/>
+      <c r="W8" s="151"/>
+      <c r="X8" s="151"/>
+      <c r="Y8" s="151"/>
+      <c r="Z8" s="151"/>
+      <c r="AA8" s="151"/>
+      <c r="AB8" s="151"/>
+      <c r="AC8" s="151"/>
+      <c r="AD8" s="151"/>
+      <c r="AE8" s="151"/>
+      <c r="AF8" s="151"/>
+      <c r="AG8" s="152"/>
+      <c r="AH8" s="150" t="s">
         <v>22</v>
       </c>
-      <c r="AI8" s="152"/>
-      <c r="AJ8" s="152"/>
-      <c r="AK8" s="152"/>
-      <c r="AL8" s="152"/>
-      <c r="AM8" s="153"/>
+      <c r="AI8" s="151"/>
+      <c r="AJ8" s="151"/>
+      <c r="AK8" s="151"/>
+      <c r="AL8" s="151"/>
+      <c r="AM8" s="152"/>
       <c r="AN8" s="29" t="s">
         <v>23</v>
       </c>
@@ -2082,45 +2088,45 @@
       <c r="AV8" s="22"/>
     </row>
     <row r="9" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="109"/>
-      <c r="B9" s="139"/>
-      <c r="C9" s="140"/>
-      <c r="D9" s="140"/>
-      <c r="E9" s="140"/>
-      <c r="F9" s="140"/>
-      <c r="G9" s="141"/>
-      <c r="H9" s="140"/>
-      <c r="I9" s="142"/>
-      <c r="J9" s="143"/>
-      <c r="K9" s="144"/>
-      <c r="L9" s="144"/>
-      <c r="M9" s="144"/>
-      <c r="N9" s="144"/>
-      <c r="O9" s="144"/>
-      <c r="P9" s="144"/>
-      <c r="Q9" s="144"/>
-      <c r="R9" s="144"/>
-      <c r="S9" s="144"/>
-      <c r="T9" s="144"/>
-      <c r="U9" s="144"/>
-      <c r="V9" s="144"/>
-      <c r="W9" s="144"/>
-      <c r="X9" s="144"/>
-      <c r="Y9" s="144"/>
-      <c r="Z9" s="144"/>
-      <c r="AA9" s="144"/>
-      <c r="AB9" s="144"/>
-      <c r="AC9" s="144"/>
-      <c r="AD9" s="144"/>
-      <c r="AE9" s="144"/>
-      <c r="AF9" s="144"/>
-      <c r="AG9" s="145"/>
-      <c r="AH9" s="143"/>
-      <c r="AI9" s="144"/>
-      <c r="AJ9" s="144"/>
-      <c r="AK9" s="144"/>
-      <c r="AL9" s="144"/>
-      <c r="AM9" s="145"/>
+      <c r="A9" s="108"/>
+      <c r="B9" s="153"/>
+      <c r="C9" s="154"/>
+      <c r="D9" s="154"/>
+      <c r="E9" s="154"/>
+      <c r="F9" s="154"/>
+      <c r="G9" s="169"/>
+      <c r="H9" s="154"/>
+      <c r="I9" s="155"/>
+      <c r="J9" s="170"/>
+      <c r="K9" s="171"/>
+      <c r="L9" s="171"/>
+      <c r="M9" s="171"/>
+      <c r="N9" s="171"/>
+      <c r="O9" s="171"/>
+      <c r="P9" s="171"/>
+      <c r="Q9" s="171"/>
+      <c r="R9" s="171"/>
+      <c r="S9" s="171"/>
+      <c r="T9" s="171"/>
+      <c r="U9" s="171"/>
+      <c r="V9" s="171"/>
+      <c r="W9" s="171"/>
+      <c r="X9" s="171"/>
+      <c r="Y9" s="171"/>
+      <c r="Z9" s="171"/>
+      <c r="AA9" s="171"/>
+      <c r="AB9" s="171"/>
+      <c r="AC9" s="171"/>
+      <c r="AD9" s="171"/>
+      <c r="AE9" s="171"/>
+      <c r="AF9" s="171"/>
+      <c r="AG9" s="172"/>
+      <c r="AH9" s="170"/>
+      <c r="AI9" s="171"/>
+      <c r="AJ9" s="171"/>
+      <c r="AK9" s="171"/>
+      <c r="AL9" s="171"/>
+      <c r="AM9" s="172"/>
       <c r="AN9" s="35"/>
       <c r="AO9" s="2"/>
       <c r="AP9" s="2"/>
@@ -2132,45 +2138,45 @@
       <c r="AV9" s="22"/>
     </row>
     <row r="10" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="109"/>
-      <c r="B10" s="139"/>
-      <c r="C10" s="140"/>
-      <c r="D10" s="140"/>
-      <c r="E10" s="140"/>
-      <c r="F10" s="140"/>
-      <c r="G10" s="141"/>
-      <c r="H10" s="140"/>
-      <c r="I10" s="142"/>
-      <c r="J10" s="143"/>
-      <c r="K10" s="144"/>
-      <c r="L10" s="144"/>
-      <c r="M10" s="144"/>
-      <c r="N10" s="144"/>
-      <c r="O10" s="144"/>
-      <c r="P10" s="144"/>
-      <c r="Q10" s="144"/>
-      <c r="R10" s="144"/>
-      <c r="S10" s="144"/>
-      <c r="T10" s="144"/>
-      <c r="U10" s="144"/>
-      <c r="V10" s="144"/>
-      <c r="W10" s="144"/>
-      <c r="X10" s="144"/>
-      <c r="Y10" s="144"/>
-      <c r="Z10" s="144"/>
-      <c r="AA10" s="144"/>
-      <c r="AB10" s="144"/>
-      <c r="AC10" s="144"/>
-      <c r="AD10" s="144"/>
-      <c r="AE10" s="144"/>
-      <c r="AF10" s="144"/>
-      <c r="AG10" s="145"/>
-      <c r="AH10" s="143"/>
-      <c r="AI10" s="144"/>
-      <c r="AJ10" s="144"/>
-      <c r="AK10" s="144"/>
-      <c r="AL10" s="144"/>
-      <c r="AM10" s="145"/>
+      <c r="A10" s="108"/>
+      <c r="B10" s="153"/>
+      <c r="C10" s="154"/>
+      <c r="D10" s="154"/>
+      <c r="E10" s="154"/>
+      <c r="F10" s="154"/>
+      <c r="G10" s="169"/>
+      <c r="H10" s="154"/>
+      <c r="I10" s="155"/>
+      <c r="J10" s="170"/>
+      <c r="K10" s="171"/>
+      <c r="L10" s="171"/>
+      <c r="M10" s="171"/>
+      <c r="N10" s="171"/>
+      <c r="O10" s="171"/>
+      <c r="P10" s="171"/>
+      <c r="Q10" s="171"/>
+      <c r="R10" s="171"/>
+      <c r="S10" s="171"/>
+      <c r="T10" s="171"/>
+      <c r="U10" s="171"/>
+      <c r="V10" s="171"/>
+      <c r="W10" s="171"/>
+      <c r="X10" s="171"/>
+      <c r="Y10" s="171"/>
+      <c r="Z10" s="171"/>
+      <c r="AA10" s="171"/>
+      <c r="AB10" s="171"/>
+      <c r="AC10" s="171"/>
+      <c r="AD10" s="171"/>
+      <c r="AE10" s="171"/>
+      <c r="AF10" s="171"/>
+      <c r="AG10" s="172"/>
+      <c r="AH10" s="170"/>
+      <c r="AI10" s="171"/>
+      <c r="AJ10" s="171"/>
+      <c r="AK10" s="171"/>
+      <c r="AL10" s="171"/>
+      <c r="AM10" s="172"/>
       <c r="AN10" s="35"/>
       <c r="AO10" s="2"/>
       <c r="AP10" s="2"/>
@@ -2182,45 +2188,45 @@
       <c r="AV10" s="22"/>
     </row>
     <row r="11" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="109"/>
-      <c r="B11" s="139"/>
-      <c r="C11" s="140"/>
-      <c r="D11" s="140"/>
-      <c r="E11" s="140"/>
-      <c r="F11" s="140"/>
-      <c r="G11" s="141"/>
-      <c r="H11" s="140"/>
-      <c r="I11" s="142"/>
-      <c r="J11" s="143"/>
-      <c r="K11" s="144"/>
-      <c r="L11" s="144"/>
-      <c r="M11" s="144"/>
-      <c r="N11" s="144"/>
-      <c r="O11" s="144"/>
-      <c r="P11" s="144"/>
-      <c r="Q11" s="144"/>
-      <c r="R11" s="144"/>
-      <c r="S11" s="144"/>
-      <c r="T11" s="144"/>
-      <c r="U11" s="144"/>
-      <c r="V11" s="144"/>
-      <c r="W11" s="144"/>
-      <c r="X11" s="144"/>
-      <c r="Y11" s="144"/>
-      <c r="Z11" s="144"/>
-      <c r="AA11" s="144"/>
-      <c r="AB11" s="144"/>
-      <c r="AC11" s="144"/>
-      <c r="AD11" s="144"/>
-      <c r="AE11" s="144"/>
-      <c r="AF11" s="144"/>
-      <c r="AG11" s="145"/>
-      <c r="AH11" s="143"/>
-      <c r="AI11" s="144"/>
-      <c r="AJ11" s="144"/>
-      <c r="AK11" s="144"/>
-      <c r="AL11" s="144"/>
-      <c r="AM11" s="145"/>
+      <c r="A11" s="108"/>
+      <c r="B11" s="153"/>
+      <c r="C11" s="154"/>
+      <c r="D11" s="154"/>
+      <c r="E11" s="154"/>
+      <c r="F11" s="154"/>
+      <c r="G11" s="169"/>
+      <c r="H11" s="154"/>
+      <c r="I11" s="155"/>
+      <c r="J11" s="170"/>
+      <c r="K11" s="171"/>
+      <c r="L11" s="171"/>
+      <c r="M11" s="171"/>
+      <c r="N11" s="171"/>
+      <c r="O11" s="171"/>
+      <c r="P11" s="171"/>
+      <c r="Q11" s="171"/>
+      <c r="R11" s="171"/>
+      <c r="S11" s="171"/>
+      <c r="T11" s="171"/>
+      <c r="U11" s="171"/>
+      <c r="V11" s="171"/>
+      <c r="W11" s="171"/>
+      <c r="X11" s="171"/>
+      <c r="Y11" s="171"/>
+      <c r="Z11" s="171"/>
+      <c r="AA11" s="171"/>
+      <c r="AB11" s="171"/>
+      <c r="AC11" s="171"/>
+      <c r="AD11" s="171"/>
+      <c r="AE11" s="171"/>
+      <c r="AF11" s="171"/>
+      <c r="AG11" s="172"/>
+      <c r="AH11" s="170"/>
+      <c r="AI11" s="171"/>
+      <c r="AJ11" s="171"/>
+      <c r="AK11" s="171"/>
+      <c r="AL11" s="171"/>
+      <c r="AM11" s="172"/>
       <c r="AN11" s="18" t="s">
         <v>24</v>
       </c>
@@ -2234,45 +2240,45 @@
       <c r="AV11" s="36"/>
     </row>
     <row r="12" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="109"/>
-      <c r="B12" s="139"/>
-      <c r="C12" s="140"/>
-      <c r="D12" s="140"/>
-      <c r="E12" s="140"/>
-      <c r="F12" s="140"/>
-      <c r="G12" s="141"/>
-      <c r="H12" s="140"/>
-      <c r="I12" s="142"/>
-      <c r="J12" s="143"/>
-      <c r="K12" s="144"/>
-      <c r="L12" s="144"/>
-      <c r="M12" s="144"/>
-      <c r="N12" s="144"/>
-      <c r="O12" s="144"/>
-      <c r="P12" s="144"/>
-      <c r="Q12" s="144"/>
-      <c r="R12" s="144"/>
-      <c r="S12" s="144"/>
-      <c r="T12" s="144"/>
-      <c r="U12" s="144"/>
-      <c r="V12" s="144"/>
-      <c r="W12" s="144"/>
-      <c r="X12" s="144"/>
-      <c r="Y12" s="144"/>
-      <c r="Z12" s="144"/>
-      <c r="AA12" s="144"/>
-      <c r="AB12" s="144"/>
-      <c r="AC12" s="144"/>
-      <c r="AD12" s="144"/>
-      <c r="AE12" s="144"/>
-      <c r="AF12" s="144"/>
-      <c r="AG12" s="145"/>
-      <c r="AH12" s="143"/>
-      <c r="AI12" s="144"/>
-      <c r="AJ12" s="144"/>
-      <c r="AK12" s="144"/>
-      <c r="AL12" s="144"/>
-      <c r="AM12" s="145"/>
+      <c r="A12" s="108"/>
+      <c r="B12" s="153"/>
+      <c r="C12" s="154"/>
+      <c r="D12" s="154"/>
+      <c r="E12" s="154"/>
+      <c r="F12" s="154"/>
+      <c r="G12" s="169"/>
+      <c r="H12" s="154"/>
+      <c r="I12" s="155"/>
+      <c r="J12" s="170"/>
+      <c r="K12" s="171"/>
+      <c r="L12" s="171"/>
+      <c r="M12" s="171"/>
+      <c r="N12" s="171"/>
+      <c r="O12" s="171"/>
+      <c r="P12" s="171"/>
+      <c r="Q12" s="171"/>
+      <c r="R12" s="171"/>
+      <c r="S12" s="171"/>
+      <c r="T12" s="171"/>
+      <c r="U12" s="171"/>
+      <c r="V12" s="171"/>
+      <c r="W12" s="171"/>
+      <c r="X12" s="171"/>
+      <c r="Y12" s="171"/>
+      <c r="Z12" s="171"/>
+      <c r="AA12" s="171"/>
+      <c r="AB12" s="171"/>
+      <c r="AC12" s="171"/>
+      <c r="AD12" s="171"/>
+      <c r="AE12" s="171"/>
+      <c r="AF12" s="171"/>
+      <c r="AG12" s="172"/>
+      <c r="AH12" s="170"/>
+      <c r="AI12" s="171"/>
+      <c r="AJ12" s="171"/>
+      <c r="AK12" s="171"/>
+      <c r="AL12" s="171"/>
+      <c r="AM12" s="172"/>
       <c r="AN12" s="35"/>
       <c r="AO12" s="2"/>
       <c r="AP12" s="2"/>
@@ -2284,45 +2290,45 @@
       <c r="AV12" s="22"/>
     </row>
     <row r="13" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="109"/>
-      <c r="B13" s="139"/>
-      <c r="C13" s="140"/>
-      <c r="D13" s="140"/>
-      <c r="E13" s="140"/>
-      <c r="F13" s="140"/>
-      <c r="G13" s="141"/>
-      <c r="H13" s="140"/>
-      <c r="I13" s="142"/>
-      <c r="J13" s="143"/>
-      <c r="K13" s="144"/>
-      <c r="L13" s="144"/>
-      <c r="M13" s="144"/>
-      <c r="N13" s="144"/>
-      <c r="O13" s="144"/>
-      <c r="P13" s="144"/>
-      <c r="Q13" s="144"/>
-      <c r="R13" s="144"/>
-      <c r="S13" s="144"/>
-      <c r="T13" s="144"/>
-      <c r="U13" s="144"/>
-      <c r="V13" s="144"/>
-      <c r="W13" s="144"/>
-      <c r="X13" s="144"/>
-      <c r="Y13" s="144"/>
-      <c r="Z13" s="144"/>
-      <c r="AA13" s="144"/>
-      <c r="AB13" s="144"/>
-      <c r="AC13" s="144"/>
-      <c r="AD13" s="144"/>
-      <c r="AE13" s="144"/>
-      <c r="AF13" s="144"/>
-      <c r="AG13" s="145"/>
-      <c r="AH13" s="143"/>
-      <c r="AI13" s="144"/>
-      <c r="AJ13" s="144"/>
-      <c r="AK13" s="144"/>
-      <c r="AL13" s="144"/>
-      <c r="AM13" s="145"/>
+      <c r="A13" s="108"/>
+      <c r="B13" s="153"/>
+      <c r="C13" s="154"/>
+      <c r="D13" s="154"/>
+      <c r="E13" s="154"/>
+      <c r="F13" s="154"/>
+      <c r="G13" s="169"/>
+      <c r="H13" s="154"/>
+      <c r="I13" s="155"/>
+      <c r="J13" s="170"/>
+      <c r="K13" s="171"/>
+      <c r="L13" s="171"/>
+      <c r="M13" s="171"/>
+      <c r="N13" s="171"/>
+      <c r="O13" s="171"/>
+      <c r="P13" s="171"/>
+      <c r="Q13" s="171"/>
+      <c r="R13" s="171"/>
+      <c r="S13" s="171"/>
+      <c r="T13" s="171"/>
+      <c r="U13" s="171"/>
+      <c r="V13" s="171"/>
+      <c r="W13" s="171"/>
+      <c r="X13" s="171"/>
+      <c r="Y13" s="171"/>
+      <c r="Z13" s="171"/>
+      <c r="AA13" s="171"/>
+      <c r="AB13" s="171"/>
+      <c r="AC13" s="171"/>
+      <c r="AD13" s="171"/>
+      <c r="AE13" s="171"/>
+      <c r="AF13" s="171"/>
+      <c r="AG13" s="172"/>
+      <c r="AH13" s="170"/>
+      <c r="AI13" s="171"/>
+      <c r="AJ13" s="171"/>
+      <c r="AK13" s="171"/>
+      <c r="AL13" s="171"/>
+      <c r="AM13" s="172"/>
       <c r="AN13" s="23"/>
       <c r="AO13" s="37"/>
       <c r="AP13" s="37"/>
@@ -2334,47 +2340,47 @@
       <c r="AV13" s="38"/>
     </row>
     <row r="14" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="146" t="s">
+      <c r="A14" s="173" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="147"/>
-      <c r="C14" s="147"/>
-      <c r="D14" s="147"/>
-      <c r="E14" s="147"/>
-      <c r="F14" s="147"/>
-      <c r="G14" s="147"/>
-      <c r="H14" s="147"/>
-      <c r="I14" s="147"/>
-      <c r="J14" s="147"/>
-      <c r="K14" s="147"/>
-      <c r="L14" s="147"/>
-      <c r="M14" s="147"/>
-      <c r="N14" s="147"/>
-      <c r="O14" s="147"/>
-      <c r="P14" s="147"/>
-      <c r="Q14" s="147"/>
-      <c r="R14" s="147"/>
-      <c r="S14" s="147"/>
-      <c r="T14" s="147"/>
-      <c r="U14" s="147"/>
-      <c r="V14" s="147"/>
-      <c r="W14" s="147"/>
-      <c r="X14" s="147"/>
-      <c r="Y14" s="147"/>
-      <c r="Z14" s="147"/>
-      <c r="AA14" s="147"/>
-      <c r="AB14" s="147"/>
-      <c r="AC14" s="147"/>
-      <c r="AD14" s="147"/>
-      <c r="AE14" s="147"/>
-      <c r="AF14" s="147"/>
-      <c r="AG14" s="147"/>
-      <c r="AH14" s="147"/>
-      <c r="AI14" s="147"/>
-      <c r="AJ14" s="147"/>
-      <c r="AK14" s="147"/>
-      <c r="AL14" s="147"/>
-      <c r="AM14" s="138"/>
+      <c r="B14" s="174"/>
+      <c r="C14" s="174"/>
+      <c r="D14" s="174"/>
+      <c r="E14" s="174"/>
+      <c r="F14" s="174"/>
+      <c r="G14" s="174"/>
+      <c r="H14" s="174"/>
+      <c r="I14" s="174"/>
+      <c r="J14" s="174"/>
+      <c r="K14" s="174"/>
+      <c r="L14" s="174"/>
+      <c r="M14" s="174"/>
+      <c r="N14" s="174"/>
+      <c r="O14" s="174"/>
+      <c r="P14" s="174"/>
+      <c r="Q14" s="174"/>
+      <c r="R14" s="174"/>
+      <c r="S14" s="174"/>
+      <c r="T14" s="174"/>
+      <c r="U14" s="174"/>
+      <c r="V14" s="174"/>
+      <c r="W14" s="174"/>
+      <c r="X14" s="174"/>
+      <c r="Y14" s="174"/>
+      <c r="Z14" s="174"/>
+      <c r="AA14" s="174"/>
+      <c r="AB14" s="174"/>
+      <c r="AC14" s="174"/>
+      <c r="AD14" s="174"/>
+      <c r="AE14" s="174"/>
+      <c r="AF14" s="174"/>
+      <c r="AG14" s="174"/>
+      <c r="AH14" s="174"/>
+      <c r="AI14" s="174"/>
+      <c r="AJ14" s="174"/>
+      <c r="AK14" s="174"/>
+      <c r="AL14" s="174"/>
+      <c r="AM14" s="175"/>
       <c r="AN14" s="39"/>
       <c r="AO14" s="21"/>
       <c r="AP14" s="21"/>
@@ -2386,104 +2392,104 @@
       <c r="AV14" s="36"/>
     </row>
     <row r="15" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="148"/>
-      <c r="B15" s="149"/>
-      <c r="C15" s="149"/>
-      <c r="D15" s="149"/>
-      <c r="E15" s="149"/>
-      <c r="F15" s="149"/>
-      <c r="G15" s="149"/>
-      <c r="H15" s="149"/>
-      <c r="I15" s="149"/>
-      <c r="J15" s="150"/>
-      <c r="K15" s="150"/>
-      <c r="L15" s="150"/>
-      <c r="M15" s="150"/>
-      <c r="N15" s="150"/>
-      <c r="O15" s="150"/>
-      <c r="P15" s="150"/>
-      <c r="Q15" s="150"/>
-      <c r="R15" s="150"/>
-      <c r="S15" s="150"/>
-      <c r="T15" s="150"/>
-      <c r="U15" s="150"/>
-      <c r="V15" s="150"/>
-      <c r="W15" s="150"/>
-      <c r="X15" s="150"/>
-      <c r="Y15" s="150"/>
-      <c r="Z15" s="150"/>
-      <c r="AA15" s="150"/>
-      <c r="AB15" s="150"/>
-      <c r="AC15" s="150"/>
-      <c r="AD15" s="150"/>
-      <c r="AE15" s="150"/>
-      <c r="AF15" s="150"/>
-      <c r="AG15" s="150"/>
-      <c r="AH15" s="150"/>
-      <c r="AI15" s="150"/>
-      <c r="AJ15" s="150"/>
-      <c r="AK15" s="150"/>
-      <c r="AL15" s="150"/>
-      <c r="AM15" s="138"/>
-      <c r="AN15" s="136"/>
-      <c r="AO15" s="137"/>
-      <c r="AP15" s="137"/>
-      <c r="AQ15" s="137"/>
-      <c r="AR15" s="137"/>
-      <c r="AS15" s="137"/>
-      <c r="AT15" s="137"/>
-      <c r="AU15" s="137"/>
-      <c r="AV15" s="138"/>
+      <c r="A15" s="176"/>
+      <c r="B15" s="166"/>
+      <c r="C15" s="166"/>
+      <c r="D15" s="166"/>
+      <c r="E15" s="166"/>
+      <c r="F15" s="166"/>
+      <c r="G15" s="166"/>
+      <c r="H15" s="166"/>
+      <c r="I15" s="166"/>
+      <c r="J15" s="177"/>
+      <c r="K15" s="177"/>
+      <c r="L15" s="177"/>
+      <c r="M15" s="177"/>
+      <c r="N15" s="177"/>
+      <c r="O15" s="177"/>
+      <c r="P15" s="177"/>
+      <c r="Q15" s="177"/>
+      <c r="R15" s="177"/>
+      <c r="S15" s="177"/>
+      <c r="T15" s="177"/>
+      <c r="U15" s="177"/>
+      <c r="V15" s="177"/>
+      <c r="W15" s="177"/>
+      <c r="X15" s="177"/>
+      <c r="Y15" s="177"/>
+      <c r="Z15" s="177"/>
+      <c r="AA15" s="177"/>
+      <c r="AB15" s="177"/>
+      <c r="AC15" s="177"/>
+      <c r="AD15" s="177"/>
+      <c r="AE15" s="177"/>
+      <c r="AF15" s="177"/>
+      <c r="AG15" s="177"/>
+      <c r="AH15" s="177"/>
+      <c r="AI15" s="177"/>
+      <c r="AJ15" s="177"/>
+      <c r="AK15" s="177"/>
+      <c r="AL15" s="177"/>
+      <c r="AM15" s="175"/>
+      <c r="AN15" s="178"/>
+      <c r="AO15" s="179"/>
+      <c r="AP15" s="179"/>
+      <c r="AQ15" s="179"/>
+      <c r="AR15" s="179"/>
+      <c r="AS15" s="179"/>
+      <c r="AT15" s="179"/>
+      <c r="AU15" s="179"/>
+      <c r="AV15" s="175"/>
     </row>
     <row r="16" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="110"/>
+      <c r="A16" s="109"/>
       <c r="B16" s="83"/>
       <c r="C16" s="83"/>
-      <c r="D16" s="118"/>
-      <c r="E16" s="84"/>
+      <c r="D16" s="117"/>
+      <c r="E16" s="117"/>
       <c r="F16" s="84"/>
       <c r="G16" s="84"/>
-      <c r="H16" s="169"/>
-      <c r="I16" s="118"/>
+      <c r="H16" s="126"/>
+      <c r="I16" s="117"/>
       <c r="J16" s="63"/>
       <c r="K16" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="L16" s="133"/>
-      <c r="M16" s="134"/>
-      <c r="N16" s="134"/>
+      <c r="L16" s="142"/>
+      <c r="M16" s="143"/>
+      <c r="N16" s="143"/>
       <c r="O16" s="65"/>
       <c r="P16" s="66"/>
       <c r="Q16" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="R16" s="133"/>
-      <c r="S16" s="134"/>
-      <c r="T16" s="134"/>
+      <c r="R16" s="142"/>
+      <c r="S16" s="143"/>
+      <c r="T16" s="143"/>
       <c r="U16" s="65"/>
       <c r="V16" s="66"/>
       <c r="W16" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="X16" s="133"/>
-      <c r="Y16" s="134"/>
-      <c r="Z16" s="134"/>
+      <c r="X16" s="142"/>
+      <c r="Y16" s="143"/>
+      <c r="Z16" s="143"/>
       <c r="AA16" s="65"/>
       <c r="AB16" s="68"/>
       <c r="AC16" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="AD16" s="133"/>
-      <c r="AE16" s="134"/>
-      <c r="AF16" s="134"/>
+      <c r="AD16" s="142"/>
+      <c r="AE16" s="143"/>
+      <c r="AF16" s="143"/>
       <c r="AG16" s="65"/>
       <c r="AH16" s="68"/>
       <c r="AI16" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="AJ16" s="133"/>
-      <c r="AK16" s="134"/>
-      <c r="AL16" s="134"/>
+      <c r="AJ16" s="142"/>
+      <c r="AK16" s="143"/>
+      <c r="AL16" s="143"/>
       <c r="AM16" s="69"/>
       <c r="AN16" s="61"/>
       <c r="AO16" s="2"/>
@@ -2496,15 +2502,15 @@
       <c r="AV16" s="22"/>
     </row>
     <row r="17" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="111"/>
-      <c r="B17" s="172"/>
+      <c r="A17" s="110"/>
+      <c r="B17" s="129"/>
       <c r="C17" s="85"/>
-      <c r="D17" s="119"/>
-      <c r="E17" s="85"/>
+      <c r="D17" s="118"/>
+      <c r="E17" s="118"/>
       <c r="F17" s="85"/>
       <c r="G17" s="85"/>
-      <c r="H17" s="170"/>
-      <c r="I17" s="119"/>
+      <c r="H17" s="127"/>
+      <c r="I17" s="118"/>
       <c r="J17" s="70"/>
       <c r="K17" s="71"/>
       <c r="L17" s="72"/>
@@ -2546,44 +2552,44 @@
       <c r="AV17" s="22"/>
     </row>
     <row r="18" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="112"/>
-      <c r="B18" s="173"/>
+      <c r="A18" s="111"/>
+      <c r="B18" s="130"/>
       <c r="C18" s="86"/>
-      <c r="D18" s="175"/>
-      <c r="E18" s="86"/>
+      <c r="D18" s="132"/>
+      <c r="E18" s="132"/>
       <c r="F18" s="86"/>
-      <c r="G18" s="168"/>
-      <c r="H18" s="178"/>
-      <c r="I18" s="120"/>
+      <c r="G18" s="125"/>
+      <c r="H18" s="135"/>
+      <c r="I18" s="119"/>
       <c r="J18" s="74"/>
-      <c r="K18" s="132"/>
-      <c r="L18" s="132"/>
-      <c r="M18" s="132"/>
-      <c r="N18" s="132"/>
+      <c r="K18" s="147"/>
+      <c r="L18" s="147"/>
+      <c r="M18" s="147"/>
+      <c r="N18" s="147"/>
       <c r="O18" s="43"/>
       <c r="P18" s="72"/>
-      <c r="Q18" s="132"/>
-      <c r="R18" s="132"/>
-      <c r="S18" s="132"/>
-      <c r="T18" s="132"/>
+      <c r="Q18" s="147"/>
+      <c r="R18" s="147"/>
+      <c r="S18" s="147"/>
+      <c r="T18" s="147"/>
       <c r="U18" s="43"/>
       <c r="V18" s="72"/>
-      <c r="W18" s="132"/>
-      <c r="X18" s="132"/>
-      <c r="Y18" s="132"/>
-      <c r="Z18" s="132"/>
+      <c r="W18" s="147"/>
+      <c r="X18" s="147"/>
+      <c r="Y18" s="147"/>
+      <c r="Z18" s="147"/>
       <c r="AA18" s="43"/>
       <c r="AB18" s="72"/>
-      <c r="AC18" s="132"/>
-      <c r="AD18" s="132"/>
-      <c r="AE18" s="132"/>
-      <c r="AF18" s="132"/>
+      <c r="AC18" s="147"/>
+      <c r="AD18" s="147"/>
+      <c r="AE18" s="147"/>
+      <c r="AF18" s="147"/>
       <c r="AG18" s="43"/>
       <c r="AH18" s="72"/>
-      <c r="AI18" s="132"/>
-      <c r="AJ18" s="132"/>
-      <c r="AK18" s="132"/>
-      <c r="AL18" s="132"/>
+      <c r="AI18" s="147"/>
+      <c r="AJ18" s="147"/>
+      <c r="AK18" s="147"/>
+      <c r="AL18" s="147"/>
       <c r="AM18" s="73"/>
       <c r="AN18" s="61"/>
       <c r="AO18" s="2"/>
@@ -2596,44 +2602,44 @@
       <c r="AV18" s="22"/>
     </row>
     <row r="19" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="112"/>
-      <c r="B19" s="173"/>
+      <c r="A19" s="111"/>
+      <c r="B19" s="130"/>
       <c r="C19" s="86"/>
-      <c r="D19" s="175"/>
-      <c r="E19" s="86"/>
+      <c r="D19" s="132"/>
+      <c r="E19" s="132"/>
       <c r="F19" s="86"/>
       <c r="G19" s="88"/>
       <c r="H19" s="87"/>
-      <c r="I19" s="120"/>
+      <c r="I19" s="119"/>
       <c r="J19" s="70"/>
-      <c r="K19" s="132"/>
-      <c r="L19" s="132"/>
-      <c r="M19" s="132"/>
-      <c r="N19" s="132"/>
+      <c r="K19" s="147"/>
+      <c r="L19" s="147"/>
+      <c r="M19" s="147"/>
+      <c r="N19" s="147"/>
       <c r="O19" s="43"/>
       <c r="P19" s="72"/>
-      <c r="Q19" s="132"/>
-      <c r="R19" s="132"/>
-      <c r="S19" s="132"/>
-      <c r="T19" s="132"/>
+      <c r="Q19" s="147"/>
+      <c r="R19" s="147"/>
+      <c r="S19" s="147"/>
+      <c r="T19" s="147"/>
       <c r="U19" s="43"/>
       <c r="V19" s="72"/>
-      <c r="W19" s="132"/>
-      <c r="X19" s="132"/>
-      <c r="Y19" s="132"/>
-      <c r="Z19" s="132"/>
+      <c r="W19" s="147"/>
+      <c r="X19" s="147"/>
+      <c r="Y19" s="147"/>
+      <c r="Z19" s="147"/>
       <c r="AA19" s="43"/>
       <c r="AB19" s="72"/>
-      <c r="AC19" s="132"/>
-      <c r="AD19" s="132"/>
-      <c r="AE19" s="132"/>
-      <c r="AF19" s="132"/>
+      <c r="AC19" s="147"/>
+      <c r="AD19" s="147"/>
+      <c r="AE19" s="147"/>
+      <c r="AF19" s="147"/>
       <c r="AG19" s="43"/>
       <c r="AH19" s="72"/>
-      <c r="AI19" s="132"/>
-      <c r="AJ19" s="132"/>
-      <c r="AK19" s="132"/>
-      <c r="AL19" s="132"/>
+      <c r="AI19" s="147"/>
+      <c r="AJ19" s="147"/>
+      <c r="AK19" s="147"/>
+      <c r="AL19" s="147"/>
       <c r="AM19" s="73"/>
       <c r="AN19" s="61"/>
       <c r="AO19" s="2"/>
@@ -2646,44 +2652,44 @@
       <c r="AV19" s="22"/>
     </row>
     <row r="20" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="112"/>
-      <c r="B20" s="173"/>
+      <c r="A20" s="111"/>
+      <c r="B20" s="130"/>
       <c r="C20" s="86"/>
-      <c r="D20" s="175"/>
-      <c r="E20" s="86"/>
+      <c r="D20" s="132"/>
+      <c r="E20" s="132"/>
       <c r="F20" s="86"/>
       <c r="G20" s="88"/>
       <c r="H20" s="87"/>
-      <c r="I20" s="120"/>
+      <c r="I20" s="119"/>
       <c r="J20" s="74"/>
-      <c r="K20" s="132"/>
-      <c r="L20" s="132"/>
-      <c r="M20" s="132"/>
-      <c r="N20" s="132"/>
+      <c r="K20" s="147"/>
+      <c r="L20" s="147"/>
+      <c r="M20" s="147"/>
+      <c r="N20" s="147"/>
       <c r="O20" s="43"/>
       <c r="P20" s="72"/>
-      <c r="Q20" s="132"/>
-      <c r="R20" s="132"/>
-      <c r="S20" s="132"/>
-      <c r="T20" s="132"/>
+      <c r="Q20" s="147"/>
+      <c r="R20" s="147"/>
+      <c r="S20" s="147"/>
+      <c r="T20" s="147"/>
       <c r="U20" s="43"/>
       <c r="V20" s="72"/>
-      <c r="W20" s="132"/>
-      <c r="X20" s="132"/>
-      <c r="Y20" s="132"/>
-      <c r="Z20" s="132"/>
+      <c r="W20" s="147"/>
+      <c r="X20" s="147"/>
+      <c r="Y20" s="147"/>
+      <c r="Z20" s="147"/>
       <c r="AA20" s="43"/>
       <c r="AB20" s="72"/>
-      <c r="AC20" s="132"/>
-      <c r="AD20" s="132"/>
-      <c r="AE20" s="132"/>
-      <c r="AF20" s="132"/>
+      <c r="AC20" s="147"/>
+      <c r="AD20" s="147"/>
+      <c r="AE20" s="147"/>
+      <c r="AF20" s="147"/>
       <c r="AG20" s="43"/>
       <c r="AH20" s="72"/>
-      <c r="AI20" s="132"/>
-      <c r="AJ20" s="132"/>
-      <c r="AK20" s="132"/>
-      <c r="AL20" s="132"/>
+      <c r="AI20" s="147"/>
+      <c r="AJ20" s="147"/>
+      <c r="AK20" s="147"/>
+      <c r="AL20" s="147"/>
       <c r="AM20" s="73"/>
       <c r="AN20" s="61"/>
       <c r="AO20" s="2"/>
@@ -2696,44 +2702,44 @@
       <c r="AV20" s="22"/>
     </row>
     <row r="21" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="110"/>
+      <c r="A21" s="109"/>
       <c r="B21" s="83"/>
       <c r="C21" s="89"/>
-      <c r="D21" s="121"/>
-      <c r="E21" s="89"/>
+      <c r="D21" s="120"/>
+      <c r="E21" s="120"/>
       <c r="F21" s="89"/>
       <c r="G21" s="89"/>
-      <c r="H21" s="171"/>
-      <c r="I21" s="121"/>
+      <c r="H21" s="128"/>
+      <c r="I21" s="120"/>
       <c r="J21" s="74"/>
-      <c r="K21" s="132"/>
-      <c r="L21" s="132"/>
-      <c r="M21" s="132"/>
-      <c r="N21" s="132"/>
+      <c r="K21" s="147"/>
+      <c r="L21" s="147"/>
+      <c r="M21" s="147"/>
+      <c r="N21" s="147"/>
       <c r="O21" s="43"/>
       <c r="P21" s="72"/>
-      <c r="Q21" s="132"/>
-      <c r="R21" s="132"/>
-      <c r="S21" s="132"/>
-      <c r="T21" s="132"/>
+      <c r="Q21" s="147"/>
+      <c r="R21" s="147"/>
+      <c r="S21" s="147"/>
+      <c r="T21" s="147"/>
       <c r="U21" s="43"/>
       <c r="V21" s="72"/>
-      <c r="W21" s="132"/>
-      <c r="X21" s="132"/>
-      <c r="Y21" s="132"/>
-      <c r="Z21" s="132"/>
+      <c r="W21" s="147"/>
+      <c r="X21" s="147"/>
+      <c r="Y21" s="147"/>
+      <c r="Z21" s="147"/>
       <c r="AA21" s="43"/>
       <c r="AB21" s="72"/>
-      <c r="AC21" s="132"/>
-      <c r="AD21" s="132"/>
-      <c r="AE21" s="132"/>
-      <c r="AF21" s="132"/>
+      <c r="AC21" s="147"/>
+      <c r="AD21" s="147"/>
+      <c r="AE21" s="147"/>
+      <c r="AF21" s="147"/>
       <c r="AG21" s="43"/>
       <c r="AH21" s="72"/>
-      <c r="AI21" s="132"/>
-      <c r="AJ21" s="132"/>
-      <c r="AK21" s="132"/>
-      <c r="AL21" s="132"/>
+      <c r="AI21" s="147"/>
+      <c r="AJ21" s="147"/>
+      <c r="AK21" s="147"/>
+      <c r="AL21" s="147"/>
       <c r="AM21" s="73"/>
       <c r="AN21" s="61"/>
       <c r="AO21" s="2"/>
@@ -2746,44 +2752,44 @@
       <c r="AV21" s="22"/>
     </row>
     <row r="22" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="112"/>
-      <c r="B22" s="173"/>
+      <c r="A22" s="111"/>
+      <c r="B22" s="130"/>
       <c r="C22" s="86"/>
-      <c r="D22" s="175"/>
-      <c r="E22" s="86"/>
+      <c r="D22" s="132"/>
+      <c r="E22" s="132"/>
       <c r="F22" s="86"/>
       <c r="G22" s="88"/>
       <c r="H22" s="87"/>
-      <c r="I22" s="120"/>
+      <c r="I22" s="119"/>
       <c r="J22" s="74"/>
-      <c r="K22" s="132"/>
-      <c r="L22" s="132"/>
-      <c r="M22" s="132"/>
-      <c r="N22" s="132"/>
+      <c r="K22" s="147"/>
+      <c r="L22" s="147"/>
+      <c r="M22" s="147"/>
+      <c r="N22" s="147"/>
       <c r="O22" s="43"/>
       <c r="P22" s="72"/>
-      <c r="Q22" s="132"/>
-      <c r="R22" s="132"/>
-      <c r="S22" s="132"/>
-      <c r="T22" s="132"/>
+      <c r="Q22" s="147"/>
+      <c r="R22" s="147"/>
+      <c r="S22" s="147"/>
+      <c r="T22" s="147"/>
       <c r="U22" s="43"/>
       <c r="V22" s="72"/>
-      <c r="W22" s="132"/>
-      <c r="X22" s="132"/>
-      <c r="Y22" s="132"/>
-      <c r="Z22" s="132"/>
+      <c r="W22" s="147"/>
+      <c r="X22" s="147"/>
+      <c r="Y22" s="147"/>
+      <c r="Z22" s="147"/>
       <c r="AA22" s="43"/>
       <c r="AB22" s="72"/>
-      <c r="AC22" s="132"/>
-      <c r="AD22" s="132"/>
-      <c r="AE22" s="132"/>
-      <c r="AF22" s="132"/>
+      <c r="AC22" s="147"/>
+      <c r="AD22" s="147"/>
+      <c r="AE22" s="147"/>
+      <c r="AF22" s="147"/>
       <c r="AG22" s="43"/>
       <c r="AH22" s="72"/>
-      <c r="AI22" s="132"/>
-      <c r="AJ22" s="132"/>
-      <c r="AK22" s="132"/>
-      <c r="AL22" s="132"/>
+      <c r="AI22" s="147"/>
+      <c r="AJ22" s="147"/>
+      <c r="AK22" s="147"/>
+      <c r="AL22" s="147"/>
       <c r="AM22" s="73"/>
       <c r="AN22" s="61"/>
       <c r="AO22" s="2"/>
@@ -2796,44 +2802,44 @@
       <c r="AV22" s="22"/>
     </row>
     <row r="23" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="112"/>
-      <c r="B23" s="173"/>
+      <c r="A23" s="111"/>
+      <c r="B23" s="130"/>
       <c r="C23" s="86"/>
-      <c r="D23" s="175"/>
-      <c r="E23" s="86"/>
+      <c r="D23" s="132"/>
+      <c r="E23" s="132"/>
       <c r="F23" s="86"/>
       <c r="G23" s="88"/>
       <c r="H23" s="87"/>
-      <c r="I23" s="120"/>
+      <c r="I23" s="119"/>
       <c r="J23" s="70"/>
-      <c r="K23" s="132"/>
-      <c r="L23" s="132"/>
-      <c r="M23" s="132"/>
-      <c r="N23" s="132"/>
+      <c r="K23" s="147"/>
+      <c r="L23" s="147"/>
+      <c r="M23" s="147"/>
+      <c r="N23" s="147"/>
       <c r="O23" s="43"/>
       <c r="P23" s="72"/>
-      <c r="Q23" s="132"/>
-      <c r="R23" s="132"/>
-      <c r="S23" s="132"/>
-      <c r="T23" s="132"/>
+      <c r="Q23" s="147"/>
+      <c r="R23" s="147"/>
+      <c r="S23" s="147"/>
+      <c r="T23" s="147"/>
       <c r="U23" s="43"/>
       <c r="V23" s="72"/>
-      <c r="W23" s="132"/>
-      <c r="X23" s="132"/>
-      <c r="Y23" s="132"/>
-      <c r="Z23" s="132"/>
+      <c r="W23" s="147"/>
+      <c r="X23" s="147"/>
+      <c r="Y23" s="147"/>
+      <c r="Z23" s="147"/>
       <c r="AA23" s="43"/>
       <c r="AB23" s="72"/>
-      <c r="AC23" s="132"/>
-      <c r="AD23" s="132"/>
-      <c r="AE23" s="132"/>
-      <c r="AF23" s="132"/>
+      <c r="AC23" s="147"/>
+      <c r="AD23" s="147"/>
+      <c r="AE23" s="147"/>
+      <c r="AF23" s="147"/>
       <c r="AG23" s="43"/>
       <c r="AH23" s="72"/>
-      <c r="AI23" s="132"/>
-      <c r="AJ23" s="132"/>
-      <c r="AK23" s="132"/>
-      <c r="AL23" s="132"/>
+      <c r="AI23" s="147"/>
+      <c r="AJ23" s="147"/>
+      <c r="AK23" s="147"/>
+      <c r="AL23" s="147"/>
       <c r="AM23" s="73"/>
       <c r="AN23" s="61"/>
       <c r="AO23" s="2"/>
@@ -2846,54 +2852,54 @@
       <c r="AV23" s="22"/>
     </row>
     <row r="24" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="112"/>
-      <c r="B24" s="173"/>
+      <c r="A24" s="111"/>
+      <c r="B24" s="130"/>
       <c r="C24" s="86"/>
-      <c r="D24" s="175"/>
-      <c r="E24" s="86"/>
+      <c r="D24" s="132"/>
+      <c r="E24" s="132"/>
       <c r="F24" s="86"/>
       <c r="G24" s="88"/>
       <c r="H24" s="87"/>
-      <c r="I24" s="120"/>
+      <c r="I24" s="119"/>
       <c r="J24" s="74"/>
-      <c r="K24" s="128" t="s">
+      <c r="K24" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="L24" s="127"/>
-      <c r="M24" s="126"/>
-      <c r="N24" s="127"/>
+      <c r="L24" s="145"/>
+      <c r="M24" s="146"/>
+      <c r="N24" s="145"/>
       <c r="O24" s="43"/>
       <c r="P24" s="72"/>
-      <c r="Q24" s="128" t="s">
+      <c r="Q24" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="R24" s="127"/>
-      <c r="S24" s="126"/>
-      <c r="T24" s="127"/>
+      <c r="R24" s="145"/>
+      <c r="S24" s="146"/>
+      <c r="T24" s="145"/>
       <c r="U24" s="43"/>
       <c r="V24" s="72"/>
-      <c r="W24" s="128" t="s">
+      <c r="W24" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="X24" s="127"/>
-      <c r="Y24" s="126"/>
-      <c r="Z24" s="127"/>
+      <c r="X24" s="145"/>
+      <c r="Y24" s="146"/>
+      <c r="Z24" s="145"/>
       <c r="AA24" s="43"/>
       <c r="AB24" s="72"/>
-      <c r="AC24" s="128" t="s">
+      <c r="AC24" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AD24" s="127"/>
-      <c r="AE24" s="126"/>
-      <c r="AF24" s="127"/>
+      <c r="AD24" s="145"/>
+      <c r="AE24" s="146"/>
+      <c r="AF24" s="145"/>
       <c r="AG24" s="43"/>
       <c r="AH24" s="72"/>
-      <c r="AI24" s="128" t="s">
+      <c r="AI24" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AJ24" s="127"/>
-      <c r="AK24" s="126"/>
-      <c r="AL24" s="127"/>
+      <c r="AJ24" s="145"/>
+      <c r="AK24" s="146"/>
+      <c r="AL24" s="145"/>
       <c r="AM24" s="73"/>
       <c r="AN24" s="61"/>
       <c r="AO24" s="2"/>
@@ -2906,54 +2912,54 @@
       <c r="AV24" s="22"/>
     </row>
     <row r="25" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="112"/>
-      <c r="B25" s="173"/>
+      <c r="A25" s="111"/>
+      <c r="B25" s="130"/>
       <c r="C25" s="86"/>
-      <c r="D25" s="175"/>
-      <c r="E25" s="86"/>
+      <c r="D25" s="132"/>
+      <c r="E25" s="132"/>
       <c r="F25" s="86"/>
       <c r="G25" s="88"/>
       <c r="H25" s="87"/>
-      <c r="I25" s="120"/>
+      <c r="I25" s="119"/>
       <c r="J25" s="74"/>
       <c r="K25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="L25" s="72"/>
-      <c r="M25" s="126"/>
-      <c r="N25" s="127"/>
+      <c r="M25" s="146"/>
+      <c r="N25" s="145"/>
       <c r="O25" s="43"/>
       <c r="P25" s="72"/>
       <c r="Q25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="R25" s="72"/>
-      <c r="S25" s="126"/>
-      <c r="T25" s="127"/>
+      <c r="S25" s="146"/>
+      <c r="T25" s="145"/>
       <c r="U25" s="43"/>
       <c r="V25" s="72"/>
       <c r="W25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="X25" s="72"/>
-      <c r="Y25" s="126"/>
-      <c r="Z25" s="127"/>
+      <c r="Y25" s="146"/>
+      <c r="Z25" s="145"/>
       <c r="AA25" s="43"/>
       <c r="AB25" s="72"/>
       <c r="AC25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AD25" s="72"/>
-      <c r="AE25" s="126"/>
-      <c r="AF25" s="127"/>
+      <c r="AE25" s="146"/>
+      <c r="AF25" s="145"/>
       <c r="AG25" s="43"/>
       <c r="AH25" s="72"/>
       <c r="AI25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AJ25" s="72"/>
-      <c r="AK25" s="126"/>
-      <c r="AL25" s="127"/>
+      <c r="AK25" s="146"/>
+      <c r="AL25" s="145"/>
       <c r="AM25" s="73"/>
       <c r="AN25" s="61"/>
       <c r="AO25" s="2"/>
@@ -2966,75 +2972,75 @@
       <c r="AV25" s="22"/>
     </row>
     <row r="26" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="112"/>
-      <c r="B26" s="173"/>
+      <c r="A26" s="111"/>
+      <c r="B26" s="130"/>
       <c r="C26" s="86"/>
-      <c r="D26" s="175"/>
-      <c r="E26" s="86"/>
+      <c r="D26" s="132"/>
+      <c r="E26" s="132"/>
       <c r="F26" s="86"/>
       <c r="G26" s="88"/>
       <c r="H26" s="87"/>
-      <c r="I26" s="120"/>
+      <c r="I26" s="119"/>
       <c r="J26" s="76"/>
       <c r="K26" s="48" t="s">
         <v>33</v>
       </c>
-      <c r="L26" s="135"/>
-      <c r="M26" s="135"/>
-      <c r="N26" s="135"/>
+      <c r="L26" s="148"/>
+      <c r="M26" s="148"/>
+      <c r="N26" s="148"/>
       <c r="O26" s="60"/>
       <c r="P26" s="41"/>
       <c r="Q26" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="R26" s="133"/>
-      <c r="S26" s="134"/>
-      <c r="T26" s="134"/>
+      <c r="R26" s="142"/>
+      <c r="S26" s="143"/>
+      <c r="T26" s="143"/>
       <c r="U26" s="40"/>
       <c r="V26" s="41"/>
       <c r="W26" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="X26" s="135"/>
-      <c r="Y26" s="135"/>
-      <c r="Z26" s="135"/>
+      <c r="X26" s="148"/>
+      <c r="Y26" s="148"/>
+      <c r="Z26" s="148"/>
       <c r="AA26" s="40"/>
       <c r="AB26" s="41"/>
       <c r="AC26" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="AD26" s="133"/>
-      <c r="AE26" s="134"/>
-      <c r="AF26" s="134"/>
+      <c r="AD26" s="142"/>
+      <c r="AE26" s="143"/>
+      <c r="AF26" s="143"/>
       <c r="AG26" s="40"/>
       <c r="AH26" s="41"/>
       <c r="AI26" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="AJ26" s="133"/>
-      <c r="AK26" s="134"/>
-      <c r="AL26" s="134"/>
+      <c r="AJ26" s="142"/>
+      <c r="AK26" s="143"/>
+      <c r="AL26" s="143"/>
       <c r="AM26" s="77"/>
       <c r="AN26" s="61"/>
-      <c r="AO26" s="129"/>
-      <c r="AP26" s="130"/>
-      <c r="AQ26" s="130"/>
-      <c r="AR26" s="130"/>
-      <c r="AS26" s="130"/>
-      <c r="AT26" s="130"/>
-      <c r="AU26" s="130"/>
+      <c r="AO26" s="180"/>
+      <c r="AP26" s="181"/>
+      <c r="AQ26" s="181"/>
+      <c r="AR26" s="181"/>
+      <c r="AS26" s="181"/>
+      <c r="AT26" s="181"/>
+      <c r="AU26" s="181"/>
       <c r="AV26" s="22"/>
     </row>
     <row r="27" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="113"/>
+      <c r="A27" s="112"/>
       <c r="B27" s="45"/>
       <c r="C27" s="42"/>
-      <c r="D27" s="176"/>
-      <c r="E27" s="42"/>
+      <c r="D27" s="133"/>
+      <c r="E27" s="133"/>
       <c r="F27" s="42"/>
       <c r="G27" s="46"/>
-      <c r="H27" s="179"/>
-      <c r="I27" s="122"/>
+      <c r="H27" s="136"/>
+      <c r="I27" s="121"/>
       <c r="J27" s="74"/>
       <c r="K27" s="71"/>
       <c r="L27" s="72"/>
@@ -3066,505 +3072,505 @@
       <c r="AL27" s="72"/>
       <c r="AM27" s="73"/>
       <c r="AN27" s="61"/>
-      <c r="AO27" s="130"/>
-      <c r="AP27" s="130"/>
-      <c r="AQ27" s="130"/>
-      <c r="AR27" s="130"/>
-      <c r="AS27" s="130"/>
-      <c r="AT27" s="130"/>
-      <c r="AU27" s="130"/>
+      <c r="AO27" s="181"/>
+      <c r="AP27" s="181"/>
+      <c r="AQ27" s="181"/>
+      <c r="AR27" s="181"/>
+      <c r="AS27" s="181"/>
+      <c r="AT27" s="181"/>
+      <c r="AU27" s="181"/>
       <c r="AV27" s="22"/>
     </row>
     <row r="28" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="114"/>
+      <c r="A28" s="113"/>
       <c r="B28" s="80"/>
       <c r="C28" s="81"/>
-      <c r="D28" s="177"/>
-      <c r="E28" s="81"/>
+      <c r="D28" s="134"/>
+      <c r="E28" s="134"/>
       <c r="F28" s="81"/>
-      <c r="G28" s="92"/>
-      <c r="H28" s="180"/>
-      <c r="I28" s="123"/>
+      <c r="G28" s="91"/>
+      <c r="H28" s="137"/>
+      <c r="I28" s="122"/>
       <c r="J28" s="74"/>
-      <c r="K28" s="132"/>
-      <c r="L28" s="132"/>
-      <c r="M28" s="132"/>
-      <c r="N28" s="132"/>
+      <c r="K28" s="147"/>
+      <c r="L28" s="147"/>
+      <c r="M28" s="147"/>
+      <c r="N28" s="147"/>
       <c r="O28" s="43"/>
       <c r="P28" s="72"/>
-      <c r="Q28" s="132"/>
-      <c r="R28" s="132"/>
-      <c r="S28" s="132"/>
-      <c r="T28" s="132"/>
+      <c r="Q28" s="147"/>
+      <c r="R28" s="147"/>
+      <c r="S28" s="147"/>
+      <c r="T28" s="147"/>
       <c r="U28" s="43"/>
       <c r="V28" s="72"/>
-      <c r="W28" s="132"/>
-      <c r="X28" s="132"/>
-      <c r="Y28" s="132"/>
-      <c r="Z28" s="132"/>
+      <c r="W28" s="147"/>
+      <c r="X28" s="147"/>
+      <c r="Y28" s="147"/>
+      <c r="Z28" s="147"/>
       <c r="AA28" s="43"/>
       <c r="AB28" s="72"/>
-      <c r="AC28" s="132"/>
-      <c r="AD28" s="132"/>
-      <c r="AE28" s="132"/>
-      <c r="AF28" s="132"/>
+      <c r="AC28" s="147"/>
+      <c r="AD28" s="147"/>
+      <c r="AE28" s="147"/>
+      <c r="AF28" s="147"/>
       <c r="AG28" s="43"/>
       <c r="AH28" s="72"/>
-      <c r="AI28" s="132"/>
-      <c r="AJ28" s="132"/>
-      <c r="AK28" s="132"/>
-      <c r="AL28" s="132"/>
+      <c r="AI28" s="147"/>
+      <c r="AJ28" s="147"/>
+      <c r="AK28" s="147"/>
+      <c r="AL28" s="147"/>
       <c r="AM28" s="73"/>
       <c r="AN28" s="61"/>
-      <c r="AO28" s="130"/>
-      <c r="AP28" s="130"/>
-      <c r="AQ28" s="130"/>
-      <c r="AR28" s="130"/>
-      <c r="AS28" s="130"/>
-      <c r="AT28" s="130"/>
-      <c r="AU28" s="130"/>
+      <c r="AO28" s="181"/>
+      <c r="AP28" s="181"/>
+      <c r="AQ28" s="181"/>
+      <c r="AR28" s="181"/>
+      <c r="AS28" s="181"/>
+      <c r="AT28" s="181"/>
+      <c r="AU28" s="181"/>
       <c r="AV28" s="22"/>
     </row>
     <row r="29" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="112"/>
-      <c r="B29" s="173"/>
+      <c r="A29" s="111"/>
+      <c r="B29" s="130"/>
       <c r="C29" s="86"/>
-      <c r="D29" s="175"/>
-      <c r="E29" s="86"/>
+      <c r="D29" s="132"/>
+      <c r="E29" s="132"/>
       <c r="F29" s="86"/>
       <c r="G29" s="88"/>
       <c r="H29" s="87"/>
-      <c r="I29" s="120"/>
+      <c r="I29" s="119"/>
       <c r="J29" s="70"/>
-      <c r="K29" s="132"/>
-      <c r="L29" s="132"/>
-      <c r="M29" s="132"/>
-      <c r="N29" s="132"/>
+      <c r="K29" s="147"/>
+      <c r="L29" s="147"/>
+      <c r="M29" s="147"/>
+      <c r="N29" s="147"/>
       <c r="O29" s="43"/>
       <c r="P29" s="72"/>
-      <c r="Q29" s="132"/>
-      <c r="R29" s="132"/>
-      <c r="S29" s="132"/>
-      <c r="T29" s="132"/>
+      <c r="Q29" s="147"/>
+      <c r="R29" s="147"/>
+      <c r="S29" s="147"/>
+      <c r="T29" s="147"/>
       <c r="U29" s="43"/>
       <c r="V29" s="72"/>
-      <c r="W29" s="132"/>
-      <c r="X29" s="132"/>
-      <c r="Y29" s="132"/>
-      <c r="Z29" s="132"/>
+      <c r="W29" s="147"/>
+      <c r="X29" s="147"/>
+      <c r="Y29" s="147"/>
+      <c r="Z29" s="147"/>
       <c r="AA29" s="43"/>
       <c r="AB29" s="72"/>
-      <c r="AC29" s="132"/>
-      <c r="AD29" s="132"/>
-      <c r="AE29" s="132"/>
-      <c r="AF29" s="132"/>
+      <c r="AC29" s="147"/>
+      <c r="AD29" s="147"/>
+      <c r="AE29" s="147"/>
+      <c r="AF29" s="147"/>
       <c r="AG29" s="43"/>
       <c r="AH29" s="72"/>
-      <c r="AI29" s="132"/>
-      <c r="AJ29" s="132"/>
-      <c r="AK29" s="132"/>
-      <c r="AL29" s="132"/>
+      <c r="AI29" s="147"/>
+      <c r="AJ29" s="147"/>
+      <c r="AK29" s="147"/>
+      <c r="AL29" s="147"/>
       <c r="AM29" s="73"/>
       <c r="AN29" s="61"/>
-      <c r="AO29" s="130"/>
-      <c r="AP29" s="130"/>
-      <c r="AQ29" s="130"/>
-      <c r="AR29" s="130"/>
-      <c r="AS29" s="130"/>
-      <c r="AT29" s="130"/>
-      <c r="AU29" s="130"/>
+      <c r="AO29" s="181"/>
+      <c r="AP29" s="181"/>
+      <c r="AQ29" s="181"/>
+      <c r="AR29" s="181"/>
+      <c r="AS29" s="181"/>
+      <c r="AT29" s="181"/>
+      <c r="AU29" s="181"/>
       <c r="AV29" s="22"/>
     </row>
     <row r="30" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="112"/>
-      <c r="B30" s="173"/>
+      <c r="A30" s="111"/>
+      <c r="B30" s="130"/>
       <c r="C30" s="86"/>
-      <c r="D30" s="175"/>
-      <c r="E30" s="86"/>
+      <c r="D30" s="132"/>
+      <c r="E30" s="132"/>
       <c r="F30" s="86"/>
       <c r="G30" s="88"/>
       <c r="H30" s="87"/>
-      <c r="I30" s="120"/>
+      <c r="I30" s="119"/>
       <c r="J30" s="74"/>
-      <c r="K30" s="132"/>
-      <c r="L30" s="132"/>
-      <c r="M30" s="132"/>
-      <c r="N30" s="132"/>
+      <c r="K30" s="147"/>
+      <c r="L30" s="147"/>
+      <c r="M30" s="147"/>
+      <c r="N30" s="147"/>
       <c r="O30" s="43"/>
       <c r="P30" s="72"/>
-      <c r="Q30" s="132"/>
-      <c r="R30" s="132"/>
-      <c r="S30" s="132"/>
-      <c r="T30" s="132"/>
+      <c r="Q30" s="147"/>
+      <c r="R30" s="147"/>
+      <c r="S30" s="147"/>
+      <c r="T30" s="147"/>
       <c r="U30" s="43"/>
       <c r="V30" s="72"/>
-      <c r="W30" s="132"/>
-      <c r="X30" s="132"/>
-      <c r="Y30" s="132"/>
-      <c r="Z30" s="132"/>
+      <c r="W30" s="147"/>
+      <c r="X30" s="147"/>
+      <c r="Y30" s="147"/>
+      <c r="Z30" s="147"/>
       <c r="AA30" s="43"/>
       <c r="AB30" s="72"/>
-      <c r="AC30" s="132"/>
-      <c r="AD30" s="132"/>
-      <c r="AE30" s="132"/>
-      <c r="AF30" s="132"/>
+      <c r="AC30" s="147"/>
+      <c r="AD30" s="147"/>
+      <c r="AE30" s="147"/>
+      <c r="AF30" s="147"/>
       <c r="AG30" s="43"/>
       <c r="AH30" s="72"/>
-      <c r="AI30" s="132"/>
-      <c r="AJ30" s="132"/>
-      <c r="AK30" s="132"/>
-      <c r="AL30" s="132"/>
+      <c r="AI30" s="147"/>
+      <c r="AJ30" s="147"/>
+      <c r="AK30" s="147"/>
+      <c r="AL30" s="147"/>
       <c r="AM30" s="73"/>
       <c r="AN30" s="62"/>
-      <c r="AO30" s="130"/>
-      <c r="AP30" s="130"/>
-      <c r="AQ30" s="130"/>
-      <c r="AR30" s="130"/>
-      <c r="AS30" s="130"/>
-      <c r="AT30" s="130"/>
-      <c r="AU30" s="130"/>
+      <c r="AO30" s="181"/>
+      <c r="AP30" s="181"/>
+      <c r="AQ30" s="181"/>
+      <c r="AR30" s="181"/>
+      <c r="AS30" s="181"/>
+      <c r="AT30" s="181"/>
+      <c r="AU30" s="181"/>
       <c r="AV30" s="22"/>
     </row>
     <row r="31" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="112"/>
-      <c r="B31" s="173"/>
+      <c r="A31" s="111"/>
+      <c r="B31" s="130"/>
       <c r="C31" s="86"/>
-      <c r="D31" s="175"/>
-      <c r="E31" s="86"/>
+      <c r="D31" s="132"/>
+      <c r="E31" s="132"/>
       <c r="F31" s="86"/>
       <c r="G31" s="88"/>
       <c r="H31" s="87"/>
-      <c r="I31" s="120"/>
+      <c r="I31" s="119"/>
       <c r="J31" s="74"/>
-      <c r="K31" s="132"/>
-      <c r="L31" s="132"/>
-      <c r="M31" s="132"/>
-      <c r="N31" s="132"/>
+      <c r="K31" s="147"/>
+      <c r="L31" s="147"/>
+      <c r="M31" s="147"/>
+      <c r="N31" s="147"/>
       <c r="O31" s="43"/>
       <c r="P31" s="72"/>
-      <c r="Q31" s="132"/>
-      <c r="R31" s="132"/>
-      <c r="S31" s="132"/>
-      <c r="T31" s="132"/>
+      <c r="Q31" s="147"/>
+      <c r="R31" s="147"/>
+      <c r="S31" s="147"/>
+      <c r="T31" s="147"/>
       <c r="U31" s="43"/>
       <c r="V31" s="72"/>
-      <c r="W31" s="132"/>
-      <c r="X31" s="132"/>
-      <c r="Y31" s="132"/>
-      <c r="Z31" s="132"/>
+      <c r="W31" s="147"/>
+      <c r="X31" s="147"/>
+      <c r="Y31" s="147"/>
+      <c r="Z31" s="147"/>
       <c r="AA31" s="43"/>
       <c r="AB31" s="72"/>
-      <c r="AC31" s="132"/>
-      <c r="AD31" s="132"/>
-      <c r="AE31" s="132"/>
-      <c r="AF31" s="132"/>
+      <c r="AC31" s="147"/>
+      <c r="AD31" s="147"/>
+      <c r="AE31" s="147"/>
+      <c r="AF31" s="147"/>
       <c r="AG31" s="43"/>
       <c r="AH31" s="72"/>
-      <c r="AI31" s="132"/>
-      <c r="AJ31" s="132"/>
-      <c r="AK31" s="132"/>
-      <c r="AL31" s="132"/>
+      <c r="AI31" s="147"/>
+      <c r="AJ31" s="147"/>
+      <c r="AK31" s="147"/>
+      <c r="AL31" s="147"/>
       <c r="AM31" s="73"/>
       <c r="AN31" s="61"/>
-      <c r="AO31" s="130"/>
-      <c r="AP31" s="130"/>
-      <c r="AQ31" s="130"/>
-      <c r="AR31" s="130"/>
-      <c r="AS31" s="130"/>
-      <c r="AT31" s="130"/>
-      <c r="AU31" s="130"/>
+      <c r="AO31" s="181"/>
+      <c r="AP31" s="181"/>
+      <c r="AQ31" s="181"/>
+      <c r="AR31" s="181"/>
+      <c r="AS31" s="181"/>
+      <c r="AT31" s="181"/>
+      <c r="AU31" s="181"/>
       <c r="AV31" s="22"/>
     </row>
     <row r="32" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="112"/>
-      <c r="B32" s="173"/>
+      <c r="A32" s="111"/>
+      <c r="B32" s="130"/>
       <c r="C32" s="86"/>
-      <c r="D32" s="175"/>
-      <c r="E32" s="86"/>
+      <c r="D32" s="132"/>
+      <c r="E32" s="132"/>
       <c r="F32" s="86"/>
       <c r="G32" s="88"/>
       <c r="H32" s="87"/>
-      <c r="I32" s="120"/>
+      <c r="I32" s="119"/>
       <c r="J32" s="74"/>
-      <c r="K32" s="132"/>
-      <c r="L32" s="132"/>
-      <c r="M32" s="132"/>
-      <c r="N32" s="132"/>
+      <c r="K32" s="147"/>
+      <c r="L32" s="147"/>
+      <c r="M32" s="147"/>
+      <c r="N32" s="147"/>
       <c r="O32" s="43"/>
       <c r="P32" s="72"/>
-      <c r="Q32" s="132"/>
-      <c r="R32" s="132"/>
-      <c r="S32" s="132"/>
-      <c r="T32" s="132"/>
+      <c r="Q32" s="147"/>
+      <c r="R32" s="147"/>
+      <c r="S32" s="147"/>
+      <c r="T32" s="147"/>
       <c r="U32" s="43"/>
       <c r="V32" s="72"/>
-      <c r="W32" s="132"/>
-      <c r="X32" s="132"/>
-      <c r="Y32" s="132"/>
-      <c r="Z32" s="132"/>
+      <c r="W32" s="147"/>
+      <c r="X32" s="147"/>
+      <c r="Y32" s="147"/>
+      <c r="Z32" s="147"/>
       <c r="AA32" s="43"/>
       <c r="AB32" s="72"/>
-      <c r="AC32" s="132"/>
-      <c r="AD32" s="132"/>
-      <c r="AE32" s="132"/>
-      <c r="AF32" s="132"/>
+      <c r="AC32" s="147"/>
+      <c r="AD32" s="147"/>
+      <c r="AE32" s="147"/>
+      <c r="AF32" s="147"/>
       <c r="AG32" s="43"/>
       <c r="AH32" s="72"/>
-      <c r="AI32" s="132"/>
-      <c r="AJ32" s="132"/>
-      <c r="AK32" s="132"/>
-      <c r="AL32" s="132"/>
+      <c r="AI32" s="147"/>
+      <c r="AJ32" s="147"/>
+      <c r="AK32" s="147"/>
+      <c r="AL32" s="147"/>
       <c r="AM32" s="73"/>
       <c r="AN32" s="61"/>
-      <c r="AO32" s="130"/>
-      <c r="AP32" s="130"/>
-      <c r="AQ32" s="130"/>
-      <c r="AR32" s="130"/>
-      <c r="AS32" s="130"/>
-      <c r="AT32" s="130"/>
-      <c r="AU32" s="130"/>
+      <c r="AO32" s="181"/>
+      <c r="AP32" s="181"/>
+      <c r="AQ32" s="181"/>
+      <c r="AR32" s="181"/>
+      <c r="AS32" s="181"/>
+      <c r="AT32" s="181"/>
+      <c r="AU32" s="181"/>
       <c r="AV32" s="22"/>
     </row>
     <row r="33" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="112"/>
-      <c r="B33" s="173"/>
+      <c r="A33" s="111"/>
+      <c r="B33" s="130"/>
       <c r="C33" s="86"/>
-      <c r="D33" s="175"/>
-      <c r="E33" s="86"/>
+      <c r="D33" s="132"/>
+      <c r="E33" s="132"/>
       <c r="F33" s="86"/>
       <c r="G33" s="88"/>
       <c r="H33" s="87"/>
-      <c r="I33" s="120"/>
+      <c r="I33" s="119"/>
       <c r="J33" s="70"/>
-      <c r="K33" s="132"/>
-      <c r="L33" s="132"/>
-      <c r="M33" s="132"/>
-      <c r="N33" s="132"/>
+      <c r="K33" s="147"/>
+      <c r="L33" s="147"/>
+      <c r="M33" s="147"/>
+      <c r="N33" s="147"/>
       <c r="O33" s="43"/>
       <c r="P33" s="72"/>
-      <c r="Q33" s="132"/>
-      <c r="R33" s="132"/>
-      <c r="S33" s="132"/>
-      <c r="T33" s="132"/>
+      <c r="Q33" s="147"/>
+      <c r="R33" s="147"/>
+      <c r="S33" s="147"/>
+      <c r="T33" s="147"/>
       <c r="U33" s="43"/>
       <c r="V33" s="72"/>
-      <c r="W33" s="132"/>
-      <c r="X33" s="132"/>
-      <c r="Y33" s="132"/>
-      <c r="Z33" s="132"/>
+      <c r="W33" s="147"/>
+      <c r="X33" s="147"/>
+      <c r="Y33" s="147"/>
+      <c r="Z33" s="147"/>
       <c r="AA33" s="43"/>
       <c r="AB33" s="72"/>
-      <c r="AC33" s="132"/>
-      <c r="AD33" s="132"/>
-      <c r="AE33" s="132"/>
-      <c r="AF33" s="132"/>
+      <c r="AC33" s="147"/>
+      <c r="AD33" s="147"/>
+      <c r="AE33" s="147"/>
+      <c r="AF33" s="147"/>
       <c r="AG33" s="43"/>
       <c r="AH33" s="72"/>
-      <c r="AI33" s="132"/>
-      <c r="AJ33" s="132"/>
-      <c r="AK33" s="132"/>
-      <c r="AL33" s="132"/>
+      <c r="AI33" s="147"/>
+      <c r="AJ33" s="147"/>
+      <c r="AK33" s="147"/>
+      <c r="AL33" s="147"/>
       <c r="AM33" s="73"/>
       <c r="AN33" s="61"/>
-      <c r="AO33" s="130"/>
-      <c r="AP33" s="130"/>
-      <c r="AQ33" s="130"/>
-      <c r="AR33" s="130"/>
-      <c r="AS33" s="130"/>
-      <c r="AT33" s="130"/>
-      <c r="AU33" s="130"/>
+      <c r="AO33" s="181"/>
+      <c r="AP33" s="181"/>
+      <c r="AQ33" s="181"/>
+      <c r="AR33" s="181"/>
+      <c r="AS33" s="181"/>
+      <c r="AT33" s="181"/>
+      <c r="AU33" s="181"/>
       <c r="AV33" s="22"/>
     </row>
     <row r="34" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="112"/>
-      <c r="B34" s="173"/>
+      <c r="A34" s="111"/>
+      <c r="B34" s="130"/>
       <c r="C34" s="86"/>
-      <c r="D34" s="175"/>
-      <c r="E34" s="86"/>
+      <c r="D34" s="132"/>
+      <c r="E34" s="132"/>
       <c r="F34" s="86"/>
       <c r="G34" s="88"/>
       <c r="H34" s="87"/>
-      <c r="I34" s="120"/>
+      <c r="I34" s="119"/>
       <c r="J34" s="78"/>
-      <c r="K34" s="128" t="s">
+      <c r="K34" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="L34" s="127"/>
-      <c r="M34" s="126"/>
-      <c r="N34" s="127"/>
+      <c r="L34" s="145"/>
+      <c r="M34" s="146"/>
+      <c r="N34" s="145"/>
       <c r="O34" s="43"/>
       <c r="P34" s="72"/>
-      <c r="Q34" s="128" t="s">
+      <c r="Q34" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="R34" s="127"/>
-      <c r="S34" s="126"/>
-      <c r="T34" s="127"/>
+      <c r="R34" s="145"/>
+      <c r="S34" s="146"/>
+      <c r="T34" s="145"/>
       <c r="U34" s="43"/>
       <c r="V34" s="72"/>
-      <c r="W34" s="128" t="s">
+      <c r="W34" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="X34" s="127"/>
-      <c r="Y34" s="126"/>
-      <c r="Z34" s="127"/>
+      <c r="X34" s="145"/>
+      <c r="Y34" s="146"/>
+      <c r="Z34" s="145"/>
       <c r="AA34" s="43"/>
       <c r="AB34" s="72"/>
-      <c r="AC34" s="128" t="s">
+      <c r="AC34" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AD34" s="127"/>
-      <c r="AE34" s="126"/>
-      <c r="AF34" s="127"/>
+      <c r="AD34" s="145"/>
+      <c r="AE34" s="146"/>
+      <c r="AF34" s="145"/>
       <c r="AG34" s="43"/>
       <c r="AH34" s="72"/>
-      <c r="AI34" s="128" t="s">
+      <c r="AI34" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AJ34" s="127"/>
-      <c r="AK34" s="126"/>
-      <c r="AL34" s="127"/>
+      <c r="AJ34" s="145"/>
+      <c r="AK34" s="146"/>
+      <c r="AL34" s="145"/>
       <c r="AM34" s="43"/>
       <c r="AN34" s="61"/>
-      <c r="AO34" s="130"/>
-      <c r="AP34" s="130"/>
-      <c r="AQ34" s="130"/>
-      <c r="AR34" s="130"/>
-      <c r="AS34" s="130"/>
-      <c r="AT34" s="130"/>
-      <c r="AU34" s="130"/>
+      <c r="AO34" s="181"/>
+      <c r="AP34" s="181"/>
+      <c r="AQ34" s="181"/>
+      <c r="AR34" s="181"/>
+      <c r="AS34" s="181"/>
+      <c r="AT34" s="181"/>
+      <c r="AU34" s="181"/>
       <c r="AV34" s="22"/>
     </row>
     <row r="35" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="112"/>
-      <c r="B35" s="173"/>
+      <c r="A35" s="111"/>
+      <c r="B35" s="130"/>
       <c r="C35" s="86"/>
-      <c r="D35" s="175"/>
-      <c r="E35" s="86"/>
+      <c r="D35" s="132"/>
+      <c r="E35" s="132"/>
       <c r="F35" s="86"/>
       <c r="G35" s="88"/>
       <c r="H35" s="87"/>
-      <c r="I35" s="120"/>
+      <c r="I35" s="119"/>
       <c r="J35" s="78"/>
       <c r="K35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="L35" s="72"/>
-      <c r="M35" s="126"/>
-      <c r="N35" s="127"/>
+      <c r="M35" s="146"/>
+      <c r="N35" s="145"/>
       <c r="O35" s="43"/>
       <c r="P35" s="72"/>
       <c r="Q35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="R35" s="72"/>
-      <c r="S35" s="126"/>
-      <c r="T35" s="127"/>
+      <c r="S35" s="146"/>
+      <c r="T35" s="145"/>
       <c r="U35" s="43"/>
       <c r="V35" s="72"/>
       <c r="W35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="X35" s="72"/>
-      <c r="Y35" s="126"/>
-      <c r="Z35" s="127"/>
+      <c r="Y35" s="146"/>
+      <c r="Z35" s="145"/>
       <c r="AA35" s="43"/>
       <c r="AB35" s="72"/>
       <c r="AC35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AD35" s="72"/>
-      <c r="AE35" s="126"/>
-      <c r="AF35" s="127"/>
+      <c r="AE35" s="146"/>
+      <c r="AF35" s="145"/>
       <c r="AG35" s="43"/>
       <c r="AH35" s="72"/>
       <c r="AI35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AJ35" s="72"/>
-      <c r="AK35" s="126"/>
-      <c r="AL35" s="127"/>
-      <c r="AM35" s="131"/>
+      <c r="AK35" s="146"/>
+      <c r="AL35" s="145"/>
+      <c r="AM35" s="149"/>
       <c r="AN35" s="61"/>
-      <c r="AO35" s="130"/>
-      <c r="AP35" s="130"/>
-      <c r="AQ35" s="130"/>
-      <c r="AR35" s="130"/>
-      <c r="AS35" s="130"/>
-      <c r="AT35" s="130"/>
-      <c r="AU35" s="130"/>
+      <c r="AO35" s="181"/>
+      <c r="AP35" s="181"/>
+      <c r="AQ35" s="181"/>
+      <c r="AR35" s="181"/>
+      <c r="AS35" s="181"/>
+      <c r="AT35" s="181"/>
+      <c r="AU35" s="181"/>
       <c r="AV35" s="30"/>
     </row>
     <row r="36" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="112"/>
-      <c r="B36" s="173"/>
+      <c r="A36" s="111"/>
+      <c r="B36" s="130"/>
       <c r="C36" s="86"/>
-      <c r="D36" s="175"/>
-      <c r="E36" s="86"/>
+      <c r="D36" s="132"/>
+      <c r="E36" s="132"/>
       <c r="F36" s="86"/>
       <c r="G36" s="88"/>
       <c r="H36" s="87"/>
-      <c r="I36" s="120"/>
+      <c r="I36" s="119"/>
       <c r="J36" s="76"/>
       <c r="K36" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="L36" s="133"/>
-      <c r="M36" s="134"/>
-      <c r="N36" s="134"/>
+      <c r="L36" s="142"/>
+      <c r="M36" s="143"/>
+      <c r="N36" s="143"/>
       <c r="O36" s="65"/>
       <c r="P36" s="41"/>
       <c r="Q36" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="R36" s="133"/>
-      <c r="S36" s="134"/>
-      <c r="T36" s="134"/>
+      <c r="R36" s="142"/>
+      <c r="S36" s="143"/>
+      <c r="T36" s="143"/>
       <c r="U36" s="40"/>
       <c r="V36" s="41"/>
       <c r="W36" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="X36" s="135"/>
-      <c r="Y36" s="135"/>
-      <c r="Z36" s="135"/>
+      <c r="X36" s="148"/>
+      <c r="Y36" s="148"/>
+      <c r="Z36" s="148"/>
       <c r="AA36" s="40"/>
       <c r="AB36" s="41"/>
       <c r="AC36" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="AD36" s="133"/>
-      <c r="AE36" s="134"/>
-      <c r="AF36" s="134"/>
+      <c r="AD36" s="142"/>
+      <c r="AE36" s="143"/>
+      <c r="AF36" s="143"/>
       <c r="AG36" s="40"/>
       <c r="AH36" s="41"/>
       <c r="AI36" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="AJ36" s="133"/>
-      <c r="AK36" s="134"/>
-      <c r="AL36" s="134"/>
+      <c r="AJ36" s="142"/>
+      <c r="AK36" s="143"/>
+      <c r="AL36" s="143"/>
       <c r="AM36" s="77"/>
       <c r="AN36" s="2"/>
-      <c r="AO36" s="130"/>
-      <c r="AP36" s="130"/>
-      <c r="AQ36" s="130"/>
-      <c r="AR36" s="130"/>
-      <c r="AS36" s="130"/>
-      <c r="AT36" s="130"/>
-      <c r="AU36" s="130"/>
+      <c r="AO36" s="181"/>
+      <c r="AP36" s="181"/>
+      <c r="AQ36" s="181"/>
+      <c r="AR36" s="181"/>
+      <c r="AS36" s="181"/>
+      <c r="AT36" s="181"/>
+      <c r="AU36" s="181"/>
       <c r="AV36" s="22"/>
     </row>
     <row r="37" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="115"/>
+      <c r="A37" s="114"/>
       <c r="B37" s="45"/>
       <c r="C37" s="42"/>
-      <c r="D37" s="176"/>
-      <c r="E37" s="42"/>
+      <c r="D37" s="133"/>
+      <c r="E37" s="133"/>
       <c r="F37" s="42"/>
       <c r="G37" s="42"/>
-      <c r="H37" s="181"/>
-      <c r="I37" s="124"/>
+      <c r="H37" s="138"/>
+      <c r="I37" s="123"/>
       <c r="J37" s="74"/>
       <c r="K37" s="71"/>
       <c r="L37" s="72"/>
@@ -3596,484 +3602,484 @@
       <c r="AL37" s="72"/>
       <c r="AM37" s="73"/>
       <c r="AN37" s="2"/>
-      <c r="AO37" s="130"/>
-      <c r="AP37" s="130"/>
-      <c r="AQ37" s="130"/>
-      <c r="AR37" s="130"/>
-      <c r="AS37" s="130"/>
-      <c r="AT37" s="130"/>
-      <c r="AU37" s="130"/>
+      <c r="AO37" s="181"/>
+      <c r="AP37" s="181"/>
+      <c r="AQ37" s="181"/>
+      <c r="AR37" s="181"/>
+      <c r="AS37" s="181"/>
+      <c r="AT37" s="181"/>
+      <c r="AU37" s="181"/>
       <c r="AV37" s="22"/>
     </row>
     <row r="38" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="116"/>
-      <c r="B38" s="174"/>
+      <c r="A38" s="115"/>
+      <c r="B38" s="131"/>
       <c r="C38" s="81"/>
-      <c r="D38" s="177"/>
-      <c r="E38" s="91"/>
+      <c r="D38" s="134"/>
+      <c r="E38" s="182"/>
       <c r="F38" s="90"/>
       <c r="G38" s="81"/>
-      <c r="H38" s="182"/>
-      <c r="I38" s="125"/>
+      <c r="H38" s="139"/>
+      <c r="I38" s="124"/>
       <c r="J38" s="74"/>
-      <c r="K38" s="132"/>
-      <c r="L38" s="132"/>
-      <c r="M38" s="132"/>
-      <c r="N38" s="132"/>
+      <c r="K38" s="147"/>
+      <c r="L38" s="147"/>
+      <c r="M38" s="147"/>
+      <c r="N38" s="147"/>
       <c r="O38" s="43"/>
       <c r="P38" s="72"/>
-      <c r="Q38" s="132"/>
-      <c r="R38" s="132"/>
-      <c r="S38" s="132"/>
-      <c r="T38" s="132"/>
+      <c r="Q38" s="147"/>
+      <c r="R38" s="147"/>
+      <c r="S38" s="147"/>
+      <c r="T38" s="147"/>
       <c r="U38" s="43"/>
       <c r="V38" s="72"/>
-      <c r="W38" s="132"/>
-      <c r="X38" s="132"/>
-      <c r="Y38" s="132"/>
-      <c r="Z38" s="132"/>
+      <c r="W38" s="147"/>
+      <c r="X38" s="147"/>
+      <c r="Y38" s="147"/>
+      <c r="Z38" s="147"/>
       <c r="AA38" s="43"/>
       <c r="AB38" s="72"/>
-      <c r="AC38" s="132"/>
-      <c r="AD38" s="132"/>
-      <c r="AE38" s="132"/>
-      <c r="AF38" s="132"/>
+      <c r="AC38" s="147"/>
+      <c r="AD38" s="147"/>
+      <c r="AE38" s="147"/>
+      <c r="AF38" s="147"/>
       <c r="AG38" s="43"/>
       <c r="AH38" s="72"/>
-      <c r="AI38" s="132"/>
-      <c r="AJ38" s="132"/>
-      <c r="AK38" s="132"/>
-      <c r="AL38" s="132"/>
+      <c r="AI38" s="147"/>
+      <c r="AJ38" s="147"/>
+      <c r="AK38" s="147"/>
+      <c r="AL38" s="147"/>
       <c r="AM38" s="73"/>
       <c r="AN38" s="2"/>
-      <c r="AO38" s="130"/>
-      <c r="AP38" s="130"/>
-      <c r="AQ38" s="130"/>
-      <c r="AR38" s="130"/>
-      <c r="AS38" s="130"/>
-      <c r="AT38" s="130"/>
-      <c r="AU38" s="130"/>
+      <c r="AO38" s="181"/>
+      <c r="AP38" s="181"/>
+      <c r="AQ38" s="181"/>
+      <c r="AR38" s="181"/>
+      <c r="AS38" s="181"/>
+      <c r="AT38" s="181"/>
+      <c r="AU38" s="181"/>
       <c r="AV38" s="22"/>
     </row>
     <row r="39" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="112"/>
-      <c r="B39" s="173"/>
+      <c r="A39" s="111"/>
+      <c r="B39" s="130"/>
       <c r="C39" s="86"/>
-      <c r="D39" s="175"/>
-      <c r="E39" s="86"/>
+      <c r="D39" s="132"/>
+      <c r="E39" s="132"/>
       <c r="F39" s="86"/>
       <c r="G39" s="88"/>
       <c r="H39" s="87"/>
-      <c r="I39" s="120"/>
+      <c r="I39" s="119"/>
       <c r="J39" s="70"/>
-      <c r="K39" s="132"/>
-      <c r="L39" s="132"/>
-      <c r="M39" s="132"/>
-      <c r="N39" s="132"/>
+      <c r="K39" s="147"/>
+      <c r="L39" s="147"/>
+      <c r="M39" s="147"/>
+      <c r="N39" s="147"/>
       <c r="O39" s="43"/>
       <c r="P39" s="72"/>
-      <c r="Q39" s="132"/>
-      <c r="R39" s="132"/>
-      <c r="S39" s="132"/>
-      <c r="T39" s="132"/>
+      <c r="Q39" s="147"/>
+      <c r="R39" s="147"/>
+      <c r="S39" s="147"/>
+      <c r="T39" s="147"/>
       <c r="U39" s="43"/>
       <c r="V39" s="72"/>
-      <c r="W39" s="132"/>
-      <c r="X39" s="132"/>
-      <c r="Y39" s="132"/>
-      <c r="Z39" s="132"/>
+      <c r="W39" s="147"/>
+      <c r="X39" s="147"/>
+      <c r="Y39" s="147"/>
+      <c r="Z39" s="147"/>
       <c r="AA39" s="43"/>
       <c r="AB39" s="72"/>
-      <c r="AC39" s="132"/>
-      <c r="AD39" s="132"/>
-      <c r="AE39" s="132"/>
-      <c r="AF39" s="132"/>
+      <c r="AC39" s="147"/>
+      <c r="AD39" s="147"/>
+      <c r="AE39" s="147"/>
+      <c r="AF39" s="147"/>
       <c r="AG39" s="43"/>
       <c r="AH39" s="72"/>
-      <c r="AI39" s="132"/>
-      <c r="AJ39" s="132"/>
-      <c r="AK39" s="132"/>
-      <c r="AL39" s="132"/>
+      <c r="AI39" s="147"/>
+      <c r="AJ39" s="147"/>
+      <c r="AK39" s="147"/>
+      <c r="AL39" s="147"/>
       <c r="AM39" s="73"/>
       <c r="AN39" s="2"/>
-      <c r="AO39" s="130"/>
-      <c r="AP39" s="130"/>
-      <c r="AQ39" s="130"/>
-      <c r="AR39" s="130"/>
-      <c r="AS39" s="130"/>
-      <c r="AT39" s="130"/>
-      <c r="AU39" s="130"/>
+      <c r="AO39" s="181"/>
+      <c r="AP39" s="181"/>
+      <c r="AQ39" s="181"/>
+      <c r="AR39" s="181"/>
+      <c r="AS39" s="181"/>
+      <c r="AT39" s="181"/>
+      <c r="AU39" s="181"/>
       <c r="AV39" s="22"/>
     </row>
     <row r="40" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="112"/>
-      <c r="B40" s="173"/>
+      <c r="A40" s="111"/>
+      <c r="B40" s="130"/>
       <c r="C40" s="86"/>
-      <c r="D40" s="175"/>
-      <c r="E40" s="86"/>
+      <c r="D40" s="132"/>
+      <c r="E40" s="132"/>
       <c r="F40" s="86"/>
       <c r="G40" s="88"/>
       <c r="H40" s="87"/>
-      <c r="I40" s="120"/>
+      <c r="I40" s="119"/>
       <c r="J40" s="74"/>
-      <c r="K40" s="132"/>
-      <c r="L40" s="132"/>
-      <c r="M40" s="132"/>
-      <c r="N40" s="132"/>
+      <c r="K40" s="147"/>
+      <c r="L40" s="147"/>
+      <c r="M40" s="147"/>
+      <c r="N40" s="147"/>
       <c r="O40" s="43"/>
       <c r="P40" s="72"/>
-      <c r="Q40" s="132"/>
-      <c r="R40" s="132"/>
-      <c r="S40" s="132"/>
-      <c r="T40" s="132"/>
+      <c r="Q40" s="147"/>
+      <c r="R40" s="147"/>
+      <c r="S40" s="147"/>
+      <c r="T40" s="147"/>
       <c r="U40" s="43"/>
       <c r="V40" s="72"/>
-      <c r="W40" s="132"/>
-      <c r="X40" s="132"/>
-      <c r="Y40" s="132"/>
-      <c r="Z40" s="132"/>
+      <c r="W40" s="147"/>
+      <c r="X40" s="147"/>
+      <c r="Y40" s="147"/>
+      <c r="Z40" s="147"/>
       <c r="AA40" s="43"/>
       <c r="AB40" s="72"/>
-      <c r="AC40" s="132"/>
-      <c r="AD40" s="132"/>
-      <c r="AE40" s="132"/>
-      <c r="AF40" s="132"/>
+      <c r="AC40" s="147"/>
+      <c r="AD40" s="147"/>
+      <c r="AE40" s="147"/>
+      <c r="AF40" s="147"/>
       <c r="AG40" s="43"/>
       <c r="AH40" s="72"/>
-      <c r="AI40" s="132"/>
-      <c r="AJ40" s="132"/>
-      <c r="AK40" s="132"/>
-      <c r="AL40" s="132"/>
+      <c r="AI40" s="147"/>
+      <c r="AJ40" s="147"/>
+      <c r="AK40" s="147"/>
+      <c r="AL40" s="147"/>
       <c r="AM40" s="73"/>
       <c r="AN40" s="2"/>
-      <c r="AO40" s="130"/>
-      <c r="AP40" s="130"/>
-      <c r="AQ40" s="130"/>
-      <c r="AR40" s="130"/>
-      <c r="AS40" s="130"/>
-      <c r="AT40" s="130"/>
-      <c r="AU40" s="130"/>
+      <c r="AO40" s="181"/>
+      <c r="AP40" s="181"/>
+      <c r="AQ40" s="181"/>
+      <c r="AR40" s="181"/>
+      <c r="AS40" s="181"/>
+      <c r="AT40" s="181"/>
+      <c r="AU40" s="181"/>
       <c r="AV40" s="22"/>
     </row>
     <row r="41" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="112"/>
-      <c r="B41" s="173"/>
+      <c r="A41" s="111"/>
+      <c r="B41" s="130"/>
       <c r="C41" s="86"/>
-      <c r="D41" s="175"/>
-      <c r="E41" s="86"/>
+      <c r="D41" s="132"/>
+      <c r="E41" s="132"/>
       <c r="F41" s="86"/>
       <c r="G41" s="88"/>
       <c r="H41" s="87"/>
-      <c r="I41" s="120"/>
+      <c r="I41" s="119"/>
       <c r="J41" s="74"/>
-      <c r="K41" s="132"/>
-      <c r="L41" s="132"/>
-      <c r="M41" s="132"/>
-      <c r="N41" s="132"/>
+      <c r="K41" s="147"/>
+      <c r="L41" s="147"/>
+      <c r="M41" s="147"/>
+      <c r="N41" s="147"/>
       <c r="O41" s="43"/>
       <c r="P41" s="72"/>
-      <c r="Q41" s="132"/>
-      <c r="R41" s="132"/>
-      <c r="S41" s="132"/>
-      <c r="T41" s="132"/>
+      <c r="Q41" s="147"/>
+      <c r="R41" s="147"/>
+      <c r="S41" s="147"/>
+      <c r="T41" s="147"/>
       <c r="U41" s="43"/>
       <c r="V41" s="72"/>
-      <c r="W41" s="132"/>
-      <c r="X41" s="132"/>
-      <c r="Y41" s="132"/>
-      <c r="Z41" s="132"/>
+      <c r="W41" s="147"/>
+      <c r="X41" s="147"/>
+      <c r="Y41" s="147"/>
+      <c r="Z41" s="147"/>
       <c r="AA41" s="43"/>
       <c r="AB41" s="72"/>
-      <c r="AC41" s="132"/>
-      <c r="AD41" s="132"/>
-      <c r="AE41" s="132"/>
-      <c r="AF41" s="132"/>
+      <c r="AC41" s="147"/>
+      <c r="AD41" s="147"/>
+      <c r="AE41" s="147"/>
+      <c r="AF41" s="147"/>
       <c r="AG41" s="43"/>
       <c r="AH41" s="72"/>
-      <c r="AI41" s="132"/>
-      <c r="AJ41" s="132"/>
-      <c r="AK41" s="132"/>
-      <c r="AL41" s="132"/>
+      <c r="AI41" s="147"/>
+      <c r="AJ41" s="147"/>
+      <c r="AK41" s="147"/>
+      <c r="AL41" s="147"/>
       <c r="AM41" s="73"/>
       <c r="AN41" s="2"/>
-      <c r="AO41" s="130"/>
-      <c r="AP41" s="130"/>
-      <c r="AQ41" s="130"/>
-      <c r="AR41" s="130"/>
-      <c r="AS41" s="130"/>
-      <c r="AT41" s="130"/>
-      <c r="AU41" s="130"/>
+      <c r="AO41" s="181"/>
+      <c r="AP41" s="181"/>
+      <c r="AQ41" s="181"/>
+      <c r="AR41" s="181"/>
+      <c r="AS41" s="181"/>
+      <c r="AT41" s="181"/>
+      <c r="AU41" s="181"/>
       <c r="AV41" s="22"/>
     </row>
     <row r="42" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="112"/>
-      <c r="B42" s="173"/>
+      <c r="A42" s="111"/>
+      <c r="B42" s="130"/>
       <c r="C42" s="86"/>
-      <c r="D42" s="175"/>
-      <c r="E42" s="86"/>
+      <c r="D42" s="132"/>
+      <c r="E42" s="132"/>
       <c r="F42" s="86"/>
       <c r="G42" s="88"/>
       <c r="H42" s="87"/>
-      <c r="I42" s="120"/>
+      <c r="I42" s="119"/>
       <c r="J42" s="74"/>
-      <c r="K42" s="132"/>
-      <c r="L42" s="132"/>
-      <c r="M42" s="132"/>
-      <c r="N42" s="132"/>
+      <c r="K42" s="147"/>
+      <c r="L42" s="147"/>
+      <c r="M42" s="147"/>
+      <c r="N42" s="147"/>
       <c r="O42" s="43"/>
       <c r="P42" s="72"/>
-      <c r="Q42" s="132"/>
-      <c r="R42" s="132"/>
-      <c r="S42" s="132"/>
-      <c r="T42" s="132"/>
+      <c r="Q42" s="147"/>
+      <c r="R42" s="147"/>
+      <c r="S42" s="147"/>
+      <c r="T42" s="147"/>
       <c r="U42" s="43"/>
       <c r="V42" s="72"/>
-      <c r="W42" s="132"/>
-      <c r="X42" s="132"/>
-      <c r="Y42" s="132"/>
-      <c r="Z42" s="132"/>
+      <c r="W42" s="147"/>
+      <c r="X42" s="147"/>
+      <c r="Y42" s="147"/>
+      <c r="Z42" s="147"/>
       <c r="AA42" s="43"/>
       <c r="AB42" s="72"/>
-      <c r="AC42" s="132"/>
-      <c r="AD42" s="132"/>
-      <c r="AE42" s="132"/>
-      <c r="AF42" s="132"/>
+      <c r="AC42" s="147"/>
+      <c r="AD42" s="147"/>
+      <c r="AE42" s="147"/>
+      <c r="AF42" s="147"/>
       <c r="AG42" s="43"/>
       <c r="AH42" s="72"/>
-      <c r="AI42" s="132"/>
-      <c r="AJ42" s="132"/>
-      <c r="AK42" s="132"/>
-      <c r="AL42" s="132"/>
+      <c r="AI42" s="147"/>
+      <c r="AJ42" s="147"/>
+      <c r="AK42" s="147"/>
+      <c r="AL42" s="147"/>
       <c r="AM42" s="73"/>
       <c r="AN42" s="2"/>
-      <c r="AO42" s="130"/>
-      <c r="AP42" s="130"/>
-      <c r="AQ42" s="130"/>
-      <c r="AR42" s="130"/>
-      <c r="AS42" s="130"/>
-      <c r="AT42" s="130"/>
-      <c r="AU42" s="130"/>
+      <c r="AO42" s="181"/>
+      <c r="AP42" s="181"/>
+      <c r="AQ42" s="181"/>
+      <c r="AR42" s="181"/>
+      <c r="AS42" s="181"/>
+      <c r="AT42" s="181"/>
+      <c r="AU42" s="181"/>
       <c r="AV42" s="22"/>
     </row>
     <row r="43" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="112"/>
-      <c r="B43" s="173"/>
+      <c r="A43" s="111"/>
+      <c r="B43" s="130"/>
       <c r="C43" s="86"/>
-      <c r="D43" s="175"/>
-      <c r="E43" s="86"/>
+      <c r="D43" s="132"/>
+      <c r="E43" s="132"/>
       <c r="F43" s="86"/>
       <c r="G43" s="88"/>
       <c r="H43" s="87"/>
-      <c r="I43" s="120"/>
+      <c r="I43" s="119"/>
       <c r="J43" s="70"/>
-      <c r="K43" s="132"/>
-      <c r="L43" s="132"/>
-      <c r="M43" s="132"/>
-      <c r="N43" s="132"/>
+      <c r="K43" s="147"/>
+      <c r="L43" s="147"/>
+      <c r="M43" s="147"/>
+      <c r="N43" s="147"/>
       <c r="O43" s="43"/>
       <c r="P43" s="72"/>
-      <c r="Q43" s="132"/>
-      <c r="R43" s="132"/>
-      <c r="S43" s="132"/>
-      <c r="T43" s="132"/>
+      <c r="Q43" s="147"/>
+      <c r="R43" s="147"/>
+      <c r="S43" s="147"/>
+      <c r="T43" s="147"/>
       <c r="U43" s="43"/>
       <c r="V43" s="72"/>
-      <c r="W43" s="132"/>
-      <c r="X43" s="132"/>
-      <c r="Y43" s="132"/>
-      <c r="Z43" s="132"/>
+      <c r="W43" s="147"/>
+      <c r="X43" s="147"/>
+      <c r="Y43" s="147"/>
+      <c r="Z43" s="147"/>
       <c r="AA43" s="43"/>
       <c r="AB43" s="72"/>
-      <c r="AC43" s="132"/>
-      <c r="AD43" s="132"/>
-      <c r="AE43" s="132"/>
-      <c r="AF43" s="132"/>
+      <c r="AC43" s="147"/>
+      <c r="AD43" s="147"/>
+      <c r="AE43" s="147"/>
+      <c r="AF43" s="147"/>
       <c r="AG43" s="43"/>
       <c r="AH43" s="72"/>
-      <c r="AI43" s="132"/>
-      <c r="AJ43" s="132"/>
-      <c r="AK43" s="132"/>
-      <c r="AL43" s="132"/>
+      <c r="AI43" s="147"/>
+      <c r="AJ43" s="147"/>
+      <c r="AK43" s="147"/>
+      <c r="AL43" s="147"/>
       <c r="AM43" s="73"/>
       <c r="AN43" s="2"/>
-      <c r="AO43" s="130"/>
-      <c r="AP43" s="130"/>
-      <c r="AQ43" s="130"/>
-      <c r="AR43" s="130"/>
-      <c r="AS43" s="130"/>
-      <c r="AT43" s="130"/>
-      <c r="AU43" s="130"/>
+      <c r="AO43" s="181"/>
+      <c r="AP43" s="181"/>
+      <c r="AQ43" s="181"/>
+      <c r="AR43" s="181"/>
+      <c r="AS43" s="181"/>
+      <c r="AT43" s="181"/>
+      <c r="AU43" s="181"/>
       <c r="AV43" s="22"/>
     </row>
     <row r="44" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="112"/>
-      <c r="B44" s="173"/>
+      <c r="A44" s="111"/>
+      <c r="B44" s="130"/>
       <c r="C44" s="86"/>
-      <c r="D44" s="175"/>
-      <c r="E44" s="86"/>
+      <c r="D44" s="132"/>
+      <c r="E44" s="132"/>
       <c r="F44" s="86"/>
       <c r="G44" s="88"/>
       <c r="H44" s="87"/>
-      <c r="I44" s="120"/>
+      <c r="I44" s="119"/>
       <c r="J44" s="78"/>
-      <c r="K44" s="128" t="s">
+      <c r="K44" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="L44" s="127"/>
-      <c r="M44" s="126"/>
-      <c r="N44" s="127"/>
+      <c r="L44" s="145"/>
+      <c r="M44" s="146"/>
+      <c r="N44" s="145"/>
       <c r="O44" s="43"/>
       <c r="P44" s="72"/>
-      <c r="Q44" s="128" t="s">
+      <c r="Q44" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="R44" s="127"/>
-      <c r="S44" s="126"/>
-      <c r="T44" s="127"/>
+      <c r="R44" s="145"/>
+      <c r="S44" s="146"/>
+      <c r="T44" s="145"/>
       <c r="U44" s="43"/>
       <c r="V44" s="72"/>
-      <c r="W44" s="128" t="s">
+      <c r="W44" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="X44" s="127"/>
-      <c r="Y44" s="126"/>
-      <c r="Z44" s="127"/>
+      <c r="X44" s="145"/>
+      <c r="Y44" s="146"/>
+      <c r="Z44" s="145"/>
       <c r="AA44" s="43"/>
       <c r="AB44" s="72"/>
-      <c r="AC44" s="128" t="s">
+      <c r="AC44" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AD44" s="127"/>
-      <c r="AE44" s="126"/>
-      <c r="AF44" s="127"/>
+      <c r="AD44" s="145"/>
+      <c r="AE44" s="146"/>
+      <c r="AF44" s="145"/>
       <c r="AG44" s="43"/>
       <c r="AH44" s="72"/>
-      <c r="AI44" s="128" t="s">
+      <c r="AI44" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AJ44" s="127"/>
-      <c r="AK44" s="126"/>
-      <c r="AL44" s="127"/>
+      <c r="AJ44" s="145"/>
+      <c r="AK44" s="146"/>
+      <c r="AL44" s="145"/>
       <c r="AM44" s="43"/>
       <c r="AN44" s="2"/>
-      <c r="AO44" s="130"/>
-      <c r="AP44" s="130"/>
-      <c r="AQ44" s="130"/>
-      <c r="AR44" s="130"/>
-      <c r="AS44" s="130"/>
-      <c r="AT44" s="130"/>
-      <c r="AU44" s="130"/>
+      <c r="AO44" s="181"/>
+      <c r="AP44" s="181"/>
+      <c r="AQ44" s="181"/>
+      <c r="AR44" s="181"/>
+      <c r="AS44" s="181"/>
+      <c r="AT44" s="181"/>
+      <c r="AU44" s="181"/>
       <c r="AV44" s="22"/>
     </row>
     <row r="45" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="112"/>
-      <c r="B45" s="173"/>
+      <c r="A45" s="111"/>
+      <c r="B45" s="130"/>
       <c r="C45" s="86"/>
-      <c r="D45" s="175"/>
-      <c r="E45" s="86"/>
+      <c r="D45" s="132"/>
+      <c r="E45" s="132"/>
       <c r="F45" s="86"/>
       <c r="G45" s="88"/>
       <c r="H45" s="87"/>
-      <c r="I45" s="120"/>
+      <c r="I45" s="119"/>
       <c r="J45" s="78"/>
       <c r="K45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="L45" s="72"/>
-      <c r="M45" s="126"/>
-      <c r="N45" s="127"/>
+      <c r="M45" s="146"/>
+      <c r="N45" s="145"/>
       <c r="O45" s="43"/>
       <c r="P45" s="72"/>
       <c r="Q45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="R45" s="72"/>
-      <c r="S45" s="126"/>
-      <c r="T45" s="127"/>
+      <c r="S45" s="146"/>
+      <c r="T45" s="145"/>
       <c r="U45" s="43"/>
       <c r="V45" s="72"/>
       <c r="W45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="X45" s="72"/>
-      <c r="Y45" s="126"/>
-      <c r="Z45" s="127"/>
+      <c r="Y45" s="146"/>
+      <c r="Z45" s="145"/>
       <c r="AA45" s="43"/>
       <c r="AB45" s="72"/>
       <c r="AC45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AD45" s="72"/>
-      <c r="AE45" s="126"/>
-      <c r="AF45" s="127"/>
+      <c r="AE45" s="146"/>
+      <c r="AF45" s="145"/>
       <c r="AG45" s="43"/>
       <c r="AH45" s="72"/>
       <c r="AI45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AJ45" s="72"/>
-      <c r="AK45" s="126"/>
-      <c r="AL45" s="127"/>
-      <c r="AM45" s="131"/>
+      <c r="AK45" s="146"/>
+      <c r="AL45" s="145"/>
+      <c r="AM45" s="149"/>
       <c r="AN45" s="2"/>
-      <c r="AO45" s="130"/>
-      <c r="AP45" s="130"/>
-      <c r="AQ45" s="130"/>
-      <c r="AR45" s="130"/>
-      <c r="AS45" s="130"/>
-      <c r="AT45" s="130"/>
-      <c r="AU45" s="130"/>
+      <c r="AO45" s="181"/>
+      <c r="AP45" s="181"/>
+      <c r="AQ45" s="181"/>
+      <c r="AR45" s="181"/>
+      <c r="AS45" s="181"/>
+      <c r="AT45" s="181"/>
+      <c r="AU45" s="181"/>
       <c r="AV45" s="22"/>
     </row>
     <row r="46" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="112"/>
-      <c r="B46" s="173"/>
+      <c r="A46" s="111"/>
+      <c r="B46" s="130"/>
       <c r="C46" s="86"/>
-      <c r="D46" s="175"/>
-      <c r="E46" s="86"/>
+      <c r="D46" s="132"/>
+      <c r="E46" s="132"/>
       <c r="F46" s="86"/>
       <c r="G46" s="88"/>
       <c r="H46" s="87"/>
-      <c r="I46" s="120"/>
+      <c r="I46" s="119"/>
       <c r="J46" s="76"/>
       <c r="K46" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="L46" s="135"/>
-      <c r="M46" s="135"/>
-      <c r="N46" s="135"/>
+      <c r="L46" s="148"/>
+      <c r="M46" s="148"/>
+      <c r="N46" s="148"/>
       <c r="O46" s="40"/>
       <c r="P46" s="41"/>
       <c r="Q46" s="48" t="s">
         <v>45</v>
       </c>
-      <c r="R46" s="133"/>
-      <c r="S46" s="134"/>
-      <c r="T46" s="134"/>
+      <c r="R46" s="142"/>
+      <c r="S46" s="143"/>
+      <c r="T46" s="143"/>
       <c r="U46" s="40"/>
       <c r="V46" s="41"/>
       <c r="W46" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="X46" s="135"/>
-      <c r="Y46" s="135"/>
-      <c r="Z46" s="135"/>
+      <c r="X46" s="148"/>
+      <c r="Y46" s="148"/>
+      <c r="Z46" s="148"/>
       <c r="AA46" s="40"/>
       <c r="AB46" s="41"/>
       <c r="AC46" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="AD46" s="133"/>
-      <c r="AE46" s="134"/>
-      <c r="AF46" s="134"/>
+      <c r="AD46" s="142"/>
+      <c r="AE46" s="143"/>
+      <c r="AF46" s="143"/>
       <c r="AG46" s="40"/>
       <c r="AH46" s="41"/>
       <c r="AI46" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="AJ46" s="133"/>
-      <c r="AK46" s="134"/>
-      <c r="AL46" s="134"/>
+      <c r="AJ46" s="142"/>
+      <c r="AK46" s="143"/>
+      <c r="AL46" s="143"/>
       <c r="AM46" s="40"/>
       <c r="AN46" s="51"/>
       <c r="AO46" s="51"/>
@@ -4086,15 +4092,15 @@
       <c r="AV46" s="52"/>
     </row>
     <row r="47" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="115"/>
+      <c r="A47" s="114"/>
       <c r="B47" s="45"/>
       <c r="C47" s="42"/>
-      <c r="D47" s="176"/>
-      <c r="E47" s="47"/>
+      <c r="D47" s="133"/>
+      <c r="E47" s="183"/>
       <c r="F47" s="47"/>
       <c r="G47" s="42"/>
-      <c r="H47" s="181"/>
-      <c r="I47" s="124"/>
+      <c r="H47" s="138"/>
+      <c r="I47" s="123"/>
       <c r="J47" s="74"/>
       <c r="K47" s="71"/>
       <c r="L47" s="72"/>
@@ -4136,44 +4142,44 @@
       <c r="AV47" s="54"/>
     </row>
     <row r="48" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="117"/>
+      <c r="A48" s="116"/>
       <c r="B48" s="80"/>
       <c r="C48" s="81"/>
-      <c r="D48" s="177"/>
-      <c r="E48" s="90"/>
+      <c r="D48" s="134"/>
+      <c r="E48" s="184"/>
       <c r="F48" s="90"/>
       <c r="G48" s="81"/>
-      <c r="H48" s="182"/>
-      <c r="I48" s="125"/>
+      <c r="H48" s="139"/>
+      <c r="I48" s="124"/>
       <c r="J48" s="74"/>
-      <c r="K48" s="132"/>
-      <c r="L48" s="132"/>
-      <c r="M48" s="132"/>
-      <c r="N48" s="132"/>
+      <c r="K48" s="147"/>
+      <c r="L48" s="147"/>
+      <c r="M48" s="147"/>
+      <c r="N48" s="147"/>
       <c r="O48" s="43"/>
       <c r="P48" s="72"/>
-      <c r="Q48" s="132"/>
-      <c r="R48" s="132"/>
-      <c r="S48" s="132"/>
-      <c r="T48" s="132"/>
+      <c r="Q48" s="147"/>
+      <c r="R48" s="147"/>
+      <c r="S48" s="147"/>
+      <c r="T48" s="147"/>
       <c r="U48" s="43"/>
       <c r="V48" s="72"/>
-      <c r="W48" s="132"/>
-      <c r="X48" s="132"/>
-      <c r="Y48" s="132"/>
-      <c r="Z48" s="132"/>
+      <c r="W48" s="147"/>
+      <c r="X48" s="147"/>
+      <c r="Y48" s="147"/>
+      <c r="Z48" s="147"/>
       <c r="AA48" s="43"/>
       <c r="AB48" s="72"/>
-      <c r="AC48" s="132"/>
-      <c r="AD48" s="132"/>
-      <c r="AE48" s="132"/>
-      <c r="AF48" s="132"/>
+      <c r="AC48" s="147"/>
+      <c r="AD48" s="147"/>
+      <c r="AE48" s="147"/>
+      <c r="AF48" s="147"/>
       <c r="AG48" s="43"/>
       <c r="AH48" s="72"/>
-      <c r="AI48" s="132"/>
-      <c r="AJ48" s="132"/>
-      <c r="AK48" s="132"/>
-      <c r="AL48" s="132"/>
+      <c r="AI48" s="147"/>
+      <c r="AJ48" s="147"/>
+      <c r="AK48" s="147"/>
+      <c r="AL48" s="147"/>
       <c r="AM48" s="73"/>
       <c r="AN48" s="53"/>
       <c r="AO48" s="53"/>
@@ -4186,44 +4192,44 @@
       <c r="AV48" s="54"/>
     </row>
     <row r="49" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="112"/>
-      <c r="B49" s="173"/>
+      <c r="A49" s="111"/>
+      <c r="B49" s="130"/>
       <c r="C49" s="86"/>
-      <c r="D49" s="175"/>
-      <c r="E49" s="86"/>
+      <c r="D49" s="132"/>
+      <c r="E49" s="132"/>
       <c r="F49" s="86"/>
       <c r="G49" s="88"/>
       <c r="H49" s="87"/>
-      <c r="I49" s="120"/>
+      <c r="I49" s="119"/>
       <c r="J49" s="70"/>
-      <c r="K49" s="132"/>
-      <c r="L49" s="132"/>
-      <c r="M49" s="132"/>
-      <c r="N49" s="132"/>
+      <c r="K49" s="147"/>
+      <c r="L49" s="147"/>
+      <c r="M49" s="147"/>
+      <c r="N49" s="147"/>
       <c r="O49" s="43"/>
       <c r="P49" s="72"/>
-      <c r="Q49" s="132"/>
-      <c r="R49" s="132"/>
-      <c r="S49" s="132"/>
-      <c r="T49" s="132"/>
+      <c r="Q49" s="147"/>
+      <c r="R49" s="147"/>
+      <c r="S49" s="147"/>
+      <c r="T49" s="147"/>
       <c r="U49" s="43"/>
       <c r="V49" s="72"/>
-      <c r="W49" s="132"/>
-      <c r="X49" s="132"/>
-      <c r="Y49" s="132"/>
-      <c r="Z49" s="132"/>
+      <c r="W49" s="147"/>
+      <c r="X49" s="147"/>
+      <c r="Y49" s="147"/>
+      <c r="Z49" s="147"/>
       <c r="AA49" s="43"/>
       <c r="AB49" s="72"/>
-      <c r="AC49" s="132"/>
-      <c r="AD49" s="132"/>
-      <c r="AE49" s="132"/>
-      <c r="AF49" s="132"/>
+      <c r="AC49" s="147"/>
+      <c r="AD49" s="147"/>
+      <c r="AE49" s="147"/>
+      <c r="AF49" s="147"/>
       <c r="AG49" s="43"/>
       <c r="AH49" s="72"/>
-      <c r="AI49" s="132"/>
-      <c r="AJ49" s="132"/>
-      <c r="AK49" s="132"/>
-      <c r="AL49" s="132"/>
+      <c r="AI49" s="147"/>
+      <c r="AJ49" s="147"/>
+      <c r="AK49" s="147"/>
+      <c r="AL49" s="147"/>
       <c r="AM49" s="73"/>
       <c r="AN49" s="53"/>
       <c r="AO49" s="53"/>
@@ -4236,44 +4242,44 @@
       <c r="AV49" s="57"/>
     </row>
     <row r="50" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="112"/>
-      <c r="B50" s="173"/>
+      <c r="A50" s="111"/>
+      <c r="B50" s="130"/>
       <c r="C50" s="86"/>
-      <c r="D50" s="175"/>
-      <c r="E50" s="86"/>
+      <c r="D50" s="132"/>
+      <c r="E50" s="132"/>
       <c r="F50" s="86"/>
       <c r="G50" s="88"/>
       <c r="H50" s="87"/>
-      <c r="I50" s="120"/>
+      <c r="I50" s="119"/>
       <c r="J50" s="74"/>
-      <c r="K50" s="132"/>
-      <c r="L50" s="132"/>
-      <c r="M50" s="132"/>
-      <c r="N50" s="132"/>
+      <c r="K50" s="147"/>
+      <c r="L50" s="147"/>
+      <c r="M50" s="147"/>
+      <c r="N50" s="147"/>
       <c r="O50" s="43"/>
       <c r="P50" s="72"/>
-      <c r="Q50" s="132"/>
-      <c r="R50" s="132"/>
-      <c r="S50" s="132"/>
-      <c r="T50" s="132"/>
+      <c r="Q50" s="147"/>
+      <c r="R50" s="147"/>
+      <c r="S50" s="147"/>
+      <c r="T50" s="147"/>
       <c r="U50" s="43"/>
       <c r="V50" s="72"/>
-      <c r="W50" s="132"/>
-      <c r="X50" s="132"/>
-      <c r="Y50" s="132"/>
-      <c r="Z50" s="132"/>
+      <c r="W50" s="147"/>
+      <c r="X50" s="147"/>
+      <c r="Y50" s="147"/>
+      <c r="Z50" s="147"/>
       <c r="AA50" s="43"/>
       <c r="AB50" s="72"/>
-      <c r="AC50" s="132"/>
-      <c r="AD50" s="132"/>
-      <c r="AE50" s="132"/>
-      <c r="AF50" s="132"/>
+      <c r="AC50" s="147"/>
+      <c r="AD50" s="147"/>
+      <c r="AE50" s="147"/>
+      <c r="AF50" s="147"/>
       <c r="AG50" s="43"/>
       <c r="AH50" s="72"/>
-      <c r="AI50" s="132"/>
-      <c r="AJ50" s="132"/>
-      <c r="AK50" s="132"/>
-      <c r="AL50" s="132"/>
+      <c r="AI50" s="147"/>
+      <c r="AJ50" s="147"/>
+      <c r="AK50" s="147"/>
+      <c r="AL50" s="147"/>
       <c r="AM50" s="73"/>
       <c r="AN50" s="53"/>
       <c r="AO50" s="53"/>
@@ -4286,44 +4292,44 @@
       <c r="AV50" s="57"/>
     </row>
     <row r="51" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="112"/>
-      <c r="B51" s="173"/>
+      <c r="A51" s="111"/>
+      <c r="B51" s="130"/>
       <c r="C51" s="86"/>
-      <c r="D51" s="175"/>
-      <c r="E51" s="86"/>
+      <c r="D51" s="132"/>
+      <c r="E51" s="132"/>
       <c r="F51" s="86"/>
       <c r="G51" s="88"/>
       <c r="H51" s="87"/>
-      <c r="I51" s="120"/>
+      <c r="I51" s="119"/>
       <c r="J51" s="74"/>
-      <c r="K51" s="132"/>
-      <c r="L51" s="132"/>
-      <c r="M51" s="132"/>
-      <c r="N51" s="132"/>
+      <c r="K51" s="147"/>
+      <c r="L51" s="147"/>
+      <c r="M51" s="147"/>
+      <c r="N51" s="147"/>
       <c r="O51" s="43"/>
       <c r="P51" s="72"/>
-      <c r="Q51" s="132"/>
-      <c r="R51" s="132"/>
-      <c r="S51" s="132"/>
-      <c r="T51" s="132"/>
+      <c r="Q51" s="147"/>
+      <c r="R51" s="147"/>
+      <c r="S51" s="147"/>
+      <c r="T51" s="147"/>
       <c r="U51" s="43"/>
       <c r="V51" s="72"/>
-      <c r="W51" s="132"/>
-      <c r="X51" s="132"/>
-      <c r="Y51" s="132"/>
-      <c r="Z51" s="132"/>
+      <c r="W51" s="147"/>
+      <c r="X51" s="147"/>
+      <c r="Y51" s="147"/>
+      <c r="Z51" s="147"/>
       <c r="AA51" s="43"/>
       <c r="AB51" s="72"/>
-      <c r="AC51" s="132"/>
-      <c r="AD51" s="132"/>
-      <c r="AE51" s="132"/>
-      <c r="AF51" s="132"/>
+      <c r="AC51" s="147"/>
+      <c r="AD51" s="147"/>
+      <c r="AE51" s="147"/>
+      <c r="AF51" s="147"/>
       <c r="AG51" s="43"/>
       <c r="AH51" s="72"/>
-      <c r="AI51" s="132"/>
-      <c r="AJ51" s="132"/>
-      <c r="AK51" s="132"/>
-      <c r="AL51" s="132"/>
+      <c r="AI51" s="147"/>
+      <c r="AJ51" s="147"/>
+      <c r="AK51" s="147"/>
+      <c r="AL51" s="147"/>
       <c r="AM51" s="73"/>
       <c r="AN51" s="51"/>
       <c r="AO51" s="51"/>
@@ -4336,224 +4342,224 @@
       <c r="AV51" s="52"/>
     </row>
     <row r="52" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="112"/>
-      <c r="B52" s="173"/>
+      <c r="A52" s="111"/>
+      <c r="B52" s="130"/>
       <c r="C52" s="86"/>
-      <c r="D52" s="175"/>
-      <c r="E52" s="86"/>
+      <c r="D52" s="132"/>
+      <c r="E52" s="132"/>
       <c r="F52" s="86"/>
       <c r="G52" s="88"/>
       <c r="H52" s="87"/>
-      <c r="I52" s="120"/>
+      <c r="I52" s="119"/>
       <c r="J52" s="74"/>
-      <c r="K52" s="132"/>
-      <c r="L52" s="132"/>
-      <c r="M52" s="132"/>
-      <c r="N52" s="132"/>
+      <c r="K52" s="147"/>
+      <c r="L52" s="147"/>
+      <c r="M52" s="147"/>
+      <c r="N52" s="147"/>
       <c r="O52" s="43"/>
       <c r="P52" s="72"/>
-      <c r="Q52" s="132"/>
-      <c r="R52" s="132"/>
-      <c r="S52" s="132"/>
-      <c r="T52" s="132"/>
+      <c r="Q52" s="147"/>
+      <c r="R52" s="147"/>
+      <c r="S52" s="147"/>
+      <c r="T52" s="147"/>
       <c r="U52" s="43"/>
       <c r="V52" s="72"/>
-      <c r="W52" s="132"/>
-      <c r="X52" s="132"/>
-      <c r="Y52" s="132"/>
-      <c r="Z52" s="132"/>
+      <c r="W52" s="147"/>
+      <c r="X52" s="147"/>
+      <c r="Y52" s="147"/>
+      <c r="Z52" s="147"/>
       <c r="AA52" s="43"/>
       <c r="AB52" s="72"/>
-      <c r="AC52" s="132"/>
-      <c r="AD52" s="132"/>
-      <c r="AE52" s="132"/>
-      <c r="AF52" s="132"/>
+      <c r="AC52" s="147"/>
+      <c r="AD52" s="147"/>
+      <c r="AE52" s="147"/>
+      <c r="AF52" s="147"/>
       <c r="AG52" s="43"/>
       <c r="AH52" s="72"/>
-      <c r="AI52" s="132"/>
-      <c r="AJ52" s="132"/>
-      <c r="AK52" s="132"/>
-      <c r="AL52" s="132"/>
+      <c r="AI52" s="147"/>
+      <c r="AJ52" s="147"/>
+      <c r="AK52" s="147"/>
+      <c r="AL52" s="147"/>
       <c r="AM52" s="73"/>
-      <c r="AN52" s="93"/>
-      <c r="AO52" s="93"/>
-      <c r="AP52" s="93"/>
-      <c r="AQ52" s="93"/>
-      <c r="AR52" s="93"/>
-      <c r="AS52" s="93"/>
-      <c r="AT52" s="93"/>
-      <c r="AU52" s="93"/>
+      <c r="AN52" s="92"/>
+      <c r="AO52" s="92"/>
+      <c r="AP52" s="92"/>
+      <c r="AQ52" s="92"/>
+      <c r="AR52" s="92"/>
+      <c r="AS52" s="92"/>
+      <c r="AT52" s="92"/>
+      <c r="AU52" s="92"/>
       <c r="AV52" s="52"/>
     </row>
     <row r="53" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="112"/>
-      <c r="B53" s="173"/>
+      <c r="A53" s="111"/>
+      <c r="B53" s="130"/>
       <c r="C53" s="86"/>
-      <c r="D53" s="175"/>
-      <c r="E53" s="86"/>
+      <c r="D53" s="132"/>
+      <c r="E53" s="132"/>
       <c r="F53" s="86"/>
       <c r="G53" s="88"/>
       <c r="H53" s="87"/>
-      <c r="I53" s="120"/>
+      <c r="I53" s="119"/>
       <c r="J53" s="70"/>
-      <c r="K53" s="132"/>
-      <c r="L53" s="132"/>
-      <c r="M53" s="132"/>
-      <c r="N53" s="132"/>
+      <c r="K53" s="147"/>
+      <c r="L53" s="147"/>
+      <c r="M53" s="147"/>
+      <c r="N53" s="147"/>
       <c r="O53" s="43"/>
       <c r="P53" s="72"/>
-      <c r="Q53" s="132"/>
-      <c r="R53" s="132"/>
-      <c r="S53" s="132"/>
-      <c r="T53" s="132"/>
+      <c r="Q53" s="147"/>
+      <c r="R53" s="147"/>
+      <c r="S53" s="147"/>
+      <c r="T53" s="147"/>
       <c r="U53" s="43"/>
       <c r="V53" s="72"/>
-      <c r="W53" s="132"/>
-      <c r="X53" s="132"/>
-      <c r="Y53" s="132"/>
-      <c r="Z53" s="132"/>
+      <c r="W53" s="147"/>
+      <c r="X53" s="147"/>
+      <c r="Y53" s="147"/>
+      <c r="Z53" s="147"/>
       <c r="AA53" s="43"/>
       <c r="AB53" s="72"/>
-      <c r="AC53" s="132"/>
-      <c r="AD53" s="132"/>
-      <c r="AE53" s="132"/>
-      <c r="AF53" s="132"/>
+      <c r="AC53" s="147"/>
+      <c r="AD53" s="147"/>
+      <c r="AE53" s="147"/>
+      <c r="AF53" s="147"/>
       <c r="AG53" s="43"/>
       <c r="AH53" s="72"/>
-      <c r="AI53" s="132"/>
-      <c r="AJ53" s="132"/>
-      <c r="AK53" s="132"/>
-      <c r="AL53" s="132"/>
+      <c r="AI53" s="147"/>
+      <c r="AJ53" s="147"/>
+      <c r="AK53" s="147"/>
+      <c r="AL53" s="147"/>
       <c r="AM53" s="72"/>
-      <c r="AN53" s="98"/>
-      <c r="AO53" s="94"/>
-      <c r="AP53" s="94"/>
-      <c r="AQ53" s="94"/>
-      <c r="AR53" s="94"/>
-      <c r="AS53" s="94"/>
-      <c r="AT53" s="94"/>
-      <c r="AU53" s="94"/>
-      <c r="AV53" s="99"/>
+      <c r="AN53" s="97"/>
+      <c r="AO53" s="93"/>
+      <c r="AP53" s="93"/>
+      <c r="AQ53" s="93"/>
+      <c r="AR53" s="93"/>
+      <c r="AS53" s="93"/>
+      <c r="AT53" s="93"/>
+      <c r="AU53" s="93"/>
+      <c r="AV53" s="98"/>
     </row>
     <row r="54" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="112"/>
-      <c r="B54" s="173"/>
+      <c r="A54" s="111"/>
+      <c r="B54" s="130"/>
       <c r="C54" s="86"/>
-      <c r="D54" s="175"/>
-      <c r="E54" s="86"/>
+      <c r="D54" s="132"/>
+      <c r="E54" s="132"/>
       <c r="F54" s="86"/>
       <c r="G54" s="88"/>
       <c r="H54" s="87"/>
-      <c r="I54" s="120"/>
+      <c r="I54" s="119"/>
       <c r="J54" s="78"/>
-      <c r="K54" s="128" t="s">
+      <c r="K54" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="L54" s="127"/>
-      <c r="M54" s="126"/>
-      <c r="N54" s="127"/>
+      <c r="L54" s="145"/>
+      <c r="M54" s="146"/>
+      <c r="N54" s="145"/>
       <c r="O54" s="43"/>
       <c r="P54" s="72"/>
-      <c r="Q54" s="128" t="s">
+      <c r="Q54" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="R54" s="127"/>
-      <c r="S54" s="126"/>
-      <c r="T54" s="127"/>
+      <c r="R54" s="145"/>
+      <c r="S54" s="146"/>
+      <c r="T54" s="145"/>
       <c r="U54" s="43"/>
       <c r="V54" s="72"/>
-      <c r="W54" s="128" t="s">
+      <c r="W54" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="X54" s="127"/>
-      <c r="Y54" s="126"/>
-      <c r="Z54" s="127"/>
+      <c r="X54" s="145"/>
+      <c r="Y54" s="146"/>
+      <c r="Z54" s="145"/>
       <c r="AA54" s="43"/>
       <c r="AB54" s="72"/>
-      <c r="AC54" s="128" t="s">
+      <c r="AC54" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AD54" s="127"/>
-      <c r="AE54" s="126"/>
-      <c r="AF54" s="127"/>
+      <c r="AD54" s="145"/>
+      <c r="AE54" s="146"/>
+      <c r="AF54" s="145"/>
       <c r="AG54" s="43"/>
       <c r="AH54" s="72"/>
-      <c r="AI54" s="128" t="s">
+      <c r="AI54" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AJ54" s="127"/>
-      <c r="AK54" s="126"/>
-      <c r="AL54" s="127"/>
+      <c r="AJ54" s="145"/>
+      <c r="AK54" s="146"/>
+      <c r="AL54" s="145"/>
       <c r="AM54" s="72"/>
-      <c r="AN54" s="100"/>
-      <c r="AO54" s="95"/>
-      <c r="AP54" s="96"/>
-      <c r="AQ54" s="97"/>
-      <c r="AR54" s="96"/>
-      <c r="AS54" s="96"/>
-      <c r="AT54" s="96"/>
-      <c r="AU54" s="96"/>
-      <c r="AV54" s="101"/>
+      <c r="AN54" s="99"/>
+      <c r="AO54" s="94"/>
+      <c r="AP54" s="95"/>
+      <c r="AQ54" s="96"/>
+      <c r="AR54" s="95"/>
+      <c r="AS54" s="95"/>
+      <c r="AT54" s="95"/>
+      <c r="AU54" s="95"/>
+      <c r="AV54" s="100"/>
     </row>
     <row r="55" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="112"/>
-      <c r="B55" s="173"/>
+      <c r="A55" s="111"/>
+      <c r="B55" s="130"/>
       <c r="C55" s="86"/>
-      <c r="D55" s="175"/>
-      <c r="E55" s="86"/>
+      <c r="D55" s="132"/>
+      <c r="E55" s="132"/>
       <c r="F55" s="86"/>
       <c r="G55" s="88"/>
       <c r="H55" s="87"/>
-      <c r="I55" s="120"/>
+      <c r="I55" s="119"/>
       <c r="J55" s="79"/>
       <c r="K55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="L55" s="81"/>
-      <c r="M55" s="166"/>
-      <c r="N55" s="167"/>
+      <c r="M55" s="140"/>
+      <c r="N55" s="141"/>
       <c r="O55" s="82"/>
       <c r="P55" s="81"/>
       <c r="Q55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="R55" s="81"/>
-      <c r="S55" s="166"/>
-      <c r="T55" s="167"/>
+      <c r="S55" s="140"/>
+      <c r="T55" s="141"/>
       <c r="U55" s="82"/>
       <c r="V55" s="81"/>
       <c r="W55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="X55" s="81"/>
-      <c r="Y55" s="166"/>
-      <c r="Z55" s="167"/>
+      <c r="Y55" s="140"/>
+      <c r="Z55" s="141"/>
       <c r="AA55" s="82"/>
       <c r="AB55" s="81"/>
       <c r="AC55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="AD55" s="81"/>
-      <c r="AE55" s="166"/>
-      <c r="AF55" s="167"/>
+      <c r="AE55" s="140"/>
+      <c r="AF55" s="141"/>
       <c r="AG55" s="82"/>
       <c r="AH55" s="81"/>
       <c r="AI55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="AJ55" s="81"/>
-      <c r="AK55" s="166"/>
-      <c r="AL55" s="167"/>
-      <c r="AM55" s="167"/>
-      <c r="AN55" s="102"/>
-      <c r="AO55" s="103"/>
-      <c r="AP55" s="104"/>
-      <c r="AQ55" s="105"/>
-      <c r="AR55" s="104"/>
-      <c r="AS55" s="104"/>
-      <c r="AT55" s="104"/>
-      <c r="AU55" s="104"/>
-      <c r="AV55" s="106"/>
+      <c r="AK55" s="140"/>
+      <c r="AL55" s="141"/>
+      <c r="AM55" s="141"/>
+      <c r="AN55" s="101"/>
+      <c r="AO55" s="102"/>
+      <c r="AP55" s="103"/>
+      <c r="AQ55" s="104"/>
+      <c r="AR55" s="103"/>
+      <c r="AS55" s="103"/>
+      <c r="AT55" s="103"/>
+      <c r="AU55" s="103"/>
+      <c r="AV55" s="105"/>
     </row>
     <row r="56" spans="1:48" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A56" s="45" t="s">
@@ -4609,107 +4615,16 @@
     </row>
   </sheetData>
   <mergeCells count="135">
-    <mergeCell ref="M55:N55"/>
-    <mergeCell ref="S55:T55"/>
-    <mergeCell ref="Y55:Z55"/>
-    <mergeCell ref="AE55:AF55"/>
-    <mergeCell ref="AK55:AM55"/>
-    <mergeCell ref="R46:T46"/>
-    <mergeCell ref="K54:L54"/>
-    <mergeCell ref="M54:N54"/>
-    <mergeCell ref="Q54:R54"/>
-    <mergeCell ref="S54:T54"/>
-    <mergeCell ref="W54:X54"/>
-    <mergeCell ref="Y54:Z54"/>
-    <mergeCell ref="K48:N53"/>
-    <mergeCell ref="Q48:T53"/>
-    <mergeCell ref="W48:Z53"/>
-    <mergeCell ref="L46:N46"/>
-    <mergeCell ref="X46:Z46"/>
-    <mergeCell ref="M45:N45"/>
-    <mergeCell ref="S45:T45"/>
-    <mergeCell ref="Y45:Z45"/>
-    <mergeCell ref="AE45:AF45"/>
-    <mergeCell ref="AK45:AM45"/>
-    <mergeCell ref="R36:T36"/>
-    <mergeCell ref="K44:L44"/>
-    <mergeCell ref="M44:N44"/>
-    <mergeCell ref="Q44:R44"/>
-    <mergeCell ref="S44:T44"/>
-    <mergeCell ref="W44:X44"/>
-    <mergeCell ref="Y44:Z44"/>
-    <mergeCell ref="K38:N43"/>
-    <mergeCell ref="Q38:T43"/>
-    <mergeCell ref="W38:Z43"/>
-    <mergeCell ref="L36:N36"/>
-    <mergeCell ref="X36:Z36"/>
-    <mergeCell ref="AJ36:AL36"/>
-    <mergeCell ref="AH3:AM3"/>
-    <mergeCell ref="AN3:AP3"/>
-    <mergeCell ref="AQ3:AS3"/>
-    <mergeCell ref="AT3:AV3"/>
-    <mergeCell ref="AH4:AM4"/>
-    <mergeCell ref="AN4:AP7"/>
-    <mergeCell ref="AQ4:AS7"/>
-    <mergeCell ref="AT4:AV7"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="J8:AG8"/>
-    <mergeCell ref="AH8:AM8"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="J9:AG9"/>
-    <mergeCell ref="AH9:AM9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="J10:AG10"/>
-    <mergeCell ref="AH10:AM10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:AG11"/>
-    <mergeCell ref="AH11:AM11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="J12:AG12"/>
-    <mergeCell ref="AH12:AM12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="J13:AG13"/>
-    <mergeCell ref="AH13:AM13"/>
-    <mergeCell ref="A14:AM15"/>
-    <mergeCell ref="AN15:AV15"/>
-    <mergeCell ref="L16:N16"/>
-    <mergeCell ref="R16:T16"/>
-    <mergeCell ref="X16:Z16"/>
-    <mergeCell ref="AD16:AF16"/>
-    <mergeCell ref="AJ16:AL16"/>
-    <mergeCell ref="AI24:AJ24"/>
-    <mergeCell ref="AK24:AL24"/>
-    <mergeCell ref="K18:N23"/>
-    <mergeCell ref="Q18:T23"/>
-    <mergeCell ref="W18:Z23"/>
-    <mergeCell ref="AC18:AF23"/>
-    <mergeCell ref="AI18:AL23"/>
-    <mergeCell ref="W24:X24"/>
-    <mergeCell ref="Y24:Z24"/>
-    <mergeCell ref="AC24:AD24"/>
-    <mergeCell ref="AE24:AF24"/>
-    <mergeCell ref="X26:Z26"/>
-    <mergeCell ref="L26:N26"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="S24:T24"/>
-    <mergeCell ref="Q34:R34"/>
-    <mergeCell ref="S34:T34"/>
-    <mergeCell ref="W34:X34"/>
-    <mergeCell ref="R26:T26"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="S25:T25"/>
-    <mergeCell ref="Y25:Z25"/>
-    <mergeCell ref="K28:N33"/>
-    <mergeCell ref="Q28:T33"/>
-    <mergeCell ref="W28:Z33"/>
+    <mergeCell ref="AK34:AL34"/>
+    <mergeCell ref="AC34:AD34"/>
+    <mergeCell ref="AE34:AF34"/>
+    <mergeCell ref="AI34:AJ34"/>
+    <mergeCell ref="Y34:Z34"/>
+    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="S35:T35"/>
+    <mergeCell ref="Y35:Z35"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="M34:N34"/>
     <mergeCell ref="AE25:AF25"/>
     <mergeCell ref="AK25:AL25"/>
     <mergeCell ref="AO26:AU45"/>
@@ -4734,16 +4649,107 @@
     <mergeCell ref="AC38:AF43"/>
     <mergeCell ref="AI38:AL43"/>
     <mergeCell ref="AD36:AF36"/>
-    <mergeCell ref="AK34:AL34"/>
-    <mergeCell ref="AC34:AD34"/>
-    <mergeCell ref="AE34:AF34"/>
-    <mergeCell ref="AI34:AJ34"/>
-    <mergeCell ref="Y34:Z34"/>
-    <mergeCell ref="M35:N35"/>
-    <mergeCell ref="S35:T35"/>
-    <mergeCell ref="Y35:Z35"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="X26:Z26"/>
+    <mergeCell ref="L26:N26"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="Q34:R34"/>
+    <mergeCell ref="S34:T34"/>
+    <mergeCell ref="W34:X34"/>
+    <mergeCell ref="R26:T26"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="S25:T25"/>
+    <mergeCell ref="Y25:Z25"/>
+    <mergeCell ref="K28:N33"/>
+    <mergeCell ref="Q28:T33"/>
+    <mergeCell ref="W28:Z33"/>
+    <mergeCell ref="AN15:AV15"/>
+    <mergeCell ref="L16:N16"/>
+    <mergeCell ref="R16:T16"/>
+    <mergeCell ref="X16:Z16"/>
+    <mergeCell ref="AD16:AF16"/>
+    <mergeCell ref="AJ16:AL16"/>
+    <mergeCell ref="AI24:AJ24"/>
+    <mergeCell ref="AK24:AL24"/>
+    <mergeCell ref="K18:N23"/>
+    <mergeCell ref="Q18:T23"/>
+    <mergeCell ref="W18:Z23"/>
+    <mergeCell ref="AC18:AF23"/>
+    <mergeCell ref="AI18:AL23"/>
+    <mergeCell ref="W24:X24"/>
+    <mergeCell ref="Y24:Z24"/>
+    <mergeCell ref="AC24:AD24"/>
+    <mergeCell ref="AE24:AF24"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="J12:AG12"/>
+    <mergeCell ref="AH12:AM12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="J13:AG13"/>
+    <mergeCell ref="AH13:AM13"/>
+    <mergeCell ref="A14:AM15"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="J9:AG9"/>
+    <mergeCell ref="AH9:AM9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="J10:AG10"/>
+    <mergeCell ref="AH10:AM10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:AG11"/>
+    <mergeCell ref="AH11:AM11"/>
+    <mergeCell ref="AH3:AM3"/>
+    <mergeCell ref="AN3:AP3"/>
+    <mergeCell ref="AQ3:AS3"/>
+    <mergeCell ref="AT3:AV3"/>
+    <mergeCell ref="AH4:AM4"/>
+    <mergeCell ref="AN4:AP7"/>
+    <mergeCell ref="AQ4:AS7"/>
+    <mergeCell ref="AT4:AV7"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="J8:AG8"/>
+    <mergeCell ref="AH8:AM8"/>
+    <mergeCell ref="M45:N45"/>
+    <mergeCell ref="S45:T45"/>
+    <mergeCell ref="Y45:Z45"/>
+    <mergeCell ref="AE45:AF45"/>
+    <mergeCell ref="AK45:AM45"/>
+    <mergeCell ref="R36:T36"/>
+    <mergeCell ref="K44:L44"/>
+    <mergeCell ref="M44:N44"/>
+    <mergeCell ref="Q44:R44"/>
+    <mergeCell ref="S44:T44"/>
+    <mergeCell ref="W44:X44"/>
+    <mergeCell ref="Y44:Z44"/>
+    <mergeCell ref="K38:N43"/>
+    <mergeCell ref="Q38:T43"/>
+    <mergeCell ref="W38:Z43"/>
+    <mergeCell ref="L36:N36"/>
+    <mergeCell ref="X36:Z36"/>
+    <mergeCell ref="AJ36:AL36"/>
+    <mergeCell ref="M55:N55"/>
+    <mergeCell ref="S55:T55"/>
+    <mergeCell ref="Y55:Z55"/>
+    <mergeCell ref="AE55:AF55"/>
+    <mergeCell ref="AK55:AM55"/>
+    <mergeCell ref="R46:T46"/>
+    <mergeCell ref="K54:L54"/>
+    <mergeCell ref="M54:N54"/>
+    <mergeCell ref="Q54:R54"/>
+    <mergeCell ref="S54:T54"/>
+    <mergeCell ref="W54:X54"/>
+    <mergeCell ref="Y54:Z54"/>
+    <mergeCell ref="K48:N53"/>
+    <mergeCell ref="Q48:T53"/>
+    <mergeCell ref="W48:Z53"/>
+    <mergeCell ref="L46:N46"/>
+    <mergeCell ref="X46:Z46"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.1" right="0.1" top="0.1" bottom="0.1" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
Resolved template header in SDS-V2
</commit_message>
<xml_diff>
--- a/apps/ENG-Backend/api/engineer/mtc/templates/sds_template.xlsx
+++ b/apps/ENG-Backend/api/engineer/mtc/templates/sds_template.xlsx
@@ -205,7 +205,7 @@
     <numFmt numFmtId="190" formatCode="0.000"/>
     <numFmt numFmtId="191" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="29" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -362,12 +362,6 @@
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
     <font>
@@ -1140,13 +1134,10 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="190" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1155,139 +1146,142 @@
     <xf numFmtId="190" fontId="16" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="190" fontId="26" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="189" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="1" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="188" fontId="1" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="189" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="190" fontId="26" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="190" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1785,29 +1779,29 @@
       <c r="AE3" s="11"/>
       <c r="AF3" s="11"/>
       <c r="AG3" s="16"/>
-      <c r="AH3" s="150" t="s">
+      <c r="AH3" s="167" t="s">
         <v>6</v>
       </c>
-      <c r="AI3" s="151"/>
-      <c r="AJ3" s="151"/>
-      <c r="AK3" s="151"/>
-      <c r="AL3" s="151"/>
-      <c r="AM3" s="152"/>
-      <c r="AN3" s="150" t="s">
+      <c r="AI3" s="168"/>
+      <c r="AJ3" s="168"/>
+      <c r="AK3" s="168"/>
+      <c r="AL3" s="168"/>
+      <c r="AM3" s="169"/>
+      <c r="AN3" s="167" t="s">
         <v>7</v>
       </c>
-      <c r="AO3" s="151"/>
-      <c r="AP3" s="152"/>
-      <c r="AQ3" s="150" t="s">
+      <c r="AO3" s="168"/>
+      <c r="AP3" s="169"/>
+      <c r="AQ3" s="167" t="s">
         <v>8</v>
       </c>
-      <c r="AR3" s="151"/>
-      <c r="AS3" s="152"/>
-      <c r="AT3" s="150" t="s">
+      <c r="AR3" s="168"/>
+      <c r="AS3" s="169"/>
+      <c r="AT3" s="167" t="s">
         <v>9</v>
       </c>
-      <c r="AU3" s="151"/>
-      <c r="AV3" s="152"/>
+      <c r="AU3" s="168"/>
+      <c r="AV3" s="169"/>
     </row>
     <row r="4" spans="1:48" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
@@ -1851,21 +1845,21 @@
       <c r="AE4" s="11"/>
       <c r="AF4" s="11"/>
       <c r="AG4" s="11"/>
-      <c r="AH4" s="153"/>
-      <c r="AI4" s="154"/>
-      <c r="AJ4" s="154"/>
-      <c r="AK4" s="154"/>
-      <c r="AL4" s="154"/>
-      <c r="AM4" s="155"/>
-      <c r="AN4" s="156"/>
-      <c r="AO4" s="157"/>
-      <c r="AP4" s="157"/>
-      <c r="AQ4" s="156"/>
-      <c r="AR4" s="157"/>
-      <c r="AS4" s="162"/>
-      <c r="AT4" s="156"/>
-      <c r="AU4" s="157"/>
-      <c r="AV4" s="162"/>
+      <c r="AH4" s="155"/>
+      <c r="AI4" s="156"/>
+      <c r="AJ4" s="156"/>
+      <c r="AK4" s="156"/>
+      <c r="AL4" s="156"/>
+      <c r="AM4" s="158"/>
+      <c r="AN4" s="170"/>
+      <c r="AO4" s="171"/>
+      <c r="AP4" s="171"/>
+      <c r="AQ4" s="170"/>
+      <c r="AR4" s="171"/>
+      <c r="AS4" s="176"/>
+      <c r="AT4" s="170"/>
+      <c r="AU4" s="171"/>
+      <c r="AV4" s="176"/>
     </row>
     <row r="5" spans="1:48" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
@@ -1913,15 +1907,15 @@
       <c r="AK5" s="3"/>
       <c r="AL5" s="3"/>
       <c r="AM5" s="27"/>
-      <c r="AN5" s="158"/>
-      <c r="AO5" s="159"/>
-      <c r="AP5" s="159"/>
-      <c r="AQ5" s="158"/>
-      <c r="AR5" s="159"/>
-      <c r="AS5" s="163"/>
-      <c r="AT5" s="158"/>
-      <c r="AU5" s="159"/>
-      <c r="AV5" s="163"/>
+      <c r="AN5" s="172"/>
+      <c r="AO5" s="173"/>
+      <c r="AP5" s="173"/>
+      <c r="AQ5" s="172"/>
+      <c r="AR5" s="173"/>
+      <c r="AS5" s="177"/>
+      <c r="AT5" s="172"/>
+      <c r="AU5" s="173"/>
+      <c r="AV5" s="177"/>
     </row>
     <row r="6" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
@@ -1965,15 +1959,15 @@
       <c r="AK6" s="1"/>
       <c r="AL6" s="1"/>
       <c r="AM6" s="30"/>
-      <c r="AN6" s="158"/>
-      <c r="AO6" s="159"/>
-      <c r="AP6" s="159"/>
-      <c r="AQ6" s="158"/>
-      <c r="AR6" s="159"/>
-      <c r="AS6" s="163"/>
-      <c r="AT6" s="158"/>
-      <c r="AU6" s="159"/>
-      <c r="AV6" s="163"/>
+      <c r="AN6" s="172"/>
+      <c r="AO6" s="173"/>
+      <c r="AP6" s="173"/>
+      <c r="AQ6" s="172"/>
+      <c r="AR6" s="173"/>
+      <c r="AS6" s="177"/>
+      <c r="AT6" s="172"/>
+      <c r="AU6" s="173"/>
+      <c r="AV6" s="177"/>
     </row>
     <row r="7" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="31"/>
@@ -2015,66 +2009,66 @@
       <c r="AK7" s="32"/>
       <c r="AL7" s="32"/>
       <c r="AM7" s="33"/>
-      <c r="AN7" s="160"/>
-      <c r="AO7" s="161"/>
-      <c r="AP7" s="161"/>
-      <c r="AQ7" s="160"/>
-      <c r="AR7" s="161"/>
-      <c r="AS7" s="164"/>
-      <c r="AT7" s="160"/>
-      <c r="AU7" s="161"/>
-      <c r="AV7" s="164"/>
+      <c r="AN7" s="174"/>
+      <c r="AO7" s="175"/>
+      <c r="AP7" s="175"/>
+      <c r="AQ7" s="174"/>
+      <c r="AR7" s="175"/>
+      <c r="AS7" s="178"/>
+      <c r="AT7" s="174"/>
+      <c r="AU7" s="175"/>
+      <c r="AV7" s="178"/>
     </row>
     <row r="8" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="165" t="s">
+      <c r="B8" s="179" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="166"/>
-      <c r="D8" s="166"/>
-      <c r="E8" s="166"/>
-      <c r="F8" s="166"/>
-      <c r="G8" s="167" t="s">
+      <c r="C8" s="165"/>
+      <c r="D8" s="165"/>
+      <c r="E8" s="165"/>
+      <c r="F8" s="165"/>
+      <c r="G8" s="180" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="166"/>
-      <c r="I8" s="168"/>
-      <c r="J8" s="150" t="s">
+      <c r="H8" s="165"/>
+      <c r="I8" s="181"/>
+      <c r="J8" s="167" t="s">
         <v>21</v>
       </c>
-      <c r="K8" s="151"/>
-      <c r="L8" s="151"/>
-      <c r="M8" s="151"/>
-      <c r="N8" s="151"/>
-      <c r="O8" s="151"/>
-      <c r="P8" s="151"/>
-      <c r="Q8" s="151"/>
-      <c r="R8" s="151"/>
-      <c r="S8" s="151"/>
-      <c r="T8" s="151"/>
-      <c r="U8" s="151"/>
-      <c r="V8" s="151"/>
-      <c r="W8" s="151"/>
-      <c r="X8" s="151"/>
-      <c r="Y8" s="151"/>
-      <c r="Z8" s="151"/>
-      <c r="AA8" s="151"/>
-      <c r="AB8" s="151"/>
-      <c r="AC8" s="151"/>
-      <c r="AD8" s="151"/>
-      <c r="AE8" s="151"/>
-      <c r="AF8" s="151"/>
-      <c r="AG8" s="152"/>
-      <c r="AH8" s="150" t="s">
+      <c r="K8" s="168"/>
+      <c r="L8" s="168"/>
+      <c r="M8" s="168"/>
+      <c r="N8" s="168"/>
+      <c r="O8" s="168"/>
+      <c r="P8" s="168"/>
+      <c r="Q8" s="168"/>
+      <c r="R8" s="168"/>
+      <c r="S8" s="168"/>
+      <c r="T8" s="168"/>
+      <c r="U8" s="168"/>
+      <c r="V8" s="168"/>
+      <c r="W8" s="168"/>
+      <c r="X8" s="168"/>
+      <c r="Y8" s="168"/>
+      <c r="Z8" s="168"/>
+      <c r="AA8" s="168"/>
+      <c r="AB8" s="168"/>
+      <c r="AC8" s="168"/>
+      <c r="AD8" s="168"/>
+      <c r="AE8" s="168"/>
+      <c r="AF8" s="168"/>
+      <c r="AG8" s="169"/>
+      <c r="AH8" s="167" t="s">
         <v>22</v>
       </c>
-      <c r="AI8" s="151"/>
-      <c r="AJ8" s="151"/>
-      <c r="AK8" s="151"/>
-      <c r="AL8" s="151"/>
-      <c r="AM8" s="152"/>
+      <c r="AI8" s="168"/>
+      <c r="AJ8" s="168"/>
+      <c r="AK8" s="168"/>
+      <c r="AL8" s="168"/>
+      <c r="AM8" s="169"/>
       <c r="AN8" s="29" t="s">
         <v>23</v>
       </c>
@@ -2089,44 +2083,44 @@
     </row>
     <row r="9" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="108"/>
-      <c r="B9" s="153"/>
-      <c r="C9" s="154"/>
-      <c r="D9" s="154"/>
-      <c r="E9" s="154"/>
-      <c r="F9" s="154"/>
-      <c r="G9" s="169"/>
-      <c r="H9" s="154"/>
-      <c r="I9" s="155"/>
-      <c r="J9" s="170"/>
-      <c r="K9" s="171"/>
-      <c r="L9" s="171"/>
-      <c r="M9" s="171"/>
-      <c r="N9" s="171"/>
-      <c r="O9" s="171"/>
-      <c r="P9" s="171"/>
-      <c r="Q9" s="171"/>
-      <c r="R9" s="171"/>
-      <c r="S9" s="171"/>
-      <c r="T9" s="171"/>
-      <c r="U9" s="171"/>
-      <c r="V9" s="171"/>
-      <c r="W9" s="171"/>
-      <c r="X9" s="171"/>
-      <c r="Y9" s="171"/>
-      <c r="Z9" s="171"/>
-      <c r="AA9" s="171"/>
-      <c r="AB9" s="171"/>
-      <c r="AC9" s="171"/>
-      <c r="AD9" s="171"/>
-      <c r="AE9" s="171"/>
-      <c r="AF9" s="171"/>
-      <c r="AG9" s="172"/>
-      <c r="AH9" s="170"/>
-      <c r="AI9" s="171"/>
-      <c r="AJ9" s="171"/>
-      <c r="AK9" s="171"/>
-      <c r="AL9" s="171"/>
-      <c r="AM9" s="172"/>
+      <c r="B9" s="155"/>
+      <c r="C9" s="156"/>
+      <c r="D9" s="156"/>
+      <c r="E9" s="156"/>
+      <c r="F9" s="156"/>
+      <c r="G9" s="157"/>
+      <c r="H9" s="156"/>
+      <c r="I9" s="158"/>
+      <c r="J9" s="159"/>
+      <c r="K9" s="160"/>
+      <c r="L9" s="160"/>
+      <c r="M9" s="160"/>
+      <c r="N9" s="160"/>
+      <c r="O9" s="160"/>
+      <c r="P9" s="160"/>
+      <c r="Q9" s="160"/>
+      <c r="R9" s="160"/>
+      <c r="S9" s="160"/>
+      <c r="T9" s="160"/>
+      <c r="U9" s="160"/>
+      <c r="V9" s="160"/>
+      <c r="W9" s="160"/>
+      <c r="X9" s="160"/>
+      <c r="Y9" s="160"/>
+      <c r="Z9" s="160"/>
+      <c r="AA9" s="160"/>
+      <c r="AB9" s="160"/>
+      <c r="AC9" s="160"/>
+      <c r="AD9" s="160"/>
+      <c r="AE9" s="160"/>
+      <c r="AF9" s="160"/>
+      <c r="AG9" s="161"/>
+      <c r="AH9" s="159"/>
+      <c r="AI9" s="160"/>
+      <c r="AJ9" s="160"/>
+      <c r="AK9" s="160"/>
+      <c r="AL9" s="160"/>
+      <c r="AM9" s="161"/>
       <c r="AN9" s="35"/>
       <c r="AO9" s="2"/>
       <c r="AP9" s="2"/>
@@ -2139,44 +2133,44 @@
     </row>
     <row r="10" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="108"/>
-      <c r="B10" s="153"/>
-      <c r="C10" s="154"/>
-      <c r="D10" s="154"/>
-      <c r="E10" s="154"/>
-      <c r="F10" s="154"/>
-      <c r="G10" s="169"/>
-      <c r="H10" s="154"/>
-      <c r="I10" s="155"/>
-      <c r="J10" s="170"/>
-      <c r="K10" s="171"/>
-      <c r="L10" s="171"/>
-      <c r="M10" s="171"/>
-      <c r="N10" s="171"/>
-      <c r="O10" s="171"/>
-      <c r="P10" s="171"/>
-      <c r="Q10" s="171"/>
-      <c r="R10" s="171"/>
-      <c r="S10" s="171"/>
-      <c r="T10" s="171"/>
-      <c r="U10" s="171"/>
-      <c r="V10" s="171"/>
-      <c r="W10" s="171"/>
-      <c r="X10" s="171"/>
-      <c r="Y10" s="171"/>
-      <c r="Z10" s="171"/>
-      <c r="AA10" s="171"/>
-      <c r="AB10" s="171"/>
-      <c r="AC10" s="171"/>
-      <c r="AD10" s="171"/>
-      <c r="AE10" s="171"/>
-      <c r="AF10" s="171"/>
-      <c r="AG10" s="172"/>
-      <c r="AH10" s="170"/>
-      <c r="AI10" s="171"/>
-      <c r="AJ10" s="171"/>
-      <c r="AK10" s="171"/>
-      <c r="AL10" s="171"/>
-      <c r="AM10" s="172"/>
+      <c r="B10" s="155"/>
+      <c r="C10" s="156"/>
+      <c r="D10" s="156"/>
+      <c r="E10" s="156"/>
+      <c r="F10" s="156"/>
+      <c r="G10" s="157"/>
+      <c r="H10" s="156"/>
+      <c r="I10" s="158"/>
+      <c r="J10" s="159"/>
+      <c r="K10" s="160"/>
+      <c r="L10" s="160"/>
+      <c r="M10" s="160"/>
+      <c r="N10" s="160"/>
+      <c r="O10" s="160"/>
+      <c r="P10" s="160"/>
+      <c r="Q10" s="160"/>
+      <c r="R10" s="160"/>
+      <c r="S10" s="160"/>
+      <c r="T10" s="160"/>
+      <c r="U10" s="160"/>
+      <c r="V10" s="160"/>
+      <c r="W10" s="160"/>
+      <c r="X10" s="160"/>
+      <c r="Y10" s="160"/>
+      <c r="Z10" s="160"/>
+      <c r="AA10" s="160"/>
+      <c r="AB10" s="160"/>
+      <c r="AC10" s="160"/>
+      <c r="AD10" s="160"/>
+      <c r="AE10" s="160"/>
+      <c r="AF10" s="160"/>
+      <c r="AG10" s="161"/>
+      <c r="AH10" s="159"/>
+      <c r="AI10" s="160"/>
+      <c r="AJ10" s="160"/>
+      <c r="AK10" s="160"/>
+      <c r="AL10" s="160"/>
+      <c r="AM10" s="161"/>
       <c r="AN10" s="35"/>
       <c r="AO10" s="2"/>
       <c r="AP10" s="2"/>
@@ -2189,44 +2183,44 @@
     </row>
     <row r="11" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="108"/>
-      <c r="B11" s="153"/>
-      <c r="C11" s="154"/>
-      <c r="D11" s="154"/>
-      <c r="E11" s="154"/>
-      <c r="F11" s="154"/>
-      <c r="G11" s="169"/>
-      <c r="H11" s="154"/>
-      <c r="I11" s="155"/>
-      <c r="J11" s="170"/>
-      <c r="K11" s="171"/>
-      <c r="L11" s="171"/>
-      <c r="M11" s="171"/>
-      <c r="N11" s="171"/>
-      <c r="O11" s="171"/>
-      <c r="P11" s="171"/>
-      <c r="Q11" s="171"/>
-      <c r="R11" s="171"/>
-      <c r="S11" s="171"/>
-      <c r="T11" s="171"/>
-      <c r="U11" s="171"/>
-      <c r="V11" s="171"/>
-      <c r="W11" s="171"/>
-      <c r="X11" s="171"/>
-      <c r="Y11" s="171"/>
-      <c r="Z11" s="171"/>
-      <c r="AA11" s="171"/>
-      <c r="AB11" s="171"/>
-      <c r="AC11" s="171"/>
-      <c r="AD11" s="171"/>
-      <c r="AE11" s="171"/>
-      <c r="AF11" s="171"/>
-      <c r="AG11" s="172"/>
-      <c r="AH11" s="170"/>
-      <c r="AI11" s="171"/>
-      <c r="AJ11" s="171"/>
-      <c r="AK11" s="171"/>
-      <c r="AL11" s="171"/>
-      <c r="AM11" s="172"/>
+      <c r="B11" s="155"/>
+      <c r="C11" s="156"/>
+      <c r="D11" s="156"/>
+      <c r="E11" s="156"/>
+      <c r="F11" s="156"/>
+      <c r="G11" s="157"/>
+      <c r="H11" s="156"/>
+      <c r="I11" s="158"/>
+      <c r="J11" s="159"/>
+      <c r="K11" s="160"/>
+      <c r="L11" s="160"/>
+      <c r="M11" s="160"/>
+      <c r="N11" s="160"/>
+      <c r="O11" s="160"/>
+      <c r="P11" s="160"/>
+      <c r="Q11" s="160"/>
+      <c r="R11" s="160"/>
+      <c r="S11" s="160"/>
+      <c r="T11" s="160"/>
+      <c r="U11" s="160"/>
+      <c r="V11" s="160"/>
+      <c r="W11" s="160"/>
+      <c r="X11" s="160"/>
+      <c r="Y11" s="160"/>
+      <c r="Z11" s="160"/>
+      <c r="AA11" s="160"/>
+      <c r="AB11" s="160"/>
+      <c r="AC11" s="160"/>
+      <c r="AD11" s="160"/>
+      <c r="AE11" s="160"/>
+      <c r="AF11" s="160"/>
+      <c r="AG11" s="161"/>
+      <c r="AH11" s="159"/>
+      <c r="AI11" s="160"/>
+      <c r="AJ11" s="160"/>
+      <c r="AK11" s="160"/>
+      <c r="AL11" s="160"/>
+      <c r="AM11" s="161"/>
       <c r="AN11" s="18" t="s">
         <v>24</v>
       </c>
@@ -2241,44 +2235,44 @@
     </row>
     <row r="12" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="108"/>
-      <c r="B12" s="153"/>
-      <c r="C12" s="154"/>
-      <c r="D12" s="154"/>
-      <c r="E12" s="154"/>
-      <c r="F12" s="154"/>
-      <c r="G12" s="169"/>
-      <c r="H12" s="154"/>
-      <c r="I12" s="155"/>
-      <c r="J12" s="170"/>
-      <c r="K12" s="171"/>
-      <c r="L12" s="171"/>
-      <c r="M12" s="171"/>
-      <c r="N12" s="171"/>
-      <c r="O12" s="171"/>
-      <c r="P12" s="171"/>
-      <c r="Q12" s="171"/>
-      <c r="R12" s="171"/>
-      <c r="S12" s="171"/>
-      <c r="T12" s="171"/>
-      <c r="U12" s="171"/>
-      <c r="V12" s="171"/>
-      <c r="W12" s="171"/>
-      <c r="X12" s="171"/>
-      <c r="Y12" s="171"/>
-      <c r="Z12" s="171"/>
-      <c r="AA12" s="171"/>
-      <c r="AB12" s="171"/>
-      <c r="AC12" s="171"/>
-      <c r="AD12" s="171"/>
-      <c r="AE12" s="171"/>
-      <c r="AF12" s="171"/>
-      <c r="AG12" s="172"/>
-      <c r="AH12" s="170"/>
-      <c r="AI12" s="171"/>
-      <c r="AJ12" s="171"/>
-      <c r="AK12" s="171"/>
-      <c r="AL12" s="171"/>
-      <c r="AM12" s="172"/>
+      <c r="B12" s="155"/>
+      <c r="C12" s="156"/>
+      <c r="D12" s="156"/>
+      <c r="E12" s="156"/>
+      <c r="F12" s="156"/>
+      <c r="G12" s="157"/>
+      <c r="H12" s="156"/>
+      <c r="I12" s="158"/>
+      <c r="J12" s="159"/>
+      <c r="K12" s="160"/>
+      <c r="L12" s="160"/>
+      <c r="M12" s="160"/>
+      <c r="N12" s="160"/>
+      <c r="O12" s="160"/>
+      <c r="P12" s="160"/>
+      <c r="Q12" s="160"/>
+      <c r="R12" s="160"/>
+      <c r="S12" s="160"/>
+      <c r="T12" s="160"/>
+      <c r="U12" s="160"/>
+      <c r="V12" s="160"/>
+      <c r="W12" s="160"/>
+      <c r="X12" s="160"/>
+      <c r="Y12" s="160"/>
+      <c r="Z12" s="160"/>
+      <c r="AA12" s="160"/>
+      <c r="AB12" s="160"/>
+      <c r="AC12" s="160"/>
+      <c r="AD12" s="160"/>
+      <c r="AE12" s="160"/>
+      <c r="AF12" s="160"/>
+      <c r="AG12" s="161"/>
+      <c r="AH12" s="159"/>
+      <c r="AI12" s="160"/>
+      <c r="AJ12" s="160"/>
+      <c r="AK12" s="160"/>
+      <c r="AL12" s="160"/>
+      <c r="AM12" s="161"/>
       <c r="AN12" s="35"/>
       <c r="AO12" s="2"/>
       <c r="AP12" s="2"/>
@@ -2291,44 +2285,44 @@
     </row>
     <row r="13" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="108"/>
-      <c r="B13" s="153"/>
-      <c r="C13" s="154"/>
-      <c r="D13" s="154"/>
-      <c r="E13" s="154"/>
-      <c r="F13" s="154"/>
-      <c r="G13" s="169"/>
-      <c r="H13" s="154"/>
-      <c r="I13" s="155"/>
-      <c r="J13" s="170"/>
-      <c r="K13" s="171"/>
-      <c r="L13" s="171"/>
-      <c r="M13" s="171"/>
-      <c r="N13" s="171"/>
-      <c r="O13" s="171"/>
-      <c r="P13" s="171"/>
-      <c r="Q13" s="171"/>
-      <c r="R13" s="171"/>
-      <c r="S13" s="171"/>
-      <c r="T13" s="171"/>
-      <c r="U13" s="171"/>
-      <c r="V13" s="171"/>
-      <c r="W13" s="171"/>
-      <c r="X13" s="171"/>
-      <c r="Y13" s="171"/>
-      <c r="Z13" s="171"/>
-      <c r="AA13" s="171"/>
-      <c r="AB13" s="171"/>
-      <c r="AC13" s="171"/>
-      <c r="AD13" s="171"/>
-      <c r="AE13" s="171"/>
-      <c r="AF13" s="171"/>
-      <c r="AG13" s="172"/>
-      <c r="AH13" s="170"/>
-      <c r="AI13" s="171"/>
-      <c r="AJ13" s="171"/>
-      <c r="AK13" s="171"/>
-      <c r="AL13" s="171"/>
-      <c r="AM13" s="172"/>
+      <c r="B13" s="155"/>
+      <c r="C13" s="156"/>
+      <c r="D13" s="156"/>
+      <c r="E13" s="156"/>
+      <c r="F13" s="156"/>
+      <c r="G13" s="157"/>
+      <c r="H13" s="156"/>
+      <c r="I13" s="158"/>
+      <c r="J13" s="159"/>
+      <c r="K13" s="160"/>
+      <c r="L13" s="160"/>
+      <c r="M13" s="160"/>
+      <c r="N13" s="160"/>
+      <c r="O13" s="160"/>
+      <c r="P13" s="160"/>
+      <c r="Q13" s="160"/>
+      <c r="R13" s="160"/>
+      <c r="S13" s="160"/>
+      <c r="T13" s="160"/>
+      <c r="U13" s="160"/>
+      <c r="V13" s="160"/>
+      <c r="W13" s="160"/>
+      <c r="X13" s="160"/>
+      <c r="Y13" s="160"/>
+      <c r="Z13" s="160"/>
+      <c r="AA13" s="160"/>
+      <c r="AB13" s="160"/>
+      <c r="AC13" s="160"/>
+      <c r="AD13" s="160"/>
+      <c r="AE13" s="160"/>
+      <c r="AF13" s="160"/>
+      <c r="AG13" s="161"/>
+      <c r="AH13" s="159"/>
+      <c r="AI13" s="160"/>
+      <c r="AJ13" s="160"/>
+      <c r="AK13" s="160"/>
+      <c r="AL13" s="160"/>
+      <c r="AM13" s="161"/>
       <c r="AN13" s="23"/>
       <c r="AO13" s="37"/>
       <c r="AP13" s="37"/>
@@ -2340,47 +2334,47 @@
       <c r="AV13" s="38"/>
     </row>
     <row r="14" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="173" t="s">
+      <c r="A14" s="162" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="174"/>
-      <c r="C14" s="174"/>
-      <c r="D14" s="174"/>
-      <c r="E14" s="174"/>
-      <c r="F14" s="174"/>
-      <c r="G14" s="174"/>
-      <c r="H14" s="174"/>
-      <c r="I14" s="174"/>
-      <c r="J14" s="174"/>
-      <c r="K14" s="174"/>
-      <c r="L14" s="174"/>
-      <c r="M14" s="174"/>
-      <c r="N14" s="174"/>
-      <c r="O14" s="174"/>
-      <c r="P14" s="174"/>
-      <c r="Q14" s="174"/>
-      <c r="R14" s="174"/>
-      <c r="S14" s="174"/>
-      <c r="T14" s="174"/>
-      <c r="U14" s="174"/>
-      <c r="V14" s="174"/>
-      <c r="W14" s="174"/>
-      <c r="X14" s="174"/>
-      <c r="Y14" s="174"/>
-      <c r="Z14" s="174"/>
-      <c r="AA14" s="174"/>
-      <c r="AB14" s="174"/>
-      <c r="AC14" s="174"/>
-      <c r="AD14" s="174"/>
-      <c r="AE14" s="174"/>
-      <c r="AF14" s="174"/>
-      <c r="AG14" s="174"/>
-      <c r="AH14" s="174"/>
-      <c r="AI14" s="174"/>
-      <c r="AJ14" s="174"/>
-      <c r="AK14" s="174"/>
-      <c r="AL14" s="174"/>
-      <c r="AM14" s="175"/>
+      <c r="B14" s="163"/>
+      <c r="C14" s="163"/>
+      <c r="D14" s="163"/>
+      <c r="E14" s="163"/>
+      <c r="F14" s="163"/>
+      <c r="G14" s="163"/>
+      <c r="H14" s="163"/>
+      <c r="I14" s="163"/>
+      <c r="J14" s="163"/>
+      <c r="K14" s="163"/>
+      <c r="L14" s="163"/>
+      <c r="M14" s="163"/>
+      <c r="N14" s="163"/>
+      <c r="O14" s="163"/>
+      <c r="P14" s="163"/>
+      <c r="Q14" s="163"/>
+      <c r="R14" s="163"/>
+      <c r="S14" s="163"/>
+      <c r="T14" s="163"/>
+      <c r="U14" s="163"/>
+      <c r="V14" s="163"/>
+      <c r="W14" s="163"/>
+      <c r="X14" s="163"/>
+      <c r="Y14" s="163"/>
+      <c r="Z14" s="163"/>
+      <c r="AA14" s="163"/>
+      <c r="AB14" s="163"/>
+      <c r="AC14" s="163"/>
+      <c r="AD14" s="163"/>
+      <c r="AE14" s="163"/>
+      <c r="AF14" s="163"/>
+      <c r="AG14" s="163"/>
+      <c r="AH14" s="163"/>
+      <c r="AI14" s="163"/>
+      <c r="AJ14" s="163"/>
+      <c r="AK14" s="163"/>
+      <c r="AL14" s="163"/>
+      <c r="AM14" s="154"/>
       <c r="AN14" s="39"/>
       <c r="AO14" s="21"/>
       <c r="AP14" s="21"/>
@@ -2392,54 +2386,54 @@
       <c r="AV14" s="36"/>
     </row>
     <row r="15" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="176"/>
-      <c r="B15" s="166"/>
-      <c r="C15" s="166"/>
-      <c r="D15" s="166"/>
-      <c r="E15" s="166"/>
-      <c r="F15" s="166"/>
-      <c r="G15" s="166"/>
-      <c r="H15" s="166"/>
-      <c r="I15" s="166"/>
-      <c r="J15" s="177"/>
-      <c r="K15" s="177"/>
-      <c r="L15" s="177"/>
-      <c r="M15" s="177"/>
-      <c r="N15" s="177"/>
-      <c r="O15" s="177"/>
-      <c r="P15" s="177"/>
-      <c r="Q15" s="177"/>
-      <c r="R15" s="177"/>
-      <c r="S15" s="177"/>
-      <c r="T15" s="177"/>
-      <c r="U15" s="177"/>
-      <c r="V15" s="177"/>
-      <c r="W15" s="177"/>
-      <c r="X15" s="177"/>
-      <c r="Y15" s="177"/>
-      <c r="Z15" s="177"/>
-      <c r="AA15" s="177"/>
-      <c r="AB15" s="177"/>
-      <c r="AC15" s="177"/>
-      <c r="AD15" s="177"/>
-      <c r="AE15" s="177"/>
-      <c r="AF15" s="177"/>
-      <c r="AG15" s="177"/>
-      <c r="AH15" s="177"/>
-      <c r="AI15" s="177"/>
-      <c r="AJ15" s="177"/>
-      <c r="AK15" s="177"/>
-      <c r="AL15" s="177"/>
-      <c r="AM15" s="175"/>
-      <c r="AN15" s="178"/>
-      <c r="AO15" s="179"/>
-      <c r="AP15" s="179"/>
-      <c r="AQ15" s="179"/>
-      <c r="AR15" s="179"/>
-      <c r="AS15" s="179"/>
-      <c r="AT15" s="179"/>
-      <c r="AU15" s="179"/>
-      <c r="AV15" s="175"/>
+      <c r="A15" s="164"/>
+      <c r="B15" s="165"/>
+      <c r="C15" s="165"/>
+      <c r="D15" s="165"/>
+      <c r="E15" s="165"/>
+      <c r="F15" s="165"/>
+      <c r="G15" s="165"/>
+      <c r="H15" s="165"/>
+      <c r="I15" s="165"/>
+      <c r="J15" s="166"/>
+      <c r="K15" s="166"/>
+      <c r="L15" s="166"/>
+      <c r="M15" s="166"/>
+      <c r="N15" s="166"/>
+      <c r="O15" s="166"/>
+      <c r="P15" s="166"/>
+      <c r="Q15" s="166"/>
+      <c r="R15" s="166"/>
+      <c r="S15" s="166"/>
+      <c r="T15" s="166"/>
+      <c r="U15" s="166"/>
+      <c r="V15" s="166"/>
+      <c r="W15" s="166"/>
+      <c r="X15" s="166"/>
+      <c r="Y15" s="166"/>
+      <c r="Z15" s="166"/>
+      <c r="AA15" s="166"/>
+      <c r="AB15" s="166"/>
+      <c r="AC15" s="166"/>
+      <c r="AD15" s="166"/>
+      <c r="AE15" s="166"/>
+      <c r="AF15" s="166"/>
+      <c r="AG15" s="166"/>
+      <c r="AH15" s="166"/>
+      <c r="AI15" s="166"/>
+      <c r="AJ15" s="166"/>
+      <c r="AK15" s="166"/>
+      <c r="AL15" s="166"/>
+      <c r="AM15" s="154"/>
+      <c r="AN15" s="152"/>
+      <c r="AO15" s="153"/>
+      <c r="AP15" s="153"/>
+      <c r="AQ15" s="153"/>
+      <c r="AR15" s="153"/>
+      <c r="AS15" s="153"/>
+      <c r="AT15" s="153"/>
+      <c r="AU15" s="153"/>
+      <c r="AV15" s="154"/>
     </row>
     <row r="16" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="109"/>
@@ -2455,41 +2449,41 @@
       <c r="K16" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="L16" s="142"/>
-      <c r="M16" s="143"/>
-      <c r="N16" s="143"/>
+      <c r="L16" s="149"/>
+      <c r="M16" s="150"/>
+      <c r="N16" s="150"/>
       <c r="O16" s="65"/>
       <c r="P16" s="66"/>
       <c r="Q16" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="R16" s="142"/>
-      <c r="S16" s="143"/>
-      <c r="T16" s="143"/>
+      <c r="R16" s="149"/>
+      <c r="S16" s="150"/>
+      <c r="T16" s="150"/>
       <c r="U16" s="65"/>
       <c r="V16" s="66"/>
       <c r="W16" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="X16" s="142"/>
-      <c r="Y16" s="143"/>
-      <c r="Z16" s="143"/>
+      <c r="X16" s="149"/>
+      <c r="Y16" s="150"/>
+      <c r="Z16" s="150"/>
       <c r="AA16" s="65"/>
       <c r="AB16" s="68"/>
       <c r="AC16" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="AD16" s="142"/>
-      <c r="AE16" s="143"/>
-      <c r="AF16" s="143"/>
+      <c r="AD16" s="149"/>
+      <c r="AE16" s="150"/>
+      <c r="AF16" s="150"/>
       <c r="AG16" s="65"/>
       <c r="AH16" s="68"/>
       <c r="AI16" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="AJ16" s="142"/>
-      <c r="AK16" s="143"/>
-      <c r="AL16" s="143"/>
+      <c r="AJ16" s="149"/>
+      <c r="AK16" s="150"/>
+      <c r="AL16" s="150"/>
       <c r="AM16" s="69"/>
       <c r="AN16" s="61"/>
       <c r="AO16" s="2"/>
@@ -2559,37 +2553,37 @@
       <c r="E18" s="132"/>
       <c r="F18" s="86"/>
       <c r="G18" s="125"/>
-      <c r="H18" s="135"/>
+      <c r="H18" s="184"/>
       <c r="I18" s="119"/>
       <c r="J18" s="74"/>
-      <c r="K18" s="147"/>
-      <c r="L18" s="147"/>
-      <c r="M18" s="147"/>
-      <c r="N18" s="147"/>
+      <c r="K18" s="148"/>
+      <c r="L18" s="148"/>
+      <c r="M18" s="148"/>
+      <c r="N18" s="148"/>
       <c r="O18" s="43"/>
       <c r="P18" s="72"/>
-      <c r="Q18" s="147"/>
-      <c r="R18" s="147"/>
-      <c r="S18" s="147"/>
-      <c r="T18" s="147"/>
+      <c r="Q18" s="148"/>
+      <c r="R18" s="148"/>
+      <c r="S18" s="148"/>
+      <c r="T18" s="148"/>
       <c r="U18" s="43"/>
       <c r="V18" s="72"/>
-      <c r="W18" s="147"/>
-      <c r="X18" s="147"/>
-      <c r="Y18" s="147"/>
-      <c r="Z18" s="147"/>
+      <c r="W18" s="148"/>
+      <c r="X18" s="148"/>
+      <c r="Y18" s="148"/>
+      <c r="Z18" s="148"/>
       <c r="AA18" s="43"/>
       <c r="AB18" s="72"/>
-      <c r="AC18" s="147"/>
-      <c r="AD18" s="147"/>
-      <c r="AE18" s="147"/>
-      <c r="AF18" s="147"/>
+      <c r="AC18" s="148"/>
+      <c r="AD18" s="148"/>
+      <c r="AE18" s="148"/>
+      <c r="AF18" s="148"/>
       <c r="AG18" s="43"/>
       <c r="AH18" s="72"/>
-      <c r="AI18" s="147"/>
-      <c r="AJ18" s="147"/>
-      <c r="AK18" s="147"/>
-      <c r="AL18" s="147"/>
+      <c r="AI18" s="148"/>
+      <c r="AJ18" s="148"/>
+      <c r="AK18" s="148"/>
+      <c r="AL18" s="148"/>
       <c r="AM18" s="73"/>
       <c r="AN18" s="61"/>
       <c r="AO18" s="2"/>
@@ -2612,34 +2606,34 @@
       <c r="H19" s="87"/>
       <c r="I19" s="119"/>
       <c r="J19" s="70"/>
-      <c r="K19" s="147"/>
-      <c r="L19" s="147"/>
-      <c r="M19" s="147"/>
-      <c r="N19" s="147"/>
+      <c r="K19" s="148"/>
+      <c r="L19" s="148"/>
+      <c r="M19" s="148"/>
+      <c r="N19" s="148"/>
       <c r="O19" s="43"/>
       <c r="P19" s="72"/>
-      <c r="Q19" s="147"/>
-      <c r="R19" s="147"/>
-      <c r="S19" s="147"/>
-      <c r="T19" s="147"/>
+      <c r="Q19" s="148"/>
+      <c r="R19" s="148"/>
+      <c r="S19" s="148"/>
+      <c r="T19" s="148"/>
       <c r="U19" s="43"/>
       <c r="V19" s="72"/>
-      <c r="W19" s="147"/>
-      <c r="X19" s="147"/>
-      <c r="Y19" s="147"/>
-      <c r="Z19" s="147"/>
+      <c r="W19" s="148"/>
+      <c r="X19" s="148"/>
+      <c r="Y19" s="148"/>
+      <c r="Z19" s="148"/>
       <c r="AA19" s="43"/>
       <c r="AB19" s="72"/>
-      <c r="AC19" s="147"/>
-      <c r="AD19" s="147"/>
-      <c r="AE19" s="147"/>
-      <c r="AF19" s="147"/>
+      <c r="AC19" s="148"/>
+      <c r="AD19" s="148"/>
+      <c r="AE19" s="148"/>
+      <c r="AF19" s="148"/>
       <c r="AG19" s="43"/>
       <c r="AH19" s="72"/>
-      <c r="AI19" s="147"/>
-      <c r="AJ19" s="147"/>
-      <c r="AK19" s="147"/>
-      <c r="AL19" s="147"/>
+      <c r="AI19" s="148"/>
+      <c r="AJ19" s="148"/>
+      <c r="AK19" s="148"/>
+      <c r="AL19" s="148"/>
       <c r="AM19" s="73"/>
       <c r="AN19" s="61"/>
       <c r="AO19" s="2"/>
@@ -2662,34 +2656,34 @@
       <c r="H20" s="87"/>
       <c r="I20" s="119"/>
       <c r="J20" s="74"/>
-      <c r="K20" s="147"/>
-      <c r="L20" s="147"/>
-      <c r="M20" s="147"/>
-      <c r="N20" s="147"/>
+      <c r="K20" s="148"/>
+      <c r="L20" s="148"/>
+      <c r="M20" s="148"/>
+      <c r="N20" s="148"/>
       <c r="O20" s="43"/>
       <c r="P20" s="72"/>
-      <c r="Q20" s="147"/>
-      <c r="R20" s="147"/>
-      <c r="S20" s="147"/>
-      <c r="T20" s="147"/>
+      <c r="Q20" s="148"/>
+      <c r="R20" s="148"/>
+      <c r="S20" s="148"/>
+      <c r="T20" s="148"/>
       <c r="U20" s="43"/>
       <c r="V20" s="72"/>
-      <c r="W20" s="147"/>
-      <c r="X20" s="147"/>
-      <c r="Y20" s="147"/>
-      <c r="Z20" s="147"/>
+      <c r="W20" s="148"/>
+      <c r="X20" s="148"/>
+      <c r="Y20" s="148"/>
+      <c r="Z20" s="148"/>
       <c r="AA20" s="43"/>
       <c r="AB20" s="72"/>
-      <c r="AC20" s="147"/>
-      <c r="AD20" s="147"/>
-      <c r="AE20" s="147"/>
-      <c r="AF20" s="147"/>
+      <c r="AC20" s="148"/>
+      <c r="AD20" s="148"/>
+      <c r="AE20" s="148"/>
+      <c r="AF20" s="148"/>
       <c r="AG20" s="43"/>
       <c r="AH20" s="72"/>
-      <c r="AI20" s="147"/>
-      <c r="AJ20" s="147"/>
-      <c r="AK20" s="147"/>
-      <c r="AL20" s="147"/>
+      <c r="AI20" s="148"/>
+      <c r="AJ20" s="148"/>
+      <c r="AK20" s="148"/>
+      <c r="AL20" s="148"/>
       <c r="AM20" s="73"/>
       <c r="AN20" s="61"/>
       <c r="AO20" s="2"/>
@@ -2712,34 +2706,34 @@
       <c r="H21" s="128"/>
       <c r="I21" s="120"/>
       <c r="J21" s="74"/>
-      <c r="K21" s="147"/>
-      <c r="L21" s="147"/>
-      <c r="M21" s="147"/>
-      <c r="N21" s="147"/>
+      <c r="K21" s="148"/>
+      <c r="L21" s="148"/>
+      <c r="M21" s="148"/>
+      <c r="N21" s="148"/>
       <c r="O21" s="43"/>
       <c r="P21" s="72"/>
-      <c r="Q21" s="147"/>
-      <c r="R21" s="147"/>
-      <c r="S21" s="147"/>
-      <c r="T21" s="147"/>
+      <c r="Q21" s="148"/>
+      <c r="R21" s="148"/>
+      <c r="S21" s="148"/>
+      <c r="T21" s="148"/>
       <c r="U21" s="43"/>
       <c r="V21" s="72"/>
-      <c r="W21" s="147"/>
-      <c r="X21" s="147"/>
-      <c r="Y21" s="147"/>
-      <c r="Z21" s="147"/>
+      <c r="W21" s="148"/>
+      <c r="X21" s="148"/>
+      <c r="Y21" s="148"/>
+      <c r="Z21" s="148"/>
       <c r="AA21" s="43"/>
       <c r="AB21" s="72"/>
-      <c r="AC21" s="147"/>
-      <c r="AD21" s="147"/>
-      <c r="AE21" s="147"/>
-      <c r="AF21" s="147"/>
+      <c r="AC21" s="148"/>
+      <c r="AD21" s="148"/>
+      <c r="AE21" s="148"/>
+      <c r="AF21" s="148"/>
       <c r="AG21" s="43"/>
       <c r="AH21" s="72"/>
-      <c r="AI21" s="147"/>
-      <c r="AJ21" s="147"/>
-      <c r="AK21" s="147"/>
-      <c r="AL21" s="147"/>
+      <c r="AI21" s="148"/>
+      <c r="AJ21" s="148"/>
+      <c r="AK21" s="148"/>
+      <c r="AL21" s="148"/>
       <c r="AM21" s="73"/>
       <c r="AN21" s="61"/>
       <c r="AO21" s="2"/>
@@ -2762,34 +2756,34 @@
       <c r="H22" s="87"/>
       <c r="I22" s="119"/>
       <c r="J22" s="74"/>
-      <c r="K22" s="147"/>
-      <c r="L22" s="147"/>
-      <c r="M22" s="147"/>
-      <c r="N22" s="147"/>
+      <c r="K22" s="148"/>
+      <c r="L22" s="148"/>
+      <c r="M22" s="148"/>
+      <c r="N22" s="148"/>
       <c r="O22" s="43"/>
       <c r="P22" s="72"/>
-      <c r="Q22" s="147"/>
-      <c r="R22" s="147"/>
-      <c r="S22" s="147"/>
-      <c r="T22" s="147"/>
+      <c r="Q22" s="148"/>
+      <c r="R22" s="148"/>
+      <c r="S22" s="148"/>
+      <c r="T22" s="148"/>
       <c r="U22" s="43"/>
       <c r="V22" s="72"/>
-      <c r="W22" s="147"/>
-      <c r="X22" s="147"/>
-      <c r="Y22" s="147"/>
-      <c r="Z22" s="147"/>
+      <c r="W22" s="148"/>
+      <c r="X22" s="148"/>
+      <c r="Y22" s="148"/>
+      <c r="Z22" s="148"/>
       <c r="AA22" s="43"/>
       <c r="AB22" s="72"/>
-      <c r="AC22" s="147"/>
-      <c r="AD22" s="147"/>
-      <c r="AE22" s="147"/>
-      <c r="AF22" s="147"/>
+      <c r="AC22" s="148"/>
+      <c r="AD22" s="148"/>
+      <c r="AE22" s="148"/>
+      <c r="AF22" s="148"/>
       <c r="AG22" s="43"/>
       <c r="AH22" s="72"/>
-      <c r="AI22" s="147"/>
-      <c r="AJ22" s="147"/>
-      <c r="AK22" s="147"/>
-      <c r="AL22" s="147"/>
+      <c r="AI22" s="148"/>
+      <c r="AJ22" s="148"/>
+      <c r="AK22" s="148"/>
+      <c r="AL22" s="148"/>
       <c r="AM22" s="73"/>
       <c r="AN22" s="61"/>
       <c r="AO22" s="2"/>
@@ -2812,34 +2806,34 @@
       <c r="H23" s="87"/>
       <c r="I23" s="119"/>
       <c r="J23" s="70"/>
-      <c r="K23" s="147"/>
-      <c r="L23" s="147"/>
-      <c r="M23" s="147"/>
-      <c r="N23" s="147"/>
+      <c r="K23" s="148"/>
+      <c r="L23" s="148"/>
+      <c r="M23" s="148"/>
+      <c r="N23" s="148"/>
       <c r="O23" s="43"/>
       <c r="P23" s="72"/>
-      <c r="Q23" s="147"/>
-      <c r="R23" s="147"/>
-      <c r="S23" s="147"/>
-      <c r="T23" s="147"/>
+      <c r="Q23" s="148"/>
+      <c r="R23" s="148"/>
+      <c r="S23" s="148"/>
+      <c r="T23" s="148"/>
       <c r="U23" s="43"/>
       <c r="V23" s="72"/>
-      <c r="W23" s="147"/>
-      <c r="X23" s="147"/>
-      <c r="Y23" s="147"/>
-      <c r="Z23" s="147"/>
+      <c r="W23" s="148"/>
+      <c r="X23" s="148"/>
+      <c r="Y23" s="148"/>
+      <c r="Z23" s="148"/>
       <c r="AA23" s="43"/>
       <c r="AB23" s="72"/>
-      <c r="AC23" s="147"/>
-      <c r="AD23" s="147"/>
-      <c r="AE23" s="147"/>
-      <c r="AF23" s="147"/>
+      <c r="AC23" s="148"/>
+      <c r="AD23" s="148"/>
+      <c r="AE23" s="148"/>
+      <c r="AF23" s="148"/>
       <c r="AG23" s="43"/>
       <c r="AH23" s="72"/>
-      <c r="AI23" s="147"/>
-      <c r="AJ23" s="147"/>
-      <c r="AK23" s="147"/>
-      <c r="AL23" s="147"/>
+      <c r="AI23" s="148"/>
+      <c r="AJ23" s="148"/>
+      <c r="AK23" s="148"/>
+      <c r="AL23" s="148"/>
       <c r="AM23" s="73"/>
       <c r="AN23" s="61"/>
       <c r="AO23" s="2"/>
@@ -2865,41 +2859,41 @@
       <c r="K24" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="L24" s="145"/>
-      <c r="M24" s="146"/>
-      <c r="N24" s="145"/>
+      <c r="L24" s="143"/>
+      <c r="M24" s="142"/>
+      <c r="N24" s="143"/>
       <c r="O24" s="43"/>
       <c r="P24" s="72"/>
       <c r="Q24" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="R24" s="145"/>
-      <c r="S24" s="146"/>
-      <c r="T24" s="145"/>
+      <c r="R24" s="143"/>
+      <c r="S24" s="142"/>
+      <c r="T24" s="143"/>
       <c r="U24" s="43"/>
       <c r="V24" s="72"/>
       <c r="W24" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="X24" s="145"/>
-      <c r="Y24" s="146"/>
-      <c r="Z24" s="145"/>
+      <c r="X24" s="143"/>
+      <c r="Y24" s="142"/>
+      <c r="Z24" s="143"/>
       <c r="AA24" s="43"/>
       <c r="AB24" s="72"/>
       <c r="AC24" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AD24" s="145"/>
-      <c r="AE24" s="146"/>
-      <c r="AF24" s="145"/>
+      <c r="AD24" s="143"/>
+      <c r="AE24" s="142"/>
+      <c r="AF24" s="143"/>
       <c r="AG24" s="43"/>
       <c r="AH24" s="72"/>
       <c r="AI24" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AJ24" s="145"/>
-      <c r="AK24" s="146"/>
-      <c r="AL24" s="145"/>
+      <c r="AJ24" s="143"/>
+      <c r="AK24" s="142"/>
+      <c r="AL24" s="143"/>
       <c r="AM24" s="73"/>
       <c r="AN24" s="61"/>
       <c r="AO24" s="2"/>
@@ -2926,40 +2920,40 @@
         <v>32</v>
       </c>
       <c r="L25" s="72"/>
-      <c r="M25" s="146"/>
-      <c r="N25" s="145"/>
+      <c r="M25" s="142"/>
+      <c r="N25" s="143"/>
       <c r="O25" s="43"/>
       <c r="P25" s="72"/>
       <c r="Q25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="R25" s="72"/>
-      <c r="S25" s="146"/>
-      <c r="T25" s="145"/>
+      <c r="S25" s="142"/>
+      <c r="T25" s="143"/>
       <c r="U25" s="43"/>
       <c r="V25" s="72"/>
       <c r="W25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="X25" s="72"/>
-      <c r="Y25" s="146"/>
-      <c r="Z25" s="145"/>
+      <c r="Y25" s="142"/>
+      <c r="Z25" s="143"/>
       <c r="AA25" s="43"/>
       <c r="AB25" s="72"/>
       <c r="AC25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AD25" s="72"/>
-      <c r="AE25" s="146"/>
-      <c r="AF25" s="145"/>
+      <c r="AE25" s="142"/>
+      <c r="AF25" s="143"/>
       <c r="AG25" s="43"/>
       <c r="AH25" s="72"/>
       <c r="AI25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AJ25" s="72"/>
-      <c r="AK25" s="146"/>
-      <c r="AL25" s="145"/>
+      <c r="AK25" s="142"/>
+      <c r="AL25" s="143"/>
       <c r="AM25" s="73"/>
       <c r="AN25" s="61"/>
       <c r="AO25" s="2"/>
@@ -2985,50 +2979,50 @@
       <c r="K26" s="48" t="s">
         <v>33</v>
       </c>
-      <c r="L26" s="148"/>
-      <c r="M26" s="148"/>
-      <c r="N26" s="148"/>
+      <c r="L26" s="151"/>
+      <c r="M26" s="151"/>
+      <c r="N26" s="151"/>
       <c r="O26" s="60"/>
       <c r="P26" s="41"/>
       <c r="Q26" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="R26" s="142"/>
-      <c r="S26" s="143"/>
-      <c r="T26" s="143"/>
+      <c r="R26" s="149"/>
+      <c r="S26" s="150"/>
+      <c r="T26" s="150"/>
       <c r="U26" s="40"/>
       <c r="V26" s="41"/>
       <c r="W26" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="X26" s="148"/>
-      <c r="Y26" s="148"/>
-      <c r="Z26" s="148"/>
+      <c r="X26" s="151"/>
+      <c r="Y26" s="151"/>
+      <c r="Z26" s="151"/>
       <c r="AA26" s="40"/>
       <c r="AB26" s="41"/>
       <c r="AC26" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="AD26" s="142"/>
-      <c r="AE26" s="143"/>
-      <c r="AF26" s="143"/>
+      <c r="AD26" s="149"/>
+      <c r="AE26" s="150"/>
+      <c r="AF26" s="150"/>
       <c r="AG26" s="40"/>
       <c r="AH26" s="41"/>
       <c r="AI26" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="AJ26" s="142"/>
-      <c r="AK26" s="143"/>
-      <c r="AL26" s="143"/>
+      <c r="AJ26" s="149"/>
+      <c r="AK26" s="150"/>
+      <c r="AL26" s="150"/>
       <c r="AM26" s="77"/>
       <c r="AN26" s="61"/>
-      <c r="AO26" s="180"/>
-      <c r="AP26" s="181"/>
-      <c r="AQ26" s="181"/>
-      <c r="AR26" s="181"/>
-      <c r="AS26" s="181"/>
-      <c r="AT26" s="181"/>
-      <c r="AU26" s="181"/>
+      <c r="AO26" s="145"/>
+      <c r="AP26" s="146"/>
+      <c r="AQ26" s="146"/>
+      <c r="AR26" s="146"/>
+      <c r="AS26" s="146"/>
+      <c r="AT26" s="146"/>
+      <c r="AU26" s="146"/>
       <c r="AV26" s="22"/>
     </row>
     <row r="27" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3039,7 +3033,7 @@
       <c r="E27" s="133"/>
       <c r="F27" s="42"/>
       <c r="G27" s="46"/>
-      <c r="H27" s="136"/>
+      <c r="H27" s="135"/>
       <c r="I27" s="121"/>
       <c r="J27" s="74"/>
       <c r="K27" s="71"/>
@@ -3072,13 +3066,13 @@
       <c r="AL27" s="72"/>
       <c r="AM27" s="73"/>
       <c r="AN27" s="61"/>
-      <c r="AO27" s="181"/>
-      <c r="AP27" s="181"/>
-      <c r="AQ27" s="181"/>
-      <c r="AR27" s="181"/>
-      <c r="AS27" s="181"/>
-      <c r="AT27" s="181"/>
-      <c r="AU27" s="181"/>
+      <c r="AO27" s="146"/>
+      <c r="AP27" s="146"/>
+      <c r="AQ27" s="146"/>
+      <c r="AR27" s="146"/>
+      <c r="AS27" s="146"/>
+      <c r="AT27" s="146"/>
+      <c r="AU27" s="146"/>
       <c r="AV27" s="22"/>
     </row>
     <row r="28" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3089,46 +3083,46 @@
       <c r="E28" s="134"/>
       <c r="F28" s="81"/>
       <c r="G28" s="91"/>
-      <c r="H28" s="137"/>
+      <c r="H28" s="136"/>
       <c r="I28" s="122"/>
       <c r="J28" s="74"/>
-      <c r="K28" s="147"/>
-      <c r="L28" s="147"/>
-      <c r="M28" s="147"/>
-      <c r="N28" s="147"/>
+      <c r="K28" s="148"/>
+      <c r="L28" s="148"/>
+      <c r="M28" s="148"/>
+      <c r="N28" s="148"/>
       <c r="O28" s="43"/>
       <c r="P28" s="72"/>
-      <c r="Q28" s="147"/>
-      <c r="R28" s="147"/>
-      <c r="S28" s="147"/>
-      <c r="T28" s="147"/>
+      <c r="Q28" s="148"/>
+      <c r="R28" s="148"/>
+      <c r="S28" s="148"/>
+      <c r="T28" s="148"/>
       <c r="U28" s="43"/>
       <c r="V28" s="72"/>
-      <c r="W28" s="147"/>
-      <c r="X28" s="147"/>
-      <c r="Y28" s="147"/>
-      <c r="Z28" s="147"/>
+      <c r="W28" s="148"/>
+      <c r="X28" s="148"/>
+      <c r="Y28" s="148"/>
+      <c r="Z28" s="148"/>
       <c r="AA28" s="43"/>
       <c r="AB28" s="72"/>
-      <c r="AC28" s="147"/>
-      <c r="AD28" s="147"/>
-      <c r="AE28" s="147"/>
-      <c r="AF28" s="147"/>
+      <c r="AC28" s="148"/>
+      <c r="AD28" s="148"/>
+      <c r="AE28" s="148"/>
+      <c r="AF28" s="148"/>
       <c r="AG28" s="43"/>
       <c r="AH28" s="72"/>
-      <c r="AI28" s="147"/>
-      <c r="AJ28" s="147"/>
-      <c r="AK28" s="147"/>
-      <c r="AL28" s="147"/>
+      <c r="AI28" s="148"/>
+      <c r="AJ28" s="148"/>
+      <c r="AK28" s="148"/>
+      <c r="AL28" s="148"/>
       <c r="AM28" s="73"/>
       <c r="AN28" s="61"/>
-      <c r="AO28" s="181"/>
-      <c r="AP28" s="181"/>
-      <c r="AQ28" s="181"/>
-      <c r="AR28" s="181"/>
-      <c r="AS28" s="181"/>
-      <c r="AT28" s="181"/>
-      <c r="AU28" s="181"/>
+      <c r="AO28" s="146"/>
+      <c r="AP28" s="146"/>
+      <c r="AQ28" s="146"/>
+      <c r="AR28" s="146"/>
+      <c r="AS28" s="146"/>
+      <c r="AT28" s="146"/>
+      <c r="AU28" s="146"/>
       <c r="AV28" s="22"/>
     </row>
     <row r="29" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3142,43 +3136,43 @@
       <c r="H29" s="87"/>
       <c r="I29" s="119"/>
       <c r="J29" s="70"/>
-      <c r="K29" s="147"/>
-      <c r="L29" s="147"/>
-      <c r="M29" s="147"/>
-      <c r="N29" s="147"/>
+      <c r="K29" s="148"/>
+      <c r="L29" s="148"/>
+      <c r="M29" s="148"/>
+      <c r="N29" s="148"/>
       <c r="O29" s="43"/>
       <c r="P29" s="72"/>
-      <c r="Q29" s="147"/>
-      <c r="R29" s="147"/>
-      <c r="S29" s="147"/>
-      <c r="T29" s="147"/>
+      <c r="Q29" s="148"/>
+      <c r="R29" s="148"/>
+      <c r="S29" s="148"/>
+      <c r="T29" s="148"/>
       <c r="U29" s="43"/>
       <c r="V29" s="72"/>
-      <c r="W29" s="147"/>
-      <c r="X29" s="147"/>
-      <c r="Y29" s="147"/>
-      <c r="Z29" s="147"/>
+      <c r="W29" s="148"/>
+      <c r="X29" s="148"/>
+      <c r="Y29" s="148"/>
+      <c r="Z29" s="148"/>
       <c r="AA29" s="43"/>
       <c r="AB29" s="72"/>
-      <c r="AC29" s="147"/>
-      <c r="AD29" s="147"/>
-      <c r="AE29" s="147"/>
-      <c r="AF29" s="147"/>
+      <c r="AC29" s="148"/>
+      <c r="AD29" s="148"/>
+      <c r="AE29" s="148"/>
+      <c r="AF29" s="148"/>
       <c r="AG29" s="43"/>
       <c r="AH29" s="72"/>
-      <c r="AI29" s="147"/>
-      <c r="AJ29" s="147"/>
-      <c r="AK29" s="147"/>
-      <c r="AL29" s="147"/>
+      <c r="AI29" s="148"/>
+      <c r="AJ29" s="148"/>
+      <c r="AK29" s="148"/>
+      <c r="AL29" s="148"/>
       <c r="AM29" s="73"/>
       <c r="AN29" s="61"/>
-      <c r="AO29" s="181"/>
-      <c r="AP29" s="181"/>
-      <c r="AQ29" s="181"/>
-      <c r="AR29" s="181"/>
-      <c r="AS29" s="181"/>
-      <c r="AT29" s="181"/>
-      <c r="AU29" s="181"/>
+      <c r="AO29" s="146"/>
+      <c r="AP29" s="146"/>
+      <c r="AQ29" s="146"/>
+      <c r="AR29" s="146"/>
+      <c r="AS29" s="146"/>
+      <c r="AT29" s="146"/>
+      <c r="AU29" s="146"/>
       <c r="AV29" s="22"/>
     </row>
     <row r="30" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3192,43 +3186,43 @@
       <c r="H30" s="87"/>
       <c r="I30" s="119"/>
       <c r="J30" s="74"/>
-      <c r="K30" s="147"/>
-      <c r="L30" s="147"/>
-      <c r="M30" s="147"/>
-      <c r="N30" s="147"/>
+      <c r="K30" s="148"/>
+      <c r="L30" s="148"/>
+      <c r="M30" s="148"/>
+      <c r="N30" s="148"/>
       <c r="O30" s="43"/>
       <c r="P30" s="72"/>
-      <c r="Q30" s="147"/>
-      <c r="R30" s="147"/>
-      <c r="S30" s="147"/>
-      <c r="T30" s="147"/>
+      <c r="Q30" s="148"/>
+      <c r="R30" s="148"/>
+      <c r="S30" s="148"/>
+      <c r="T30" s="148"/>
       <c r="U30" s="43"/>
       <c r="V30" s="72"/>
-      <c r="W30" s="147"/>
-      <c r="X30" s="147"/>
-      <c r="Y30" s="147"/>
-      <c r="Z30" s="147"/>
+      <c r="W30" s="148"/>
+      <c r="X30" s="148"/>
+      <c r="Y30" s="148"/>
+      <c r="Z30" s="148"/>
       <c r="AA30" s="43"/>
       <c r="AB30" s="72"/>
-      <c r="AC30" s="147"/>
-      <c r="AD30" s="147"/>
-      <c r="AE30" s="147"/>
-      <c r="AF30" s="147"/>
+      <c r="AC30" s="148"/>
+      <c r="AD30" s="148"/>
+      <c r="AE30" s="148"/>
+      <c r="AF30" s="148"/>
       <c r="AG30" s="43"/>
       <c r="AH30" s="72"/>
-      <c r="AI30" s="147"/>
-      <c r="AJ30" s="147"/>
-      <c r="AK30" s="147"/>
-      <c r="AL30" s="147"/>
+      <c r="AI30" s="148"/>
+      <c r="AJ30" s="148"/>
+      <c r="AK30" s="148"/>
+      <c r="AL30" s="148"/>
       <c r="AM30" s="73"/>
       <c r="AN30" s="62"/>
-      <c r="AO30" s="181"/>
-      <c r="AP30" s="181"/>
-      <c r="AQ30" s="181"/>
-      <c r="AR30" s="181"/>
-      <c r="AS30" s="181"/>
-      <c r="AT30" s="181"/>
-      <c r="AU30" s="181"/>
+      <c r="AO30" s="146"/>
+      <c r="AP30" s="146"/>
+      <c r="AQ30" s="146"/>
+      <c r="AR30" s="146"/>
+      <c r="AS30" s="146"/>
+      <c r="AT30" s="146"/>
+      <c r="AU30" s="146"/>
       <c r="AV30" s="22"/>
     </row>
     <row r="31" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3242,43 +3236,43 @@
       <c r="H31" s="87"/>
       <c r="I31" s="119"/>
       <c r="J31" s="74"/>
-      <c r="K31" s="147"/>
-      <c r="L31" s="147"/>
-      <c r="M31" s="147"/>
-      <c r="N31" s="147"/>
+      <c r="K31" s="148"/>
+      <c r="L31" s="148"/>
+      <c r="M31" s="148"/>
+      <c r="N31" s="148"/>
       <c r="O31" s="43"/>
       <c r="P31" s="72"/>
-      <c r="Q31" s="147"/>
-      <c r="R31" s="147"/>
-      <c r="S31" s="147"/>
-      <c r="T31" s="147"/>
+      <c r="Q31" s="148"/>
+      <c r="R31" s="148"/>
+      <c r="S31" s="148"/>
+      <c r="T31" s="148"/>
       <c r="U31" s="43"/>
       <c r="V31" s="72"/>
-      <c r="W31" s="147"/>
-      <c r="X31" s="147"/>
-      <c r="Y31" s="147"/>
-      <c r="Z31" s="147"/>
+      <c r="W31" s="148"/>
+      <c r="X31" s="148"/>
+      <c r="Y31" s="148"/>
+      <c r="Z31" s="148"/>
       <c r="AA31" s="43"/>
       <c r="AB31" s="72"/>
-      <c r="AC31" s="147"/>
-      <c r="AD31" s="147"/>
-      <c r="AE31" s="147"/>
-      <c r="AF31" s="147"/>
+      <c r="AC31" s="148"/>
+      <c r="AD31" s="148"/>
+      <c r="AE31" s="148"/>
+      <c r="AF31" s="148"/>
       <c r="AG31" s="43"/>
       <c r="AH31" s="72"/>
-      <c r="AI31" s="147"/>
-      <c r="AJ31" s="147"/>
-      <c r="AK31" s="147"/>
-      <c r="AL31" s="147"/>
+      <c r="AI31" s="148"/>
+      <c r="AJ31" s="148"/>
+      <c r="AK31" s="148"/>
+      <c r="AL31" s="148"/>
       <c r="AM31" s="73"/>
       <c r="AN31" s="61"/>
-      <c r="AO31" s="181"/>
-      <c r="AP31" s="181"/>
-      <c r="AQ31" s="181"/>
-      <c r="AR31" s="181"/>
-      <c r="AS31" s="181"/>
-      <c r="AT31" s="181"/>
-      <c r="AU31" s="181"/>
+      <c r="AO31" s="146"/>
+      <c r="AP31" s="146"/>
+      <c r="AQ31" s="146"/>
+      <c r="AR31" s="146"/>
+      <c r="AS31" s="146"/>
+      <c r="AT31" s="146"/>
+      <c r="AU31" s="146"/>
       <c r="AV31" s="22"/>
     </row>
     <row r="32" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3292,43 +3286,43 @@
       <c r="H32" s="87"/>
       <c r="I32" s="119"/>
       <c r="J32" s="74"/>
-      <c r="K32" s="147"/>
-      <c r="L32" s="147"/>
-      <c r="M32" s="147"/>
-      <c r="N32" s="147"/>
+      <c r="K32" s="148"/>
+      <c r="L32" s="148"/>
+      <c r="M32" s="148"/>
+      <c r="N32" s="148"/>
       <c r="O32" s="43"/>
       <c r="P32" s="72"/>
-      <c r="Q32" s="147"/>
-      <c r="R32" s="147"/>
-      <c r="S32" s="147"/>
-      <c r="T32" s="147"/>
+      <c r="Q32" s="148"/>
+      <c r="R32" s="148"/>
+      <c r="S32" s="148"/>
+      <c r="T32" s="148"/>
       <c r="U32" s="43"/>
       <c r="V32" s="72"/>
-      <c r="W32" s="147"/>
-      <c r="X32" s="147"/>
-      <c r="Y32" s="147"/>
-      <c r="Z32" s="147"/>
+      <c r="W32" s="148"/>
+      <c r="X32" s="148"/>
+      <c r="Y32" s="148"/>
+      <c r="Z32" s="148"/>
       <c r="AA32" s="43"/>
       <c r="AB32" s="72"/>
-      <c r="AC32" s="147"/>
-      <c r="AD32" s="147"/>
-      <c r="AE32" s="147"/>
-      <c r="AF32" s="147"/>
+      <c r="AC32" s="148"/>
+      <c r="AD32" s="148"/>
+      <c r="AE32" s="148"/>
+      <c r="AF32" s="148"/>
       <c r="AG32" s="43"/>
       <c r="AH32" s="72"/>
-      <c r="AI32" s="147"/>
-      <c r="AJ32" s="147"/>
-      <c r="AK32" s="147"/>
-      <c r="AL32" s="147"/>
+      <c r="AI32" s="148"/>
+      <c r="AJ32" s="148"/>
+      <c r="AK32" s="148"/>
+      <c r="AL32" s="148"/>
       <c r="AM32" s="73"/>
       <c r="AN32" s="61"/>
-      <c r="AO32" s="181"/>
-      <c r="AP32" s="181"/>
-      <c r="AQ32" s="181"/>
-      <c r="AR32" s="181"/>
-      <c r="AS32" s="181"/>
-      <c r="AT32" s="181"/>
-      <c r="AU32" s="181"/>
+      <c r="AO32" s="146"/>
+      <c r="AP32" s="146"/>
+      <c r="AQ32" s="146"/>
+      <c r="AR32" s="146"/>
+      <c r="AS32" s="146"/>
+      <c r="AT32" s="146"/>
+      <c r="AU32" s="146"/>
       <c r="AV32" s="22"/>
     </row>
     <row r="33" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3342,43 +3336,43 @@
       <c r="H33" s="87"/>
       <c r="I33" s="119"/>
       <c r="J33" s="70"/>
-      <c r="K33" s="147"/>
-      <c r="L33" s="147"/>
-      <c r="M33" s="147"/>
-      <c r="N33" s="147"/>
+      <c r="K33" s="148"/>
+      <c r="L33" s="148"/>
+      <c r="M33" s="148"/>
+      <c r="N33" s="148"/>
       <c r="O33" s="43"/>
       <c r="P33" s="72"/>
-      <c r="Q33" s="147"/>
-      <c r="R33" s="147"/>
-      <c r="S33" s="147"/>
-      <c r="T33" s="147"/>
+      <c r="Q33" s="148"/>
+      <c r="R33" s="148"/>
+      <c r="S33" s="148"/>
+      <c r="T33" s="148"/>
       <c r="U33" s="43"/>
       <c r="V33" s="72"/>
-      <c r="W33" s="147"/>
-      <c r="X33" s="147"/>
-      <c r="Y33" s="147"/>
-      <c r="Z33" s="147"/>
+      <c r="W33" s="148"/>
+      <c r="X33" s="148"/>
+      <c r="Y33" s="148"/>
+      <c r="Z33" s="148"/>
       <c r="AA33" s="43"/>
       <c r="AB33" s="72"/>
-      <c r="AC33" s="147"/>
-      <c r="AD33" s="147"/>
-      <c r="AE33" s="147"/>
-      <c r="AF33" s="147"/>
+      <c r="AC33" s="148"/>
+      <c r="AD33" s="148"/>
+      <c r="AE33" s="148"/>
+      <c r="AF33" s="148"/>
       <c r="AG33" s="43"/>
       <c r="AH33" s="72"/>
-      <c r="AI33" s="147"/>
-      <c r="AJ33" s="147"/>
-      <c r="AK33" s="147"/>
-      <c r="AL33" s="147"/>
+      <c r="AI33" s="148"/>
+      <c r="AJ33" s="148"/>
+      <c r="AK33" s="148"/>
+      <c r="AL33" s="148"/>
       <c r="AM33" s="73"/>
       <c r="AN33" s="61"/>
-      <c r="AO33" s="181"/>
-      <c r="AP33" s="181"/>
-      <c r="AQ33" s="181"/>
-      <c r="AR33" s="181"/>
-      <c r="AS33" s="181"/>
-      <c r="AT33" s="181"/>
-      <c r="AU33" s="181"/>
+      <c r="AO33" s="146"/>
+      <c r="AP33" s="146"/>
+      <c r="AQ33" s="146"/>
+      <c r="AR33" s="146"/>
+      <c r="AS33" s="146"/>
+      <c r="AT33" s="146"/>
+      <c r="AU33" s="146"/>
       <c r="AV33" s="22"/>
     </row>
     <row r="34" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3395,50 +3389,50 @@
       <c r="K34" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="L34" s="145"/>
-      <c r="M34" s="146"/>
-      <c r="N34" s="145"/>
+      <c r="L34" s="143"/>
+      <c r="M34" s="142"/>
+      <c r="N34" s="143"/>
       <c r="O34" s="43"/>
       <c r="P34" s="72"/>
       <c r="Q34" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="R34" s="145"/>
-      <c r="S34" s="146"/>
-      <c r="T34" s="145"/>
+      <c r="R34" s="143"/>
+      <c r="S34" s="142"/>
+      <c r="T34" s="143"/>
       <c r="U34" s="43"/>
       <c r="V34" s="72"/>
       <c r="W34" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="X34" s="145"/>
-      <c r="Y34" s="146"/>
-      <c r="Z34" s="145"/>
+      <c r="X34" s="143"/>
+      <c r="Y34" s="142"/>
+      <c r="Z34" s="143"/>
       <c r="AA34" s="43"/>
       <c r="AB34" s="72"/>
       <c r="AC34" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AD34" s="145"/>
-      <c r="AE34" s="146"/>
-      <c r="AF34" s="145"/>
+      <c r="AD34" s="143"/>
+      <c r="AE34" s="142"/>
+      <c r="AF34" s="143"/>
       <c r="AG34" s="43"/>
       <c r="AH34" s="72"/>
       <c r="AI34" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AJ34" s="145"/>
-      <c r="AK34" s="146"/>
-      <c r="AL34" s="145"/>
+      <c r="AJ34" s="143"/>
+      <c r="AK34" s="142"/>
+      <c r="AL34" s="143"/>
       <c r="AM34" s="43"/>
       <c r="AN34" s="61"/>
-      <c r="AO34" s="181"/>
-      <c r="AP34" s="181"/>
-      <c r="AQ34" s="181"/>
-      <c r="AR34" s="181"/>
-      <c r="AS34" s="181"/>
-      <c r="AT34" s="181"/>
-      <c r="AU34" s="181"/>
+      <c r="AO34" s="146"/>
+      <c r="AP34" s="146"/>
+      <c r="AQ34" s="146"/>
+      <c r="AR34" s="146"/>
+      <c r="AS34" s="146"/>
+      <c r="AT34" s="146"/>
+      <c r="AU34" s="146"/>
       <c r="AV34" s="22"/>
     </row>
     <row r="35" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3456,49 +3450,49 @@
         <v>32</v>
       </c>
       <c r="L35" s="72"/>
-      <c r="M35" s="146"/>
-      <c r="N35" s="145"/>
+      <c r="M35" s="142"/>
+      <c r="N35" s="143"/>
       <c r="O35" s="43"/>
       <c r="P35" s="72"/>
       <c r="Q35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="R35" s="72"/>
-      <c r="S35" s="146"/>
-      <c r="T35" s="145"/>
+      <c r="S35" s="142"/>
+      <c r="T35" s="143"/>
       <c r="U35" s="43"/>
       <c r="V35" s="72"/>
       <c r="W35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="X35" s="72"/>
-      <c r="Y35" s="146"/>
-      <c r="Z35" s="145"/>
+      <c r="Y35" s="142"/>
+      <c r="Z35" s="143"/>
       <c r="AA35" s="43"/>
       <c r="AB35" s="72"/>
       <c r="AC35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AD35" s="72"/>
-      <c r="AE35" s="146"/>
-      <c r="AF35" s="145"/>
+      <c r="AE35" s="142"/>
+      <c r="AF35" s="143"/>
       <c r="AG35" s="43"/>
       <c r="AH35" s="72"/>
       <c r="AI35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AJ35" s="72"/>
-      <c r="AK35" s="146"/>
-      <c r="AL35" s="145"/>
-      <c r="AM35" s="149"/>
+      <c r="AK35" s="142"/>
+      <c r="AL35" s="143"/>
+      <c r="AM35" s="147"/>
       <c r="AN35" s="61"/>
-      <c r="AO35" s="181"/>
-      <c r="AP35" s="181"/>
-      <c r="AQ35" s="181"/>
-      <c r="AR35" s="181"/>
-      <c r="AS35" s="181"/>
-      <c r="AT35" s="181"/>
-      <c r="AU35" s="181"/>
+      <c r="AO35" s="146"/>
+      <c r="AP35" s="146"/>
+      <c r="AQ35" s="146"/>
+      <c r="AR35" s="146"/>
+      <c r="AS35" s="146"/>
+      <c r="AT35" s="146"/>
+      <c r="AU35" s="146"/>
       <c r="AV35" s="30"/>
     </row>
     <row r="36" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3515,50 +3509,50 @@
       <c r="K36" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="L36" s="142"/>
-      <c r="M36" s="143"/>
-      <c r="N36" s="143"/>
+      <c r="L36" s="149"/>
+      <c r="M36" s="150"/>
+      <c r="N36" s="150"/>
       <c r="O36" s="65"/>
       <c r="P36" s="41"/>
       <c r="Q36" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="R36" s="142"/>
-      <c r="S36" s="143"/>
-      <c r="T36" s="143"/>
+      <c r="R36" s="149"/>
+      <c r="S36" s="150"/>
+      <c r="T36" s="150"/>
       <c r="U36" s="40"/>
       <c r="V36" s="41"/>
       <c r="W36" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="X36" s="148"/>
-      <c r="Y36" s="148"/>
-      <c r="Z36" s="148"/>
+      <c r="X36" s="151"/>
+      <c r="Y36" s="151"/>
+      <c r="Z36" s="151"/>
       <c r="AA36" s="40"/>
       <c r="AB36" s="41"/>
       <c r="AC36" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="AD36" s="142"/>
-      <c r="AE36" s="143"/>
-      <c r="AF36" s="143"/>
+      <c r="AD36" s="149"/>
+      <c r="AE36" s="150"/>
+      <c r="AF36" s="150"/>
       <c r="AG36" s="40"/>
       <c r="AH36" s="41"/>
       <c r="AI36" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="AJ36" s="142"/>
-      <c r="AK36" s="143"/>
-      <c r="AL36" s="143"/>
+      <c r="AJ36" s="149"/>
+      <c r="AK36" s="150"/>
+      <c r="AL36" s="150"/>
       <c r="AM36" s="77"/>
       <c r="AN36" s="2"/>
-      <c r="AO36" s="181"/>
-      <c r="AP36" s="181"/>
-      <c r="AQ36" s="181"/>
-      <c r="AR36" s="181"/>
-      <c r="AS36" s="181"/>
-      <c r="AT36" s="181"/>
-      <c r="AU36" s="181"/>
+      <c r="AO36" s="146"/>
+      <c r="AP36" s="146"/>
+      <c r="AQ36" s="146"/>
+      <c r="AR36" s="146"/>
+      <c r="AS36" s="146"/>
+      <c r="AT36" s="146"/>
+      <c r="AU36" s="146"/>
       <c r="AV36" s="22"/>
     </row>
     <row r="37" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3569,7 +3563,7 @@
       <c r="E37" s="133"/>
       <c r="F37" s="42"/>
       <c r="G37" s="42"/>
-      <c r="H37" s="138"/>
+      <c r="H37" s="137"/>
       <c r="I37" s="123"/>
       <c r="J37" s="74"/>
       <c r="K37" s="71"/>
@@ -3602,13 +3596,13 @@
       <c r="AL37" s="72"/>
       <c r="AM37" s="73"/>
       <c r="AN37" s="2"/>
-      <c r="AO37" s="181"/>
-      <c r="AP37" s="181"/>
-      <c r="AQ37" s="181"/>
-      <c r="AR37" s="181"/>
-      <c r="AS37" s="181"/>
-      <c r="AT37" s="181"/>
-      <c r="AU37" s="181"/>
+      <c r="AO37" s="146"/>
+      <c r="AP37" s="146"/>
+      <c r="AQ37" s="146"/>
+      <c r="AR37" s="146"/>
+      <c r="AS37" s="146"/>
+      <c r="AT37" s="146"/>
+      <c r="AU37" s="146"/>
       <c r="AV37" s="22"/>
     </row>
     <row r="38" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3616,49 +3610,49 @@
       <c r="B38" s="131"/>
       <c r="C38" s="81"/>
       <c r="D38" s="134"/>
-      <c r="E38" s="182"/>
+      <c r="E38" s="139"/>
       <c r="F38" s="90"/>
       <c r="G38" s="81"/>
-      <c r="H38" s="139"/>
+      <c r="H38" s="138"/>
       <c r="I38" s="124"/>
       <c r="J38" s="74"/>
-      <c r="K38" s="147"/>
-      <c r="L38" s="147"/>
-      <c r="M38" s="147"/>
-      <c r="N38" s="147"/>
+      <c r="K38" s="148"/>
+      <c r="L38" s="148"/>
+      <c r="M38" s="148"/>
+      <c r="N38" s="148"/>
       <c r="O38" s="43"/>
       <c r="P38" s="72"/>
-      <c r="Q38" s="147"/>
-      <c r="R38" s="147"/>
-      <c r="S38" s="147"/>
-      <c r="T38" s="147"/>
+      <c r="Q38" s="148"/>
+      <c r="R38" s="148"/>
+      <c r="S38" s="148"/>
+      <c r="T38" s="148"/>
       <c r="U38" s="43"/>
       <c r="V38" s="72"/>
-      <c r="W38" s="147"/>
-      <c r="X38" s="147"/>
-      <c r="Y38" s="147"/>
-      <c r="Z38" s="147"/>
+      <c r="W38" s="148"/>
+      <c r="X38" s="148"/>
+      <c r="Y38" s="148"/>
+      <c r="Z38" s="148"/>
       <c r="AA38" s="43"/>
       <c r="AB38" s="72"/>
-      <c r="AC38" s="147"/>
-      <c r="AD38" s="147"/>
-      <c r="AE38" s="147"/>
-      <c r="AF38" s="147"/>
+      <c r="AC38" s="148"/>
+      <c r="AD38" s="148"/>
+      <c r="AE38" s="148"/>
+      <c r="AF38" s="148"/>
       <c r="AG38" s="43"/>
       <c r="AH38" s="72"/>
-      <c r="AI38" s="147"/>
-      <c r="AJ38" s="147"/>
-      <c r="AK38" s="147"/>
-      <c r="AL38" s="147"/>
+      <c r="AI38" s="148"/>
+      <c r="AJ38" s="148"/>
+      <c r="AK38" s="148"/>
+      <c r="AL38" s="148"/>
       <c r="AM38" s="73"/>
       <c r="AN38" s="2"/>
-      <c r="AO38" s="181"/>
-      <c r="AP38" s="181"/>
-      <c r="AQ38" s="181"/>
-      <c r="AR38" s="181"/>
-      <c r="AS38" s="181"/>
-      <c r="AT38" s="181"/>
-      <c r="AU38" s="181"/>
+      <c r="AO38" s="146"/>
+      <c r="AP38" s="146"/>
+      <c r="AQ38" s="146"/>
+      <c r="AR38" s="146"/>
+      <c r="AS38" s="146"/>
+      <c r="AT38" s="146"/>
+      <c r="AU38" s="146"/>
       <c r="AV38" s="22"/>
     </row>
     <row r="39" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3672,43 +3666,43 @@
       <c r="H39" s="87"/>
       <c r="I39" s="119"/>
       <c r="J39" s="70"/>
-      <c r="K39" s="147"/>
-      <c r="L39" s="147"/>
-      <c r="M39" s="147"/>
-      <c r="N39" s="147"/>
+      <c r="K39" s="148"/>
+      <c r="L39" s="148"/>
+      <c r="M39" s="148"/>
+      <c r="N39" s="148"/>
       <c r="O39" s="43"/>
       <c r="P39" s="72"/>
-      <c r="Q39" s="147"/>
-      <c r="R39" s="147"/>
-      <c r="S39" s="147"/>
-      <c r="T39" s="147"/>
+      <c r="Q39" s="148"/>
+      <c r="R39" s="148"/>
+      <c r="S39" s="148"/>
+      <c r="T39" s="148"/>
       <c r="U39" s="43"/>
       <c r="V39" s="72"/>
-      <c r="W39" s="147"/>
-      <c r="X39" s="147"/>
-      <c r="Y39" s="147"/>
-      <c r="Z39" s="147"/>
+      <c r="W39" s="148"/>
+      <c r="X39" s="148"/>
+      <c r="Y39" s="148"/>
+      <c r="Z39" s="148"/>
       <c r="AA39" s="43"/>
       <c r="AB39" s="72"/>
-      <c r="AC39" s="147"/>
-      <c r="AD39" s="147"/>
-      <c r="AE39" s="147"/>
-      <c r="AF39" s="147"/>
+      <c r="AC39" s="148"/>
+      <c r="AD39" s="148"/>
+      <c r="AE39" s="148"/>
+      <c r="AF39" s="148"/>
       <c r="AG39" s="43"/>
       <c r="AH39" s="72"/>
-      <c r="AI39" s="147"/>
-      <c r="AJ39" s="147"/>
-      <c r="AK39" s="147"/>
-      <c r="AL39" s="147"/>
+      <c r="AI39" s="148"/>
+      <c r="AJ39" s="148"/>
+      <c r="AK39" s="148"/>
+      <c r="AL39" s="148"/>
       <c r="AM39" s="73"/>
       <c r="AN39" s="2"/>
-      <c r="AO39" s="181"/>
-      <c r="AP39" s="181"/>
-      <c r="AQ39" s="181"/>
-      <c r="AR39" s="181"/>
-      <c r="AS39" s="181"/>
-      <c r="AT39" s="181"/>
-      <c r="AU39" s="181"/>
+      <c r="AO39" s="146"/>
+      <c r="AP39" s="146"/>
+      <c r="AQ39" s="146"/>
+      <c r="AR39" s="146"/>
+      <c r="AS39" s="146"/>
+      <c r="AT39" s="146"/>
+      <c r="AU39" s="146"/>
       <c r="AV39" s="22"/>
     </row>
     <row r="40" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3722,43 +3716,43 @@
       <c r="H40" s="87"/>
       <c r="I40" s="119"/>
       <c r="J40" s="74"/>
-      <c r="K40" s="147"/>
-      <c r="L40" s="147"/>
-      <c r="M40" s="147"/>
-      <c r="N40" s="147"/>
+      <c r="K40" s="148"/>
+      <c r="L40" s="148"/>
+      <c r="M40" s="148"/>
+      <c r="N40" s="148"/>
       <c r="O40" s="43"/>
       <c r="P40" s="72"/>
-      <c r="Q40" s="147"/>
-      <c r="R40" s="147"/>
-      <c r="S40" s="147"/>
-      <c r="T40" s="147"/>
+      <c r="Q40" s="148"/>
+      <c r="R40" s="148"/>
+      <c r="S40" s="148"/>
+      <c r="T40" s="148"/>
       <c r="U40" s="43"/>
       <c r="V40" s="72"/>
-      <c r="W40" s="147"/>
-      <c r="X40" s="147"/>
-      <c r="Y40" s="147"/>
-      <c r="Z40" s="147"/>
+      <c r="W40" s="148"/>
+      <c r="X40" s="148"/>
+      <c r="Y40" s="148"/>
+      <c r="Z40" s="148"/>
       <c r="AA40" s="43"/>
       <c r="AB40" s="72"/>
-      <c r="AC40" s="147"/>
-      <c r="AD40" s="147"/>
-      <c r="AE40" s="147"/>
-      <c r="AF40" s="147"/>
+      <c r="AC40" s="148"/>
+      <c r="AD40" s="148"/>
+      <c r="AE40" s="148"/>
+      <c r="AF40" s="148"/>
       <c r="AG40" s="43"/>
       <c r="AH40" s="72"/>
-      <c r="AI40" s="147"/>
-      <c r="AJ40" s="147"/>
-      <c r="AK40" s="147"/>
-      <c r="AL40" s="147"/>
+      <c r="AI40" s="148"/>
+      <c r="AJ40" s="148"/>
+      <c r="AK40" s="148"/>
+      <c r="AL40" s="148"/>
       <c r="AM40" s="73"/>
       <c r="AN40" s="2"/>
-      <c r="AO40" s="181"/>
-      <c r="AP40" s="181"/>
-      <c r="AQ40" s="181"/>
-      <c r="AR40" s="181"/>
-      <c r="AS40" s="181"/>
-      <c r="AT40" s="181"/>
-      <c r="AU40" s="181"/>
+      <c r="AO40" s="146"/>
+      <c r="AP40" s="146"/>
+      <c r="AQ40" s="146"/>
+      <c r="AR40" s="146"/>
+      <c r="AS40" s="146"/>
+      <c r="AT40" s="146"/>
+      <c r="AU40" s="146"/>
       <c r="AV40" s="22"/>
     </row>
     <row r="41" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3772,43 +3766,43 @@
       <c r="H41" s="87"/>
       <c r="I41" s="119"/>
       <c r="J41" s="74"/>
-      <c r="K41" s="147"/>
-      <c r="L41" s="147"/>
-      <c r="M41" s="147"/>
-      <c r="N41" s="147"/>
+      <c r="K41" s="148"/>
+      <c r="L41" s="148"/>
+      <c r="M41" s="148"/>
+      <c r="N41" s="148"/>
       <c r="O41" s="43"/>
       <c r="P41" s="72"/>
-      <c r="Q41" s="147"/>
-      <c r="R41" s="147"/>
-      <c r="S41" s="147"/>
-      <c r="T41" s="147"/>
+      <c r="Q41" s="148"/>
+      <c r="R41" s="148"/>
+      <c r="S41" s="148"/>
+      <c r="T41" s="148"/>
       <c r="U41" s="43"/>
       <c r="V41" s="72"/>
-      <c r="W41" s="147"/>
-      <c r="X41" s="147"/>
-      <c r="Y41" s="147"/>
-      <c r="Z41" s="147"/>
+      <c r="W41" s="148"/>
+      <c r="X41" s="148"/>
+      <c r="Y41" s="148"/>
+      <c r="Z41" s="148"/>
       <c r="AA41" s="43"/>
       <c r="AB41" s="72"/>
-      <c r="AC41" s="147"/>
-      <c r="AD41" s="147"/>
-      <c r="AE41" s="147"/>
-      <c r="AF41" s="147"/>
+      <c r="AC41" s="148"/>
+      <c r="AD41" s="148"/>
+      <c r="AE41" s="148"/>
+      <c r="AF41" s="148"/>
       <c r="AG41" s="43"/>
       <c r="AH41" s="72"/>
-      <c r="AI41" s="147"/>
-      <c r="AJ41" s="147"/>
-      <c r="AK41" s="147"/>
-      <c r="AL41" s="147"/>
+      <c r="AI41" s="148"/>
+      <c r="AJ41" s="148"/>
+      <c r="AK41" s="148"/>
+      <c r="AL41" s="148"/>
       <c r="AM41" s="73"/>
       <c r="AN41" s="2"/>
-      <c r="AO41" s="181"/>
-      <c r="AP41" s="181"/>
-      <c r="AQ41" s="181"/>
-      <c r="AR41" s="181"/>
-      <c r="AS41" s="181"/>
-      <c r="AT41" s="181"/>
-      <c r="AU41" s="181"/>
+      <c r="AO41" s="146"/>
+      <c r="AP41" s="146"/>
+      <c r="AQ41" s="146"/>
+      <c r="AR41" s="146"/>
+      <c r="AS41" s="146"/>
+      <c r="AT41" s="146"/>
+      <c r="AU41" s="146"/>
       <c r="AV41" s="22"/>
     </row>
     <row r="42" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3822,43 +3816,43 @@
       <c r="H42" s="87"/>
       <c r="I42" s="119"/>
       <c r="J42" s="74"/>
-      <c r="K42" s="147"/>
-      <c r="L42" s="147"/>
-      <c r="M42" s="147"/>
-      <c r="N42" s="147"/>
+      <c r="K42" s="148"/>
+      <c r="L42" s="148"/>
+      <c r="M42" s="148"/>
+      <c r="N42" s="148"/>
       <c r="O42" s="43"/>
       <c r="P42" s="72"/>
-      <c r="Q42" s="147"/>
-      <c r="R42" s="147"/>
-      <c r="S42" s="147"/>
-      <c r="T42" s="147"/>
+      <c r="Q42" s="148"/>
+      <c r="R42" s="148"/>
+      <c r="S42" s="148"/>
+      <c r="T42" s="148"/>
       <c r="U42" s="43"/>
       <c r="V42" s="72"/>
-      <c r="W42" s="147"/>
-      <c r="X42" s="147"/>
-      <c r="Y42" s="147"/>
-      <c r="Z42" s="147"/>
+      <c r="W42" s="148"/>
+      <c r="X42" s="148"/>
+      <c r="Y42" s="148"/>
+      <c r="Z42" s="148"/>
       <c r="AA42" s="43"/>
       <c r="AB42" s="72"/>
-      <c r="AC42" s="147"/>
-      <c r="AD42" s="147"/>
-      <c r="AE42" s="147"/>
-      <c r="AF42" s="147"/>
+      <c r="AC42" s="148"/>
+      <c r="AD42" s="148"/>
+      <c r="AE42" s="148"/>
+      <c r="AF42" s="148"/>
       <c r="AG42" s="43"/>
       <c r="AH42" s="72"/>
-      <c r="AI42" s="147"/>
-      <c r="AJ42" s="147"/>
-      <c r="AK42" s="147"/>
-      <c r="AL42" s="147"/>
+      <c r="AI42" s="148"/>
+      <c r="AJ42" s="148"/>
+      <c r="AK42" s="148"/>
+      <c r="AL42" s="148"/>
       <c r="AM42" s="73"/>
       <c r="AN42" s="2"/>
-      <c r="AO42" s="181"/>
-      <c r="AP42" s="181"/>
-      <c r="AQ42" s="181"/>
-      <c r="AR42" s="181"/>
-      <c r="AS42" s="181"/>
-      <c r="AT42" s="181"/>
-      <c r="AU42" s="181"/>
+      <c r="AO42" s="146"/>
+      <c r="AP42" s="146"/>
+      <c r="AQ42" s="146"/>
+      <c r="AR42" s="146"/>
+      <c r="AS42" s="146"/>
+      <c r="AT42" s="146"/>
+      <c r="AU42" s="146"/>
       <c r="AV42" s="22"/>
     </row>
     <row r="43" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3872,43 +3866,43 @@
       <c r="H43" s="87"/>
       <c r="I43" s="119"/>
       <c r="J43" s="70"/>
-      <c r="K43" s="147"/>
-      <c r="L43" s="147"/>
-      <c r="M43" s="147"/>
-      <c r="N43" s="147"/>
+      <c r="K43" s="148"/>
+      <c r="L43" s="148"/>
+      <c r="M43" s="148"/>
+      <c r="N43" s="148"/>
       <c r="O43" s="43"/>
       <c r="P43" s="72"/>
-      <c r="Q43" s="147"/>
-      <c r="R43" s="147"/>
-      <c r="S43" s="147"/>
-      <c r="T43" s="147"/>
+      <c r="Q43" s="148"/>
+      <c r="R43" s="148"/>
+      <c r="S43" s="148"/>
+      <c r="T43" s="148"/>
       <c r="U43" s="43"/>
       <c r="V43" s="72"/>
-      <c r="W43" s="147"/>
-      <c r="X43" s="147"/>
-      <c r="Y43" s="147"/>
-      <c r="Z43" s="147"/>
+      <c r="W43" s="148"/>
+      <c r="X43" s="148"/>
+      <c r="Y43" s="148"/>
+      <c r="Z43" s="148"/>
       <c r="AA43" s="43"/>
       <c r="AB43" s="72"/>
-      <c r="AC43" s="147"/>
-      <c r="AD43" s="147"/>
-      <c r="AE43" s="147"/>
-      <c r="AF43" s="147"/>
+      <c r="AC43" s="148"/>
+      <c r="AD43" s="148"/>
+      <c r="AE43" s="148"/>
+      <c r="AF43" s="148"/>
       <c r="AG43" s="43"/>
       <c r="AH43" s="72"/>
-      <c r="AI43" s="147"/>
-      <c r="AJ43" s="147"/>
-      <c r="AK43" s="147"/>
-      <c r="AL43" s="147"/>
+      <c r="AI43" s="148"/>
+      <c r="AJ43" s="148"/>
+      <c r="AK43" s="148"/>
+      <c r="AL43" s="148"/>
       <c r="AM43" s="73"/>
       <c r="AN43" s="2"/>
-      <c r="AO43" s="181"/>
-      <c r="AP43" s="181"/>
-      <c r="AQ43" s="181"/>
-      <c r="AR43" s="181"/>
-      <c r="AS43" s="181"/>
-      <c r="AT43" s="181"/>
-      <c r="AU43" s="181"/>
+      <c r="AO43" s="146"/>
+      <c r="AP43" s="146"/>
+      <c r="AQ43" s="146"/>
+      <c r="AR43" s="146"/>
+      <c r="AS43" s="146"/>
+      <c r="AT43" s="146"/>
+      <c r="AU43" s="146"/>
       <c r="AV43" s="22"/>
     </row>
     <row r="44" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3925,50 +3919,50 @@
       <c r="K44" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="L44" s="145"/>
-      <c r="M44" s="146"/>
-      <c r="N44" s="145"/>
+      <c r="L44" s="143"/>
+      <c r="M44" s="142"/>
+      <c r="N44" s="143"/>
       <c r="O44" s="43"/>
       <c r="P44" s="72"/>
       <c r="Q44" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="R44" s="145"/>
-      <c r="S44" s="146"/>
-      <c r="T44" s="145"/>
+      <c r="R44" s="143"/>
+      <c r="S44" s="142"/>
+      <c r="T44" s="143"/>
       <c r="U44" s="43"/>
       <c r="V44" s="72"/>
       <c r="W44" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="X44" s="145"/>
-      <c r="Y44" s="146"/>
-      <c r="Z44" s="145"/>
+      <c r="X44" s="143"/>
+      <c r="Y44" s="142"/>
+      <c r="Z44" s="143"/>
       <c r="AA44" s="43"/>
       <c r="AB44" s="72"/>
       <c r="AC44" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AD44" s="145"/>
-      <c r="AE44" s="146"/>
-      <c r="AF44" s="145"/>
+      <c r="AD44" s="143"/>
+      <c r="AE44" s="142"/>
+      <c r="AF44" s="143"/>
       <c r="AG44" s="43"/>
       <c r="AH44" s="72"/>
       <c r="AI44" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AJ44" s="145"/>
-      <c r="AK44" s="146"/>
-      <c r="AL44" s="145"/>
+      <c r="AJ44" s="143"/>
+      <c r="AK44" s="142"/>
+      <c r="AL44" s="143"/>
       <c r="AM44" s="43"/>
       <c r="AN44" s="2"/>
-      <c r="AO44" s="181"/>
-      <c r="AP44" s="181"/>
-      <c r="AQ44" s="181"/>
-      <c r="AR44" s="181"/>
-      <c r="AS44" s="181"/>
-      <c r="AT44" s="181"/>
-      <c r="AU44" s="181"/>
+      <c r="AO44" s="146"/>
+      <c r="AP44" s="146"/>
+      <c r="AQ44" s="146"/>
+      <c r="AR44" s="146"/>
+      <c r="AS44" s="146"/>
+      <c r="AT44" s="146"/>
+      <c r="AU44" s="146"/>
       <c r="AV44" s="22"/>
     </row>
     <row r="45" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3986,49 +3980,49 @@
         <v>32</v>
       </c>
       <c r="L45" s="72"/>
-      <c r="M45" s="146"/>
-      <c r="N45" s="145"/>
+      <c r="M45" s="142"/>
+      <c r="N45" s="143"/>
       <c r="O45" s="43"/>
       <c r="P45" s="72"/>
       <c r="Q45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="R45" s="72"/>
-      <c r="S45" s="146"/>
-      <c r="T45" s="145"/>
+      <c r="S45" s="142"/>
+      <c r="T45" s="143"/>
       <c r="U45" s="43"/>
       <c r="V45" s="72"/>
       <c r="W45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="X45" s="72"/>
-      <c r="Y45" s="146"/>
-      <c r="Z45" s="145"/>
+      <c r="Y45" s="142"/>
+      <c r="Z45" s="143"/>
       <c r="AA45" s="43"/>
       <c r="AB45" s="72"/>
       <c r="AC45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AD45" s="72"/>
-      <c r="AE45" s="146"/>
-      <c r="AF45" s="145"/>
+      <c r="AE45" s="142"/>
+      <c r="AF45" s="143"/>
       <c r="AG45" s="43"/>
       <c r="AH45" s="72"/>
       <c r="AI45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AJ45" s="72"/>
-      <c r="AK45" s="146"/>
-      <c r="AL45" s="145"/>
-      <c r="AM45" s="149"/>
+      <c r="AK45" s="142"/>
+      <c r="AL45" s="143"/>
+      <c r="AM45" s="147"/>
       <c r="AN45" s="2"/>
-      <c r="AO45" s="181"/>
-      <c r="AP45" s="181"/>
-      <c r="AQ45" s="181"/>
-      <c r="AR45" s="181"/>
-      <c r="AS45" s="181"/>
-      <c r="AT45" s="181"/>
-      <c r="AU45" s="181"/>
+      <c r="AO45" s="146"/>
+      <c r="AP45" s="146"/>
+      <c r="AQ45" s="146"/>
+      <c r="AR45" s="146"/>
+      <c r="AS45" s="146"/>
+      <c r="AT45" s="146"/>
+      <c r="AU45" s="146"/>
       <c r="AV45" s="22"/>
     </row>
     <row r="46" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4045,41 +4039,41 @@
       <c r="K46" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="L46" s="148"/>
-      <c r="M46" s="148"/>
-      <c r="N46" s="148"/>
+      <c r="L46" s="151"/>
+      <c r="M46" s="151"/>
+      <c r="N46" s="151"/>
       <c r="O46" s="40"/>
       <c r="P46" s="41"/>
       <c r="Q46" s="48" t="s">
         <v>45</v>
       </c>
-      <c r="R46" s="142"/>
-      <c r="S46" s="143"/>
-      <c r="T46" s="143"/>
+      <c r="R46" s="149"/>
+      <c r="S46" s="150"/>
+      <c r="T46" s="150"/>
       <c r="U46" s="40"/>
       <c r="V46" s="41"/>
       <c r="W46" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="X46" s="148"/>
-      <c r="Y46" s="148"/>
-      <c r="Z46" s="148"/>
+      <c r="X46" s="151"/>
+      <c r="Y46" s="151"/>
+      <c r="Z46" s="151"/>
       <c r="AA46" s="40"/>
       <c r="AB46" s="41"/>
       <c r="AC46" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="AD46" s="142"/>
-      <c r="AE46" s="143"/>
-      <c r="AF46" s="143"/>
+      <c r="AD46" s="149"/>
+      <c r="AE46" s="150"/>
+      <c r="AF46" s="150"/>
       <c r="AG46" s="40"/>
       <c r="AH46" s="41"/>
       <c r="AI46" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="AJ46" s="142"/>
-      <c r="AK46" s="143"/>
-      <c r="AL46" s="143"/>
+      <c r="AJ46" s="149"/>
+      <c r="AK46" s="150"/>
+      <c r="AL46" s="150"/>
       <c r="AM46" s="40"/>
       <c r="AN46" s="51"/>
       <c r="AO46" s="51"/>
@@ -4096,10 +4090,10 @@
       <c r="B47" s="45"/>
       <c r="C47" s="42"/>
       <c r="D47" s="133"/>
-      <c r="E47" s="183"/>
+      <c r="E47" s="140"/>
       <c r="F47" s="47"/>
       <c r="G47" s="42"/>
-      <c r="H47" s="138"/>
+      <c r="H47" s="137"/>
       <c r="I47" s="123"/>
       <c r="J47" s="74"/>
       <c r="K47" s="71"/>
@@ -4146,40 +4140,40 @@
       <c r="B48" s="80"/>
       <c r="C48" s="81"/>
       <c r="D48" s="134"/>
-      <c r="E48" s="184"/>
+      <c r="E48" s="141"/>
       <c r="F48" s="90"/>
       <c r="G48" s="81"/>
-      <c r="H48" s="139"/>
+      <c r="H48" s="138"/>
       <c r="I48" s="124"/>
       <c r="J48" s="74"/>
-      <c r="K48" s="147"/>
-      <c r="L48" s="147"/>
-      <c r="M48" s="147"/>
-      <c r="N48" s="147"/>
+      <c r="K48" s="148"/>
+      <c r="L48" s="148"/>
+      <c r="M48" s="148"/>
+      <c r="N48" s="148"/>
       <c r="O48" s="43"/>
       <c r="P48" s="72"/>
-      <c r="Q48" s="147"/>
-      <c r="R48" s="147"/>
-      <c r="S48" s="147"/>
-      <c r="T48" s="147"/>
+      <c r="Q48" s="148"/>
+      <c r="R48" s="148"/>
+      <c r="S48" s="148"/>
+      <c r="T48" s="148"/>
       <c r="U48" s="43"/>
       <c r="V48" s="72"/>
-      <c r="W48" s="147"/>
-      <c r="X48" s="147"/>
-      <c r="Y48" s="147"/>
-      <c r="Z48" s="147"/>
+      <c r="W48" s="148"/>
+      <c r="X48" s="148"/>
+      <c r="Y48" s="148"/>
+      <c r="Z48" s="148"/>
       <c r="AA48" s="43"/>
       <c r="AB48" s="72"/>
-      <c r="AC48" s="147"/>
-      <c r="AD48" s="147"/>
-      <c r="AE48" s="147"/>
-      <c r="AF48" s="147"/>
+      <c r="AC48" s="148"/>
+      <c r="AD48" s="148"/>
+      <c r="AE48" s="148"/>
+      <c r="AF48" s="148"/>
       <c r="AG48" s="43"/>
       <c r="AH48" s="72"/>
-      <c r="AI48" s="147"/>
-      <c r="AJ48" s="147"/>
-      <c r="AK48" s="147"/>
-      <c r="AL48" s="147"/>
+      <c r="AI48" s="148"/>
+      <c r="AJ48" s="148"/>
+      <c r="AK48" s="148"/>
+      <c r="AL48" s="148"/>
       <c r="AM48" s="73"/>
       <c r="AN48" s="53"/>
       <c r="AO48" s="53"/>
@@ -4202,34 +4196,34 @@
       <c r="H49" s="87"/>
       <c r="I49" s="119"/>
       <c r="J49" s="70"/>
-      <c r="K49" s="147"/>
-      <c r="L49" s="147"/>
-      <c r="M49" s="147"/>
-      <c r="N49" s="147"/>
+      <c r="K49" s="148"/>
+      <c r="L49" s="148"/>
+      <c r="M49" s="148"/>
+      <c r="N49" s="148"/>
       <c r="O49" s="43"/>
       <c r="P49" s="72"/>
-      <c r="Q49" s="147"/>
-      <c r="R49" s="147"/>
-      <c r="S49" s="147"/>
-      <c r="T49" s="147"/>
+      <c r="Q49" s="148"/>
+      <c r="R49" s="148"/>
+      <c r="S49" s="148"/>
+      <c r="T49" s="148"/>
       <c r="U49" s="43"/>
       <c r="V49" s="72"/>
-      <c r="W49" s="147"/>
-      <c r="X49" s="147"/>
-      <c r="Y49" s="147"/>
-      <c r="Z49" s="147"/>
+      <c r="W49" s="148"/>
+      <c r="X49" s="148"/>
+      <c r="Y49" s="148"/>
+      <c r="Z49" s="148"/>
       <c r="AA49" s="43"/>
       <c r="AB49" s="72"/>
-      <c r="AC49" s="147"/>
-      <c r="AD49" s="147"/>
-      <c r="AE49" s="147"/>
-      <c r="AF49" s="147"/>
+      <c r="AC49" s="148"/>
+      <c r="AD49" s="148"/>
+      <c r="AE49" s="148"/>
+      <c r="AF49" s="148"/>
       <c r="AG49" s="43"/>
       <c r="AH49" s="72"/>
-      <c r="AI49" s="147"/>
-      <c r="AJ49" s="147"/>
-      <c r="AK49" s="147"/>
-      <c r="AL49" s="147"/>
+      <c r="AI49" s="148"/>
+      <c r="AJ49" s="148"/>
+      <c r="AK49" s="148"/>
+      <c r="AL49" s="148"/>
       <c r="AM49" s="73"/>
       <c r="AN49" s="53"/>
       <c r="AO49" s="53"/>
@@ -4252,34 +4246,34 @@
       <c r="H50" s="87"/>
       <c r="I50" s="119"/>
       <c r="J50" s="74"/>
-      <c r="K50" s="147"/>
-      <c r="L50" s="147"/>
-      <c r="M50" s="147"/>
-      <c r="N50" s="147"/>
+      <c r="K50" s="148"/>
+      <c r="L50" s="148"/>
+      <c r="M50" s="148"/>
+      <c r="N50" s="148"/>
       <c r="O50" s="43"/>
       <c r="P50" s="72"/>
-      <c r="Q50" s="147"/>
-      <c r="R50" s="147"/>
-      <c r="S50" s="147"/>
-      <c r="T50" s="147"/>
+      <c r="Q50" s="148"/>
+      <c r="R50" s="148"/>
+      <c r="S50" s="148"/>
+      <c r="T50" s="148"/>
       <c r="U50" s="43"/>
       <c r="V50" s="72"/>
-      <c r="W50" s="147"/>
-      <c r="X50" s="147"/>
-      <c r="Y50" s="147"/>
-      <c r="Z50" s="147"/>
+      <c r="W50" s="148"/>
+      <c r="X50" s="148"/>
+      <c r="Y50" s="148"/>
+      <c r="Z50" s="148"/>
       <c r="AA50" s="43"/>
       <c r="AB50" s="72"/>
-      <c r="AC50" s="147"/>
-      <c r="AD50" s="147"/>
-      <c r="AE50" s="147"/>
-      <c r="AF50" s="147"/>
+      <c r="AC50" s="148"/>
+      <c r="AD50" s="148"/>
+      <c r="AE50" s="148"/>
+      <c r="AF50" s="148"/>
       <c r="AG50" s="43"/>
       <c r="AH50" s="72"/>
-      <c r="AI50" s="147"/>
-      <c r="AJ50" s="147"/>
-      <c r="AK50" s="147"/>
-      <c r="AL50" s="147"/>
+      <c r="AI50" s="148"/>
+      <c r="AJ50" s="148"/>
+      <c r="AK50" s="148"/>
+      <c r="AL50" s="148"/>
       <c r="AM50" s="73"/>
       <c r="AN50" s="53"/>
       <c r="AO50" s="53"/>
@@ -4302,34 +4296,34 @@
       <c r="H51" s="87"/>
       <c r="I51" s="119"/>
       <c r="J51" s="74"/>
-      <c r="K51" s="147"/>
-      <c r="L51" s="147"/>
-      <c r="M51" s="147"/>
-      <c r="N51" s="147"/>
+      <c r="K51" s="148"/>
+      <c r="L51" s="148"/>
+      <c r="M51" s="148"/>
+      <c r="N51" s="148"/>
       <c r="O51" s="43"/>
       <c r="P51" s="72"/>
-      <c r="Q51" s="147"/>
-      <c r="R51" s="147"/>
-      <c r="S51" s="147"/>
-      <c r="T51" s="147"/>
+      <c r="Q51" s="148"/>
+      <c r="R51" s="148"/>
+      <c r="S51" s="148"/>
+      <c r="T51" s="148"/>
       <c r="U51" s="43"/>
       <c r="V51" s="72"/>
-      <c r="W51" s="147"/>
-      <c r="X51" s="147"/>
-      <c r="Y51" s="147"/>
-      <c r="Z51" s="147"/>
+      <c r="W51" s="148"/>
+      <c r="X51" s="148"/>
+      <c r="Y51" s="148"/>
+      <c r="Z51" s="148"/>
       <c r="AA51" s="43"/>
       <c r="AB51" s="72"/>
-      <c r="AC51" s="147"/>
-      <c r="AD51" s="147"/>
-      <c r="AE51" s="147"/>
-      <c r="AF51" s="147"/>
+      <c r="AC51" s="148"/>
+      <c r="AD51" s="148"/>
+      <c r="AE51" s="148"/>
+      <c r="AF51" s="148"/>
       <c r="AG51" s="43"/>
       <c r="AH51" s="72"/>
-      <c r="AI51" s="147"/>
-      <c r="AJ51" s="147"/>
-      <c r="AK51" s="147"/>
-      <c r="AL51" s="147"/>
+      <c r="AI51" s="148"/>
+      <c r="AJ51" s="148"/>
+      <c r="AK51" s="148"/>
+      <c r="AL51" s="148"/>
       <c r="AM51" s="73"/>
       <c r="AN51" s="51"/>
       <c r="AO51" s="51"/>
@@ -4352,34 +4346,34 @@
       <c r="H52" s="87"/>
       <c r="I52" s="119"/>
       <c r="J52" s="74"/>
-      <c r="K52" s="147"/>
-      <c r="L52" s="147"/>
-      <c r="M52" s="147"/>
-      <c r="N52" s="147"/>
+      <c r="K52" s="148"/>
+      <c r="L52" s="148"/>
+      <c r="M52" s="148"/>
+      <c r="N52" s="148"/>
       <c r="O52" s="43"/>
       <c r="P52" s="72"/>
-      <c r="Q52" s="147"/>
-      <c r="R52" s="147"/>
-      <c r="S52" s="147"/>
-      <c r="T52" s="147"/>
+      <c r="Q52" s="148"/>
+      <c r="R52" s="148"/>
+      <c r="S52" s="148"/>
+      <c r="T52" s="148"/>
       <c r="U52" s="43"/>
       <c r="V52" s="72"/>
-      <c r="W52" s="147"/>
-      <c r="X52" s="147"/>
-      <c r="Y52" s="147"/>
-      <c r="Z52" s="147"/>
+      <c r="W52" s="148"/>
+      <c r="X52" s="148"/>
+      <c r="Y52" s="148"/>
+      <c r="Z52" s="148"/>
       <c r="AA52" s="43"/>
       <c r="AB52" s="72"/>
-      <c r="AC52" s="147"/>
-      <c r="AD52" s="147"/>
-      <c r="AE52" s="147"/>
-      <c r="AF52" s="147"/>
+      <c r="AC52" s="148"/>
+      <c r="AD52" s="148"/>
+      <c r="AE52" s="148"/>
+      <c r="AF52" s="148"/>
       <c r="AG52" s="43"/>
       <c r="AH52" s="72"/>
-      <c r="AI52" s="147"/>
-      <c r="AJ52" s="147"/>
-      <c r="AK52" s="147"/>
-      <c r="AL52" s="147"/>
+      <c r="AI52" s="148"/>
+      <c r="AJ52" s="148"/>
+      <c r="AK52" s="148"/>
+      <c r="AL52" s="148"/>
       <c r="AM52" s="73"/>
       <c r="AN52" s="92"/>
       <c r="AO52" s="92"/>
@@ -4402,34 +4396,34 @@
       <c r="H53" s="87"/>
       <c r="I53" s="119"/>
       <c r="J53" s="70"/>
-      <c r="K53" s="147"/>
-      <c r="L53" s="147"/>
-      <c r="M53" s="147"/>
-      <c r="N53" s="147"/>
+      <c r="K53" s="148"/>
+      <c r="L53" s="148"/>
+      <c r="M53" s="148"/>
+      <c r="N53" s="148"/>
       <c r="O53" s="43"/>
       <c r="P53" s="72"/>
-      <c r="Q53" s="147"/>
-      <c r="R53" s="147"/>
-      <c r="S53" s="147"/>
-      <c r="T53" s="147"/>
+      <c r="Q53" s="148"/>
+      <c r="R53" s="148"/>
+      <c r="S53" s="148"/>
+      <c r="T53" s="148"/>
       <c r="U53" s="43"/>
       <c r="V53" s="72"/>
-      <c r="W53" s="147"/>
-      <c r="X53" s="147"/>
-      <c r="Y53" s="147"/>
-      <c r="Z53" s="147"/>
+      <c r="W53" s="148"/>
+      <c r="X53" s="148"/>
+      <c r="Y53" s="148"/>
+      <c r="Z53" s="148"/>
       <c r="AA53" s="43"/>
       <c r="AB53" s="72"/>
-      <c r="AC53" s="147"/>
-      <c r="AD53" s="147"/>
-      <c r="AE53" s="147"/>
-      <c r="AF53" s="147"/>
+      <c r="AC53" s="148"/>
+      <c r="AD53" s="148"/>
+      <c r="AE53" s="148"/>
+      <c r="AF53" s="148"/>
       <c r="AG53" s="43"/>
       <c r="AH53" s="72"/>
-      <c r="AI53" s="147"/>
-      <c r="AJ53" s="147"/>
-      <c r="AK53" s="147"/>
-      <c r="AL53" s="147"/>
+      <c r="AI53" s="148"/>
+      <c r="AJ53" s="148"/>
+      <c r="AK53" s="148"/>
+      <c r="AL53" s="148"/>
       <c r="AM53" s="72"/>
       <c r="AN53" s="97"/>
       <c r="AO53" s="93"/>
@@ -4455,41 +4449,41 @@
       <c r="K54" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="L54" s="145"/>
-      <c r="M54" s="146"/>
-      <c r="N54" s="145"/>
+      <c r="L54" s="143"/>
+      <c r="M54" s="142"/>
+      <c r="N54" s="143"/>
       <c r="O54" s="43"/>
       <c r="P54" s="72"/>
       <c r="Q54" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="R54" s="145"/>
-      <c r="S54" s="146"/>
-      <c r="T54" s="145"/>
+      <c r="R54" s="143"/>
+      <c r="S54" s="142"/>
+      <c r="T54" s="143"/>
       <c r="U54" s="43"/>
       <c r="V54" s="72"/>
       <c r="W54" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="X54" s="145"/>
-      <c r="Y54" s="146"/>
-      <c r="Z54" s="145"/>
+      <c r="X54" s="143"/>
+      <c r="Y54" s="142"/>
+      <c r="Z54" s="143"/>
       <c r="AA54" s="43"/>
       <c r="AB54" s="72"/>
       <c r="AC54" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AD54" s="145"/>
-      <c r="AE54" s="146"/>
-      <c r="AF54" s="145"/>
+      <c r="AD54" s="143"/>
+      <c r="AE54" s="142"/>
+      <c r="AF54" s="143"/>
       <c r="AG54" s="43"/>
       <c r="AH54" s="72"/>
       <c r="AI54" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="AJ54" s="145"/>
-      <c r="AK54" s="146"/>
-      <c r="AL54" s="145"/>
+      <c r="AJ54" s="143"/>
+      <c r="AK54" s="142"/>
+      <c r="AL54" s="143"/>
       <c r="AM54" s="72"/>
       <c r="AN54" s="99"/>
       <c r="AO54" s="94"/>
@@ -4516,41 +4510,41 @@
         <v>32</v>
       </c>
       <c r="L55" s="81"/>
-      <c r="M55" s="140"/>
-      <c r="N55" s="141"/>
+      <c r="M55" s="182"/>
+      <c r="N55" s="183"/>
       <c r="O55" s="82"/>
       <c r="P55" s="81"/>
       <c r="Q55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="R55" s="81"/>
-      <c r="S55" s="140"/>
-      <c r="T55" s="141"/>
+      <c r="S55" s="182"/>
+      <c r="T55" s="183"/>
       <c r="U55" s="82"/>
       <c r="V55" s="81"/>
       <c r="W55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="X55" s="81"/>
-      <c r="Y55" s="140"/>
-      <c r="Z55" s="141"/>
+      <c r="Y55" s="182"/>
+      <c r="Z55" s="183"/>
       <c r="AA55" s="82"/>
       <c r="AB55" s="81"/>
       <c r="AC55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="AD55" s="81"/>
-      <c r="AE55" s="140"/>
-      <c r="AF55" s="141"/>
+      <c r="AE55" s="182"/>
+      <c r="AF55" s="183"/>
       <c r="AG55" s="82"/>
       <c r="AH55" s="81"/>
       <c r="AI55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="AJ55" s="81"/>
-      <c r="AK55" s="140"/>
-      <c r="AL55" s="141"/>
-      <c r="AM55" s="141"/>
+      <c r="AK55" s="182"/>
+      <c r="AL55" s="183"/>
+      <c r="AM55" s="183"/>
       <c r="AN55" s="101"/>
       <c r="AO55" s="102"/>
       <c r="AP55" s="103"/>
@@ -4615,16 +4609,107 @@
     </row>
   </sheetData>
   <mergeCells count="135">
-    <mergeCell ref="AK34:AL34"/>
-    <mergeCell ref="AC34:AD34"/>
-    <mergeCell ref="AE34:AF34"/>
-    <mergeCell ref="AI34:AJ34"/>
-    <mergeCell ref="Y34:Z34"/>
-    <mergeCell ref="M35:N35"/>
-    <mergeCell ref="S35:T35"/>
-    <mergeCell ref="Y35:Z35"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="M55:N55"/>
+    <mergeCell ref="S55:T55"/>
+    <mergeCell ref="Y55:Z55"/>
+    <mergeCell ref="AE55:AF55"/>
+    <mergeCell ref="AK55:AM55"/>
+    <mergeCell ref="R46:T46"/>
+    <mergeCell ref="K54:L54"/>
+    <mergeCell ref="M54:N54"/>
+    <mergeCell ref="Q54:R54"/>
+    <mergeCell ref="S54:T54"/>
+    <mergeCell ref="W54:X54"/>
+    <mergeCell ref="Y54:Z54"/>
+    <mergeCell ref="K48:N53"/>
+    <mergeCell ref="Q48:T53"/>
+    <mergeCell ref="W48:Z53"/>
+    <mergeCell ref="L46:N46"/>
+    <mergeCell ref="X46:Z46"/>
+    <mergeCell ref="M45:N45"/>
+    <mergeCell ref="S45:T45"/>
+    <mergeCell ref="Y45:Z45"/>
+    <mergeCell ref="AE45:AF45"/>
+    <mergeCell ref="AK45:AM45"/>
+    <mergeCell ref="R36:T36"/>
+    <mergeCell ref="K44:L44"/>
+    <mergeCell ref="M44:N44"/>
+    <mergeCell ref="Q44:R44"/>
+    <mergeCell ref="S44:T44"/>
+    <mergeCell ref="W44:X44"/>
+    <mergeCell ref="Y44:Z44"/>
+    <mergeCell ref="K38:N43"/>
+    <mergeCell ref="Q38:T43"/>
+    <mergeCell ref="W38:Z43"/>
+    <mergeCell ref="L36:N36"/>
+    <mergeCell ref="X36:Z36"/>
+    <mergeCell ref="AJ36:AL36"/>
+    <mergeCell ref="AH3:AM3"/>
+    <mergeCell ref="AN3:AP3"/>
+    <mergeCell ref="AQ3:AS3"/>
+    <mergeCell ref="AT3:AV3"/>
+    <mergeCell ref="AH4:AM4"/>
+    <mergeCell ref="AN4:AP7"/>
+    <mergeCell ref="AQ4:AS7"/>
+    <mergeCell ref="AT4:AV7"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="J8:AG8"/>
+    <mergeCell ref="AH8:AM8"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="J9:AG9"/>
+    <mergeCell ref="AH9:AM9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="J10:AG10"/>
+    <mergeCell ref="AH10:AM10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:AG11"/>
+    <mergeCell ref="AH11:AM11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="J12:AG12"/>
+    <mergeCell ref="AH12:AM12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="J13:AG13"/>
+    <mergeCell ref="AH13:AM13"/>
+    <mergeCell ref="A14:AM15"/>
+    <mergeCell ref="AN15:AV15"/>
+    <mergeCell ref="L16:N16"/>
+    <mergeCell ref="R16:T16"/>
+    <mergeCell ref="X16:Z16"/>
+    <mergeCell ref="AD16:AF16"/>
+    <mergeCell ref="AJ16:AL16"/>
+    <mergeCell ref="AI24:AJ24"/>
+    <mergeCell ref="AK24:AL24"/>
+    <mergeCell ref="K18:N23"/>
+    <mergeCell ref="Q18:T23"/>
+    <mergeCell ref="W18:Z23"/>
+    <mergeCell ref="AC18:AF23"/>
+    <mergeCell ref="AI18:AL23"/>
+    <mergeCell ref="W24:X24"/>
+    <mergeCell ref="Y24:Z24"/>
+    <mergeCell ref="AC24:AD24"/>
+    <mergeCell ref="AE24:AF24"/>
+    <mergeCell ref="X26:Z26"/>
+    <mergeCell ref="L26:N26"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="Q34:R34"/>
+    <mergeCell ref="S34:T34"/>
+    <mergeCell ref="W34:X34"/>
+    <mergeCell ref="R26:T26"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="S25:T25"/>
+    <mergeCell ref="Y25:Z25"/>
+    <mergeCell ref="K28:N33"/>
+    <mergeCell ref="Q28:T33"/>
+    <mergeCell ref="W28:Z33"/>
     <mergeCell ref="AE25:AF25"/>
     <mergeCell ref="AK25:AL25"/>
     <mergeCell ref="AO26:AU45"/>
@@ -4649,107 +4734,16 @@
     <mergeCell ref="AC38:AF43"/>
     <mergeCell ref="AI38:AL43"/>
     <mergeCell ref="AD36:AF36"/>
-    <mergeCell ref="X26:Z26"/>
-    <mergeCell ref="L26:N26"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="S24:T24"/>
-    <mergeCell ref="Q34:R34"/>
-    <mergeCell ref="S34:T34"/>
-    <mergeCell ref="W34:X34"/>
-    <mergeCell ref="R26:T26"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="S25:T25"/>
-    <mergeCell ref="Y25:Z25"/>
-    <mergeCell ref="K28:N33"/>
-    <mergeCell ref="Q28:T33"/>
-    <mergeCell ref="W28:Z33"/>
-    <mergeCell ref="AN15:AV15"/>
-    <mergeCell ref="L16:N16"/>
-    <mergeCell ref="R16:T16"/>
-    <mergeCell ref="X16:Z16"/>
-    <mergeCell ref="AD16:AF16"/>
-    <mergeCell ref="AJ16:AL16"/>
-    <mergeCell ref="AI24:AJ24"/>
-    <mergeCell ref="AK24:AL24"/>
-    <mergeCell ref="K18:N23"/>
-    <mergeCell ref="Q18:T23"/>
-    <mergeCell ref="W18:Z23"/>
-    <mergeCell ref="AC18:AF23"/>
-    <mergeCell ref="AI18:AL23"/>
-    <mergeCell ref="W24:X24"/>
-    <mergeCell ref="Y24:Z24"/>
-    <mergeCell ref="AC24:AD24"/>
-    <mergeCell ref="AE24:AF24"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="J12:AG12"/>
-    <mergeCell ref="AH12:AM12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="J13:AG13"/>
-    <mergeCell ref="AH13:AM13"/>
-    <mergeCell ref="A14:AM15"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="J9:AG9"/>
-    <mergeCell ref="AH9:AM9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="J10:AG10"/>
-    <mergeCell ref="AH10:AM10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:AG11"/>
-    <mergeCell ref="AH11:AM11"/>
-    <mergeCell ref="AH3:AM3"/>
-    <mergeCell ref="AN3:AP3"/>
-    <mergeCell ref="AQ3:AS3"/>
-    <mergeCell ref="AT3:AV3"/>
-    <mergeCell ref="AH4:AM4"/>
-    <mergeCell ref="AN4:AP7"/>
-    <mergeCell ref="AQ4:AS7"/>
-    <mergeCell ref="AT4:AV7"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="J8:AG8"/>
-    <mergeCell ref="AH8:AM8"/>
-    <mergeCell ref="M45:N45"/>
-    <mergeCell ref="S45:T45"/>
-    <mergeCell ref="Y45:Z45"/>
-    <mergeCell ref="AE45:AF45"/>
-    <mergeCell ref="AK45:AM45"/>
-    <mergeCell ref="R36:T36"/>
-    <mergeCell ref="K44:L44"/>
-    <mergeCell ref="M44:N44"/>
-    <mergeCell ref="Q44:R44"/>
-    <mergeCell ref="S44:T44"/>
-    <mergeCell ref="W44:X44"/>
-    <mergeCell ref="Y44:Z44"/>
-    <mergeCell ref="K38:N43"/>
-    <mergeCell ref="Q38:T43"/>
-    <mergeCell ref="W38:Z43"/>
-    <mergeCell ref="L36:N36"/>
-    <mergeCell ref="X36:Z36"/>
-    <mergeCell ref="AJ36:AL36"/>
-    <mergeCell ref="M55:N55"/>
-    <mergeCell ref="S55:T55"/>
-    <mergeCell ref="Y55:Z55"/>
-    <mergeCell ref="AE55:AF55"/>
-    <mergeCell ref="AK55:AM55"/>
-    <mergeCell ref="R46:T46"/>
-    <mergeCell ref="K54:L54"/>
-    <mergeCell ref="M54:N54"/>
-    <mergeCell ref="Q54:R54"/>
-    <mergeCell ref="S54:T54"/>
-    <mergeCell ref="W54:X54"/>
-    <mergeCell ref="Y54:Z54"/>
-    <mergeCell ref="K48:N53"/>
-    <mergeCell ref="Q48:T53"/>
-    <mergeCell ref="W48:Z53"/>
-    <mergeCell ref="L46:N46"/>
-    <mergeCell ref="X46:Z46"/>
+    <mergeCell ref="AK34:AL34"/>
+    <mergeCell ref="AC34:AD34"/>
+    <mergeCell ref="AE34:AF34"/>
+    <mergeCell ref="AI34:AJ34"/>
+    <mergeCell ref="Y34:Z34"/>
+    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="S35:T35"/>
+    <mergeCell ref="Y35:Z35"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="M34:N34"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.1" right="0.1" top="0.1" bottom="0.1" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
Wip: minor update => Setup data sheet
</commit_message>
<xml_diff>
--- a/apps/ENG-Backend/api/engineer/mtc/templates/sds_template.xlsx
+++ b/apps/ENG-Backend/api/engineer/mtc/templates/sds_template.xlsx
@@ -1098,12 +1098,6 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="190" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1155,14 +1149,128 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="190" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="1" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="189" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1170,118 +1278,10 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="189" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="188" fontId="1" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="190" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1779,29 +1779,29 @@
       <c r="AE3" s="11"/>
       <c r="AF3" s="11"/>
       <c r="AG3" s="16"/>
-      <c r="AH3" s="167" t="s">
+      <c r="AH3" s="151" t="s">
         <v>6</v>
       </c>
-      <c r="AI3" s="168"/>
-      <c r="AJ3" s="168"/>
-      <c r="AK3" s="168"/>
-      <c r="AL3" s="168"/>
-      <c r="AM3" s="169"/>
-      <c r="AN3" s="167" t="s">
+      <c r="AI3" s="152"/>
+      <c r="AJ3" s="152"/>
+      <c r="AK3" s="152"/>
+      <c r="AL3" s="152"/>
+      <c r="AM3" s="153"/>
+      <c r="AN3" s="151" t="s">
         <v>7</v>
       </c>
-      <c r="AO3" s="168"/>
-      <c r="AP3" s="169"/>
-      <c r="AQ3" s="167" t="s">
+      <c r="AO3" s="152"/>
+      <c r="AP3" s="153"/>
+      <c r="AQ3" s="151" t="s">
         <v>8</v>
       </c>
-      <c r="AR3" s="168"/>
-      <c r="AS3" s="169"/>
-      <c r="AT3" s="167" t="s">
+      <c r="AR3" s="152"/>
+      <c r="AS3" s="153"/>
+      <c r="AT3" s="151" t="s">
         <v>9</v>
       </c>
-      <c r="AU3" s="168"/>
-      <c r="AV3" s="169"/>
+      <c r="AU3" s="152"/>
+      <c r="AV3" s="153"/>
     </row>
     <row r="4" spans="1:48" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
@@ -1845,21 +1845,21 @@
       <c r="AE4" s="11"/>
       <c r="AF4" s="11"/>
       <c r="AG4" s="11"/>
-      <c r="AH4" s="155"/>
-      <c r="AI4" s="156"/>
-      <c r="AJ4" s="156"/>
-      <c r="AK4" s="156"/>
-      <c r="AL4" s="156"/>
-      <c r="AM4" s="158"/>
-      <c r="AN4" s="170"/>
-      <c r="AO4" s="171"/>
-      <c r="AP4" s="171"/>
-      <c r="AQ4" s="170"/>
-      <c r="AR4" s="171"/>
-      <c r="AS4" s="176"/>
-      <c r="AT4" s="170"/>
-      <c r="AU4" s="171"/>
-      <c r="AV4" s="176"/>
+      <c r="AH4" s="154"/>
+      <c r="AI4" s="155"/>
+      <c r="AJ4" s="155"/>
+      <c r="AK4" s="155"/>
+      <c r="AL4" s="155"/>
+      <c r="AM4" s="156"/>
+      <c r="AN4" s="157"/>
+      <c r="AO4" s="158"/>
+      <c r="AP4" s="158"/>
+      <c r="AQ4" s="157"/>
+      <c r="AR4" s="158"/>
+      <c r="AS4" s="163"/>
+      <c r="AT4" s="157"/>
+      <c r="AU4" s="158"/>
+      <c r="AV4" s="163"/>
     </row>
     <row r="5" spans="1:48" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
@@ -1907,15 +1907,15 @@
       <c r="AK5" s="3"/>
       <c r="AL5" s="3"/>
       <c r="AM5" s="27"/>
-      <c r="AN5" s="172"/>
-      <c r="AO5" s="173"/>
-      <c r="AP5" s="173"/>
-      <c r="AQ5" s="172"/>
-      <c r="AR5" s="173"/>
-      <c r="AS5" s="177"/>
-      <c r="AT5" s="172"/>
-      <c r="AU5" s="173"/>
-      <c r="AV5" s="177"/>
+      <c r="AN5" s="159"/>
+      <c r="AO5" s="160"/>
+      <c r="AP5" s="160"/>
+      <c r="AQ5" s="159"/>
+      <c r="AR5" s="160"/>
+      <c r="AS5" s="164"/>
+      <c r="AT5" s="159"/>
+      <c r="AU5" s="160"/>
+      <c r="AV5" s="164"/>
     </row>
     <row r="6" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
@@ -1959,15 +1959,15 @@
       <c r="AK6" s="1"/>
       <c r="AL6" s="1"/>
       <c r="AM6" s="30"/>
-      <c r="AN6" s="172"/>
-      <c r="AO6" s="173"/>
-      <c r="AP6" s="173"/>
-      <c r="AQ6" s="172"/>
-      <c r="AR6" s="173"/>
-      <c r="AS6" s="177"/>
-      <c r="AT6" s="172"/>
-      <c r="AU6" s="173"/>
-      <c r="AV6" s="177"/>
+      <c r="AN6" s="159"/>
+      <c r="AO6" s="160"/>
+      <c r="AP6" s="160"/>
+      <c r="AQ6" s="159"/>
+      <c r="AR6" s="160"/>
+      <c r="AS6" s="164"/>
+      <c r="AT6" s="159"/>
+      <c r="AU6" s="160"/>
+      <c r="AV6" s="164"/>
     </row>
     <row r="7" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="31"/>
@@ -2009,66 +2009,66 @@
       <c r="AK7" s="32"/>
       <c r="AL7" s="32"/>
       <c r="AM7" s="33"/>
-      <c r="AN7" s="174"/>
-      <c r="AO7" s="175"/>
-      <c r="AP7" s="175"/>
-      <c r="AQ7" s="174"/>
-      <c r="AR7" s="175"/>
-      <c r="AS7" s="178"/>
-      <c r="AT7" s="174"/>
-      <c r="AU7" s="175"/>
-      <c r="AV7" s="178"/>
+      <c r="AN7" s="161"/>
+      <c r="AO7" s="162"/>
+      <c r="AP7" s="162"/>
+      <c r="AQ7" s="161"/>
+      <c r="AR7" s="162"/>
+      <c r="AS7" s="165"/>
+      <c r="AT7" s="161"/>
+      <c r="AU7" s="162"/>
+      <c r="AV7" s="165"/>
     </row>
     <row r="8" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="179" t="s">
+      <c r="B8" s="166" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="165"/>
-      <c r="D8" s="165"/>
-      <c r="E8" s="165"/>
-      <c r="F8" s="165"/>
-      <c r="G8" s="180" t="s">
+      <c r="C8" s="167"/>
+      <c r="D8" s="167"/>
+      <c r="E8" s="167"/>
+      <c r="F8" s="167"/>
+      <c r="G8" s="168" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="165"/>
-      <c r="I8" s="181"/>
-      <c r="J8" s="167" t="s">
+      <c r="H8" s="167"/>
+      <c r="I8" s="169"/>
+      <c r="J8" s="151" t="s">
         <v>21</v>
       </c>
-      <c r="K8" s="168"/>
-      <c r="L8" s="168"/>
-      <c r="M8" s="168"/>
-      <c r="N8" s="168"/>
-      <c r="O8" s="168"/>
-      <c r="P8" s="168"/>
-      <c r="Q8" s="168"/>
-      <c r="R8" s="168"/>
-      <c r="S8" s="168"/>
-      <c r="T8" s="168"/>
-      <c r="U8" s="168"/>
-      <c r="V8" s="168"/>
-      <c r="W8" s="168"/>
-      <c r="X8" s="168"/>
-      <c r="Y8" s="168"/>
-      <c r="Z8" s="168"/>
-      <c r="AA8" s="168"/>
-      <c r="AB8" s="168"/>
-      <c r="AC8" s="168"/>
-      <c r="AD8" s="168"/>
-      <c r="AE8" s="168"/>
-      <c r="AF8" s="168"/>
-      <c r="AG8" s="169"/>
-      <c r="AH8" s="167" t="s">
+      <c r="K8" s="152"/>
+      <c r="L8" s="152"/>
+      <c r="M8" s="152"/>
+      <c r="N8" s="152"/>
+      <c r="O8" s="152"/>
+      <c r="P8" s="152"/>
+      <c r="Q8" s="152"/>
+      <c r="R8" s="152"/>
+      <c r="S8" s="152"/>
+      <c r="T8" s="152"/>
+      <c r="U8" s="152"/>
+      <c r="V8" s="152"/>
+      <c r="W8" s="152"/>
+      <c r="X8" s="152"/>
+      <c r="Y8" s="152"/>
+      <c r="Z8" s="152"/>
+      <c r="AA8" s="152"/>
+      <c r="AB8" s="152"/>
+      <c r="AC8" s="152"/>
+      <c r="AD8" s="152"/>
+      <c r="AE8" s="152"/>
+      <c r="AF8" s="152"/>
+      <c r="AG8" s="153"/>
+      <c r="AH8" s="151" t="s">
         <v>22</v>
       </c>
-      <c r="AI8" s="168"/>
-      <c r="AJ8" s="168"/>
-      <c r="AK8" s="168"/>
-      <c r="AL8" s="168"/>
-      <c r="AM8" s="169"/>
+      <c r="AI8" s="152"/>
+      <c r="AJ8" s="152"/>
+      <c r="AK8" s="152"/>
+      <c r="AL8" s="152"/>
+      <c r="AM8" s="153"/>
       <c r="AN8" s="29" t="s">
         <v>23</v>
       </c>
@@ -2083,44 +2083,44 @@
     </row>
     <row r="9" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="108"/>
-      <c r="B9" s="155"/>
-      <c r="C9" s="156"/>
-      <c r="D9" s="156"/>
-      <c r="E9" s="156"/>
-      <c r="F9" s="156"/>
-      <c r="G9" s="157"/>
-      <c r="H9" s="156"/>
-      <c r="I9" s="158"/>
-      <c r="J9" s="159"/>
-      <c r="K9" s="160"/>
-      <c r="L9" s="160"/>
-      <c r="M9" s="160"/>
-      <c r="N9" s="160"/>
-      <c r="O9" s="160"/>
-      <c r="P9" s="160"/>
-      <c r="Q9" s="160"/>
-      <c r="R9" s="160"/>
-      <c r="S9" s="160"/>
-      <c r="T9" s="160"/>
-      <c r="U9" s="160"/>
-      <c r="V9" s="160"/>
-      <c r="W9" s="160"/>
-      <c r="X9" s="160"/>
-      <c r="Y9" s="160"/>
-      <c r="Z9" s="160"/>
-      <c r="AA9" s="160"/>
-      <c r="AB9" s="160"/>
-      <c r="AC9" s="160"/>
-      <c r="AD9" s="160"/>
-      <c r="AE9" s="160"/>
-      <c r="AF9" s="160"/>
-      <c r="AG9" s="161"/>
-      <c r="AH9" s="159"/>
-      <c r="AI9" s="160"/>
-      <c r="AJ9" s="160"/>
-      <c r="AK9" s="160"/>
-      <c r="AL9" s="160"/>
-      <c r="AM9" s="161"/>
+      <c r="B9" s="154"/>
+      <c r="C9" s="155"/>
+      <c r="D9" s="155"/>
+      <c r="E9" s="155"/>
+      <c r="F9" s="155"/>
+      <c r="G9" s="170"/>
+      <c r="H9" s="155"/>
+      <c r="I9" s="156"/>
+      <c r="J9" s="171"/>
+      <c r="K9" s="172"/>
+      <c r="L9" s="172"/>
+      <c r="M9" s="172"/>
+      <c r="N9" s="172"/>
+      <c r="O9" s="172"/>
+      <c r="P9" s="172"/>
+      <c r="Q9" s="172"/>
+      <c r="R9" s="172"/>
+      <c r="S9" s="172"/>
+      <c r="T9" s="172"/>
+      <c r="U9" s="172"/>
+      <c r="V9" s="172"/>
+      <c r="W9" s="172"/>
+      <c r="X9" s="172"/>
+      <c r="Y9" s="172"/>
+      <c r="Z9" s="172"/>
+      <c r="AA9" s="172"/>
+      <c r="AB9" s="172"/>
+      <c r="AC9" s="172"/>
+      <c r="AD9" s="172"/>
+      <c r="AE9" s="172"/>
+      <c r="AF9" s="172"/>
+      <c r="AG9" s="173"/>
+      <c r="AH9" s="171"/>
+      <c r="AI9" s="172"/>
+      <c r="AJ9" s="172"/>
+      <c r="AK9" s="172"/>
+      <c r="AL9" s="172"/>
+      <c r="AM9" s="173"/>
       <c r="AN9" s="35"/>
       <c r="AO9" s="2"/>
       <c r="AP9" s="2"/>
@@ -2133,44 +2133,44 @@
     </row>
     <row r="10" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="108"/>
-      <c r="B10" s="155"/>
-      <c r="C10" s="156"/>
-      <c r="D10" s="156"/>
-      <c r="E10" s="156"/>
-      <c r="F10" s="156"/>
-      <c r="G10" s="157"/>
-      <c r="H10" s="156"/>
-      <c r="I10" s="158"/>
-      <c r="J10" s="159"/>
-      <c r="K10" s="160"/>
-      <c r="L10" s="160"/>
-      <c r="M10" s="160"/>
-      <c r="N10" s="160"/>
-      <c r="O10" s="160"/>
-      <c r="P10" s="160"/>
-      <c r="Q10" s="160"/>
-      <c r="R10" s="160"/>
-      <c r="S10" s="160"/>
-      <c r="T10" s="160"/>
-      <c r="U10" s="160"/>
-      <c r="V10" s="160"/>
-      <c r="W10" s="160"/>
-      <c r="X10" s="160"/>
-      <c r="Y10" s="160"/>
-      <c r="Z10" s="160"/>
-      <c r="AA10" s="160"/>
-      <c r="AB10" s="160"/>
-      <c r="AC10" s="160"/>
-      <c r="AD10" s="160"/>
-      <c r="AE10" s="160"/>
-      <c r="AF10" s="160"/>
-      <c r="AG10" s="161"/>
-      <c r="AH10" s="159"/>
-      <c r="AI10" s="160"/>
-      <c r="AJ10" s="160"/>
-      <c r="AK10" s="160"/>
-      <c r="AL10" s="160"/>
-      <c r="AM10" s="161"/>
+      <c r="B10" s="154"/>
+      <c r="C10" s="155"/>
+      <c r="D10" s="155"/>
+      <c r="E10" s="155"/>
+      <c r="F10" s="155"/>
+      <c r="G10" s="170"/>
+      <c r="H10" s="155"/>
+      <c r="I10" s="156"/>
+      <c r="J10" s="171"/>
+      <c r="K10" s="172"/>
+      <c r="L10" s="172"/>
+      <c r="M10" s="172"/>
+      <c r="N10" s="172"/>
+      <c r="O10" s="172"/>
+      <c r="P10" s="172"/>
+      <c r="Q10" s="172"/>
+      <c r="R10" s="172"/>
+      <c r="S10" s="172"/>
+      <c r="T10" s="172"/>
+      <c r="U10" s="172"/>
+      <c r="V10" s="172"/>
+      <c r="W10" s="172"/>
+      <c r="X10" s="172"/>
+      <c r="Y10" s="172"/>
+      <c r="Z10" s="172"/>
+      <c r="AA10" s="172"/>
+      <c r="AB10" s="172"/>
+      <c r="AC10" s="172"/>
+      <c r="AD10" s="172"/>
+      <c r="AE10" s="172"/>
+      <c r="AF10" s="172"/>
+      <c r="AG10" s="173"/>
+      <c r="AH10" s="171"/>
+      <c r="AI10" s="172"/>
+      <c r="AJ10" s="172"/>
+      <c r="AK10" s="172"/>
+      <c r="AL10" s="172"/>
+      <c r="AM10" s="173"/>
       <c r="AN10" s="35"/>
       <c r="AO10" s="2"/>
       <c r="AP10" s="2"/>
@@ -2183,44 +2183,44 @@
     </row>
     <row r="11" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="108"/>
-      <c r="B11" s="155"/>
-      <c r="C11" s="156"/>
-      <c r="D11" s="156"/>
-      <c r="E11" s="156"/>
-      <c r="F11" s="156"/>
-      <c r="G11" s="157"/>
-      <c r="H11" s="156"/>
-      <c r="I11" s="158"/>
-      <c r="J11" s="159"/>
-      <c r="K11" s="160"/>
-      <c r="L11" s="160"/>
-      <c r="M11" s="160"/>
-      <c r="N11" s="160"/>
-      <c r="O11" s="160"/>
-      <c r="P11" s="160"/>
-      <c r="Q11" s="160"/>
-      <c r="R11" s="160"/>
-      <c r="S11" s="160"/>
-      <c r="T11" s="160"/>
-      <c r="U11" s="160"/>
-      <c r="V11" s="160"/>
-      <c r="W11" s="160"/>
-      <c r="X11" s="160"/>
-      <c r="Y11" s="160"/>
-      <c r="Z11" s="160"/>
-      <c r="AA11" s="160"/>
-      <c r="AB11" s="160"/>
-      <c r="AC11" s="160"/>
-      <c r="AD11" s="160"/>
-      <c r="AE11" s="160"/>
-      <c r="AF11" s="160"/>
-      <c r="AG11" s="161"/>
-      <c r="AH11" s="159"/>
-      <c r="AI11" s="160"/>
-      <c r="AJ11" s="160"/>
-      <c r="AK11" s="160"/>
-      <c r="AL11" s="160"/>
-      <c r="AM11" s="161"/>
+      <c r="B11" s="154"/>
+      <c r="C11" s="155"/>
+      <c r="D11" s="155"/>
+      <c r="E11" s="155"/>
+      <c r="F11" s="155"/>
+      <c r="G11" s="170"/>
+      <c r="H11" s="155"/>
+      <c r="I11" s="156"/>
+      <c r="J11" s="171"/>
+      <c r="K11" s="172"/>
+      <c r="L11" s="172"/>
+      <c r="M11" s="172"/>
+      <c r="N11" s="172"/>
+      <c r="O11" s="172"/>
+      <c r="P11" s="172"/>
+      <c r="Q11" s="172"/>
+      <c r="R11" s="172"/>
+      <c r="S11" s="172"/>
+      <c r="T11" s="172"/>
+      <c r="U11" s="172"/>
+      <c r="V11" s="172"/>
+      <c r="W11" s="172"/>
+      <c r="X11" s="172"/>
+      <c r="Y11" s="172"/>
+      <c r="Z11" s="172"/>
+      <c r="AA11" s="172"/>
+      <c r="AB11" s="172"/>
+      <c r="AC11" s="172"/>
+      <c r="AD11" s="172"/>
+      <c r="AE11" s="172"/>
+      <c r="AF11" s="172"/>
+      <c r="AG11" s="173"/>
+      <c r="AH11" s="171"/>
+      <c r="AI11" s="172"/>
+      <c r="AJ11" s="172"/>
+      <c r="AK11" s="172"/>
+      <c r="AL11" s="172"/>
+      <c r="AM11" s="173"/>
       <c r="AN11" s="18" t="s">
         <v>24</v>
       </c>
@@ -2235,44 +2235,44 @@
     </row>
     <row r="12" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="108"/>
-      <c r="B12" s="155"/>
-      <c r="C12" s="156"/>
-      <c r="D12" s="156"/>
-      <c r="E12" s="156"/>
-      <c r="F12" s="156"/>
-      <c r="G12" s="157"/>
-      <c r="H12" s="156"/>
-      <c r="I12" s="158"/>
-      <c r="J12" s="159"/>
-      <c r="K12" s="160"/>
-      <c r="L12" s="160"/>
-      <c r="M12" s="160"/>
-      <c r="N12" s="160"/>
-      <c r="O12" s="160"/>
-      <c r="P12" s="160"/>
-      <c r="Q12" s="160"/>
-      <c r="R12" s="160"/>
-      <c r="S12" s="160"/>
-      <c r="T12" s="160"/>
-      <c r="U12" s="160"/>
-      <c r="V12" s="160"/>
-      <c r="W12" s="160"/>
-      <c r="X12" s="160"/>
-      <c r="Y12" s="160"/>
-      <c r="Z12" s="160"/>
-      <c r="AA12" s="160"/>
-      <c r="AB12" s="160"/>
-      <c r="AC12" s="160"/>
-      <c r="AD12" s="160"/>
-      <c r="AE12" s="160"/>
-      <c r="AF12" s="160"/>
-      <c r="AG12" s="161"/>
-      <c r="AH12" s="159"/>
-      <c r="AI12" s="160"/>
-      <c r="AJ12" s="160"/>
-      <c r="AK12" s="160"/>
-      <c r="AL12" s="160"/>
-      <c r="AM12" s="161"/>
+      <c r="B12" s="154"/>
+      <c r="C12" s="155"/>
+      <c r="D12" s="155"/>
+      <c r="E12" s="155"/>
+      <c r="F12" s="155"/>
+      <c r="G12" s="170"/>
+      <c r="H12" s="155"/>
+      <c r="I12" s="156"/>
+      <c r="J12" s="171"/>
+      <c r="K12" s="172"/>
+      <c r="L12" s="172"/>
+      <c r="M12" s="172"/>
+      <c r="N12" s="172"/>
+      <c r="O12" s="172"/>
+      <c r="P12" s="172"/>
+      <c r="Q12" s="172"/>
+      <c r="R12" s="172"/>
+      <c r="S12" s="172"/>
+      <c r="T12" s="172"/>
+      <c r="U12" s="172"/>
+      <c r="V12" s="172"/>
+      <c r="W12" s="172"/>
+      <c r="X12" s="172"/>
+      <c r="Y12" s="172"/>
+      <c r="Z12" s="172"/>
+      <c r="AA12" s="172"/>
+      <c r="AB12" s="172"/>
+      <c r="AC12" s="172"/>
+      <c r="AD12" s="172"/>
+      <c r="AE12" s="172"/>
+      <c r="AF12" s="172"/>
+      <c r="AG12" s="173"/>
+      <c r="AH12" s="171"/>
+      <c r="AI12" s="172"/>
+      <c r="AJ12" s="172"/>
+      <c r="AK12" s="172"/>
+      <c r="AL12" s="172"/>
+      <c r="AM12" s="173"/>
       <c r="AN12" s="35"/>
       <c r="AO12" s="2"/>
       <c r="AP12" s="2"/>
@@ -2285,44 +2285,44 @@
     </row>
     <row r="13" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="108"/>
-      <c r="B13" s="155"/>
-      <c r="C13" s="156"/>
-      <c r="D13" s="156"/>
-      <c r="E13" s="156"/>
-      <c r="F13" s="156"/>
-      <c r="G13" s="157"/>
-      <c r="H13" s="156"/>
-      <c r="I13" s="158"/>
-      <c r="J13" s="159"/>
-      <c r="K13" s="160"/>
-      <c r="L13" s="160"/>
-      <c r="M13" s="160"/>
-      <c r="N13" s="160"/>
-      <c r="O13" s="160"/>
-      <c r="P13" s="160"/>
-      <c r="Q13" s="160"/>
-      <c r="R13" s="160"/>
-      <c r="S13" s="160"/>
-      <c r="T13" s="160"/>
-      <c r="U13" s="160"/>
-      <c r="V13" s="160"/>
-      <c r="W13" s="160"/>
-      <c r="X13" s="160"/>
-      <c r="Y13" s="160"/>
-      <c r="Z13" s="160"/>
-      <c r="AA13" s="160"/>
-      <c r="AB13" s="160"/>
-      <c r="AC13" s="160"/>
-      <c r="AD13" s="160"/>
-      <c r="AE13" s="160"/>
-      <c r="AF13" s="160"/>
-      <c r="AG13" s="161"/>
-      <c r="AH13" s="159"/>
-      <c r="AI13" s="160"/>
-      <c r="AJ13" s="160"/>
-      <c r="AK13" s="160"/>
-      <c r="AL13" s="160"/>
-      <c r="AM13" s="161"/>
+      <c r="B13" s="154"/>
+      <c r="C13" s="155"/>
+      <c r="D13" s="155"/>
+      <c r="E13" s="155"/>
+      <c r="F13" s="155"/>
+      <c r="G13" s="170"/>
+      <c r="H13" s="155"/>
+      <c r="I13" s="156"/>
+      <c r="J13" s="171"/>
+      <c r="K13" s="172"/>
+      <c r="L13" s="172"/>
+      <c r="M13" s="172"/>
+      <c r="N13" s="172"/>
+      <c r="O13" s="172"/>
+      <c r="P13" s="172"/>
+      <c r="Q13" s="172"/>
+      <c r="R13" s="172"/>
+      <c r="S13" s="172"/>
+      <c r="T13" s="172"/>
+      <c r="U13" s="172"/>
+      <c r="V13" s="172"/>
+      <c r="W13" s="172"/>
+      <c r="X13" s="172"/>
+      <c r="Y13" s="172"/>
+      <c r="Z13" s="172"/>
+      <c r="AA13" s="172"/>
+      <c r="AB13" s="172"/>
+      <c r="AC13" s="172"/>
+      <c r="AD13" s="172"/>
+      <c r="AE13" s="172"/>
+      <c r="AF13" s="172"/>
+      <c r="AG13" s="173"/>
+      <c r="AH13" s="171"/>
+      <c r="AI13" s="172"/>
+      <c r="AJ13" s="172"/>
+      <c r="AK13" s="172"/>
+      <c r="AL13" s="172"/>
+      <c r="AM13" s="173"/>
       <c r="AN13" s="23"/>
       <c r="AO13" s="37"/>
       <c r="AP13" s="37"/>
@@ -2334,47 +2334,47 @@
       <c r="AV13" s="38"/>
     </row>
     <row r="14" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="162" t="s">
+      <c r="A14" s="174" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="163"/>
-      <c r="C14" s="163"/>
-      <c r="D14" s="163"/>
-      <c r="E14" s="163"/>
-      <c r="F14" s="163"/>
-      <c r="G14" s="163"/>
-      <c r="H14" s="163"/>
-      <c r="I14" s="163"/>
-      <c r="J14" s="163"/>
-      <c r="K14" s="163"/>
-      <c r="L14" s="163"/>
-      <c r="M14" s="163"/>
-      <c r="N14" s="163"/>
-      <c r="O14" s="163"/>
-      <c r="P14" s="163"/>
-      <c r="Q14" s="163"/>
-      <c r="R14" s="163"/>
-      <c r="S14" s="163"/>
-      <c r="T14" s="163"/>
-      <c r="U14" s="163"/>
-      <c r="V14" s="163"/>
-      <c r="W14" s="163"/>
-      <c r="X14" s="163"/>
-      <c r="Y14" s="163"/>
-      <c r="Z14" s="163"/>
-      <c r="AA14" s="163"/>
-      <c r="AB14" s="163"/>
-      <c r="AC14" s="163"/>
-      <c r="AD14" s="163"/>
-      <c r="AE14" s="163"/>
-      <c r="AF14" s="163"/>
-      <c r="AG14" s="163"/>
-      <c r="AH14" s="163"/>
-      <c r="AI14" s="163"/>
-      <c r="AJ14" s="163"/>
-      <c r="AK14" s="163"/>
-      <c r="AL14" s="163"/>
-      <c r="AM14" s="154"/>
+      <c r="B14" s="175"/>
+      <c r="C14" s="175"/>
+      <c r="D14" s="175"/>
+      <c r="E14" s="175"/>
+      <c r="F14" s="175"/>
+      <c r="G14" s="175"/>
+      <c r="H14" s="175"/>
+      <c r="I14" s="175"/>
+      <c r="J14" s="175"/>
+      <c r="K14" s="175"/>
+      <c r="L14" s="175"/>
+      <c r="M14" s="175"/>
+      <c r="N14" s="175"/>
+      <c r="O14" s="175"/>
+      <c r="P14" s="175"/>
+      <c r="Q14" s="175"/>
+      <c r="R14" s="175"/>
+      <c r="S14" s="175"/>
+      <c r="T14" s="175"/>
+      <c r="U14" s="175"/>
+      <c r="V14" s="175"/>
+      <c r="W14" s="175"/>
+      <c r="X14" s="175"/>
+      <c r="Y14" s="175"/>
+      <c r="Z14" s="175"/>
+      <c r="AA14" s="175"/>
+      <c r="AB14" s="175"/>
+      <c r="AC14" s="175"/>
+      <c r="AD14" s="175"/>
+      <c r="AE14" s="175"/>
+      <c r="AF14" s="175"/>
+      <c r="AG14" s="175"/>
+      <c r="AH14" s="175"/>
+      <c r="AI14" s="175"/>
+      <c r="AJ14" s="175"/>
+      <c r="AK14" s="175"/>
+      <c r="AL14" s="175"/>
+      <c r="AM14" s="176"/>
       <c r="AN14" s="39"/>
       <c r="AO14" s="21"/>
       <c r="AP14" s="21"/>
@@ -2386,54 +2386,54 @@
       <c r="AV14" s="36"/>
     </row>
     <row r="15" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="164"/>
-      <c r="B15" s="165"/>
-      <c r="C15" s="165"/>
-      <c r="D15" s="165"/>
-      <c r="E15" s="165"/>
-      <c r="F15" s="165"/>
-      <c r="G15" s="165"/>
-      <c r="H15" s="165"/>
-      <c r="I15" s="165"/>
-      <c r="J15" s="166"/>
-      <c r="K15" s="166"/>
-      <c r="L15" s="166"/>
-      <c r="M15" s="166"/>
-      <c r="N15" s="166"/>
-      <c r="O15" s="166"/>
-      <c r="P15" s="166"/>
-      <c r="Q15" s="166"/>
-      <c r="R15" s="166"/>
-      <c r="S15" s="166"/>
-      <c r="T15" s="166"/>
-      <c r="U15" s="166"/>
-      <c r="V15" s="166"/>
-      <c r="W15" s="166"/>
-      <c r="X15" s="166"/>
-      <c r="Y15" s="166"/>
-      <c r="Z15" s="166"/>
-      <c r="AA15" s="166"/>
-      <c r="AB15" s="166"/>
-      <c r="AC15" s="166"/>
-      <c r="AD15" s="166"/>
-      <c r="AE15" s="166"/>
-      <c r="AF15" s="166"/>
-      <c r="AG15" s="166"/>
-      <c r="AH15" s="166"/>
-      <c r="AI15" s="166"/>
-      <c r="AJ15" s="166"/>
-      <c r="AK15" s="166"/>
-      <c r="AL15" s="166"/>
-      <c r="AM15" s="154"/>
-      <c r="AN15" s="152"/>
-      <c r="AO15" s="153"/>
-      <c r="AP15" s="153"/>
-      <c r="AQ15" s="153"/>
-      <c r="AR15" s="153"/>
-      <c r="AS15" s="153"/>
-      <c r="AT15" s="153"/>
-      <c r="AU15" s="153"/>
-      <c r="AV15" s="154"/>
+      <c r="A15" s="177"/>
+      <c r="B15" s="167"/>
+      <c r="C15" s="167"/>
+      <c r="D15" s="167"/>
+      <c r="E15" s="167"/>
+      <c r="F15" s="167"/>
+      <c r="G15" s="167"/>
+      <c r="H15" s="167"/>
+      <c r="I15" s="167"/>
+      <c r="J15" s="178"/>
+      <c r="K15" s="178"/>
+      <c r="L15" s="178"/>
+      <c r="M15" s="178"/>
+      <c r="N15" s="178"/>
+      <c r="O15" s="178"/>
+      <c r="P15" s="178"/>
+      <c r="Q15" s="178"/>
+      <c r="R15" s="178"/>
+      <c r="S15" s="178"/>
+      <c r="T15" s="178"/>
+      <c r="U15" s="178"/>
+      <c r="V15" s="178"/>
+      <c r="W15" s="178"/>
+      <c r="X15" s="178"/>
+      <c r="Y15" s="178"/>
+      <c r="Z15" s="178"/>
+      <c r="AA15" s="178"/>
+      <c r="AB15" s="178"/>
+      <c r="AC15" s="178"/>
+      <c r="AD15" s="178"/>
+      <c r="AE15" s="178"/>
+      <c r="AF15" s="178"/>
+      <c r="AG15" s="178"/>
+      <c r="AH15" s="178"/>
+      <c r="AI15" s="178"/>
+      <c r="AJ15" s="178"/>
+      <c r="AK15" s="178"/>
+      <c r="AL15" s="178"/>
+      <c r="AM15" s="176"/>
+      <c r="AN15" s="179"/>
+      <c r="AO15" s="180"/>
+      <c r="AP15" s="180"/>
+      <c r="AQ15" s="180"/>
+      <c r="AR15" s="180"/>
+      <c r="AS15" s="180"/>
+      <c r="AT15" s="180"/>
+      <c r="AU15" s="180"/>
+      <c r="AV15" s="176"/>
     </row>
     <row r="16" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="109"/>
@@ -2443,47 +2443,47 @@
       <c r="E16" s="117"/>
       <c r="F16" s="84"/>
       <c r="G16" s="84"/>
-      <c r="H16" s="126"/>
-      <c r="I16" s="117"/>
+      <c r="H16" s="124"/>
+      <c r="I16" s="183"/>
       <c r="J16" s="63"/>
       <c r="K16" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="L16" s="149"/>
-      <c r="M16" s="150"/>
-      <c r="N16" s="150"/>
+      <c r="L16" s="143"/>
+      <c r="M16" s="144"/>
+      <c r="N16" s="144"/>
       <c r="O16" s="65"/>
       <c r="P16" s="66"/>
       <c r="Q16" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="R16" s="149"/>
-      <c r="S16" s="150"/>
-      <c r="T16" s="150"/>
+      <c r="R16" s="143"/>
+      <c r="S16" s="144"/>
+      <c r="T16" s="144"/>
       <c r="U16" s="65"/>
       <c r="V16" s="66"/>
       <c r="W16" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="X16" s="149"/>
-      <c r="Y16" s="150"/>
-      <c r="Z16" s="150"/>
+      <c r="X16" s="143"/>
+      <c r="Y16" s="144"/>
+      <c r="Z16" s="144"/>
       <c r="AA16" s="65"/>
       <c r="AB16" s="68"/>
       <c r="AC16" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="AD16" s="149"/>
-      <c r="AE16" s="150"/>
-      <c r="AF16" s="150"/>
+      <c r="AD16" s="143"/>
+      <c r="AE16" s="144"/>
+      <c r="AF16" s="144"/>
       <c r="AG16" s="65"/>
       <c r="AH16" s="68"/>
       <c r="AI16" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="AJ16" s="149"/>
-      <c r="AK16" s="150"/>
-      <c r="AL16" s="150"/>
+      <c r="AJ16" s="143"/>
+      <c r="AK16" s="144"/>
+      <c r="AL16" s="144"/>
       <c r="AM16" s="69"/>
       <c r="AN16" s="61"/>
       <c r="AO16" s="2"/>
@@ -2497,14 +2497,14 @@
     </row>
     <row r="17" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="110"/>
-      <c r="B17" s="129"/>
+      <c r="B17" s="127"/>
       <c r="C17" s="85"/>
       <c r="D17" s="118"/>
       <c r="E17" s="118"/>
       <c r="F17" s="85"/>
       <c r="G17" s="85"/>
-      <c r="H17" s="127"/>
-      <c r="I17" s="118"/>
+      <c r="H17" s="125"/>
+      <c r="I17" s="184"/>
       <c r="J17" s="70"/>
       <c r="K17" s="71"/>
       <c r="L17" s="72"/>
@@ -2547,13 +2547,13 @@
     </row>
     <row r="18" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="111"/>
-      <c r="B18" s="130"/>
+      <c r="B18" s="128"/>
       <c r="C18" s="86"/>
-      <c r="D18" s="132"/>
-      <c r="E18" s="132"/>
+      <c r="D18" s="130"/>
+      <c r="E18" s="130"/>
       <c r="F18" s="86"/>
-      <c r="G18" s="125"/>
-      <c r="H18" s="184"/>
+      <c r="G18" s="123"/>
+      <c r="H18" s="140"/>
       <c r="I18" s="119"/>
       <c r="J18" s="74"/>
       <c r="K18" s="148"/>
@@ -2597,10 +2597,10 @@
     </row>
     <row r="19" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="111"/>
-      <c r="B19" s="130"/>
+      <c r="B19" s="128"/>
       <c r="C19" s="86"/>
-      <c r="D19" s="132"/>
-      <c r="E19" s="132"/>
+      <c r="D19" s="130"/>
+      <c r="E19" s="130"/>
       <c r="F19" s="86"/>
       <c r="G19" s="88"/>
       <c r="H19" s="87"/>
@@ -2647,10 +2647,10 @@
     </row>
     <row r="20" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="111"/>
-      <c r="B20" s="130"/>
+      <c r="B20" s="128"/>
       <c r="C20" s="86"/>
-      <c r="D20" s="132"/>
-      <c r="E20" s="132"/>
+      <c r="D20" s="130"/>
+      <c r="E20" s="130"/>
       <c r="F20" s="86"/>
       <c r="G20" s="88"/>
       <c r="H20" s="87"/>
@@ -2703,8 +2703,8 @@
       <c r="E21" s="120"/>
       <c r="F21" s="89"/>
       <c r="G21" s="89"/>
-      <c r="H21" s="128"/>
-      <c r="I21" s="120"/>
+      <c r="H21" s="126"/>
+      <c r="I21" s="119"/>
       <c r="J21" s="74"/>
       <c r="K21" s="148"/>
       <c r="L21" s="148"/>
@@ -2747,10 +2747,10 @@
     </row>
     <row r="22" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="111"/>
-      <c r="B22" s="130"/>
+      <c r="B22" s="128"/>
       <c r="C22" s="86"/>
-      <c r="D22" s="132"/>
-      <c r="E22" s="132"/>
+      <c r="D22" s="130"/>
+      <c r="E22" s="130"/>
       <c r="F22" s="86"/>
       <c r="G22" s="88"/>
       <c r="H22" s="87"/>
@@ -2797,10 +2797,10 @@
     </row>
     <row r="23" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="111"/>
-      <c r="B23" s="130"/>
+      <c r="B23" s="128"/>
       <c r="C23" s="86"/>
-      <c r="D23" s="132"/>
-      <c r="E23" s="132"/>
+      <c r="D23" s="130"/>
+      <c r="E23" s="130"/>
       <c r="F23" s="86"/>
       <c r="G23" s="88"/>
       <c r="H23" s="87"/>
@@ -2847,53 +2847,53 @@
     </row>
     <row r="24" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="111"/>
-      <c r="B24" s="130"/>
+      <c r="B24" s="128"/>
       <c r="C24" s="86"/>
-      <c r="D24" s="132"/>
-      <c r="E24" s="132"/>
+      <c r="D24" s="130"/>
+      <c r="E24" s="130"/>
       <c r="F24" s="86"/>
       <c r="G24" s="88"/>
       <c r="H24" s="87"/>
       <c r="I24" s="119"/>
       <c r="J24" s="74"/>
-      <c r="K24" s="144" t="s">
+      <c r="K24" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="L24" s="143"/>
-      <c r="M24" s="142"/>
-      <c r="N24" s="143"/>
+      <c r="L24" s="146"/>
+      <c r="M24" s="147"/>
+      <c r="N24" s="146"/>
       <c r="O24" s="43"/>
       <c r="P24" s="72"/>
-      <c r="Q24" s="144" t="s">
+      <c r="Q24" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="R24" s="143"/>
-      <c r="S24" s="142"/>
-      <c r="T24" s="143"/>
+      <c r="R24" s="146"/>
+      <c r="S24" s="147"/>
+      <c r="T24" s="146"/>
       <c r="U24" s="43"/>
       <c r="V24" s="72"/>
-      <c r="W24" s="144" t="s">
+      <c r="W24" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="X24" s="143"/>
-      <c r="Y24" s="142"/>
-      <c r="Z24" s="143"/>
+      <c r="X24" s="146"/>
+      <c r="Y24" s="147"/>
+      <c r="Z24" s="146"/>
       <c r="AA24" s="43"/>
       <c r="AB24" s="72"/>
-      <c r="AC24" s="144" t="s">
+      <c r="AC24" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="AD24" s="143"/>
-      <c r="AE24" s="142"/>
-      <c r="AF24" s="143"/>
+      <c r="AD24" s="146"/>
+      <c r="AE24" s="147"/>
+      <c r="AF24" s="146"/>
       <c r="AG24" s="43"/>
       <c r="AH24" s="72"/>
-      <c r="AI24" s="144" t="s">
+      <c r="AI24" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="AJ24" s="143"/>
-      <c r="AK24" s="142"/>
-      <c r="AL24" s="143"/>
+      <c r="AJ24" s="146"/>
+      <c r="AK24" s="147"/>
+      <c r="AL24" s="146"/>
       <c r="AM24" s="73"/>
       <c r="AN24" s="61"/>
       <c r="AO24" s="2"/>
@@ -2907,10 +2907,10 @@
     </row>
     <row r="25" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="111"/>
-      <c r="B25" s="130"/>
+      <c r="B25" s="128"/>
       <c r="C25" s="86"/>
-      <c r="D25" s="132"/>
-      <c r="E25" s="132"/>
+      <c r="D25" s="130"/>
+      <c r="E25" s="130"/>
       <c r="F25" s="86"/>
       <c r="G25" s="88"/>
       <c r="H25" s="87"/>
@@ -2920,40 +2920,40 @@
         <v>32</v>
       </c>
       <c r="L25" s="72"/>
-      <c r="M25" s="142"/>
-      <c r="N25" s="143"/>
+      <c r="M25" s="147"/>
+      <c r="N25" s="146"/>
       <c r="O25" s="43"/>
       <c r="P25" s="72"/>
       <c r="Q25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="R25" s="72"/>
-      <c r="S25" s="142"/>
-      <c r="T25" s="143"/>
+      <c r="S25" s="147"/>
+      <c r="T25" s="146"/>
       <c r="U25" s="43"/>
       <c r="V25" s="72"/>
       <c r="W25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="X25" s="72"/>
-      <c r="Y25" s="142"/>
-      <c r="Z25" s="143"/>
+      <c r="Y25" s="147"/>
+      <c r="Z25" s="146"/>
       <c r="AA25" s="43"/>
       <c r="AB25" s="72"/>
       <c r="AC25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AD25" s="72"/>
-      <c r="AE25" s="142"/>
-      <c r="AF25" s="143"/>
+      <c r="AE25" s="147"/>
+      <c r="AF25" s="146"/>
       <c r="AG25" s="43"/>
       <c r="AH25" s="72"/>
       <c r="AI25" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AJ25" s="72"/>
-      <c r="AK25" s="142"/>
-      <c r="AL25" s="143"/>
+      <c r="AK25" s="147"/>
+      <c r="AL25" s="146"/>
       <c r="AM25" s="73"/>
       <c r="AN25" s="61"/>
       <c r="AO25" s="2"/>
@@ -2967,10 +2967,10 @@
     </row>
     <row r="26" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="111"/>
-      <c r="B26" s="130"/>
+      <c r="B26" s="128"/>
       <c r="C26" s="86"/>
-      <c r="D26" s="132"/>
-      <c r="E26" s="132"/>
+      <c r="D26" s="130"/>
+      <c r="E26" s="130"/>
       <c r="F26" s="86"/>
       <c r="G26" s="88"/>
       <c r="H26" s="87"/>
@@ -2979,61 +2979,61 @@
       <c r="K26" s="48" t="s">
         <v>33</v>
       </c>
-      <c r="L26" s="151"/>
-      <c r="M26" s="151"/>
-      <c r="N26" s="151"/>
+      <c r="L26" s="149"/>
+      <c r="M26" s="149"/>
+      <c r="N26" s="149"/>
       <c r="O26" s="60"/>
       <c r="P26" s="41"/>
       <c r="Q26" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="R26" s="149"/>
-      <c r="S26" s="150"/>
-      <c r="T26" s="150"/>
+      <c r="R26" s="143"/>
+      <c r="S26" s="144"/>
+      <c r="T26" s="144"/>
       <c r="U26" s="40"/>
       <c r="V26" s="41"/>
       <c r="W26" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="X26" s="151"/>
-      <c r="Y26" s="151"/>
-      <c r="Z26" s="151"/>
+      <c r="X26" s="149"/>
+      <c r="Y26" s="149"/>
+      <c r="Z26" s="149"/>
       <c r="AA26" s="40"/>
       <c r="AB26" s="41"/>
       <c r="AC26" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="AD26" s="149"/>
-      <c r="AE26" s="150"/>
-      <c r="AF26" s="150"/>
+      <c r="AD26" s="143"/>
+      <c r="AE26" s="144"/>
+      <c r="AF26" s="144"/>
       <c r="AG26" s="40"/>
       <c r="AH26" s="41"/>
       <c r="AI26" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="AJ26" s="149"/>
-      <c r="AK26" s="150"/>
-      <c r="AL26" s="150"/>
+      <c r="AJ26" s="143"/>
+      <c r="AK26" s="144"/>
+      <c r="AL26" s="144"/>
       <c r="AM26" s="77"/>
       <c r="AN26" s="61"/>
-      <c r="AO26" s="145"/>
-      <c r="AP26" s="146"/>
-      <c r="AQ26" s="146"/>
-      <c r="AR26" s="146"/>
-      <c r="AS26" s="146"/>
-      <c r="AT26" s="146"/>
-      <c r="AU26" s="146"/>
+      <c r="AO26" s="181"/>
+      <c r="AP26" s="182"/>
+      <c r="AQ26" s="182"/>
+      <c r="AR26" s="182"/>
+      <c r="AS26" s="182"/>
+      <c r="AT26" s="182"/>
+      <c r="AU26" s="182"/>
       <c r="AV26" s="22"/>
     </row>
     <row r="27" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="112"/>
       <c r="B27" s="45"/>
       <c r="C27" s="42"/>
-      <c r="D27" s="133"/>
-      <c r="E27" s="133"/>
+      <c r="D27" s="131"/>
+      <c r="E27" s="131"/>
       <c r="F27" s="42"/>
       <c r="G27" s="46"/>
-      <c r="H27" s="135"/>
+      <c r="H27" s="133"/>
       <c r="I27" s="121"/>
       <c r="J27" s="74"/>
       <c r="K27" s="71"/>
@@ -3066,24 +3066,24 @@
       <c r="AL27" s="72"/>
       <c r="AM27" s="73"/>
       <c r="AN27" s="61"/>
-      <c r="AO27" s="146"/>
-      <c r="AP27" s="146"/>
-      <c r="AQ27" s="146"/>
-      <c r="AR27" s="146"/>
-      <c r="AS27" s="146"/>
-      <c r="AT27" s="146"/>
-      <c r="AU27" s="146"/>
+      <c r="AO27" s="182"/>
+      <c r="AP27" s="182"/>
+      <c r="AQ27" s="182"/>
+      <c r="AR27" s="182"/>
+      <c r="AS27" s="182"/>
+      <c r="AT27" s="182"/>
+      <c r="AU27" s="182"/>
       <c r="AV27" s="22"/>
     </row>
     <row r="28" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="113"/>
       <c r="B28" s="80"/>
       <c r="C28" s="81"/>
-      <c r="D28" s="134"/>
-      <c r="E28" s="134"/>
+      <c r="D28" s="132"/>
+      <c r="E28" s="132"/>
       <c r="F28" s="81"/>
       <c r="G28" s="91"/>
-      <c r="H28" s="136"/>
+      <c r="H28" s="134"/>
       <c r="I28" s="122"/>
       <c r="J28" s="74"/>
       <c r="K28" s="148"/>
@@ -3116,21 +3116,21 @@
       <c r="AL28" s="148"/>
       <c r="AM28" s="73"/>
       <c r="AN28" s="61"/>
-      <c r="AO28" s="146"/>
-      <c r="AP28" s="146"/>
-      <c r="AQ28" s="146"/>
-      <c r="AR28" s="146"/>
-      <c r="AS28" s="146"/>
-      <c r="AT28" s="146"/>
-      <c r="AU28" s="146"/>
+      <c r="AO28" s="182"/>
+      <c r="AP28" s="182"/>
+      <c r="AQ28" s="182"/>
+      <c r="AR28" s="182"/>
+      <c r="AS28" s="182"/>
+      <c r="AT28" s="182"/>
+      <c r="AU28" s="182"/>
       <c r="AV28" s="22"/>
     </row>
     <row r="29" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="111"/>
-      <c r="B29" s="130"/>
+      <c r="B29" s="128"/>
       <c r="C29" s="86"/>
-      <c r="D29" s="132"/>
-      <c r="E29" s="132"/>
+      <c r="D29" s="130"/>
+      <c r="E29" s="130"/>
       <c r="F29" s="86"/>
       <c r="G29" s="88"/>
       <c r="H29" s="87"/>
@@ -3166,21 +3166,21 @@
       <c r="AL29" s="148"/>
       <c r="AM29" s="73"/>
       <c r="AN29" s="61"/>
-      <c r="AO29" s="146"/>
-      <c r="AP29" s="146"/>
-      <c r="AQ29" s="146"/>
-      <c r="AR29" s="146"/>
-      <c r="AS29" s="146"/>
-      <c r="AT29" s="146"/>
-      <c r="AU29" s="146"/>
+      <c r="AO29" s="182"/>
+      <c r="AP29" s="182"/>
+      <c r="AQ29" s="182"/>
+      <c r="AR29" s="182"/>
+      <c r="AS29" s="182"/>
+      <c r="AT29" s="182"/>
+      <c r="AU29" s="182"/>
       <c r="AV29" s="22"/>
     </row>
     <row r="30" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="111"/>
-      <c r="B30" s="130"/>
+      <c r="B30" s="128"/>
       <c r="C30" s="86"/>
-      <c r="D30" s="132"/>
-      <c r="E30" s="132"/>
+      <c r="D30" s="130"/>
+      <c r="E30" s="130"/>
       <c r="F30" s="86"/>
       <c r="G30" s="88"/>
       <c r="H30" s="87"/>
@@ -3216,21 +3216,21 @@
       <c r="AL30" s="148"/>
       <c r="AM30" s="73"/>
       <c r="AN30" s="62"/>
-      <c r="AO30" s="146"/>
-      <c r="AP30" s="146"/>
-      <c r="AQ30" s="146"/>
-      <c r="AR30" s="146"/>
-      <c r="AS30" s="146"/>
-      <c r="AT30" s="146"/>
-      <c r="AU30" s="146"/>
+      <c r="AO30" s="182"/>
+      <c r="AP30" s="182"/>
+      <c r="AQ30" s="182"/>
+      <c r="AR30" s="182"/>
+      <c r="AS30" s="182"/>
+      <c r="AT30" s="182"/>
+      <c r="AU30" s="182"/>
       <c r="AV30" s="22"/>
     </row>
     <row r="31" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="111"/>
-      <c r="B31" s="130"/>
+      <c r="B31" s="128"/>
       <c r="C31" s="86"/>
-      <c r="D31" s="132"/>
-      <c r="E31" s="132"/>
+      <c r="D31" s="130"/>
+      <c r="E31" s="130"/>
       <c r="F31" s="86"/>
       <c r="G31" s="88"/>
       <c r="H31" s="87"/>
@@ -3266,21 +3266,21 @@
       <c r="AL31" s="148"/>
       <c r="AM31" s="73"/>
       <c r="AN31" s="61"/>
-      <c r="AO31" s="146"/>
-      <c r="AP31" s="146"/>
-      <c r="AQ31" s="146"/>
-      <c r="AR31" s="146"/>
-      <c r="AS31" s="146"/>
-      <c r="AT31" s="146"/>
-      <c r="AU31" s="146"/>
+      <c r="AO31" s="182"/>
+      <c r="AP31" s="182"/>
+      <c r="AQ31" s="182"/>
+      <c r="AR31" s="182"/>
+      <c r="AS31" s="182"/>
+      <c r="AT31" s="182"/>
+      <c r="AU31" s="182"/>
       <c r="AV31" s="22"/>
     </row>
     <row r="32" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="111"/>
-      <c r="B32" s="130"/>
+      <c r="B32" s="128"/>
       <c r="C32" s="86"/>
-      <c r="D32" s="132"/>
-      <c r="E32" s="132"/>
+      <c r="D32" s="130"/>
+      <c r="E32" s="130"/>
       <c r="F32" s="86"/>
       <c r="G32" s="88"/>
       <c r="H32" s="87"/>
@@ -3316,21 +3316,21 @@
       <c r="AL32" s="148"/>
       <c r="AM32" s="73"/>
       <c r="AN32" s="61"/>
-      <c r="AO32" s="146"/>
-      <c r="AP32" s="146"/>
-      <c r="AQ32" s="146"/>
-      <c r="AR32" s="146"/>
-      <c r="AS32" s="146"/>
-      <c r="AT32" s="146"/>
-      <c r="AU32" s="146"/>
+      <c r="AO32" s="182"/>
+      <c r="AP32" s="182"/>
+      <c r="AQ32" s="182"/>
+      <c r="AR32" s="182"/>
+      <c r="AS32" s="182"/>
+      <c r="AT32" s="182"/>
+      <c r="AU32" s="182"/>
       <c r="AV32" s="22"/>
     </row>
     <row r="33" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="111"/>
-      <c r="B33" s="130"/>
+      <c r="B33" s="128"/>
       <c r="C33" s="86"/>
-      <c r="D33" s="132"/>
-      <c r="E33" s="132"/>
+      <c r="D33" s="130"/>
+      <c r="E33" s="130"/>
       <c r="F33" s="86"/>
       <c r="G33" s="88"/>
       <c r="H33" s="87"/>
@@ -3366,81 +3366,81 @@
       <c r="AL33" s="148"/>
       <c r="AM33" s="73"/>
       <c r="AN33" s="61"/>
-      <c r="AO33" s="146"/>
-      <c r="AP33" s="146"/>
-      <c r="AQ33" s="146"/>
-      <c r="AR33" s="146"/>
-      <c r="AS33" s="146"/>
-      <c r="AT33" s="146"/>
-      <c r="AU33" s="146"/>
+      <c r="AO33" s="182"/>
+      <c r="AP33" s="182"/>
+      <c r="AQ33" s="182"/>
+      <c r="AR33" s="182"/>
+      <c r="AS33" s="182"/>
+      <c r="AT33" s="182"/>
+      <c r="AU33" s="182"/>
       <c r="AV33" s="22"/>
     </row>
     <row r="34" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="111"/>
-      <c r="B34" s="130"/>
+      <c r="B34" s="128"/>
       <c r="C34" s="86"/>
-      <c r="D34" s="132"/>
-      <c r="E34" s="132"/>
+      <c r="D34" s="130"/>
+      <c r="E34" s="130"/>
       <c r="F34" s="86"/>
       <c r="G34" s="88"/>
       <c r="H34" s="87"/>
       <c r="I34" s="119"/>
       <c r="J34" s="78"/>
-      <c r="K34" s="144" t="s">
+      <c r="K34" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="L34" s="143"/>
-      <c r="M34" s="142"/>
-      <c r="N34" s="143"/>
+      <c r="L34" s="146"/>
+      <c r="M34" s="147"/>
+      <c r="N34" s="146"/>
       <c r="O34" s="43"/>
       <c r="P34" s="72"/>
-      <c r="Q34" s="144" t="s">
+      <c r="Q34" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="R34" s="143"/>
-      <c r="S34" s="142"/>
-      <c r="T34" s="143"/>
+      <c r="R34" s="146"/>
+      <c r="S34" s="147"/>
+      <c r="T34" s="146"/>
       <c r="U34" s="43"/>
       <c r="V34" s="72"/>
-      <c r="W34" s="144" t="s">
+      <c r="W34" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="X34" s="143"/>
-      <c r="Y34" s="142"/>
-      <c r="Z34" s="143"/>
+      <c r="X34" s="146"/>
+      <c r="Y34" s="147"/>
+      <c r="Z34" s="146"/>
       <c r="AA34" s="43"/>
       <c r="AB34" s="72"/>
-      <c r="AC34" s="144" t="s">
+      <c r="AC34" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="AD34" s="143"/>
-      <c r="AE34" s="142"/>
-      <c r="AF34" s="143"/>
+      <c r="AD34" s="146"/>
+      <c r="AE34" s="147"/>
+      <c r="AF34" s="146"/>
       <c r="AG34" s="43"/>
       <c r="AH34" s="72"/>
-      <c r="AI34" s="144" t="s">
+      <c r="AI34" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="AJ34" s="143"/>
-      <c r="AK34" s="142"/>
-      <c r="AL34" s="143"/>
+      <c r="AJ34" s="146"/>
+      <c r="AK34" s="147"/>
+      <c r="AL34" s="146"/>
       <c r="AM34" s="43"/>
       <c r="AN34" s="61"/>
-      <c r="AO34" s="146"/>
-      <c r="AP34" s="146"/>
-      <c r="AQ34" s="146"/>
-      <c r="AR34" s="146"/>
-      <c r="AS34" s="146"/>
-      <c r="AT34" s="146"/>
-      <c r="AU34" s="146"/>
+      <c r="AO34" s="182"/>
+      <c r="AP34" s="182"/>
+      <c r="AQ34" s="182"/>
+      <c r="AR34" s="182"/>
+      <c r="AS34" s="182"/>
+      <c r="AT34" s="182"/>
+      <c r="AU34" s="182"/>
       <c r="AV34" s="22"/>
     </row>
     <row r="35" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="111"/>
-      <c r="B35" s="130"/>
+      <c r="B35" s="128"/>
       <c r="C35" s="86"/>
-      <c r="D35" s="132"/>
-      <c r="E35" s="132"/>
+      <c r="D35" s="130"/>
+      <c r="E35" s="130"/>
       <c r="F35" s="86"/>
       <c r="G35" s="88"/>
       <c r="H35" s="87"/>
@@ -3450,57 +3450,57 @@
         <v>32</v>
       </c>
       <c r="L35" s="72"/>
-      <c r="M35" s="142"/>
-      <c r="N35" s="143"/>
+      <c r="M35" s="147"/>
+      <c r="N35" s="146"/>
       <c r="O35" s="43"/>
       <c r="P35" s="72"/>
       <c r="Q35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="R35" s="72"/>
-      <c r="S35" s="142"/>
-      <c r="T35" s="143"/>
+      <c r="S35" s="147"/>
+      <c r="T35" s="146"/>
       <c r="U35" s="43"/>
       <c r="V35" s="72"/>
       <c r="W35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="X35" s="72"/>
-      <c r="Y35" s="142"/>
-      <c r="Z35" s="143"/>
+      <c r="Y35" s="147"/>
+      <c r="Z35" s="146"/>
       <c r="AA35" s="43"/>
       <c r="AB35" s="72"/>
       <c r="AC35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AD35" s="72"/>
-      <c r="AE35" s="142"/>
-      <c r="AF35" s="143"/>
+      <c r="AE35" s="147"/>
+      <c r="AF35" s="146"/>
       <c r="AG35" s="43"/>
       <c r="AH35" s="72"/>
       <c r="AI35" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AJ35" s="72"/>
-      <c r="AK35" s="142"/>
-      <c r="AL35" s="143"/>
-      <c r="AM35" s="147"/>
+      <c r="AK35" s="147"/>
+      <c r="AL35" s="146"/>
+      <c r="AM35" s="150"/>
       <c r="AN35" s="61"/>
-      <c r="AO35" s="146"/>
-      <c r="AP35" s="146"/>
-      <c r="AQ35" s="146"/>
-      <c r="AR35" s="146"/>
-      <c r="AS35" s="146"/>
-      <c r="AT35" s="146"/>
-      <c r="AU35" s="146"/>
+      <c r="AO35" s="182"/>
+      <c r="AP35" s="182"/>
+      <c r="AQ35" s="182"/>
+      <c r="AR35" s="182"/>
+      <c r="AS35" s="182"/>
+      <c r="AT35" s="182"/>
+      <c r="AU35" s="182"/>
       <c r="AV35" s="30"/>
     </row>
     <row r="36" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="111"/>
-      <c r="B36" s="130"/>
+      <c r="B36" s="128"/>
       <c r="C36" s="86"/>
-      <c r="D36" s="132"/>
-      <c r="E36" s="132"/>
+      <c r="D36" s="130"/>
+      <c r="E36" s="130"/>
       <c r="F36" s="86"/>
       <c r="G36" s="88"/>
       <c r="H36" s="87"/>
@@ -3509,62 +3509,62 @@
       <c r="K36" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="L36" s="149"/>
-      <c r="M36" s="150"/>
-      <c r="N36" s="150"/>
+      <c r="L36" s="143"/>
+      <c r="M36" s="144"/>
+      <c r="N36" s="144"/>
       <c r="O36" s="65"/>
       <c r="P36" s="41"/>
       <c r="Q36" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="R36" s="149"/>
-      <c r="S36" s="150"/>
-      <c r="T36" s="150"/>
+      <c r="R36" s="143"/>
+      <c r="S36" s="144"/>
+      <c r="T36" s="144"/>
       <c r="U36" s="40"/>
       <c r="V36" s="41"/>
       <c r="W36" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="X36" s="151"/>
-      <c r="Y36" s="151"/>
-      <c r="Z36" s="151"/>
+      <c r="X36" s="149"/>
+      <c r="Y36" s="149"/>
+      <c r="Z36" s="149"/>
       <c r="AA36" s="40"/>
       <c r="AB36" s="41"/>
       <c r="AC36" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="AD36" s="149"/>
-      <c r="AE36" s="150"/>
-      <c r="AF36" s="150"/>
+      <c r="AD36" s="143"/>
+      <c r="AE36" s="144"/>
+      <c r="AF36" s="144"/>
       <c r="AG36" s="40"/>
       <c r="AH36" s="41"/>
       <c r="AI36" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="AJ36" s="149"/>
-      <c r="AK36" s="150"/>
-      <c r="AL36" s="150"/>
+      <c r="AJ36" s="143"/>
+      <c r="AK36" s="144"/>
+      <c r="AL36" s="144"/>
       <c r="AM36" s="77"/>
       <c r="AN36" s="2"/>
-      <c r="AO36" s="146"/>
-      <c r="AP36" s="146"/>
-      <c r="AQ36" s="146"/>
-      <c r="AR36" s="146"/>
-      <c r="AS36" s="146"/>
-      <c r="AT36" s="146"/>
-      <c r="AU36" s="146"/>
+      <c r="AO36" s="182"/>
+      <c r="AP36" s="182"/>
+      <c r="AQ36" s="182"/>
+      <c r="AR36" s="182"/>
+      <c r="AS36" s="182"/>
+      <c r="AT36" s="182"/>
+      <c r="AU36" s="182"/>
       <c r="AV36" s="22"/>
     </row>
     <row r="37" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="114"/>
       <c r="B37" s="45"/>
       <c r="C37" s="42"/>
-      <c r="D37" s="133"/>
-      <c r="E37" s="133"/>
+      <c r="D37" s="131"/>
+      <c r="E37" s="131"/>
       <c r="F37" s="42"/>
       <c r="G37" s="42"/>
-      <c r="H37" s="137"/>
-      <c r="I37" s="123"/>
+      <c r="H37" s="135"/>
+      <c r="I37" s="138"/>
       <c r="J37" s="74"/>
       <c r="K37" s="71"/>
       <c r="L37" s="72"/>
@@ -3596,25 +3596,25 @@
       <c r="AL37" s="72"/>
       <c r="AM37" s="73"/>
       <c r="AN37" s="2"/>
-      <c r="AO37" s="146"/>
-      <c r="AP37" s="146"/>
-      <c r="AQ37" s="146"/>
-      <c r="AR37" s="146"/>
-      <c r="AS37" s="146"/>
-      <c r="AT37" s="146"/>
-      <c r="AU37" s="146"/>
+      <c r="AO37" s="182"/>
+      <c r="AP37" s="182"/>
+      <c r="AQ37" s="182"/>
+      <c r="AR37" s="182"/>
+      <c r="AS37" s="182"/>
+      <c r="AT37" s="182"/>
+      <c r="AU37" s="182"/>
       <c r="AV37" s="22"/>
     </row>
     <row r="38" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="115"/>
-      <c r="B38" s="131"/>
+      <c r="B38" s="129"/>
       <c r="C38" s="81"/>
-      <c r="D38" s="134"/>
-      <c r="E38" s="139"/>
+      <c r="D38" s="132"/>
+      <c r="E38" s="137"/>
       <c r="F38" s="90"/>
       <c r="G38" s="81"/>
-      <c r="H38" s="138"/>
-      <c r="I38" s="124"/>
+      <c r="H38" s="136"/>
+      <c r="I38" s="122"/>
       <c r="J38" s="74"/>
       <c r="K38" s="148"/>
       <c r="L38" s="148"/>
@@ -3646,21 +3646,21 @@
       <c r="AL38" s="148"/>
       <c r="AM38" s="73"/>
       <c r="AN38" s="2"/>
-      <c r="AO38" s="146"/>
-      <c r="AP38" s="146"/>
-      <c r="AQ38" s="146"/>
-      <c r="AR38" s="146"/>
-      <c r="AS38" s="146"/>
-      <c r="AT38" s="146"/>
-      <c r="AU38" s="146"/>
+      <c r="AO38" s="182"/>
+      <c r="AP38" s="182"/>
+      <c r="AQ38" s="182"/>
+      <c r="AR38" s="182"/>
+      <c r="AS38" s="182"/>
+      <c r="AT38" s="182"/>
+      <c r="AU38" s="182"/>
       <c r="AV38" s="22"/>
     </row>
     <row r="39" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="111"/>
-      <c r="B39" s="130"/>
+      <c r="B39" s="128"/>
       <c r="C39" s="86"/>
-      <c r="D39" s="132"/>
-      <c r="E39" s="132"/>
+      <c r="D39" s="130"/>
+      <c r="E39" s="130"/>
       <c r="F39" s="86"/>
       <c r="G39" s="88"/>
       <c r="H39" s="87"/>
@@ -3696,21 +3696,21 @@
       <c r="AL39" s="148"/>
       <c r="AM39" s="73"/>
       <c r="AN39" s="2"/>
-      <c r="AO39" s="146"/>
-      <c r="AP39" s="146"/>
-      <c r="AQ39" s="146"/>
-      <c r="AR39" s="146"/>
-      <c r="AS39" s="146"/>
-      <c r="AT39" s="146"/>
-      <c r="AU39" s="146"/>
+      <c r="AO39" s="182"/>
+      <c r="AP39" s="182"/>
+      <c r="AQ39" s="182"/>
+      <c r="AR39" s="182"/>
+      <c r="AS39" s="182"/>
+      <c r="AT39" s="182"/>
+      <c r="AU39" s="182"/>
       <c r="AV39" s="22"/>
     </row>
     <row r="40" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="111"/>
-      <c r="B40" s="130"/>
+      <c r="B40" s="128"/>
       <c r="C40" s="86"/>
-      <c r="D40" s="132"/>
-      <c r="E40" s="132"/>
+      <c r="D40" s="130"/>
+      <c r="E40" s="130"/>
       <c r="F40" s="86"/>
       <c r="G40" s="88"/>
       <c r="H40" s="87"/>
@@ -3746,21 +3746,21 @@
       <c r="AL40" s="148"/>
       <c r="AM40" s="73"/>
       <c r="AN40" s="2"/>
-      <c r="AO40" s="146"/>
-      <c r="AP40" s="146"/>
-      <c r="AQ40" s="146"/>
-      <c r="AR40" s="146"/>
-      <c r="AS40" s="146"/>
-      <c r="AT40" s="146"/>
-      <c r="AU40" s="146"/>
+      <c r="AO40" s="182"/>
+      <c r="AP40" s="182"/>
+      <c r="AQ40" s="182"/>
+      <c r="AR40" s="182"/>
+      <c r="AS40" s="182"/>
+      <c r="AT40" s="182"/>
+      <c r="AU40" s="182"/>
       <c r="AV40" s="22"/>
     </row>
     <row r="41" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="111"/>
-      <c r="B41" s="130"/>
+      <c r="B41" s="128"/>
       <c r="C41" s="86"/>
-      <c r="D41" s="132"/>
-      <c r="E41" s="132"/>
+      <c r="D41" s="130"/>
+      <c r="E41" s="130"/>
       <c r="F41" s="86"/>
       <c r="G41" s="88"/>
       <c r="H41" s="87"/>
@@ -3796,21 +3796,21 @@
       <c r="AL41" s="148"/>
       <c r="AM41" s="73"/>
       <c r="AN41" s="2"/>
-      <c r="AO41" s="146"/>
-      <c r="AP41" s="146"/>
-      <c r="AQ41" s="146"/>
-      <c r="AR41" s="146"/>
-      <c r="AS41" s="146"/>
-      <c r="AT41" s="146"/>
-      <c r="AU41" s="146"/>
+      <c r="AO41" s="182"/>
+      <c r="AP41" s="182"/>
+      <c r="AQ41" s="182"/>
+      <c r="AR41" s="182"/>
+      <c r="AS41" s="182"/>
+      <c r="AT41" s="182"/>
+      <c r="AU41" s="182"/>
       <c r="AV41" s="22"/>
     </row>
     <row r="42" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="111"/>
-      <c r="B42" s="130"/>
+      <c r="B42" s="128"/>
       <c r="C42" s="86"/>
-      <c r="D42" s="132"/>
-      <c r="E42" s="132"/>
+      <c r="D42" s="130"/>
+      <c r="E42" s="130"/>
       <c r="F42" s="86"/>
       <c r="G42" s="88"/>
       <c r="H42" s="87"/>
@@ -3846,21 +3846,21 @@
       <c r="AL42" s="148"/>
       <c r="AM42" s="73"/>
       <c r="AN42" s="2"/>
-      <c r="AO42" s="146"/>
-      <c r="AP42" s="146"/>
-      <c r="AQ42" s="146"/>
-      <c r="AR42" s="146"/>
-      <c r="AS42" s="146"/>
-      <c r="AT42" s="146"/>
-      <c r="AU42" s="146"/>
+      <c r="AO42" s="182"/>
+      <c r="AP42" s="182"/>
+      <c r="AQ42" s="182"/>
+      <c r="AR42" s="182"/>
+      <c r="AS42" s="182"/>
+      <c r="AT42" s="182"/>
+      <c r="AU42" s="182"/>
       <c r="AV42" s="22"/>
     </row>
     <row r="43" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="111"/>
-      <c r="B43" s="130"/>
+      <c r="B43" s="128"/>
       <c r="C43" s="86"/>
-      <c r="D43" s="132"/>
-      <c r="E43" s="132"/>
+      <c r="D43" s="130"/>
+      <c r="E43" s="130"/>
       <c r="F43" s="86"/>
       <c r="G43" s="88"/>
       <c r="H43" s="87"/>
@@ -3896,81 +3896,81 @@
       <c r="AL43" s="148"/>
       <c r="AM43" s="73"/>
       <c r="AN43" s="2"/>
-      <c r="AO43" s="146"/>
-      <c r="AP43" s="146"/>
-      <c r="AQ43" s="146"/>
-      <c r="AR43" s="146"/>
-      <c r="AS43" s="146"/>
-      <c r="AT43" s="146"/>
-      <c r="AU43" s="146"/>
+      <c r="AO43" s="182"/>
+      <c r="AP43" s="182"/>
+      <c r="AQ43" s="182"/>
+      <c r="AR43" s="182"/>
+      <c r="AS43" s="182"/>
+      <c r="AT43" s="182"/>
+      <c r="AU43" s="182"/>
       <c r="AV43" s="22"/>
     </row>
     <row r="44" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="111"/>
-      <c r="B44" s="130"/>
+      <c r="B44" s="128"/>
       <c r="C44" s="86"/>
-      <c r="D44" s="132"/>
-      <c r="E44" s="132"/>
+      <c r="D44" s="130"/>
+      <c r="E44" s="130"/>
       <c r="F44" s="86"/>
       <c r="G44" s="88"/>
       <c r="H44" s="87"/>
       <c r="I44" s="119"/>
       <c r="J44" s="78"/>
-      <c r="K44" s="144" t="s">
+      <c r="K44" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="L44" s="143"/>
-      <c r="M44" s="142"/>
-      <c r="N44" s="143"/>
+      <c r="L44" s="146"/>
+      <c r="M44" s="147"/>
+      <c r="N44" s="146"/>
       <c r="O44" s="43"/>
       <c r="P44" s="72"/>
-      <c r="Q44" s="144" t="s">
+      <c r="Q44" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="R44" s="143"/>
-      <c r="S44" s="142"/>
-      <c r="T44" s="143"/>
+      <c r="R44" s="146"/>
+      <c r="S44" s="147"/>
+      <c r="T44" s="146"/>
       <c r="U44" s="43"/>
       <c r="V44" s="72"/>
-      <c r="W44" s="144" t="s">
+      <c r="W44" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="X44" s="143"/>
-      <c r="Y44" s="142"/>
-      <c r="Z44" s="143"/>
+      <c r="X44" s="146"/>
+      <c r="Y44" s="147"/>
+      <c r="Z44" s="146"/>
       <c r="AA44" s="43"/>
       <c r="AB44" s="72"/>
-      <c r="AC44" s="144" t="s">
+      <c r="AC44" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="AD44" s="143"/>
-      <c r="AE44" s="142"/>
-      <c r="AF44" s="143"/>
+      <c r="AD44" s="146"/>
+      <c r="AE44" s="147"/>
+      <c r="AF44" s="146"/>
       <c r="AG44" s="43"/>
       <c r="AH44" s="72"/>
-      <c r="AI44" s="144" t="s">
+      <c r="AI44" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="AJ44" s="143"/>
-      <c r="AK44" s="142"/>
-      <c r="AL44" s="143"/>
+      <c r="AJ44" s="146"/>
+      <c r="AK44" s="147"/>
+      <c r="AL44" s="146"/>
       <c r="AM44" s="43"/>
       <c r="AN44" s="2"/>
-      <c r="AO44" s="146"/>
-      <c r="AP44" s="146"/>
-      <c r="AQ44" s="146"/>
-      <c r="AR44" s="146"/>
-      <c r="AS44" s="146"/>
-      <c r="AT44" s="146"/>
-      <c r="AU44" s="146"/>
+      <c r="AO44" s="182"/>
+      <c r="AP44" s="182"/>
+      <c r="AQ44" s="182"/>
+      <c r="AR44" s="182"/>
+      <c r="AS44" s="182"/>
+      <c r="AT44" s="182"/>
+      <c r="AU44" s="182"/>
       <c r="AV44" s="22"/>
     </row>
     <row r="45" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="111"/>
-      <c r="B45" s="130"/>
+      <c r="B45" s="128"/>
       <c r="C45" s="86"/>
-      <c r="D45" s="132"/>
-      <c r="E45" s="132"/>
+      <c r="D45" s="130"/>
+      <c r="E45" s="130"/>
       <c r="F45" s="86"/>
       <c r="G45" s="88"/>
       <c r="H45" s="87"/>
@@ -3980,57 +3980,57 @@
         <v>32</v>
       </c>
       <c r="L45" s="72"/>
-      <c r="M45" s="142"/>
-      <c r="N45" s="143"/>
+      <c r="M45" s="147"/>
+      <c r="N45" s="146"/>
       <c r="O45" s="43"/>
       <c r="P45" s="72"/>
       <c r="Q45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="R45" s="72"/>
-      <c r="S45" s="142"/>
-      <c r="T45" s="143"/>
+      <c r="S45" s="147"/>
+      <c r="T45" s="146"/>
       <c r="U45" s="43"/>
       <c r="V45" s="72"/>
       <c r="W45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="X45" s="72"/>
-      <c r="Y45" s="142"/>
-      <c r="Z45" s="143"/>
+      <c r="Y45" s="147"/>
+      <c r="Z45" s="146"/>
       <c r="AA45" s="43"/>
       <c r="AB45" s="72"/>
       <c r="AC45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AD45" s="72"/>
-      <c r="AE45" s="142"/>
-      <c r="AF45" s="143"/>
+      <c r="AE45" s="147"/>
+      <c r="AF45" s="146"/>
       <c r="AG45" s="43"/>
       <c r="AH45" s="72"/>
       <c r="AI45" s="75" t="s">
         <v>32</v>
       </c>
       <c r="AJ45" s="72"/>
-      <c r="AK45" s="142"/>
-      <c r="AL45" s="143"/>
-      <c r="AM45" s="147"/>
+      <c r="AK45" s="147"/>
+      <c r="AL45" s="146"/>
+      <c r="AM45" s="150"/>
       <c r="AN45" s="2"/>
-      <c r="AO45" s="146"/>
-      <c r="AP45" s="146"/>
-      <c r="AQ45" s="146"/>
-      <c r="AR45" s="146"/>
-      <c r="AS45" s="146"/>
-      <c r="AT45" s="146"/>
-      <c r="AU45" s="146"/>
+      <c r="AO45" s="182"/>
+      <c r="AP45" s="182"/>
+      <c r="AQ45" s="182"/>
+      <c r="AR45" s="182"/>
+      <c r="AS45" s="182"/>
+      <c r="AT45" s="182"/>
+      <c r="AU45" s="182"/>
       <c r="AV45" s="22"/>
     </row>
     <row r="46" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="111"/>
-      <c r="B46" s="130"/>
+      <c r="B46" s="128"/>
       <c r="C46" s="86"/>
-      <c r="D46" s="132"/>
-      <c r="E46" s="132"/>
+      <c r="D46" s="130"/>
+      <c r="E46" s="130"/>
       <c r="F46" s="86"/>
       <c r="G46" s="88"/>
       <c r="H46" s="87"/>
@@ -4039,41 +4039,41 @@
       <c r="K46" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="L46" s="151"/>
-      <c r="M46" s="151"/>
-      <c r="N46" s="151"/>
+      <c r="L46" s="149"/>
+      <c r="M46" s="149"/>
+      <c r="N46" s="149"/>
       <c r="O46" s="40"/>
       <c r="P46" s="41"/>
       <c r="Q46" s="48" t="s">
         <v>45</v>
       </c>
-      <c r="R46" s="149"/>
-      <c r="S46" s="150"/>
-      <c r="T46" s="150"/>
+      <c r="R46" s="143"/>
+      <c r="S46" s="144"/>
+      <c r="T46" s="144"/>
       <c r="U46" s="40"/>
       <c r="V46" s="41"/>
       <c r="W46" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="X46" s="151"/>
-      <c r="Y46" s="151"/>
-      <c r="Z46" s="151"/>
+      <c r="X46" s="149"/>
+      <c r="Y46" s="149"/>
+      <c r="Z46" s="149"/>
       <c r="AA46" s="40"/>
       <c r="AB46" s="41"/>
       <c r="AC46" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="AD46" s="149"/>
-      <c r="AE46" s="150"/>
-      <c r="AF46" s="150"/>
+      <c r="AD46" s="143"/>
+      <c r="AE46" s="144"/>
+      <c r="AF46" s="144"/>
       <c r="AG46" s="40"/>
       <c r="AH46" s="41"/>
       <c r="AI46" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="AJ46" s="149"/>
-      <c r="AK46" s="150"/>
-      <c r="AL46" s="150"/>
+      <c r="AJ46" s="143"/>
+      <c r="AK46" s="144"/>
+      <c r="AL46" s="144"/>
       <c r="AM46" s="40"/>
       <c r="AN46" s="51"/>
       <c r="AO46" s="51"/>
@@ -4089,12 +4089,12 @@
       <c r="A47" s="114"/>
       <c r="B47" s="45"/>
       <c r="C47" s="42"/>
-      <c r="D47" s="133"/>
-      <c r="E47" s="140"/>
+      <c r="D47" s="131"/>
+      <c r="E47" s="138"/>
       <c r="F47" s="47"/>
       <c r="G47" s="42"/>
-      <c r="H47" s="137"/>
-      <c r="I47" s="123"/>
+      <c r="H47" s="135"/>
+      <c r="I47" s="138"/>
       <c r="J47" s="74"/>
       <c r="K47" s="71"/>
       <c r="L47" s="72"/>
@@ -4139,12 +4139,12 @@
       <c r="A48" s="116"/>
       <c r="B48" s="80"/>
       <c r="C48" s="81"/>
-      <c r="D48" s="134"/>
-      <c r="E48" s="141"/>
+      <c r="D48" s="132"/>
+      <c r="E48" s="139"/>
       <c r="F48" s="90"/>
       <c r="G48" s="81"/>
-      <c r="H48" s="138"/>
-      <c r="I48" s="124"/>
+      <c r="H48" s="136"/>
+      <c r="I48" s="122"/>
       <c r="J48" s="74"/>
       <c r="K48" s="148"/>
       <c r="L48" s="148"/>
@@ -4187,10 +4187,10 @@
     </row>
     <row r="49" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="111"/>
-      <c r="B49" s="130"/>
+      <c r="B49" s="128"/>
       <c r="C49" s="86"/>
-      <c r="D49" s="132"/>
-      <c r="E49" s="132"/>
+      <c r="D49" s="130"/>
+      <c r="E49" s="130"/>
       <c r="F49" s="86"/>
       <c r="G49" s="88"/>
       <c r="H49" s="87"/>
@@ -4237,10 +4237,10 @@
     </row>
     <row r="50" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="111"/>
-      <c r="B50" s="130"/>
+      <c r="B50" s="128"/>
       <c r="C50" s="86"/>
-      <c r="D50" s="132"/>
-      <c r="E50" s="132"/>
+      <c r="D50" s="130"/>
+      <c r="E50" s="130"/>
       <c r="F50" s="86"/>
       <c r="G50" s="88"/>
       <c r="H50" s="87"/>
@@ -4287,10 +4287,10 @@
     </row>
     <row r="51" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="111"/>
-      <c r="B51" s="130"/>
+      <c r="B51" s="128"/>
       <c r="C51" s="86"/>
-      <c r="D51" s="132"/>
-      <c r="E51" s="132"/>
+      <c r="D51" s="130"/>
+      <c r="E51" s="130"/>
       <c r="F51" s="86"/>
       <c r="G51" s="88"/>
       <c r="H51" s="87"/>
@@ -4337,10 +4337,10 @@
     </row>
     <row r="52" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="111"/>
-      <c r="B52" s="130"/>
+      <c r="B52" s="128"/>
       <c r="C52" s="86"/>
-      <c r="D52" s="132"/>
-      <c r="E52" s="132"/>
+      <c r="D52" s="130"/>
+      <c r="E52" s="130"/>
       <c r="F52" s="86"/>
       <c r="G52" s="88"/>
       <c r="H52" s="87"/>
@@ -4387,10 +4387,10 @@
     </row>
     <row r="53" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="111"/>
-      <c r="B53" s="130"/>
+      <c r="B53" s="128"/>
       <c r="C53" s="86"/>
-      <c r="D53" s="132"/>
-      <c r="E53" s="132"/>
+      <c r="D53" s="130"/>
+      <c r="E53" s="130"/>
       <c r="F53" s="86"/>
       <c r="G53" s="88"/>
       <c r="H53" s="87"/>
@@ -4437,53 +4437,53 @@
     </row>
     <row r="54" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="111"/>
-      <c r="B54" s="130"/>
+      <c r="B54" s="128"/>
       <c r="C54" s="86"/>
-      <c r="D54" s="132"/>
-      <c r="E54" s="132"/>
+      <c r="D54" s="130"/>
+      <c r="E54" s="130"/>
       <c r="F54" s="86"/>
       <c r="G54" s="88"/>
       <c r="H54" s="87"/>
       <c r="I54" s="119"/>
       <c r="J54" s="78"/>
-      <c r="K54" s="144" t="s">
+      <c r="K54" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="L54" s="143"/>
-      <c r="M54" s="142"/>
-      <c r="N54" s="143"/>
+      <c r="L54" s="146"/>
+      <c r="M54" s="147"/>
+      <c r="N54" s="146"/>
       <c r="O54" s="43"/>
       <c r="P54" s="72"/>
-      <c r="Q54" s="144" t="s">
+      <c r="Q54" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="R54" s="143"/>
-      <c r="S54" s="142"/>
-      <c r="T54" s="143"/>
+      <c r="R54" s="146"/>
+      <c r="S54" s="147"/>
+      <c r="T54" s="146"/>
       <c r="U54" s="43"/>
       <c r="V54" s="72"/>
-      <c r="W54" s="144" t="s">
+      <c r="W54" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="X54" s="143"/>
-      <c r="Y54" s="142"/>
-      <c r="Z54" s="143"/>
+      <c r="X54" s="146"/>
+      <c r="Y54" s="147"/>
+      <c r="Z54" s="146"/>
       <c r="AA54" s="43"/>
       <c r="AB54" s="72"/>
-      <c r="AC54" s="144" t="s">
+      <c r="AC54" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="AD54" s="143"/>
-      <c r="AE54" s="142"/>
-      <c r="AF54" s="143"/>
+      <c r="AD54" s="146"/>
+      <c r="AE54" s="147"/>
+      <c r="AF54" s="146"/>
       <c r="AG54" s="43"/>
       <c r="AH54" s="72"/>
-      <c r="AI54" s="144" t="s">
+      <c r="AI54" s="145" t="s">
         <v>31</v>
       </c>
-      <c r="AJ54" s="143"/>
-      <c r="AK54" s="142"/>
-      <c r="AL54" s="143"/>
+      <c r="AJ54" s="146"/>
+      <c r="AK54" s="147"/>
+      <c r="AL54" s="146"/>
       <c r="AM54" s="72"/>
       <c r="AN54" s="99"/>
       <c r="AO54" s="94"/>
@@ -4497,10 +4497,10 @@
     </row>
     <row r="55" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="111"/>
-      <c r="B55" s="130"/>
+      <c r="B55" s="128"/>
       <c r="C55" s="86"/>
-      <c r="D55" s="132"/>
-      <c r="E55" s="132"/>
+      <c r="D55" s="130"/>
+      <c r="E55" s="130"/>
       <c r="F55" s="86"/>
       <c r="G55" s="88"/>
       <c r="H55" s="87"/>
@@ -4510,41 +4510,41 @@
         <v>32</v>
       </c>
       <c r="L55" s="81"/>
-      <c r="M55" s="182"/>
-      <c r="N55" s="183"/>
+      <c r="M55" s="141"/>
+      <c r="N55" s="142"/>
       <c r="O55" s="82"/>
       <c r="P55" s="81"/>
       <c r="Q55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="R55" s="81"/>
-      <c r="S55" s="182"/>
-      <c r="T55" s="183"/>
+      <c r="S55" s="141"/>
+      <c r="T55" s="142"/>
       <c r="U55" s="82"/>
       <c r="V55" s="81"/>
       <c r="W55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="X55" s="81"/>
-      <c r="Y55" s="182"/>
-      <c r="Z55" s="183"/>
+      <c r="Y55" s="141"/>
+      <c r="Z55" s="142"/>
       <c r="AA55" s="82"/>
       <c r="AB55" s="81"/>
       <c r="AC55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="AD55" s="81"/>
-      <c r="AE55" s="182"/>
-      <c r="AF55" s="183"/>
+      <c r="AE55" s="141"/>
+      <c r="AF55" s="142"/>
       <c r="AG55" s="82"/>
       <c r="AH55" s="81"/>
       <c r="AI55" s="80" t="s">
         <v>32</v>
       </c>
       <c r="AJ55" s="81"/>
-      <c r="AK55" s="182"/>
-      <c r="AL55" s="183"/>
-      <c r="AM55" s="183"/>
+      <c r="AK55" s="141"/>
+      <c r="AL55" s="142"/>
+      <c r="AM55" s="142"/>
       <c r="AN55" s="101"/>
       <c r="AO55" s="102"/>
       <c r="AP55" s="103"/>
@@ -4609,107 +4609,16 @@
     </row>
   </sheetData>
   <mergeCells count="135">
-    <mergeCell ref="M55:N55"/>
-    <mergeCell ref="S55:T55"/>
-    <mergeCell ref="Y55:Z55"/>
-    <mergeCell ref="AE55:AF55"/>
-    <mergeCell ref="AK55:AM55"/>
-    <mergeCell ref="R46:T46"/>
-    <mergeCell ref="K54:L54"/>
-    <mergeCell ref="M54:N54"/>
-    <mergeCell ref="Q54:R54"/>
-    <mergeCell ref="S54:T54"/>
-    <mergeCell ref="W54:X54"/>
-    <mergeCell ref="Y54:Z54"/>
-    <mergeCell ref="K48:N53"/>
-    <mergeCell ref="Q48:T53"/>
-    <mergeCell ref="W48:Z53"/>
-    <mergeCell ref="L46:N46"/>
-    <mergeCell ref="X46:Z46"/>
-    <mergeCell ref="M45:N45"/>
-    <mergeCell ref="S45:T45"/>
-    <mergeCell ref="Y45:Z45"/>
-    <mergeCell ref="AE45:AF45"/>
-    <mergeCell ref="AK45:AM45"/>
-    <mergeCell ref="R36:T36"/>
-    <mergeCell ref="K44:L44"/>
-    <mergeCell ref="M44:N44"/>
-    <mergeCell ref="Q44:R44"/>
-    <mergeCell ref="S44:T44"/>
-    <mergeCell ref="W44:X44"/>
-    <mergeCell ref="Y44:Z44"/>
-    <mergeCell ref="K38:N43"/>
-    <mergeCell ref="Q38:T43"/>
-    <mergeCell ref="W38:Z43"/>
-    <mergeCell ref="L36:N36"/>
-    <mergeCell ref="X36:Z36"/>
-    <mergeCell ref="AJ36:AL36"/>
-    <mergeCell ref="AH3:AM3"/>
-    <mergeCell ref="AN3:AP3"/>
-    <mergeCell ref="AQ3:AS3"/>
-    <mergeCell ref="AT3:AV3"/>
-    <mergeCell ref="AH4:AM4"/>
-    <mergeCell ref="AN4:AP7"/>
-    <mergeCell ref="AQ4:AS7"/>
-    <mergeCell ref="AT4:AV7"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="J8:AG8"/>
-    <mergeCell ref="AH8:AM8"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="J9:AG9"/>
-    <mergeCell ref="AH9:AM9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="J10:AG10"/>
-    <mergeCell ref="AH10:AM10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:AG11"/>
-    <mergeCell ref="AH11:AM11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="J12:AG12"/>
-    <mergeCell ref="AH12:AM12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="J13:AG13"/>
-    <mergeCell ref="AH13:AM13"/>
-    <mergeCell ref="A14:AM15"/>
-    <mergeCell ref="AN15:AV15"/>
-    <mergeCell ref="L16:N16"/>
-    <mergeCell ref="R16:T16"/>
-    <mergeCell ref="X16:Z16"/>
-    <mergeCell ref="AD16:AF16"/>
-    <mergeCell ref="AJ16:AL16"/>
-    <mergeCell ref="AI24:AJ24"/>
-    <mergeCell ref="AK24:AL24"/>
-    <mergeCell ref="K18:N23"/>
-    <mergeCell ref="Q18:T23"/>
-    <mergeCell ref="W18:Z23"/>
-    <mergeCell ref="AC18:AF23"/>
-    <mergeCell ref="AI18:AL23"/>
-    <mergeCell ref="W24:X24"/>
-    <mergeCell ref="Y24:Z24"/>
-    <mergeCell ref="AC24:AD24"/>
-    <mergeCell ref="AE24:AF24"/>
-    <mergeCell ref="X26:Z26"/>
-    <mergeCell ref="L26:N26"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="S24:T24"/>
-    <mergeCell ref="Q34:R34"/>
-    <mergeCell ref="S34:T34"/>
-    <mergeCell ref="W34:X34"/>
-    <mergeCell ref="R26:T26"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="S25:T25"/>
-    <mergeCell ref="Y25:Z25"/>
-    <mergeCell ref="K28:N33"/>
-    <mergeCell ref="Q28:T33"/>
-    <mergeCell ref="W28:Z33"/>
+    <mergeCell ref="AK34:AL34"/>
+    <mergeCell ref="AC34:AD34"/>
+    <mergeCell ref="AE34:AF34"/>
+    <mergeCell ref="AI34:AJ34"/>
+    <mergeCell ref="Y34:Z34"/>
+    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="S35:T35"/>
+    <mergeCell ref="Y35:Z35"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="M34:N34"/>
     <mergeCell ref="AE25:AF25"/>
     <mergeCell ref="AK25:AL25"/>
     <mergeCell ref="AO26:AU45"/>
@@ -4734,16 +4643,107 @@
     <mergeCell ref="AC38:AF43"/>
     <mergeCell ref="AI38:AL43"/>
     <mergeCell ref="AD36:AF36"/>
-    <mergeCell ref="AK34:AL34"/>
-    <mergeCell ref="AC34:AD34"/>
-    <mergeCell ref="AE34:AF34"/>
-    <mergeCell ref="AI34:AJ34"/>
-    <mergeCell ref="Y34:Z34"/>
-    <mergeCell ref="M35:N35"/>
-    <mergeCell ref="S35:T35"/>
-    <mergeCell ref="Y35:Z35"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="X26:Z26"/>
+    <mergeCell ref="L26:N26"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="Q34:R34"/>
+    <mergeCell ref="S34:T34"/>
+    <mergeCell ref="W34:X34"/>
+    <mergeCell ref="R26:T26"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="S25:T25"/>
+    <mergeCell ref="Y25:Z25"/>
+    <mergeCell ref="K28:N33"/>
+    <mergeCell ref="Q28:T33"/>
+    <mergeCell ref="W28:Z33"/>
+    <mergeCell ref="AN15:AV15"/>
+    <mergeCell ref="L16:N16"/>
+    <mergeCell ref="R16:T16"/>
+    <mergeCell ref="X16:Z16"/>
+    <mergeCell ref="AD16:AF16"/>
+    <mergeCell ref="AJ16:AL16"/>
+    <mergeCell ref="AI24:AJ24"/>
+    <mergeCell ref="AK24:AL24"/>
+    <mergeCell ref="K18:N23"/>
+    <mergeCell ref="Q18:T23"/>
+    <mergeCell ref="W18:Z23"/>
+    <mergeCell ref="AC18:AF23"/>
+    <mergeCell ref="AI18:AL23"/>
+    <mergeCell ref="W24:X24"/>
+    <mergeCell ref="Y24:Z24"/>
+    <mergeCell ref="AC24:AD24"/>
+    <mergeCell ref="AE24:AF24"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="J12:AG12"/>
+    <mergeCell ref="AH12:AM12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="J13:AG13"/>
+    <mergeCell ref="AH13:AM13"/>
+    <mergeCell ref="A14:AM15"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="J9:AG9"/>
+    <mergeCell ref="AH9:AM9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="J10:AG10"/>
+    <mergeCell ref="AH10:AM10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:AG11"/>
+    <mergeCell ref="AH11:AM11"/>
+    <mergeCell ref="AH3:AM3"/>
+    <mergeCell ref="AN3:AP3"/>
+    <mergeCell ref="AQ3:AS3"/>
+    <mergeCell ref="AT3:AV3"/>
+    <mergeCell ref="AH4:AM4"/>
+    <mergeCell ref="AN4:AP7"/>
+    <mergeCell ref="AQ4:AS7"/>
+    <mergeCell ref="AT4:AV7"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="J8:AG8"/>
+    <mergeCell ref="AH8:AM8"/>
+    <mergeCell ref="M45:N45"/>
+    <mergeCell ref="S45:T45"/>
+    <mergeCell ref="Y45:Z45"/>
+    <mergeCell ref="AE45:AF45"/>
+    <mergeCell ref="AK45:AM45"/>
+    <mergeCell ref="R36:T36"/>
+    <mergeCell ref="K44:L44"/>
+    <mergeCell ref="M44:N44"/>
+    <mergeCell ref="Q44:R44"/>
+    <mergeCell ref="S44:T44"/>
+    <mergeCell ref="W44:X44"/>
+    <mergeCell ref="Y44:Z44"/>
+    <mergeCell ref="K38:N43"/>
+    <mergeCell ref="Q38:T43"/>
+    <mergeCell ref="W38:Z43"/>
+    <mergeCell ref="L36:N36"/>
+    <mergeCell ref="X36:Z36"/>
+    <mergeCell ref="AJ36:AL36"/>
+    <mergeCell ref="M55:N55"/>
+    <mergeCell ref="S55:T55"/>
+    <mergeCell ref="Y55:Z55"/>
+    <mergeCell ref="AE55:AF55"/>
+    <mergeCell ref="AK55:AM55"/>
+    <mergeCell ref="R46:T46"/>
+    <mergeCell ref="K54:L54"/>
+    <mergeCell ref="M54:N54"/>
+    <mergeCell ref="Q54:R54"/>
+    <mergeCell ref="S54:T54"/>
+    <mergeCell ref="W54:X54"/>
+    <mergeCell ref="Y54:Z54"/>
+    <mergeCell ref="K48:N53"/>
+    <mergeCell ref="Q48:T53"/>
+    <mergeCell ref="W48:Z53"/>
+    <mergeCell ref="L46:N46"/>
+    <mergeCell ref="X46:Z46"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.1" right="0.1" top="0.1" bottom="0.1" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
Update SDS - Tooling select 20260530
</commit_message>
<xml_diff>
--- a/apps/ENG-Backend/api/engineer/mtc/templates/sds_template.xlsx
+++ b/apps/ENG-Backend/api/engineer/mtc/templates/sds_template.xlsx
@@ -751,7 +751,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="180">
+  <cellXfs count="181">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1158,6 +1158,12 @@
     <xf numFmtId="190" fontId="13" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1284,11 +1290,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1785,29 +1788,29 @@
       <c r="AE3" s="11"/>
       <c r="AF3" s="11"/>
       <c r="AG3" s="16"/>
-      <c r="AH3" s="161" t="s">
+      <c r="AH3" s="163" t="s">
         <v>6</v>
       </c>
-      <c r="AI3" s="162"/>
-      <c r="AJ3" s="162"/>
-      <c r="AK3" s="162"/>
-      <c r="AL3" s="162"/>
-      <c r="AM3" s="163"/>
-      <c r="AN3" s="161" t="s">
+      <c r="AI3" s="164"/>
+      <c r="AJ3" s="164"/>
+      <c r="AK3" s="164"/>
+      <c r="AL3" s="164"/>
+      <c r="AM3" s="165"/>
+      <c r="AN3" s="163" t="s">
         <v>7</v>
       </c>
-      <c r="AO3" s="162"/>
-      <c r="AP3" s="163"/>
-      <c r="AQ3" s="161" t="s">
+      <c r="AO3" s="164"/>
+      <c r="AP3" s="165"/>
+      <c r="AQ3" s="163" t="s">
         <v>8</v>
       </c>
-      <c r="AR3" s="162"/>
-      <c r="AS3" s="163"/>
-      <c r="AT3" s="161" t="s">
+      <c r="AR3" s="164"/>
+      <c r="AS3" s="165"/>
+      <c r="AT3" s="163" t="s">
         <v>9</v>
       </c>
-      <c r="AU3" s="162"/>
-      <c r="AV3" s="163"/>
+      <c r="AU3" s="164"/>
+      <c r="AV3" s="165"/>
     </row>
     <row r="4" spans="1:48" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
@@ -1851,21 +1854,21 @@
       <c r="AE4" s="11"/>
       <c r="AF4" s="11"/>
       <c r="AG4" s="11"/>
-      <c r="AH4" s="148"/>
-      <c r="AI4" s="149"/>
-      <c r="AJ4" s="149"/>
-      <c r="AK4" s="149"/>
-      <c r="AL4" s="149"/>
-      <c r="AM4" s="151"/>
-      <c r="AN4" s="164"/>
-      <c r="AO4" s="165"/>
-      <c r="AP4" s="165"/>
-      <c r="AQ4" s="164"/>
-      <c r="AR4" s="165"/>
-      <c r="AS4" s="170"/>
-      <c r="AT4" s="164"/>
-      <c r="AU4" s="165"/>
-      <c r="AV4" s="170"/>
+      <c r="AH4" s="150"/>
+      <c r="AI4" s="151"/>
+      <c r="AJ4" s="151"/>
+      <c r="AK4" s="151"/>
+      <c r="AL4" s="151"/>
+      <c r="AM4" s="153"/>
+      <c r="AN4" s="166"/>
+      <c r="AO4" s="167"/>
+      <c r="AP4" s="167"/>
+      <c r="AQ4" s="166"/>
+      <c r="AR4" s="167"/>
+      <c r="AS4" s="172"/>
+      <c r="AT4" s="166"/>
+      <c r="AU4" s="167"/>
+      <c r="AV4" s="172"/>
     </row>
     <row r="5" spans="1:48" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
@@ -1913,15 +1916,15 @@
       <c r="AK5" s="3"/>
       <c r="AL5" s="3"/>
       <c r="AM5" s="27"/>
-      <c r="AN5" s="166"/>
-      <c r="AO5" s="167"/>
-      <c r="AP5" s="167"/>
-      <c r="AQ5" s="166"/>
-      <c r="AR5" s="167"/>
-      <c r="AS5" s="171"/>
-      <c r="AT5" s="166"/>
-      <c r="AU5" s="167"/>
-      <c r="AV5" s="171"/>
+      <c r="AN5" s="168"/>
+      <c r="AO5" s="169"/>
+      <c r="AP5" s="169"/>
+      <c r="AQ5" s="168"/>
+      <c r="AR5" s="169"/>
+      <c r="AS5" s="173"/>
+      <c r="AT5" s="168"/>
+      <c r="AU5" s="169"/>
+      <c r="AV5" s="173"/>
     </row>
     <row r="6" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
@@ -1965,15 +1968,15 @@
       <c r="AK6" s="1"/>
       <c r="AL6" s="1"/>
       <c r="AM6" s="30"/>
-      <c r="AN6" s="166"/>
-      <c r="AO6" s="167"/>
-      <c r="AP6" s="167"/>
-      <c r="AQ6" s="166"/>
-      <c r="AR6" s="167"/>
-      <c r="AS6" s="171"/>
-      <c r="AT6" s="166"/>
-      <c r="AU6" s="167"/>
-      <c r="AV6" s="171"/>
+      <c r="AN6" s="168"/>
+      <c r="AO6" s="169"/>
+      <c r="AP6" s="169"/>
+      <c r="AQ6" s="168"/>
+      <c r="AR6" s="169"/>
+      <c r="AS6" s="173"/>
+      <c r="AT6" s="168"/>
+      <c r="AU6" s="169"/>
+      <c r="AV6" s="173"/>
     </row>
     <row r="7" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="31"/>
@@ -2015,66 +2018,66 @@
       <c r="AK7" s="32"/>
       <c r="AL7" s="32"/>
       <c r="AM7" s="33"/>
-      <c r="AN7" s="168"/>
-      <c r="AO7" s="169"/>
-      <c r="AP7" s="169"/>
-      <c r="AQ7" s="168"/>
-      <c r="AR7" s="169"/>
-      <c r="AS7" s="172"/>
-      <c r="AT7" s="168"/>
-      <c r="AU7" s="169"/>
-      <c r="AV7" s="172"/>
+      <c r="AN7" s="170"/>
+      <c r="AO7" s="171"/>
+      <c r="AP7" s="171"/>
+      <c r="AQ7" s="170"/>
+      <c r="AR7" s="171"/>
+      <c r="AS7" s="174"/>
+      <c r="AT7" s="170"/>
+      <c r="AU7" s="171"/>
+      <c r="AV7" s="174"/>
     </row>
     <row r="8" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="173" t="s">
+      <c r="B8" s="175" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="159"/>
-      <c r="D8" s="159"/>
-      <c r="E8" s="159"/>
-      <c r="F8" s="159"/>
-      <c r="G8" s="174" t="s">
+      <c r="C8" s="161"/>
+      <c r="D8" s="161"/>
+      <c r="E8" s="161"/>
+      <c r="F8" s="161"/>
+      <c r="G8" s="176" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="159"/>
-      <c r="I8" s="175"/>
-      <c r="J8" s="161" t="s">
+      <c r="H8" s="161"/>
+      <c r="I8" s="177"/>
+      <c r="J8" s="163" t="s">
         <v>21</v>
       </c>
-      <c r="K8" s="162"/>
-      <c r="L8" s="162"/>
-      <c r="M8" s="162"/>
-      <c r="N8" s="162"/>
-      <c r="O8" s="162"/>
-      <c r="P8" s="162"/>
-      <c r="Q8" s="162"/>
-      <c r="R8" s="162"/>
-      <c r="S8" s="162"/>
-      <c r="T8" s="162"/>
-      <c r="U8" s="162"/>
-      <c r="V8" s="162"/>
-      <c r="W8" s="162"/>
-      <c r="X8" s="162"/>
-      <c r="Y8" s="162"/>
-      <c r="Z8" s="162"/>
-      <c r="AA8" s="162"/>
-      <c r="AB8" s="162"/>
-      <c r="AC8" s="162"/>
-      <c r="AD8" s="162"/>
-      <c r="AE8" s="162"/>
-      <c r="AF8" s="162"/>
-      <c r="AG8" s="163"/>
-      <c r="AH8" s="161" t="s">
+      <c r="K8" s="164"/>
+      <c r="L8" s="164"/>
+      <c r="M8" s="164"/>
+      <c r="N8" s="164"/>
+      <c r="O8" s="164"/>
+      <c r="P8" s="164"/>
+      <c r="Q8" s="164"/>
+      <c r="R8" s="164"/>
+      <c r="S8" s="164"/>
+      <c r="T8" s="164"/>
+      <c r="U8" s="164"/>
+      <c r="V8" s="164"/>
+      <c r="W8" s="164"/>
+      <c r="X8" s="164"/>
+      <c r="Y8" s="164"/>
+      <c r="Z8" s="164"/>
+      <c r="AA8" s="164"/>
+      <c r="AB8" s="164"/>
+      <c r="AC8" s="164"/>
+      <c r="AD8" s="164"/>
+      <c r="AE8" s="164"/>
+      <c r="AF8" s="164"/>
+      <c r="AG8" s="165"/>
+      <c r="AH8" s="163" t="s">
         <v>22</v>
       </c>
-      <c r="AI8" s="162"/>
-      <c r="AJ8" s="162"/>
-      <c r="AK8" s="162"/>
-      <c r="AL8" s="162"/>
-      <c r="AM8" s="163"/>
+      <c r="AI8" s="164"/>
+      <c r="AJ8" s="164"/>
+      <c r="AK8" s="164"/>
+      <c r="AL8" s="164"/>
+      <c r="AM8" s="165"/>
       <c r="AN8" s="29" t="s">
         <v>23</v>
       </c>
@@ -2089,44 +2092,44 @@
     </row>
     <row r="9" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="79"/>
-      <c r="B9" s="148"/>
-      <c r="C9" s="149"/>
-      <c r="D9" s="149"/>
-      <c r="E9" s="149"/>
-      <c r="F9" s="149"/>
-      <c r="G9" s="150"/>
-      <c r="H9" s="149"/>
-      <c r="I9" s="151"/>
-      <c r="J9" s="152"/>
-      <c r="K9" s="153"/>
-      <c r="L9" s="153"/>
-      <c r="M9" s="153"/>
-      <c r="N9" s="153"/>
-      <c r="O9" s="153"/>
-      <c r="P9" s="153"/>
-      <c r="Q9" s="153"/>
-      <c r="R9" s="153"/>
-      <c r="S9" s="153"/>
-      <c r="T9" s="153"/>
-      <c r="U9" s="153"/>
-      <c r="V9" s="153"/>
-      <c r="W9" s="153"/>
-      <c r="X9" s="153"/>
-      <c r="Y9" s="153"/>
-      <c r="Z9" s="153"/>
-      <c r="AA9" s="153"/>
-      <c r="AB9" s="153"/>
-      <c r="AC9" s="153"/>
-      <c r="AD9" s="153"/>
-      <c r="AE9" s="153"/>
-      <c r="AF9" s="153"/>
-      <c r="AG9" s="154"/>
-      <c r="AH9" s="152"/>
-      <c r="AI9" s="153"/>
-      <c r="AJ9" s="153"/>
-      <c r="AK9" s="153"/>
-      <c r="AL9" s="153"/>
-      <c r="AM9" s="154"/>
+      <c r="B9" s="150"/>
+      <c r="C9" s="151"/>
+      <c r="D9" s="151"/>
+      <c r="E9" s="151"/>
+      <c r="F9" s="151"/>
+      <c r="G9" s="152"/>
+      <c r="H9" s="151"/>
+      <c r="I9" s="153"/>
+      <c r="J9" s="154"/>
+      <c r="K9" s="155"/>
+      <c r="L9" s="155"/>
+      <c r="M9" s="155"/>
+      <c r="N9" s="155"/>
+      <c r="O9" s="155"/>
+      <c r="P9" s="155"/>
+      <c r="Q9" s="155"/>
+      <c r="R9" s="155"/>
+      <c r="S9" s="155"/>
+      <c r="T9" s="155"/>
+      <c r="U9" s="155"/>
+      <c r="V9" s="155"/>
+      <c r="W9" s="155"/>
+      <c r="X9" s="155"/>
+      <c r="Y9" s="155"/>
+      <c r="Z9" s="155"/>
+      <c r="AA9" s="155"/>
+      <c r="AB9" s="155"/>
+      <c r="AC9" s="155"/>
+      <c r="AD9" s="155"/>
+      <c r="AE9" s="155"/>
+      <c r="AF9" s="155"/>
+      <c r="AG9" s="156"/>
+      <c r="AH9" s="154"/>
+      <c r="AI9" s="155"/>
+      <c r="AJ9" s="155"/>
+      <c r="AK9" s="155"/>
+      <c r="AL9" s="155"/>
+      <c r="AM9" s="156"/>
       <c r="AN9" s="35"/>
       <c r="AO9" s="2"/>
       <c r="AP9" s="2"/>
@@ -2139,44 +2142,44 @@
     </row>
     <row r="10" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="79"/>
-      <c r="B10" s="148"/>
-      <c r="C10" s="149"/>
-      <c r="D10" s="149"/>
-      <c r="E10" s="149"/>
-      <c r="F10" s="149"/>
-      <c r="G10" s="150"/>
-      <c r="H10" s="149"/>
-      <c r="I10" s="151"/>
-      <c r="J10" s="152"/>
-      <c r="K10" s="153"/>
-      <c r="L10" s="153"/>
-      <c r="M10" s="153"/>
-      <c r="N10" s="153"/>
-      <c r="O10" s="153"/>
-      <c r="P10" s="153"/>
-      <c r="Q10" s="153"/>
-      <c r="R10" s="153"/>
-      <c r="S10" s="153"/>
-      <c r="T10" s="153"/>
-      <c r="U10" s="153"/>
-      <c r="V10" s="153"/>
-      <c r="W10" s="153"/>
-      <c r="X10" s="153"/>
-      <c r="Y10" s="153"/>
-      <c r="Z10" s="153"/>
-      <c r="AA10" s="153"/>
-      <c r="AB10" s="153"/>
-      <c r="AC10" s="153"/>
-      <c r="AD10" s="153"/>
-      <c r="AE10" s="153"/>
-      <c r="AF10" s="153"/>
-      <c r="AG10" s="154"/>
-      <c r="AH10" s="152"/>
-      <c r="AI10" s="153"/>
-      <c r="AJ10" s="153"/>
-      <c r="AK10" s="153"/>
-      <c r="AL10" s="153"/>
-      <c r="AM10" s="154"/>
+      <c r="B10" s="150"/>
+      <c r="C10" s="151"/>
+      <c r="D10" s="151"/>
+      <c r="E10" s="151"/>
+      <c r="F10" s="151"/>
+      <c r="G10" s="152"/>
+      <c r="H10" s="151"/>
+      <c r="I10" s="153"/>
+      <c r="J10" s="154"/>
+      <c r="K10" s="155"/>
+      <c r="L10" s="155"/>
+      <c r="M10" s="155"/>
+      <c r="N10" s="155"/>
+      <c r="O10" s="155"/>
+      <c r="P10" s="155"/>
+      <c r="Q10" s="155"/>
+      <c r="R10" s="155"/>
+      <c r="S10" s="155"/>
+      <c r="T10" s="155"/>
+      <c r="U10" s="155"/>
+      <c r="V10" s="155"/>
+      <c r="W10" s="155"/>
+      <c r="X10" s="155"/>
+      <c r="Y10" s="155"/>
+      <c r="Z10" s="155"/>
+      <c r="AA10" s="155"/>
+      <c r="AB10" s="155"/>
+      <c r="AC10" s="155"/>
+      <c r="AD10" s="155"/>
+      <c r="AE10" s="155"/>
+      <c r="AF10" s="155"/>
+      <c r="AG10" s="156"/>
+      <c r="AH10" s="154"/>
+      <c r="AI10" s="155"/>
+      <c r="AJ10" s="155"/>
+      <c r="AK10" s="155"/>
+      <c r="AL10" s="155"/>
+      <c r="AM10" s="156"/>
       <c r="AN10" s="35"/>
       <c r="AO10" s="2"/>
       <c r="AP10" s="2"/>
@@ -2189,44 +2192,44 @@
     </row>
     <row r="11" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="79"/>
-      <c r="B11" s="148"/>
-      <c r="C11" s="149"/>
-      <c r="D11" s="149"/>
-      <c r="E11" s="149"/>
-      <c r="F11" s="149"/>
-      <c r="G11" s="150"/>
-      <c r="H11" s="149"/>
-      <c r="I11" s="151"/>
-      <c r="J11" s="152"/>
-      <c r="K11" s="153"/>
-      <c r="L11" s="153"/>
-      <c r="M11" s="153"/>
-      <c r="N11" s="153"/>
-      <c r="O11" s="153"/>
-      <c r="P11" s="153"/>
-      <c r="Q11" s="153"/>
-      <c r="R11" s="153"/>
-      <c r="S11" s="153"/>
-      <c r="T11" s="153"/>
-      <c r="U11" s="153"/>
-      <c r="V11" s="153"/>
-      <c r="W11" s="153"/>
-      <c r="X11" s="153"/>
-      <c r="Y11" s="153"/>
-      <c r="Z11" s="153"/>
-      <c r="AA11" s="153"/>
-      <c r="AB11" s="153"/>
-      <c r="AC11" s="153"/>
-      <c r="AD11" s="153"/>
-      <c r="AE11" s="153"/>
-      <c r="AF11" s="153"/>
-      <c r="AG11" s="154"/>
-      <c r="AH11" s="152"/>
-      <c r="AI11" s="153"/>
-      <c r="AJ11" s="153"/>
-      <c r="AK11" s="153"/>
-      <c r="AL11" s="153"/>
-      <c r="AM11" s="154"/>
+      <c r="B11" s="150"/>
+      <c r="C11" s="151"/>
+      <c r="D11" s="151"/>
+      <c r="E11" s="151"/>
+      <c r="F11" s="151"/>
+      <c r="G11" s="152"/>
+      <c r="H11" s="151"/>
+      <c r="I11" s="153"/>
+      <c r="J11" s="154"/>
+      <c r="K11" s="155"/>
+      <c r="L11" s="155"/>
+      <c r="M11" s="155"/>
+      <c r="N11" s="155"/>
+      <c r="O11" s="155"/>
+      <c r="P11" s="155"/>
+      <c r="Q11" s="155"/>
+      <c r="R11" s="155"/>
+      <c r="S11" s="155"/>
+      <c r="T11" s="155"/>
+      <c r="U11" s="155"/>
+      <c r="V11" s="155"/>
+      <c r="W11" s="155"/>
+      <c r="X11" s="155"/>
+      <c r="Y11" s="155"/>
+      <c r="Z11" s="155"/>
+      <c r="AA11" s="155"/>
+      <c r="AB11" s="155"/>
+      <c r="AC11" s="155"/>
+      <c r="AD11" s="155"/>
+      <c r="AE11" s="155"/>
+      <c r="AF11" s="155"/>
+      <c r="AG11" s="156"/>
+      <c r="AH11" s="154"/>
+      <c r="AI11" s="155"/>
+      <c r="AJ11" s="155"/>
+      <c r="AK11" s="155"/>
+      <c r="AL11" s="155"/>
+      <c r="AM11" s="156"/>
       <c r="AN11" s="18" t="s">
         <v>24</v>
       </c>
@@ -2241,44 +2244,44 @@
     </row>
     <row r="12" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="79"/>
-      <c r="B12" s="148"/>
-      <c r="C12" s="149"/>
-      <c r="D12" s="149"/>
-      <c r="E12" s="149"/>
-      <c r="F12" s="149"/>
-      <c r="G12" s="150"/>
-      <c r="H12" s="149"/>
-      <c r="I12" s="151"/>
-      <c r="J12" s="152"/>
-      <c r="K12" s="153"/>
-      <c r="L12" s="153"/>
-      <c r="M12" s="153"/>
-      <c r="N12" s="153"/>
-      <c r="O12" s="153"/>
-      <c r="P12" s="153"/>
-      <c r="Q12" s="153"/>
-      <c r="R12" s="153"/>
-      <c r="S12" s="153"/>
-      <c r="T12" s="153"/>
-      <c r="U12" s="153"/>
-      <c r="V12" s="153"/>
-      <c r="W12" s="153"/>
-      <c r="X12" s="153"/>
-      <c r="Y12" s="153"/>
-      <c r="Z12" s="153"/>
-      <c r="AA12" s="153"/>
-      <c r="AB12" s="153"/>
-      <c r="AC12" s="153"/>
-      <c r="AD12" s="153"/>
-      <c r="AE12" s="153"/>
-      <c r="AF12" s="153"/>
-      <c r="AG12" s="154"/>
-      <c r="AH12" s="152"/>
-      <c r="AI12" s="153"/>
-      <c r="AJ12" s="153"/>
-      <c r="AK12" s="153"/>
-      <c r="AL12" s="153"/>
-      <c r="AM12" s="154"/>
+      <c r="B12" s="150"/>
+      <c r="C12" s="151"/>
+      <c r="D12" s="151"/>
+      <c r="E12" s="151"/>
+      <c r="F12" s="151"/>
+      <c r="G12" s="152"/>
+      <c r="H12" s="151"/>
+      <c r="I12" s="153"/>
+      <c r="J12" s="154"/>
+      <c r="K12" s="155"/>
+      <c r="L12" s="155"/>
+      <c r="M12" s="155"/>
+      <c r="N12" s="155"/>
+      <c r="O12" s="155"/>
+      <c r="P12" s="155"/>
+      <c r="Q12" s="155"/>
+      <c r="R12" s="155"/>
+      <c r="S12" s="155"/>
+      <c r="T12" s="155"/>
+      <c r="U12" s="155"/>
+      <c r="V12" s="155"/>
+      <c r="W12" s="155"/>
+      <c r="X12" s="155"/>
+      <c r="Y12" s="155"/>
+      <c r="Z12" s="155"/>
+      <c r="AA12" s="155"/>
+      <c r="AB12" s="155"/>
+      <c r="AC12" s="155"/>
+      <c r="AD12" s="155"/>
+      <c r="AE12" s="155"/>
+      <c r="AF12" s="155"/>
+      <c r="AG12" s="156"/>
+      <c r="AH12" s="154"/>
+      <c r="AI12" s="155"/>
+      <c r="AJ12" s="155"/>
+      <c r="AK12" s="155"/>
+      <c r="AL12" s="155"/>
+      <c r="AM12" s="156"/>
       <c r="AN12" s="35"/>
       <c r="AO12" s="2"/>
       <c r="AP12" s="2"/>
@@ -2291,44 +2294,44 @@
     </row>
     <row r="13" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="79"/>
-      <c r="B13" s="148"/>
-      <c r="C13" s="149"/>
-      <c r="D13" s="149"/>
-      <c r="E13" s="149"/>
-      <c r="F13" s="149"/>
-      <c r="G13" s="150"/>
-      <c r="H13" s="149"/>
-      <c r="I13" s="151"/>
-      <c r="J13" s="152"/>
-      <c r="K13" s="153"/>
-      <c r="L13" s="153"/>
-      <c r="M13" s="153"/>
-      <c r="N13" s="153"/>
-      <c r="O13" s="153"/>
-      <c r="P13" s="153"/>
-      <c r="Q13" s="153"/>
-      <c r="R13" s="153"/>
-      <c r="S13" s="153"/>
-      <c r="T13" s="153"/>
-      <c r="U13" s="153"/>
-      <c r="V13" s="153"/>
-      <c r="W13" s="153"/>
-      <c r="X13" s="153"/>
-      <c r="Y13" s="153"/>
-      <c r="Z13" s="153"/>
-      <c r="AA13" s="153"/>
-      <c r="AB13" s="153"/>
-      <c r="AC13" s="153"/>
-      <c r="AD13" s="153"/>
-      <c r="AE13" s="153"/>
-      <c r="AF13" s="153"/>
-      <c r="AG13" s="154"/>
-      <c r="AH13" s="152"/>
-      <c r="AI13" s="153"/>
-      <c r="AJ13" s="153"/>
-      <c r="AK13" s="153"/>
-      <c r="AL13" s="153"/>
-      <c r="AM13" s="154"/>
+      <c r="B13" s="150"/>
+      <c r="C13" s="151"/>
+      <c r="D13" s="151"/>
+      <c r="E13" s="151"/>
+      <c r="F13" s="151"/>
+      <c r="G13" s="152"/>
+      <c r="H13" s="151"/>
+      <c r="I13" s="153"/>
+      <c r="J13" s="154"/>
+      <c r="K13" s="155"/>
+      <c r="L13" s="155"/>
+      <c r="M13" s="155"/>
+      <c r="N13" s="155"/>
+      <c r="O13" s="155"/>
+      <c r="P13" s="155"/>
+      <c r="Q13" s="155"/>
+      <c r="R13" s="155"/>
+      <c r="S13" s="155"/>
+      <c r="T13" s="155"/>
+      <c r="U13" s="155"/>
+      <c r="V13" s="155"/>
+      <c r="W13" s="155"/>
+      <c r="X13" s="155"/>
+      <c r="Y13" s="155"/>
+      <c r="Z13" s="155"/>
+      <c r="AA13" s="155"/>
+      <c r="AB13" s="155"/>
+      <c r="AC13" s="155"/>
+      <c r="AD13" s="155"/>
+      <c r="AE13" s="155"/>
+      <c r="AF13" s="155"/>
+      <c r="AG13" s="156"/>
+      <c r="AH13" s="154"/>
+      <c r="AI13" s="155"/>
+      <c r="AJ13" s="155"/>
+      <c r="AK13" s="155"/>
+      <c r="AL13" s="155"/>
+      <c r="AM13" s="156"/>
       <c r="AN13" s="23"/>
       <c r="AO13" s="37"/>
       <c r="AP13" s="37"/>
@@ -2340,47 +2343,47 @@
       <c r="AV13" s="38"/>
     </row>
     <row r="14" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="155" t="s">
+      <c r="A14" s="157" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="156"/>
-      <c r="C14" s="156"/>
-      <c r="D14" s="156"/>
-      <c r="E14" s="156"/>
-      <c r="F14" s="156"/>
-      <c r="G14" s="156"/>
-      <c r="H14" s="156"/>
-      <c r="I14" s="156"/>
-      <c r="J14" s="156"/>
-      <c r="K14" s="156"/>
-      <c r="L14" s="156"/>
-      <c r="M14" s="156"/>
-      <c r="N14" s="156"/>
-      <c r="O14" s="156"/>
-      <c r="P14" s="156"/>
-      <c r="Q14" s="156"/>
-      <c r="R14" s="156"/>
-      <c r="S14" s="156"/>
-      <c r="T14" s="156"/>
-      <c r="U14" s="156"/>
-      <c r="V14" s="156"/>
-      <c r="W14" s="156"/>
-      <c r="X14" s="156"/>
-      <c r="Y14" s="156"/>
-      <c r="Z14" s="156"/>
-      <c r="AA14" s="156"/>
-      <c r="AB14" s="156"/>
-      <c r="AC14" s="156"/>
-      <c r="AD14" s="156"/>
-      <c r="AE14" s="156"/>
-      <c r="AF14" s="156"/>
-      <c r="AG14" s="156"/>
-      <c r="AH14" s="156"/>
-      <c r="AI14" s="156"/>
-      <c r="AJ14" s="156"/>
-      <c r="AK14" s="156"/>
-      <c r="AL14" s="156"/>
-      <c r="AM14" s="157"/>
+      <c r="B14" s="158"/>
+      <c r="C14" s="158"/>
+      <c r="D14" s="158"/>
+      <c r="E14" s="158"/>
+      <c r="F14" s="158"/>
+      <c r="G14" s="158"/>
+      <c r="H14" s="158"/>
+      <c r="I14" s="158"/>
+      <c r="J14" s="158"/>
+      <c r="K14" s="158"/>
+      <c r="L14" s="158"/>
+      <c r="M14" s="158"/>
+      <c r="N14" s="158"/>
+      <c r="O14" s="158"/>
+      <c r="P14" s="158"/>
+      <c r="Q14" s="158"/>
+      <c r="R14" s="158"/>
+      <c r="S14" s="158"/>
+      <c r="T14" s="158"/>
+      <c r="U14" s="158"/>
+      <c r="V14" s="158"/>
+      <c r="W14" s="158"/>
+      <c r="X14" s="158"/>
+      <c r="Y14" s="158"/>
+      <c r="Z14" s="158"/>
+      <c r="AA14" s="158"/>
+      <c r="AB14" s="158"/>
+      <c r="AC14" s="158"/>
+      <c r="AD14" s="158"/>
+      <c r="AE14" s="158"/>
+      <c r="AF14" s="158"/>
+      <c r="AG14" s="158"/>
+      <c r="AH14" s="158"/>
+      <c r="AI14" s="158"/>
+      <c r="AJ14" s="158"/>
+      <c r="AK14" s="158"/>
+      <c r="AL14" s="158"/>
+      <c r="AM14" s="159"/>
       <c r="AN14" s="101"/>
       <c r="AO14" s="102"/>
       <c r="AP14" s="102"/>
@@ -2392,59 +2395,59 @@
       <c r="AV14" s="103"/>
     </row>
     <row r="15" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="158"/>
-      <c r="B15" s="159"/>
-      <c r="C15" s="159"/>
-      <c r="D15" s="159"/>
-      <c r="E15" s="159"/>
-      <c r="F15" s="159"/>
-      <c r="G15" s="159"/>
-      <c r="H15" s="159"/>
-      <c r="I15" s="159"/>
-      <c r="J15" s="160"/>
-      <c r="K15" s="160"/>
-      <c r="L15" s="160"/>
-      <c r="M15" s="160"/>
-      <c r="N15" s="160"/>
-      <c r="O15" s="160"/>
-      <c r="P15" s="160"/>
-      <c r="Q15" s="160"/>
-      <c r="R15" s="160"/>
-      <c r="S15" s="160"/>
-      <c r="T15" s="160"/>
-      <c r="U15" s="160"/>
-      <c r="V15" s="160"/>
-      <c r="W15" s="160"/>
-      <c r="X15" s="160"/>
-      <c r="Y15" s="160"/>
-      <c r="Z15" s="160"/>
-      <c r="AA15" s="160"/>
-      <c r="AB15" s="160"/>
-      <c r="AC15" s="160"/>
-      <c r="AD15" s="160"/>
-      <c r="AE15" s="160"/>
-      <c r="AF15" s="160"/>
-      <c r="AG15" s="160"/>
-      <c r="AH15" s="160"/>
-      <c r="AI15" s="160"/>
-      <c r="AJ15" s="160"/>
-      <c r="AK15" s="160"/>
-      <c r="AL15" s="160"/>
-      <c r="AM15" s="157"/>
-      <c r="AN15" s="146"/>
-      <c r="AO15" s="140"/>
-      <c r="AP15" s="140"/>
-      <c r="AQ15" s="140"/>
-      <c r="AR15" s="140"/>
-      <c r="AS15" s="140"/>
-      <c r="AT15" s="140"/>
-      <c r="AU15" s="140"/>
-      <c r="AV15" s="147"/>
+      <c r="A15" s="160"/>
+      <c r="B15" s="161"/>
+      <c r="C15" s="161"/>
+      <c r="D15" s="161"/>
+      <c r="E15" s="161"/>
+      <c r="F15" s="161"/>
+      <c r="G15" s="161"/>
+      <c r="H15" s="161"/>
+      <c r="I15" s="161"/>
+      <c r="J15" s="162"/>
+      <c r="K15" s="162"/>
+      <c r="L15" s="162"/>
+      <c r="M15" s="162"/>
+      <c r="N15" s="162"/>
+      <c r="O15" s="162"/>
+      <c r="P15" s="162"/>
+      <c r="Q15" s="162"/>
+      <c r="R15" s="162"/>
+      <c r="S15" s="162"/>
+      <c r="T15" s="162"/>
+      <c r="U15" s="162"/>
+      <c r="V15" s="162"/>
+      <c r="W15" s="162"/>
+      <c r="X15" s="162"/>
+      <c r="Y15" s="162"/>
+      <c r="Z15" s="162"/>
+      <c r="AA15" s="162"/>
+      <c r="AB15" s="162"/>
+      <c r="AC15" s="162"/>
+      <c r="AD15" s="162"/>
+      <c r="AE15" s="162"/>
+      <c r="AF15" s="162"/>
+      <c r="AG15" s="162"/>
+      <c r="AH15" s="162"/>
+      <c r="AI15" s="162"/>
+      <c r="AJ15" s="162"/>
+      <c r="AK15" s="162"/>
+      <c r="AL15" s="162"/>
+      <c r="AM15" s="159"/>
+      <c r="AN15" s="148"/>
+      <c r="AO15" s="142"/>
+      <c r="AP15" s="142"/>
+      <c r="AQ15" s="142"/>
+      <c r="AR15" s="142"/>
+      <c r="AS15" s="142"/>
+      <c r="AT15" s="142"/>
+      <c r="AU15" s="142"/>
+      <c r="AV15" s="149"/>
     </row>
     <row r="16" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="118"/>
       <c r="B16" s="119"/>
-      <c r="C16" s="119"/>
+      <c r="C16" s="180"/>
       <c r="D16" s="120"/>
       <c r="E16" s="120"/>
       <c r="F16" s="121"/>
@@ -2455,41 +2458,41 @@
       <c r="K16" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="L16" s="143"/>
-      <c r="M16" s="144"/>
-      <c r="N16" s="144"/>
+      <c r="L16" s="145"/>
+      <c r="M16" s="146"/>
+      <c r="N16" s="146"/>
       <c r="O16" s="56"/>
       <c r="P16" s="57"/>
       <c r="Q16" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="R16" s="143"/>
-      <c r="S16" s="144"/>
-      <c r="T16" s="144"/>
+      <c r="R16" s="145"/>
+      <c r="S16" s="146"/>
+      <c r="T16" s="146"/>
       <c r="U16" s="56"/>
       <c r="V16" s="57"/>
       <c r="W16" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="X16" s="143"/>
-      <c r="Y16" s="144"/>
-      <c r="Z16" s="144"/>
+      <c r="X16" s="145"/>
+      <c r="Y16" s="146"/>
+      <c r="Z16" s="146"/>
       <c r="AA16" s="56"/>
       <c r="AB16" s="59"/>
       <c r="AC16" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="AD16" s="143"/>
-      <c r="AE16" s="144"/>
-      <c r="AF16" s="144"/>
+      <c r="AD16" s="145"/>
+      <c r="AE16" s="146"/>
+      <c r="AF16" s="146"/>
       <c r="AG16" s="56"/>
       <c r="AH16" s="59"/>
       <c r="AI16" s="58" t="s">
         <v>30</v>
       </c>
-      <c r="AJ16" s="143"/>
-      <c r="AK16" s="144"/>
-      <c r="AL16" s="144"/>
+      <c r="AJ16" s="145"/>
+      <c r="AK16" s="146"/>
+      <c r="AL16" s="146"/>
       <c r="AM16" s="60"/>
       <c r="AN16" s="104"/>
       <c r="AO16" s="89"/>
@@ -2504,7 +2507,7 @@
     <row r="17" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="123"/>
       <c r="B17" s="124"/>
-      <c r="C17" s="125"/>
+      <c r="C17" s="126"/>
       <c r="D17" s="126"/>
       <c r="E17" s="126"/>
       <c r="F17" s="125"/>
@@ -2554,7 +2557,7 @@
     <row r="18" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="80"/>
       <c r="B18" s="87"/>
-      <c r="C18" s="74"/>
+      <c r="C18" s="88"/>
       <c r="D18" s="88"/>
       <c r="E18" s="88"/>
       <c r="F18" s="74"/>
@@ -2562,34 +2565,34 @@
       <c r="H18" s="98"/>
       <c r="I18" s="83"/>
       <c r="J18" s="65"/>
-      <c r="K18" s="142"/>
-      <c r="L18" s="142"/>
-      <c r="M18" s="142"/>
-      <c r="N18" s="142"/>
+      <c r="K18" s="144"/>
+      <c r="L18" s="144"/>
+      <c r="M18" s="144"/>
+      <c r="N18" s="144"/>
       <c r="O18" s="42"/>
       <c r="P18" s="63"/>
-      <c r="Q18" s="142"/>
-      <c r="R18" s="142"/>
-      <c r="S18" s="142"/>
-      <c r="T18" s="142"/>
+      <c r="Q18" s="144"/>
+      <c r="R18" s="144"/>
+      <c r="S18" s="144"/>
+      <c r="T18" s="144"/>
       <c r="U18" s="42"/>
       <c r="V18" s="63"/>
-      <c r="W18" s="142"/>
-      <c r="X18" s="142"/>
-      <c r="Y18" s="142"/>
-      <c r="Z18" s="142"/>
+      <c r="W18" s="144"/>
+      <c r="X18" s="144"/>
+      <c r="Y18" s="144"/>
+      <c r="Z18" s="144"/>
       <c r="AA18" s="42"/>
       <c r="AB18" s="63"/>
-      <c r="AC18" s="142"/>
-      <c r="AD18" s="142"/>
-      <c r="AE18" s="142"/>
-      <c r="AF18" s="142"/>
+      <c r="AC18" s="144"/>
+      <c r="AD18" s="144"/>
+      <c r="AE18" s="144"/>
+      <c r="AF18" s="144"/>
       <c r="AG18" s="42"/>
       <c r="AH18" s="63"/>
-      <c r="AI18" s="142"/>
-      <c r="AJ18" s="142"/>
-      <c r="AK18" s="142"/>
-      <c r="AL18" s="142"/>
+      <c r="AI18" s="144"/>
+      <c r="AJ18" s="144"/>
+      <c r="AK18" s="144"/>
+      <c r="AL18" s="144"/>
       <c r="AM18" s="64"/>
       <c r="AN18" s="104"/>
       <c r="AO18" s="89"/>
@@ -2604,7 +2607,7 @@
     <row r="19" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="80"/>
       <c r="B19" s="87"/>
-      <c r="C19" s="74"/>
+      <c r="C19" s="88"/>
       <c r="D19" s="88"/>
       <c r="E19" s="88"/>
       <c r="F19" s="74"/>
@@ -2612,34 +2615,34 @@
       <c r="H19" s="75"/>
       <c r="I19" s="83"/>
       <c r="J19" s="61"/>
-      <c r="K19" s="142"/>
-      <c r="L19" s="142"/>
-      <c r="M19" s="142"/>
-      <c r="N19" s="142"/>
+      <c r="K19" s="144"/>
+      <c r="L19" s="144"/>
+      <c r="M19" s="144"/>
+      <c r="N19" s="144"/>
       <c r="O19" s="42"/>
       <c r="P19" s="63"/>
-      <c r="Q19" s="142"/>
-      <c r="R19" s="142"/>
-      <c r="S19" s="142"/>
-      <c r="T19" s="142"/>
+      <c r="Q19" s="144"/>
+      <c r="R19" s="144"/>
+      <c r="S19" s="144"/>
+      <c r="T19" s="144"/>
       <c r="U19" s="42"/>
       <c r="V19" s="63"/>
-      <c r="W19" s="142"/>
-      <c r="X19" s="142"/>
-      <c r="Y19" s="142"/>
-      <c r="Z19" s="142"/>
+      <c r="W19" s="144"/>
+      <c r="X19" s="144"/>
+      <c r="Y19" s="144"/>
+      <c r="Z19" s="144"/>
       <c r="AA19" s="42"/>
       <c r="AB19" s="63"/>
-      <c r="AC19" s="142"/>
-      <c r="AD19" s="142"/>
-      <c r="AE19" s="142"/>
-      <c r="AF19" s="142"/>
+      <c r="AC19" s="144"/>
+      <c r="AD19" s="144"/>
+      <c r="AE19" s="144"/>
+      <c r="AF19" s="144"/>
       <c r="AG19" s="42"/>
       <c r="AH19" s="63"/>
-      <c r="AI19" s="142"/>
-      <c r="AJ19" s="142"/>
-      <c r="AK19" s="142"/>
-      <c r="AL19" s="142"/>
+      <c r="AI19" s="144"/>
+      <c r="AJ19" s="144"/>
+      <c r="AK19" s="144"/>
+      <c r="AL19" s="144"/>
       <c r="AM19" s="64"/>
       <c r="AN19" s="104"/>
       <c r="AO19" s="89"/>
@@ -2654,7 +2657,7 @@
     <row r="20" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="80"/>
       <c r="B20" s="87"/>
-      <c r="C20" s="74"/>
+      <c r="C20" s="88"/>
       <c r="D20" s="88"/>
       <c r="E20" s="88"/>
       <c r="F20" s="74"/>
@@ -2662,34 +2665,34 @@
       <c r="H20" s="75"/>
       <c r="I20" s="83"/>
       <c r="J20" s="65"/>
-      <c r="K20" s="142"/>
-      <c r="L20" s="142"/>
-      <c r="M20" s="142"/>
-      <c r="N20" s="142"/>
+      <c r="K20" s="144"/>
+      <c r="L20" s="144"/>
+      <c r="M20" s="144"/>
+      <c r="N20" s="144"/>
       <c r="O20" s="42"/>
       <c r="P20" s="63"/>
-      <c r="Q20" s="142"/>
-      <c r="R20" s="142"/>
-      <c r="S20" s="142"/>
-      <c r="T20" s="142"/>
+      <c r="Q20" s="144"/>
+      <c r="R20" s="144"/>
+      <c r="S20" s="144"/>
+      <c r="T20" s="144"/>
       <c r="U20" s="42"/>
       <c r="V20" s="63"/>
-      <c r="W20" s="142"/>
-      <c r="X20" s="142"/>
-      <c r="Y20" s="142"/>
-      <c r="Z20" s="142"/>
+      <c r="W20" s="144"/>
+      <c r="X20" s="144"/>
+      <c r="Y20" s="144"/>
+      <c r="Z20" s="144"/>
       <c r="AA20" s="42"/>
       <c r="AB20" s="63"/>
-      <c r="AC20" s="142"/>
-      <c r="AD20" s="142"/>
-      <c r="AE20" s="142"/>
-      <c r="AF20" s="142"/>
+      <c r="AC20" s="144"/>
+      <c r="AD20" s="144"/>
+      <c r="AE20" s="144"/>
+      <c r="AF20" s="144"/>
       <c r="AG20" s="42"/>
       <c r="AH20" s="63"/>
-      <c r="AI20" s="142"/>
-      <c r="AJ20" s="142"/>
-      <c r="AK20" s="142"/>
-      <c r="AL20" s="142"/>
+      <c r="AI20" s="144"/>
+      <c r="AJ20" s="144"/>
+      <c r="AK20" s="144"/>
+      <c r="AL20" s="144"/>
       <c r="AM20" s="64"/>
       <c r="AN20" s="104"/>
       <c r="AO20" s="89"/>
@@ -2704,7 +2707,7 @@
     <row r="21" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="118"/>
       <c r="B21" s="119"/>
-      <c r="C21" s="74"/>
+      <c r="C21" s="88"/>
       <c r="D21" s="88"/>
       <c r="E21" s="88"/>
       <c r="F21" s="74"/>
@@ -2712,34 +2715,34 @@
       <c r="H21" s="75"/>
       <c r="I21" s="83"/>
       <c r="J21" s="65"/>
-      <c r="K21" s="142"/>
-      <c r="L21" s="142"/>
-      <c r="M21" s="142"/>
-      <c r="N21" s="142"/>
+      <c r="K21" s="144"/>
+      <c r="L21" s="144"/>
+      <c r="M21" s="144"/>
+      <c r="N21" s="144"/>
       <c r="O21" s="42"/>
       <c r="P21" s="63"/>
-      <c r="Q21" s="142"/>
-      <c r="R21" s="142"/>
-      <c r="S21" s="142"/>
-      <c r="T21" s="142"/>
+      <c r="Q21" s="144"/>
+      <c r="R21" s="144"/>
+      <c r="S21" s="144"/>
+      <c r="T21" s="144"/>
       <c r="U21" s="42"/>
       <c r="V21" s="63"/>
-      <c r="W21" s="142"/>
-      <c r="X21" s="142"/>
-      <c r="Y21" s="142"/>
-      <c r="Z21" s="142"/>
+      <c r="W21" s="144"/>
+      <c r="X21" s="144"/>
+      <c r="Y21" s="144"/>
+      <c r="Z21" s="144"/>
       <c r="AA21" s="42"/>
       <c r="AB21" s="63"/>
-      <c r="AC21" s="142"/>
-      <c r="AD21" s="142"/>
-      <c r="AE21" s="142"/>
-      <c r="AF21" s="142"/>
+      <c r="AC21" s="144"/>
+      <c r="AD21" s="144"/>
+      <c r="AE21" s="144"/>
+      <c r="AF21" s="144"/>
       <c r="AG21" s="42"/>
       <c r="AH21" s="63"/>
-      <c r="AI21" s="142"/>
-      <c r="AJ21" s="142"/>
-      <c r="AK21" s="142"/>
-      <c r="AL21" s="142"/>
+      <c r="AI21" s="144"/>
+      <c r="AJ21" s="144"/>
+      <c r="AK21" s="144"/>
+      <c r="AL21" s="144"/>
       <c r="AM21" s="64"/>
       <c r="AN21" s="104"/>
       <c r="AO21" s="89"/>
@@ -2754,7 +2757,7 @@
     <row r="22" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="80"/>
       <c r="B22" s="87"/>
-      <c r="C22" s="74"/>
+      <c r="C22" s="88"/>
       <c r="D22" s="88"/>
       <c r="E22" s="88"/>
       <c r="F22" s="74"/>
@@ -2762,34 +2765,34 @@
       <c r="H22" s="75"/>
       <c r="I22" s="83"/>
       <c r="J22" s="65"/>
-      <c r="K22" s="142"/>
-      <c r="L22" s="142"/>
-      <c r="M22" s="142"/>
-      <c r="N22" s="142"/>
+      <c r="K22" s="144"/>
+      <c r="L22" s="144"/>
+      <c r="M22" s="144"/>
+      <c r="N22" s="144"/>
       <c r="O22" s="42"/>
       <c r="P22" s="63"/>
-      <c r="Q22" s="142"/>
-      <c r="R22" s="142"/>
-      <c r="S22" s="142"/>
-      <c r="T22" s="142"/>
+      <c r="Q22" s="144"/>
+      <c r="R22" s="144"/>
+      <c r="S22" s="144"/>
+      <c r="T22" s="144"/>
       <c r="U22" s="42"/>
       <c r="V22" s="63"/>
-      <c r="W22" s="142"/>
-      <c r="X22" s="142"/>
-      <c r="Y22" s="142"/>
-      <c r="Z22" s="142"/>
+      <c r="W22" s="144"/>
+      <c r="X22" s="144"/>
+      <c r="Y22" s="144"/>
+      <c r="Z22" s="144"/>
       <c r="AA22" s="42"/>
       <c r="AB22" s="63"/>
-      <c r="AC22" s="142"/>
-      <c r="AD22" s="142"/>
-      <c r="AE22" s="142"/>
-      <c r="AF22" s="142"/>
+      <c r="AC22" s="144"/>
+      <c r="AD22" s="144"/>
+      <c r="AE22" s="144"/>
+      <c r="AF22" s="144"/>
       <c r="AG22" s="42"/>
       <c r="AH22" s="63"/>
-      <c r="AI22" s="142"/>
-      <c r="AJ22" s="142"/>
-      <c r="AK22" s="142"/>
-      <c r="AL22" s="142"/>
+      <c r="AI22" s="144"/>
+      <c r="AJ22" s="144"/>
+      <c r="AK22" s="144"/>
+      <c r="AL22" s="144"/>
       <c r="AM22" s="64"/>
       <c r="AN22" s="104"/>
       <c r="AO22" s="89"/>
@@ -2804,7 +2807,7 @@
     <row r="23" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="80"/>
       <c r="B23" s="87"/>
-      <c r="C23" s="74"/>
+      <c r="C23" s="88"/>
       <c r="D23" s="88"/>
       <c r="E23" s="88"/>
       <c r="F23" s="74"/>
@@ -2812,34 +2815,34 @@
       <c r="H23" s="75"/>
       <c r="I23" s="83"/>
       <c r="J23" s="61"/>
-      <c r="K23" s="142"/>
-      <c r="L23" s="142"/>
-      <c r="M23" s="142"/>
-      <c r="N23" s="142"/>
+      <c r="K23" s="144"/>
+      <c r="L23" s="144"/>
+      <c r="M23" s="144"/>
+      <c r="N23" s="144"/>
       <c r="O23" s="42"/>
       <c r="P23" s="63"/>
-      <c r="Q23" s="142"/>
-      <c r="R23" s="142"/>
-      <c r="S23" s="142"/>
-      <c r="T23" s="142"/>
+      <c r="Q23" s="144"/>
+      <c r="R23" s="144"/>
+      <c r="S23" s="144"/>
+      <c r="T23" s="144"/>
       <c r="U23" s="42"/>
       <c r="V23" s="63"/>
-      <c r="W23" s="142"/>
-      <c r="X23" s="142"/>
-      <c r="Y23" s="142"/>
-      <c r="Z23" s="142"/>
+      <c r="W23" s="144"/>
+      <c r="X23" s="144"/>
+      <c r="Y23" s="144"/>
+      <c r="Z23" s="144"/>
       <c r="AA23" s="42"/>
       <c r="AB23" s="63"/>
-      <c r="AC23" s="142"/>
-      <c r="AD23" s="142"/>
-      <c r="AE23" s="142"/>
-      <c r="AF23" s="142"/>
+      <c r="AC23" s="144"/>
+      <c r="AD23" s="144"/>
+      <c r="AE23" s="144"/>
+      <c r="AF23" s="144"/>
       <c r="AG23" s="42"/>
       <c r="AH23" s="63"/>
-      <c r="AI23" s="142"/>
-      <c r="AJ23" s="142"/>
-      <c r="AK23" s="142"/>
-      <c r="AL23" s="142"/>
+      <c r="AI23" s="144"/>
+      <c r="AJ23" s="144"/>
+      <c r="AK23" s="144"/>
+      <c r="AL23" s="144"/>
       <c r="AM23" s="64"/>
       <c r="AN23" s="104"/>
       <c r="AO23" s="89"/>
@@ -2854,7 +2857,7 @@
     <row r="24" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="80"/>
       <c r="B24" s="87"/>
-      <c r="C24" s="74"/>
+      <c r="C24" s="88"/>
       <c r="D24" s="88"/>
       <c r="E24" s="88"/>
       <c r="F24" s="74"/>
@@ -2862,44 +2865,44 @@
       <c r="H24" s="75"/>
       <c r="I24" s="83"/>
       <c r="J24" s="65"/>
-      <c r="K24" s="138" t="s">
+      <c r="K24" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="L24" s="137"/>
-      <c r="M24" s="136"/>
-      <c r="N24" s="137"/>
+      <c r="L24" s="139"/>
+      <c r="M24" s="138"/>
+      <c r="N24" s="139"/>
       <c r="O24" s="42"/>
       <c r="P24" s="63"/>
-      <c r="Q24" s="138" t="s">
+      <c r="Q24" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="R24" s="137"/>
-      <c r="S24" s="136"/>
-      <c r="T24" s="137"/>
+      <c r="R24" s="139"/>
+      <c r="S24" s="138"/>
+      <c r="T24" s="139"/>
       <c r="U24" s="42"/>
       <c r="V24" s="63"/>
-      <c r="W24" s="138" t="s">
+      <c r="W24" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="X24" s="137"/>
-      <c r="Y24" s="136"/>
-      <c r="Z24" s="137"/>
+      <c r="X24" s="139"/>
+      <c r="Y24" s="138"/>
+      <c r="Z24" s="139"/>
       <c r="AA24" s="42"/>
       <c r="AB24" s="63"/>
-      <c r="AC24" s="138" t="s">
+      <c r="AC24" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="AD24" s="137"/>
-      <c r="AE24" s="136"/>
-      <c r="AF24" s="137"/>
+      <c r="AD24" s="139"/>
+      <c r="AE24" s="138"/>
+      <c r="AF24" s="139"/>
       <c r="AG24" s="42"/>
       <c r="AH24" s="63"/>
-      <c r="AI24" s="138" t="s">
+      <c r="AI24" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="AJ24" s="137"/>
-      <c r="AK24" s="136"/>
-      <c r="AL24" s="137"/>
+      <c r="AJ24" s="139"/>
+      <c r="AK24" s="138"/>
+      <c r="AL24" s="139"/>
       <c r="AM24" s="64"/>
       <c r="AN24" s="104"/>
       <c r="AO24" s="89"/>
@@ -2914,7 +2917,7 @@
     <row r="25" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="80"/>
       <c r="B25" s="87"/>
-      <c r="C25" s="74"/>
+      <c r="C25" s="88"/>
       <c r="D25" s="88"/>
       <c r="E25" s="88"/>
       <c r="F25" s="74"/>
@@ -2926,40 +2929,40 @@
         <v>32</v>
       </c>
       <c r="L25" s="63"/>
-      <c r="M25" s="136"/>
-      <c r="N25" s="137"/>
+      <c r="M25" s="138"/>
+      <c r="N25" s="139"/>
       <c r="O25" s="42"/>
       <c r="P25" s="63"/>
       <c r="Q25" s="66" t="s">
         <v>32</v>
       </c>
       <c r="R25" s="63"/>
-      <c r="S25" s="136"/>
-      <c r="T25" s="137"/>
+      <c r="S25" s="138"/>
+      <c r="T25" s="139"/>
       <c r="U25" s="42"/>
       <c r="V25" s="63"/>
       <c r="W25" s="66" t="s">
         <v>32</v>
       </c>
       <c r="X25" s="63"/>
-      <c r="Y25" s="136"/>
-      <c r="Z25" s="137"/>
+      <c r="Y25" s="138"/>
+      <c r="Z25" s="139"/>
       <c r="AA25" s="42"/>
       <c r="AB25" s="63"/>
       <c r="AC25" s="66" t="s">
         <v>32</v>
       </c>
       <c r="AD25" s="63"/>
-      <c r="AE25" s="136"/>
-      <c r="AF25" s="137"/>
+      <c r="AE25" s="138"/>
+      <c r="AF25" s="139"/>
       <c r="AG25" s="42"/>
       <c r="AH25" s="63"/>
       <c r="AI25" s="66" t="s">
         <v>32</v>
       </c>
       <c r="AJ25" s="63"/>
-      <c r="AK25" s="136"/>
-      <c r="AL25" s="137"/>
+      <c r="AK25" s="138"/>
+      <c r="AL25" s="139"/>
       <c r="AM25" s="64"/>
       <c r="AN25" s="104"/>
       <c r="AO25" s="89"/>
@@ -2974,7 +2977,7 @@
     <row r="26" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="80"/>
       <c r="B26" s="87"/>
-      <c r="C26" s="74"/>
+      <c r="C26" s="88"/>
       <c r="D26" s="88"/>
       <c r="E26" s="88"/>
       <c r="F26" s="74"/>
@@ -2985,56 +2988,56 @@
       <c r="K26" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="L26" s="145"/>
-      <c r="M26" s="145"/>
-      <c r="N26" s="145"/>
+      <c r="L26" s="147"/>
+      <c r="M26" s="147"/>
+      <c r="N26" s="147"/>
       <c r="O26" s="53"/>
       <c r="P26" s="40"/>
       <c r="Q26" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="R26" s="143"/>
-      <c r="S26" s="144"/>
-      <c r="T26" s="144"/>
+      <c r="R26" s="145"/>
+      <c r="S26" s="146"/>
+      <c r="T26" s="146"/>
       <c r="U26" s="39"/>
       <c r="V26" s="40"/>
       <c r="W26" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="X26" s="145"/>
-      <c r="Y26" s="145"/>
-      <c r="Z26" s="145"/>
+      <c r="X26" s="147"/>
+      <c r="Y26" s="147"/>
+      <c r="Z26" s="147"/>
       <c r="AA26" s="39"/>
       <c r="AB26" s="40"/>
       <c r="AC26" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="AD26" s="143"/>
-      <c r="AE26" s="144"/>
-      <c r="AF26" s="144"/>
+      <c r="AD26" s="145"/>
+      <c r="AE26" s="146"/>
+      <c r="AF26" s="146"/>
       <c r="AG26" s="39"/>
       <c r="AH26" s="40"/>
       <c r="AI26" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="AJ26" s="143"/>
-      <c r="AK26" s="144"/>
-      <c r="AL26" s="144"/>
+      <c r="AJ26" s="145"/>
+      <c r="AK26" s="146"/>
+      <c r="AL26" s="146"/>
       <c r="AM26" s="68"/>
       <c r="AN26" s="104"/>
-      <c r="AO26" s="139"/>
-      <c r="AP26" s="140"/>
-      <c r="AQ26" s="140"/>
-      <c r="AR26" s="140"/>
-      <c r="AS26" s="140"/>
-      <c r="AT26" s="140"/>
-      <c r="AU26" s="140"/>
+      <c r="AO26" s="141"/>
+      <c r="AP26" s="142"/>
+      <c r="AQ26" s="142"/>
+      <c r="AR26" s="142"/>
+      <c r="AS26" s="142"/>
+      <c r="AT26" s="142"/>
+      <c r="AU26" s="142"/>
       <c r="AV26" s="105"/>
     </row>
     <row r="27" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="81"/>
       <c r="B27" s="128"/>
-      <c r="C27" s="129"/>
+      <c r="C27" s="89"/>
       <c r="D27" s="89"/>
       <c r="E27" s="89"/>
       <c r="F27" s="129"/>
@@ -3072,19 +3075,19 @@
       <c r="AL27" s="63"/>
       <c r="AM27" s="64"/>
       <c r="AN27" s="104"/>
-      <c r="AO27" s="140"/>
-      <c r="AP27" s="140"/>
-      <c r="AQ27" s="140"/>
-      <c r="AR27" s="140"/>
-      <c r="AS27" s="140"/>
-      <c r="AT27" s="140"/>
-      <c r="AU27" s="140"/>
+      <c r="AO27" s="142"/>
+      <c r="AP27" s="142"/>
+      <c r="AQ27" s="142"/>
+      <c r="AR27" s="142"/>
+      <c r="AS27" s="142"/>
+      <c r="AT27" s="142"/>
+      <c r="AU27" s="142"/>
       <c r="AV27" s="105"/>
     </row>
     <row r="28" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="82"/>
       <c r="B28" s="131"/>
-      <c r="C28" s="132"/>
+      <c r="C28" s="90"/>
       <c r="D28" s="90"/>
       <c r="E28" s="90"/>
       <c r="F28" s="132"/>
@@ -3092,49 +3095,49 @@
       <c r="H28" s="92"/>
       <c r="I28" s="85"/>
       <c r="J28" s="65"/>
-      <c r="K28" s="142"/>
-      <c r="L28" s="142"/>
-      <c r="M28" s="142"/>
-      <c r="N28" s="142"/>
+      <c r="K28" s="144"/>
+      <c r="L28" s="144"/>
+      <c r="M28" s="144"/>
+      <c r="N28" s="144"/>
       <c r="O28" s="42"/>
       <c r="P28" s="63"/>
-      <c r="Q28" s="142"/>
-      <c r="R28" s="142"/>
-      <c r="S28" s="142"/>
-      <c r="T28" s="142"/>
+      <c r="Q28" s="144"/>
+      <c r="R28" s="144"/>
+      <c r="S28" s="144"/>
+      <c r="T28" s="144"/>
       <c r="U28" s="42"/>
       <c r="V28" s="63"/>
-      <c r="W28" s="142"/>
-      <c r="X28" s="142"/>
-      <c r="Y28" s="142"/>
-      <c r="Z28" s="142"/>
+      <c r="W28" s="144"/>
+      <c r="X28" s="144"/>
+      <c r="Y28" s="144"/>
+      <c r="Z28" s="144"/>
       <c r="AA28" s="42"/>
       <c r="AB28" s="63"/>
-      <c r="AC28" s="142"/>
-      <c r="AD28" s="142"/>
-      <c r="AE28" s="142"/>
-      <c r="AF28" s="142"/>
+      <c r="AC28" s="144"/>
+      <c r="AD28" s="144"/>
+      <c r="AE28" s="144"/>
+      <c r="AF28" s="144"/>
       <c r="AG28" s="42"/>
       <c r="AH28" s="63"/>
-      <c r="AI28" s="142"/>
-      <c r="AJ28" s="142"/>
-      <c r="AK28" s="142"/>
-      <c r="AL28" s="142"/>
+      <c r="AI28" s="144"/>
+      <c r="AJ28" s="144"/>
+      <c r="AK28" s="144"/>
+      <c r="AL28" s="144"/>
       <c r="AM28" s="64"/>
       <c r="AN28" s="104"/>
-      <c r="AO28" s="140"/>
-      <c r="AP28" s="140"/>
-      <c r="AQ28" s="140"/>
-      <c r="AR28" s="140"/>
-      <c r="AS28" s="140"/>
-      <c r="AT28" s="140"/>
-      <c r="AU28" s="140"/>
+      <c r="AO28" s="142"/>
+      <c r="AP28" s="142"/>
+      <c r="AQ28" s="142"/>
+      <c r="AR28" s="142"/>
+      <c r="AS28" s="142"/>
+      <c r="AT28" s="142"/>
+      <c r="AU28" s="142"/>
       <c r="AV28" s="105"/>
     </row>
     <row r="29" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="80"/>
       <c r="B29" s="87"/>
-      <c r="C29" s="74"/>
+      <c r="C29" s="88"/>
       <c r="D29" s="88"/>
       <c r="E29" s="88"/>
       <c r="F29" s="74"/>
@@ -3142,49 +3145,49 @@
       <c r="H29" s="75"/>
       <c r="I29" s="83"/>
       <c r="J29" s="61"/>
-      <c r="K29" s="142"/>
-      <c r="L29" s="142"/>
-      <c r="M29" s="142"/>
-      <c r="N29" s="142"/>
+      <c r="K29" s="144"/>
+      <c r="L29" s="144"/>
+      <c r="M29" s="144"/>
+      <c r="N29" s="144"/>
       <c r="O29" s="42"/>
       <c r="P29" s="63"/>
-      <c r="Q29" s="142"/>
-      <c r="R29" s="142"/>
-      <c r="S29" s="142"/>
-      <c r="T29" s="142"/>
+      <c r="Q29" s="144"/>
+      <c r="R29" s="144"/>
+      <c r="S29" s="144"/>
+      <c r="T29" s="144"/>
       <c r="U29" s="42"/>
       <c r="V29" s="63"/>
-      <c r="W29" s="142"/>
-      <c r="X29" s="142"/>
-      <c r="Y29" s="142"/>
-      <c r="Z29" s="142"/>
+      <c r="W29" s="144"/>
+      <c r="X29" s="144"/>
+      <c r="Y29" s="144"/>
+      <c r="Z29" s="144"/>
       <c r="AA29" s="42"/>
       <c r="AB29" s="63"/>
-      <c r="AC29" s="142"/>
-      <c r="AD29" s="142"/>
-      <c r="AE29" s="142"/>
-      <c r="AF29" s="142"/>
+      <c r="AC29" s="144"/>
+      <c r="AD29" s="144"/>
+      <c r="AE29" s="144"/>
+      <c r="AF29" s="144"/>
       <c r="AG29" s="42"/>
       <c r="AH29" s="63"/>
-      <c r="AI29" s="142"/>
-      <c r="AJ29" s="142"/>
-      <c r="AK29" s="142"/>
-      <c r="AL29" s="142"/>
+      <c r="AI29" s="144"/>
+      <c r="AJ29" s="144"/>
+      <c r="AK29" s="144"/>
+      <c r="AL29" s="144"/>
       <c r="AM29" s="64"/>
       <c r="AN29" s="104"/>
-      <c r="AO29" s="140"/>
-      <c r="AP29" s="140"/>
-      <c r="AQ29" s="140"/>
-      <c r="AR29" s="140"/>
-      <c r="AS29" s="140"/>
-      <c r="AT29" s="140"/>
-      <c r="AU29" s="140"/>
+      <c r="AO29" s="142"/>
+      <c r="AP29" s="142"/>
+      <c r="AQ29" s="142"/>
+      <c r="AR29" s="142"/>
+      <c r="AS29" s="142"/>
+      <c r="AT29" s="142"/>
+      <c r="AU29" s="142"/>
       <c r="AV29" s="105"/>
     </row>
     <row r="30" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="80"/>
       <c r="B30" s="87"/>
-      <c r="C30" s="74"/>
+      <c r="C30" s="88"/>
       <c r="D30" s="88"/>
       <c r="E30" s="88"/>
       <c r="F30" s="74"/>
@@ -3192,49 +3195,49 @@
       <c r="H30" s="75"/>
       <c r="I30" s="83"/>
       <c r="J30" s="65"/>
-      <c r="K30" s="142"/>
-      <c r="L30" s="142"/>
-      <c r="M30" s="142"/>
-      <c r="N30" s="142"/>
+      <c r="K30" s="144"/>
+      <c r="L30" s="144"/>
+      <c r="M30" s="144"/>
+      <c r="N30" s="144"/>
       <c r="O30" s="42"/>
       <c r="P30" s="63"/>
-      <c r="Q30" s="142"/>
-      <c r="R30" s="142"/>
-      <c r="S30" s="142"/>
-      <c r="T30" s="142"/>
+      <c r="Q30" s="144"/>
+      <c r="R30" s="144"/>
+      <c r="S30" s="144"/>
+      <c r="T30" s="144"/>
       <c r="U30" s="42"/>
       <c r="V30" s="63"/>
-      <c r="W30" s="142"/>
-      <c r="X30" s="142"/>
-      <c r="Y30" s="142"/>
-      <c r="Z30" s="142"/>
+      <c r="W30" s="144"/>
+      <c r="X30" s="144"/>
+      <c r="Y30" s="144"/>
+      <c r="Z30" s="144"/>
       <c r="AA30" s="42"/>
       <c r="AB30" s="63"/>
-      <c r="AC30" s="142"/>
-      <c r="AD30" s="142"/>
-      <c r="AE30" s="142"/>
-      <c r="AF30" s="142"/>
+      <c r="AC30" s="144"/>
+      <c r="AD30" s="144"/>
+      <c r="AE30" s="144"/>
+      <c r="AF30" s="144"/>
       <c r="AG30" s="42"/>
       <c r="AH30" s="63"/>
-      <c r="AI30" s="142"/>
-      <c r="AJ30" s="142"/>
-      <c r="AK30" s="142"/>
-      <c r="AL30" s="142"/>
+      <c r="AI30" s="144"/>
+      <c r="AJ30" s="144"/>
+      <c r="AK30" s="144"/>
+      <c r="AL30" s="144"/>
       <c r="AM30" s="64"/>
       <c r="AN30" s="104"/>
-      <c r="AO30" s="140"/>
-      <c r="AP30" s="140"/>
-      <c r="AQ30" s="140"/>
-      <c r="AR30" s="140"/>
-      <c r="AS30" s="140"/>
-      <c r="AT30" s="140"/>
-      <c r="AU30" s="140"/>
+      <c r="AO30" s="142"/>
+      <c r="AP30" s="142"/>
+      <c r="AQ30" s="142"/>
+      <c r="AR30" s="142"/>
+      <c r="AS30" s="142"/>
+      <c r="AT30" s="142"/>
+      <c r="AU30" s="142"/>
       <c r="AV30" s="105"/>
     </row>
     <row r="31" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="80"/>
       <c r="B31" s="87"/>
-      <c r="C31" s="74"/>
+      <c r="C31" s="88"/>
       <c r="D31" s="88"/>
       <c r="E31" s="88"/>
       <c r="F31" s="74"/>
@@ -3242,49 +3245,49 @@
       <c r="H31" s="75"/>
       <c r="I31" s="83"/>
       <c r="J31" s="65"/>
-      <c r="K31" s="142"/>
-      <c r="L31" s="142"/>
-      <c r="M31" s="142"/>
-      <c r="N31" s="142"/>
+      <c r="K31" s="144"/>
+      <c r="L31" s="144"/>
+      <c r="M31" s="144"/>
+      <c r="N31" s="144"/>
       <c r="O31" s="42"/>
       <c r="P31" s="63"/>
-      <c r="Q31" s="142"/>
-      <c r="R31" s="142"/>
-      <c r="S31" s="142"/>
-      <c r="T31" s="142"/>
+      <c r="Q31" s="144"/>
+      <c r="R31" s="144"/>
+      <c r="S31" s="144"/>
+      <c r="T31" s="144"/>
       <c r="U31" s="42"/>
       <c r="V31" s="63"/>
-      <c r="W31" s="142"/>
-      <c r="X31" s="142"/>
-      <c r="Y31" s="142"/>
-      <c r="Z31" s="142"/>
+      <c r="W31" s="144"/>
+      <c r="X31" s="144"/>
+      <c r="Y31" s="144"/>
+      <c r="Z31" s="144"/>
       <c r="AA31" s="42"/>
       <c r="AB31" s="63"/>
-      <c r="AC31" s="142"/>
-      <c r="AD31" s="142"/>
-      <c r="AE31" s="142"/>
-      <c r="AF31" s="142"/>
+      <c r="AC31" s="144"/>
+      <c r="AD31" s="144"/>
+      <c r="AE31" s="144"/>
+      <c r="AF31" s="144"/>
       <c r="AG31" s="42"/>
       <c r="AH31" s="63"/>
-      <c r="AI31" s="142"/>
-      <c r="AJ31" s="142"/>
-      <c r="AK31" s="142"/>
-      <c r="AL31" s="142"/>
+      <c r="AI31" s="144"/>
+      <c r="AJ31" s="144"/>
+      <c r="AK31" s="144"/>
+      <c r="AL31" s="144"/>
       <c r="AM31" s="64"/>
       <c r="AN31" s="104"/>
-      <c r="AO31" s="140"/>
-      <c r="AP31" s="140"/>
-      <c r="AQ31" s="140"/>
-      <c r="AR31" s="140"/>
-      <c r="AS31" s="140"/>
-      <c r="AT31" s="140"/>
-      <c r="AU31" s="140"/>
+      <c r="AO31" s="142"/>
+      <c r="AP31" s="142"/>
+      <c r="AQ31" s="142"/>
+      <c r="AR31" s="142"/>
+      <c r="AS31" s="142"/>
+      <c r="AT31" s="142"/>
+      <c r="AU31" s="142"/>
       <c r="AV31" s="105"/>
     </row>
     <row r="32" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="80"/>
       <c r="B32" s="87"/>
-      <c r="C32" s="74"/>
+      <c r="C32" s="88"/>
       <c r="D32" s="88"/>
       <c r="E32" s="88"/>
       <c r="F32" s="74"/>
@@ -3292,49 +3295,49 @@
       <c r="H32" s="75"/>
       <c r="I32" s="83"/>
       <c r="J32" s="65"/>
-      <c r="K32" s="142"/>
-      <c r="L32" s="142"/>
-      <c r="M32" s="142"/>
-      <c r="N32" s="142"/>
+      <c r="K32" s="144"/>
+      <c r="L32" s="144"/>
+      <c r="M32" s="144"/>
+      <c r="N32" s="144"/>
       <c r="O32" s="42"/>
       <c r="P32" s="63"/>
-      <c r="Q32" s="142"/>
-      <c r="R32" s="142"/>
-      <c r="S32" s="142"/>
-      <c r="T32" s="142"/>
+      <c r="Q32" s="144"/>
+      <c r="R32" s="144"/>
+      <c r="S32" s="144"/>
+      <c r="T32" s="144"/>
       <c r="U32" s="42"/>
       <c r="V32" s="63"/>
-      <c r="W32" s="142"/>
-      <c r="X32" s="142"/>
-      <c r="Y32" s="142"/>
-      <c r="Z32" s="142"/>
+      <c r="W32" s="144"/>
+      <c r="X32" s="144"/>
+      <c r="Y32" s="144"/>
+      <c r="Z32" s="144"/>
       <c r="AA32" s="42"/>
       <c r="AB32" s="63"/>
-      <c r="AC32" s="142"/>
-      <c r="AD32" s="142"/>
-      <c r="AE32" s="142"/>
-      <c r="AF32" s="142"/>
+      <c r="AC32" s="144"/>
+      <c r="AD32" s="144"/>
+      <c r="AE32" s="144"/>
+      <c r="AF32" s="144"/>
       <c r="AG32" s="42"/>
       <c r="AH32" s="63"/>
-      <c r="AI32" s="142"/>
-      <c r="AJ32" s="142"/>
-      <c r="AK32" s="142"/>
-      <c r="AL32" s="142"/>
+      <c r="AI32" s="144"/>
+      <c r="AJ32" s="144"/>
+      <c r="AK32" s="144"/>
+      <c r="AL32" s="144"/>
       <c r="AM32" s="64"/>
       <c r="AN32" s="104"/>
-      <c r="AO32" s="140"/>
-      <c r="AP32" s="140"/>
-      <c r="AQ32" s="140"/>
-      <c r="AR32" s="140"/>
-      <c r="AS32" s="140"/>
-      <c r="AT32" s="140"/>
-      <c r="AU32" s="140"/>
+      <c r="AO32" s="142"/>
+      <c r="AP32" s="142"/>
+      <c r="AQ32" s="142"/>
+      <c r="AR32" s="142"/>
+      <c r="AS32" s="142"/>
+      <c r="AT32" s="142"/>
+      <c r="AU32" s="142"/>
       <c r="AV32" s="105"/>
     </row>
     <row r="33" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="80"/>
       <c r="B33" s="87"/>
-      <c r="C33" s="74"/>
+      <c r="C33" s="88"/>
       <c r="D33" s="88"/>
       <c r="E33" s="88"/>
       <c r="F33" s="74"/>
@@ -3342,49 +3345,49 @@
       <c r="H33" s="75"/>
       <c r="I33" s="83"/>
       <c r="J33" s="61"/>
-      <c r="K33" s="142"/>
-      <c r="L33" s="142"/>
-      <c r="M33" s="142"/>
-      <c r="N33" s="142"/>
+      <c r="K33" s="144"/>
+      <c r="L33" s="144"/>
+      <c r="M33" s="144"/>
+      <c r="N33" s="144"/>
       <c r="O33" s="42"/>
       <c r="P33" s="63"/>
-      <c r="Q33" s="142"/>
-      <c r="R33" s="142"/>
-      <c r="S33" s="142"/>
-      <c r="T33" s="142"/>
+      <c r="Q33" s="144"/>
+      <c r="R33" s="144"/>
+      <c r="S33" s="144"/>
+      <c r="T33" s="144"/>
       <c r="U33" s="42"/>
       <c r="V33" s="63"/>
-      <c r="W33" s="142"/>
-      <c r="X33" s="142"/>
-      <c r="Y33" s="142"/>
-      <c r="Z33" s="142"/>
+      <c r="W33" s="144"/>
+      <c r="X33" s="144"/>
+      <c r="Y33" s="144"/>
+      <c r="Z33" s="144"/>
       <c r="AA33" s="42"/>
       <c r="AB33" s="63"/>
-      <c r="AC33" s="142"/>
-      <c r="AD33" s="142"/>
-      <c r="AE33" s="142"/>
-      <c r="AF33" s="142"/>
+      <c r="AC33" s="144"/>
+      <c r="AD33" s="144"/>
+      <c r="AE33" s="144"/>
+      <c r="AF33" s="144"/>
       <c r="AG33" s="42"/>
       <c r="AH33" s="63"/>
-      <c r="AI33" s="142"/>
-      <c r="AJ33" s="142"/>
-      <c r="AK33" s="142"/>
-      <c r="AL33" s="142"/>
+      <c r="AI33" s="144"/>
+      <c r="AJ33" s="144"/>
+      <c r="AK33" s="144"/>
+      <c r="AL33" s="144"/>
       <c r="AM33" s="64"/>
       <c r="AN33" s="104"/>
-      <c r="AO33" s="140"/>
-      <c r="AP33" s="140"/>
-      <c r="AQ33" s="140"/>
-      <c r="AR33" s="140"/>
-      <c r="AS33" s="140"/>
-      <c r="AT33" s="140"/>
-      <c r="AU33" s="140"/>
+      <c r="AO33" s="142"/>
+      <c r="AP33" s="142"/>
+      <c r="AQ33" s="142"/>
+      <c r="AR33" s="142"/>
+      <c r="AS33" s="142"/>
+      <c r="AT33" s="142"/>
+      <c r="AU33" s="142"/>
       <c r="AV33" s="105"/>
     </row>
     <row r="34" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="80"/>
       <c r="B34" s="87"/>
-      <c r="C34" s="74"/>
+      <c r="C34" s="88"/>
       <c r="D34" s="88"/>
       <c r="E34" s="88"/>
       <c r="F34" s="74"/>
@@ -3392,59 +3395,59 @@
       <c r="H34" s="75"/>
       <c r="I34" s="83"/>
       <c r="J34" s="69"/>
-      <c r="K34" s="138" t="s">
+      <c r="K34" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="L34" s="137"/>
-      <c r="M34" s="136"/>
-      <c r="N34" s="137"/>
+      <c r="L34" s="139"/>
+      <c r="M34" s="138"/>
+      <c r="N34" s="139"/>
       <c r="O34" s="42"/>
       <c r="P34" s="63"/>
-      <c r="Q34" s="138" t="s">
+      <c r="Q34" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="R34" s="137"/>
-      <c r="S34" s="136"/>
-      <c r="T34" s="137"/>
+      <c r="R34" s="139"/>
+      <c r="S34" s="138"/>
+      <c r="T34" s="139"/>
       <c r="U34" s="42"/>
       <c r="V34" s="63"/>
-      <c r="W34" s="138" t="s">
+      <c r="W34" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="X34" s="137"/>
-      <c r="Y34" s="136"/>
-      <c r="Z34" s="137"/>
+      <c r="X34" s="139"/>
+      <c r="Y34" s="138"/>
+      <c r="Z34" s="139"/>
       <c r="AA34" s="42"/>
       <c r="AB34" s="63"/>
-      <c r="AC34" s="138" t="s">
+      <c r="AC34" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="AD34" s="137"/>
-      <c r="AE34" s="136"/>
-      <c r="AF34" s="137"/>
+      <c r="AD34" s="139"/>
+      <c r="AE34" s="138"/>
+      <c r="AF34" s="139"/>
       <c r="AG34" s="42"/>
       <c r="AH34" s="63"/>
-      <c r="AI34" s="138" t="s">
+      <c r="AI34" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="AJ34" s="137"/>
-      <c r="AK34" s="136"/>
-      <c r="AL34" s="137"/>
+      <c r="AJ34" s="139"/>
+      <c r="AK34" s="138"/>
+      <c r="AL34" s="139"/>
       <c r="AM34" s="42"/>
       <c r="AN34" s="104"/>
-      <c r="AO34" s="140"/>
-      <c r="AP34" s="140"/>
-      <c r="AQ34" s="140"/>
-      <c r="AR34" s="140"/>
-      <c r="AS34" s="140"/>
-      <c r="AT34" s="140"/>
-      <c r="AU34" s="140"/>
+      <c r="AO34" s="142"/>
+      <c r="AP34" s="142"/>
+      <c r="AQ34" s="142"/>
+      <c r="AR34" s="142"/>
+      <c r="AS34" s="142"/>
+      <c r="AT34" s="142"/>
+      <c r="AU34" s="142"/>
       <c r="AV34" s="105"/>
     </row>
     <row r="35" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="80"/>
       <c r="B35" s="87"/>
-      <c r="C35" s="74"/>
+      <c r="C35" s="88"/>
       <c r="D35" s="88"/>
       <c r="E35" s="88"/>
       <c r="F35" s="74"/>
@@ -3456,55 +3459,55 @@
         <v>32</v>
       </c>
       <c r="L35" s="63"/>
-      <c r="M35" s="136"/>
-      <c r="N35" s="137"/>
+      <c r="M35" s="138"/>
+      <c r="N35" s="139"/>
       <c r="O35" s="42"/>
       <c r="P35" s="63"/>
       <c r="Q35" s="66" t="s">
         <v>32</v>
       </c>
       <c r="R35" s="63"/>
-      <c r="S35" s="136"/>
-      <c r="T35" s="137"/>
+      <c r="S35" s="138"/>
+      <c r="T35" s="139"/>
       <c r="U35" s="42"/>
       <c r="V35" s="63"/>
       <c r="W35" s="66" t="s">
         <v>32</v>
       </c>
       <c r="X35" s="63"/>
-      <c r="Y35" s="136"/>
-      <c r="Z35" s="137"/>
+      <c r="Y35" s="138"/>
+      <c r="Z35" s="139"/>
       <c r="AA35" s="42"/>
       <c r="AB35" s="63"/>
       <c r="AC35" s="66" t="s">
         <v>32</v>
       </c>
       <c r="AD35" s="63"/>
-      <c r="AE35" s="136"/>
-      <c r="AF35" s="137"/>
+      <c r="AE35" s="138"/>
+      <c r="AF35" s="139"/>
       <c r="AG35" s="42"/>
       <c r="AH35" s="63"/>
       <c r="AI35" s="66" t="s">
         <v>32</v>
       </c>
       <c r="AJ35" s="63"/>
-      <c r="AK35" s="136"/>
-      <c r="AL35" s="137"/>
-      <c r="AM35" s="141"/>
+      <c r="AK35" s="138"/>
+      <c r="AL35" s="139"/>
+      <c r="AM35" s="143"/>
       <c r="AN35" s="104"/>
-      <c r="AO35" s="140"/>
-      <c r="AP35" s="140"/>
-      <c r="AQ35" s="140"/>
-      <c r="AR35" s="140"/>
-      <c r="AS35" s="140"/>
-      <c r="AT35" s="140"/>
-      <c r="AU35" s="140"/>
+      <c r="AO35" s="142"/>
+      <c r="AP35" s="142"/>
+      <c r="AQ35" s="142"/>
+      <c r="AR35" s="142"/>
+      <c r="AS35" s="142"/>
+      <c r="AT35" s="142"/>
+      <c r="AU35" s="142"/>
       <c r="AV35" s="105"/>
     </row>
     <row r="36" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="80"/>
       <c r="B36" s="87"/>
-      <c r="C36" s="74"/>
+      <c r="C36" s="88"/>
       <c r="D36" s="88"/>
       <c r="E36" s="88"/>
       <c r="F36" s="74"/>
@@ -3515,56 +3518,56 @@
       <c r="K36" s="46" t="s">
         <v>39</v>
       </c>
-      <c r="L36" s="143"/>
-      <c r="M36" s="144"/>
-      <c r="N36" s="144"/>
+      <c r="L36" s="145"/>
+      <c r="M36" s="146"/>
+      <c r="N36" s="146"/>
       <c r="O36" s="56"/>
       <c r="P36" s="40"/>
       <c r="Q36" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="R36" s="143"/>
-      <c r="S36" s="144"/>
-      <c r="T36" s="144"/>
+      <c r="R36" s="145"/>
+      <c r="S36" s="146"/>
+      <c r="T36" s="146"/>
       <c r="U36" s="39"/>
       <c r="V36" s="40"/>
       <c r="W36" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="X36" s="145"/>
-      <c r="Y36" s="145"/>
-      <c r="Z36" s="145"/>
+      <c r="X36" s="147"/>
+      <c r="Y36" s="147"/>
+      <c r="Z36" s="147"/>
       <c r="AA36" s="39"/>
       <c r="AB36" s="40"/>
       <c r="AC36" s="46" t="s">
         <v>42</v>
       </c>
-      <c r="AD36" s="143"/>
-      <c r="AE36" s="144"/>
-      <c r="AF36" s="144"/>
+      <c r="AD36" s="145"/>
+      <c r="AE36" s="146"/>
+      <c r="AF36" s="146"/>
       <c r="AG36" s="39"/>
       <c r="AH36" s="40"/>
       <c r="AI36" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="AJ36" s="143"/>
-      <c r="AK36" s="144"/>
-      <c r="AL36" s="144"/>
+      <c r="AJ36" s="145"/>
+      <c r="AK36" s="146"/>
+      <c r="AL36" s="146"/>
       <c r="AM36" s="68"/>
       <c r="AN36" s="89"/>
-      <c r="AO36" s="140"/>
-      <c r="AP36" s="140"/>
-      <c r="AQ36" s="140"/>
-      <c r="AR36" s="140"/>
-      <c r="AS36" s="140"/>
-      <c r="AT36" s="140"/>
-      <c r="AU36" s="140"/>
+      <c r="AO36" s="142"/>
+      <c r="AP36" s="142"/>
+      <c r="AQ36" s="142"/>
+      <c r="AR36" s="142"/>
+      <c r="AS36" s="142"/>
+      <c r="AT36" s="142"/>
+      <c r="AU36" s="142"/>
       <c r="AV36" s="105"/>
     </row>
     <row r="37" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="81"/>
       <c r="B37" s="128"/>
-      <c r="C37" s="129"/>
+      <c r="C37" s="89"/>
       <c r="D37" s="89"/>
       <c r="E37" s="89"/>
       <c r="F37" s="129"/>
@@ -3602,19 +3605,19 @@
       <c r="AL37" s="63"/>
       <c r="AM37" s="64"/>
       <c r="AN37" s="89"/>
-      <c r="AO37" s="140"/>
-      <c r="AP37" s="140"/>
-      <c r="AQ37" s="140"/>
-      <c r="AR37" s="140"/>
-      <c r="AS37" s="140"/>
-      <c r="AT37" s="140"/>
-      <c r="AU37" s="140"/>
+      <c r="AO37" s="142"/>
+      <c r="AP37" s="142"/>
+      <c r="AQ37" s="142"/>
+      <c r="AR37" s="142"/>
+      <c r="AS37" s="142"/>
+      <c r="AT37" s="142"/>
+      <c r="AU37" s="142"/>
       <c r="AV37" s="105"/>
     </row>
     <row r="38" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="134"/>
       <c r="B38" s="135"/>
-      <c r="C38" s="132"/>
+      <c r="C38" s="90"/>
       <c r="D38" s="90"/>
       <c r="E38" s="95"/>
       <c r="F38" s="92"/>
@@ -3622,49 +3625,49 @@
       <c r="H38" s="94"/>
       <c r="I38" s="85"/>
       <c r="J38" s="65"/>
-      <c r="K38" s="142"/>
-      <c r="L38" s="142"/>
-      <c r="M38" s="142"/>
-      <c r="N38" s="142"/>
+      <c r="K38" s="144"/>
+      <c r="L38" s="144"/>
+      <c r="M38" s="144"/>
+      <c r="N38" s="144"/>
       <c r="O38" s="42"/>
       <c r="P38" s="63"/>
-      <c r="Q38" s="142"/>
-      <c r="R38" s="142"/>
-      <c r="S38" s="142"/>
-      <c r="T38" s="142"/>
+      <c r="Q38" s="144"/>
+      <c r="R38" s="144"/>
+      <c r="S38" s="144"/>
+      <c r="T38" s="144"/>
       <c r="U38" s="42"/>
       <c r="V38" s="63"/>
-      <c r="W38" s="142"/>
-      <c r="X38" s="142"/>
-      <c r="Y38" s="142"/>
-      <c r="Z38" s="142"/>
+      <c r="W38" s="144"/>
+      <c r="X38" s="144"/>
+      <c r="Y38" s="144"/>
+      <c r="Z38" s="144"/>
       <c r="AA38" s="42"/>
       <c r="AB38" s="63"/>
-      <c r="AC38" s="142"/>
-      <c r="AD38" s="142"/>
-      <c r="AE38" s="142"/>
-      <c r="AF38" s="142"/>
+      <c r="AC38" s="144"/>
+      <c r="AD38" s="144"/>
+      <c r="AE38" s="144"/>
+      <c r="AF38" s="144"/>
       <c r="AG38" s="42"/>
       <c r="AH38" s="63"/>
-      <c r="AI38" s="142"/>
-      <c r="AJ38" s="142"/>
-      <c r="AK38" s="142"/>
-      <c r="AL38" s="142"/>
+      <c r="AI38" s="144"/>
+      <c r="AJ38" s="144"/>
+      <c r="AK38" s="144"/>
+      <c r="AL38" s="144"/>
       <c r="AM38" s="64"/>
       <c r="AN38" s="89"/>
-      <c r="AO38" s="140"/>
-      <c r="AP38" s="140"/>
-      <c r="AQ38" s="140"/>
-      <c r="AR38" s="140"/>
-      <c r="AS38" s="140"/>
-      <c r="AT38" s="140"/>
-      <c r="AU38" s="140"/>
+      <c r="AO38" s="142"/>
+      <c r="AP38" s="142"/>
+      <c r="AQ38" s="142"/>
+      <c r="AR38" s="142"/>
+      <c r="AS38" s="142"/>
+      <c r="AT38" s="142"/>
+      <c r="AU38" s="142"/>
       <c r="AV38" s="105"/>
     </row>
     <row r="39" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="80"/>
       <c r="B39" s="87"/>
-      <c r="C39" s="74"/>
+      <c r="C39" s="88"/>
       <c r="D39" s="88"/>
       <c r="E39" s="88"/>
       <c r="F39" s="74"/>
@@ -3672,49 +3675,49 @@
       <c r="H39" s="75"/>
       <c r="I39" s="83"/>
       <c r="J39" s="61"/>
-      <c r="K39" s="142"/>
-      <c r="L39" s="142"/>
-      <c r="M39" s="142"/>
-      <c r="N39" s="142"/>
+      <c r="K39" s="144"/>
+      <c r="L39" s="144"/>
+      <c r="M39" s="144"/>
+      <c r="N39" s="144"/>
       <c r="O39" s="42"/>
       <c r="P39" s="63"/>
-      <c r="Q39" s="142"/>
-      <c r="R39" s="142"/>
-      <c r="S39" s="142"/>
-      <c r="T39" s="142"/>
+      <c r="Q39" s="144"/>
+      <c r="R39" s="144"/>
+      <c r="S39" s="144"/>
+      <c r="T39" s="144"/>
       <c r="U39" s="42"/>
       <c r="V39" s="63"/>
-      <c r="W39" s="142"/>
-      <c r="X39" s="142"/>
-      <c r="Y39" s="142"/>
-      <c r="Z39" s="142"/>
+      <c r="W39" s="144"/>
+      <c r="X39" s="144"/>
+      <c r="Y39" s="144"/>
+      <c r="Z39" s="144"/>
       <c r="AA39" s="42"/>
       <c r="AB39" s="63"/>
-      <c r="AC39" s="142"/>
-      <c r="AD39" s="142"/>
-      <c r="AE39" s="142"/>
-      <c r="AF39" s="142"/>
+      <c r="AC39" s="144"/>
+      <c r="AD39" s="144"/>
+      <c r="AE39" s="144"/>
+      <c r="AF39" s="144"/>
       <c r="AG39" s="42"/>
       <c r="AH39" s="63"/>
-      <c r="AI39" s="142"/>
-      <c r="AJ39" s="142"/>
-      <c r="AK39" s="142"/>
-      <c r="AL39" s="142"/>
+      <c r="AI39" s="144"/>
+      <c r="AJ39" s="144"/>
+      <c r="AK39" s="144"/>
+      <c r="AL39" s="144"/>
       <c r="AM39" s="64"/>
       <c r="AN39" s="89"/>
-      <c r="AO39" s="140"/>
-      <c r="AP39" s="140"/>
-      <c r="AQ39" s="140"/>
-      <c r="AR39" s="140"/>
-      <c r="AS39" s="140"/>
-      <c r="AT39" s="140"/>
-      <c r="AU39" s="140"/>
+      <c r="AO39" s="142"/>
+      <c r="AP39" s="142"/>
+      <c r="AQ39" s="142"/>
+      <c r="AR39" s="142"/>
+      <c r="AS39" s="142"/>
+      <c r="AT39" s="142"/>
+      <c r="AU39" s="142"/>
       <c r="AV39" s="105"/>
     </row>
     <row r="40" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="80"/>
       <c r="B40" s="87"/>
-      <c r="C40" s="74"/>
+      <c r="C40" s="88"/>
       <c r="D40" s="88"/>
       <c r="E40" s="88"/>
       <c r="F40" s="74"/>
@@ -3722,49 +3725,49 @@
       <c r="H40" s="75"/>
       <c r="I40" s="83"/>
       <c r="J40" s="65"/>
-      <c r="K40" s="142"/>
-      <c r="L40" s="142"/>
-      <c r="M40" s="142"/>
-      <c r="N40" s="142"/>
+      <c r="K40" s="144"/>
+      <c r="L40" s="144"/>
+      <c r="M40" s="144"/>
+      <c r="N40" s="144"/>
       <c r="O40" s="42"/>
       <c r="P40" s="63"/>
-      <c r="Q40" s="142"/>
-      <c r="R40" s="142"/>
-      <c r="S40" s="142"/>
-      <c r="T40" s="142"/>
+      <c r="Q40" s="144"/>
+      <c r="R40" s="144"/>
+      <c r="S40" s="144"/>
+      <c r="T40" s="144"/>
       <c r="U40" s="42"/>
       <c r="V40" s="63"/>
-      <c r="W40" s="142"/>
-      <c r="X40" s="142"/>
-      <c r="Y40" s="142"/>
-      <c r="Z40" s="142"/>
+      <c r="W40" s="144"/>
+      <c r="X40" s="144"/>
+      <c r="Y40" s="144"/>
+      <c r="Z40" s="144"/>
       <c r="AA40" s="42"/>
       <c r="AB40" s="63"/>
-      <c r="AC40" s="142"/>
-      <c r="AD40" s="142"/>
-      <c r="AE40" s="142"/>
-      <c r="AF40" s="142"/>
+      <c r="AC40" s="144"/>
+      <c r="AD40" s="144"/>
+      <c r="AE40" s="144"/>
+      <c r="AF40" s="144"/>
       <c r="AG40" s="42"/>
       <c r="AH40" s="63"/>
-      <c r="AI40" s="142"/>
-      <c r="AJ40" s="142"/>
-      <c r="AK40" s="142"/>
-      <c r="AL40" s="142"/>
+      <c r="AI40" s="144"/>
+      <c r="AJ40" s="144"/>
+      <c r="AK40" s="144"/>
+      <c r="AL40" s="144"/>
       <c r="AM40" s="64"/>
       <c r="AN40" s="89"/>
-      <c r="AO40" s="140"/>
-      <c r="AP40" s="140"/>
-      <c r="AQ40" s="140"/>
-      <c r="AR40" s="140"/>
-      <c r="AS40" s="140"/>
-      <c r="AT40" s="140"/>
-      <c r="AU40" s="140"/>
+      <c r="AO40" s="142"/>
+      <c r="AP40" s="142"/>
+      <c r="AQ40" s="142"/>
+      <c r="AR40" s="142"/>
+      <c r="AS40" s="142"/>
+      <c r="AT40" s="142"/>
+      <c r="AU40" s="142"/>
       <c r="AV40" s="105"/>
     </row>
     <row r="41" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="80"/>
       <c r="B41" s="87"/>
-      <c r="C41" s="74"/>
+      <c r="C41" s="88"/>
       <c r="D41" s="88"/>
       <c r="E41" s="88"/>
       <c r="F41" s="74"/>
@@ -3772,49 +3775,49 @@
       <c r="H41" s="75"/>
       <c r="I41" s="83"/>
       <c r="J41" s="65"/>
-      <c r="K41" s="142"/>
-      <c r="L41" s="142"/>
-      <c r="M41" s="142"/>
-      <c r="N41" s="142"/>
+      <c r="K41" s="144"/>
+      <c r="L41" s="144"/>
+      <c r="M41" s="144"/>
+      <c r="N41" s="144"/>
       <c r="O41" s="42"/>
       <c r="P41" s="63"/>
-      <c r="Q41" s="142"/>
-      <c r="R41" s="142"/>
-      <c r="S41" s="142"/>
-      <c r="T41" s="142"/>
+      <c r="Q41" s="144"/>
+      <c r="R41" s="144"/>
+      <c r="S41" s="144"/>
+      <c r="T41" s="144"/>
       <c r="U41" s="42"/>
       <c r="V41" s="63"/>
-      <c r="W41" s="142"/>
-      <c r="X41" s="142"/>
-      <c r="Y41" s="142"/>
-      <c r="Z41" s="142"/>
+      <c r="W41" s="144"/>
+      <c r="X41" s="144"/>
+      <c r="Y41" s="144"/>
+      <c r="Z41" s="144"/>
       <c r="AA41" s="42"/>
       <c r="AB41" s="63"/>
-      <c r="AC41" s="142"/>
-      <c r="AD41" s="142"/>
-      <c r="AE41" s="142"/>
-      <c r="AF41" s="142"/>
+      <c r="AC41" s="144"/>
+      <c r="AD41" s="144"/>
+      <c r="AE41" s="144"/>
+      <c r="AF41" s="144"/>
       <c r="AG41" s="42"/>
       <c r="AH41" s="63"/>
-      <c r="AI41" s="142"/>
-      <c r="AJ41" s="142"/>
-      <c r="AK41" s="142"/>
-      <c r="AL41" s="142"/>
+      <c r="AI41" s="144"/>
+      <c r="AJ41" s="144"/>
+      <c r="AK41" s="144"/>
+      <c r="AL41" s="144"/>
       <c r="AM41" s="64"/>
       <c r="AN41" s="89"/>
-      <c r="AO41" s="140"/>
-      <c r="AP41" s="140"/>
-      <c r="AQ41" s="140"/>
-      <c r="AR41" s="140"/>
-      <c r="AS41" s="140"/>
-      <c r="AT41" s="140"/>
-      <c r="AU41" s="140"/>
+      <c r="AO41" s="142"/>
+      <c r="AP41" s="142"/>
+      <c r="AQ41" s="142"/>
+      <c r="AR41" s="142"/>
+      <c r="AS41" s="142"/>
+      <c r="AT41" s="142"/>
+      <c r="AU41" s="142"/>
       <c r="AV41" s="105"/>
     </row>
     <row r="42" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="80"/>
       <c r="B42" s="87"/>
-      <c r="C42" s="74"/>
+      <c r="C42" s="88"/>
       <c r="D42" s="88"/>
       <c r="E42" s="88"/>
       <c r="F42" s="74"/>
@@ -3822,49 +3825,49 @@
       <c r="H42" s="75"/>
       <c r="I42" s="83"/>
       <c r="J42" s="65"/>
-      <c r="K42" s="142"/>
-      <c r="L42" s="142"/>
-      <c r="M42" s="142"/>
-      <c r="N42" s="142"/>
+      <c r="K42" s="144"/>
+      <c r="L42" s="144"/>
+      <c r="M42" s="144"/>
+      <c r="N42" s="144"/>
       <c r="O42" s="42"/>
       <c r="P42" s="63"/>
-      <c r="Q42" s="142"/>
-      <c r="R42" s="142"/>
-      <c r="S42" s="142"/>
-      <c r="T42" s="142"/>
+      <c r="Q42" s="144"/>
+      <c r="R42" s="144"/>
+      <c r="S42" s="144"/>
+      <c r="T42" s="144"/>
       <c r="U42" s="42"/>
       <c r="V42" s="63"/>
-      <c r="W42" s="142"/>
-      <c r="X42" s="142"/>
-      <c r="Y42" s="142"/>
-      <c r="Z42" s="142"/>
+      <c r="W42" s="144"/>
+      <c r="X42" s="144"/>
+      <c r="Y42" s="144"/>
+      <c r="Z42" s="144"/>
       <c r="AA42" s="42"/>
       <c r="AB42" s="63"/>
-      <c r="AC42" s="142"/>
-      <c r="AD42" s="142"/>
-      <c r="AE42" s="142"/>
-      <c r="AF42" s="142"/>
+      <c r="AC42" s="144"/>
+      <c r="AD42" s="144"/>
+      <c r="AE42" s="144"/>
+      <c r="AF42" s="144"/>
       <c r="AG42" s="42"/>
       <c r="AH42" s="63"/>
-      <c r="AI42" s="142"/>
-      <c r="AJ42" s="142"/>
-      <c r="AK42" s="142"/>
-      <c r="AL42" s="142"/>
+      <c r="AI42" s="144"/>
+      <c r="AJ42" s="144"/>
+      <c r="AK42" s="144"/>
+      <c r="AL42" s="144"/>
       <c r="AM42" s="64"/>
       <c r="AN42" s="89"/>
-      <c r="AO42" s="140"/>
-      <c r="AP42" s="140"/>
-      <c r="AQ42" s="140"/>
-      <c r="AR42" s="140"/>
-      <c r="AS42" s="140"/>
-      <c r="AT42" s="140"/>
-      <c r="AU42" s="140"/>
+      <c r="AO42" s="142"/>
+      <c r="AP42" s="142"/>
+      <c r="AQ42" s="142"/>
+      <c r="AR42" s="142"/>
+      <c r="AS42" s="142"/>
+      <c r="AT42" s="142"/>
+      <c r="AU42" s="142"/>
       <c r="AV42" s="105"/>
     </row>
     <row r="43" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="80"/>
       <c r="B43" s="87"/>
-      <c r="C43" s="74"/>
+      <c r="C43" s="88"/>
       <c r="D43" s="88"/>
       <c r="E43" s="88"/>
       <c r="F43" s="74"/>
@@ -3872,49 +3875,49 @@
       <c r="H43" s="75"/>
       <c r="I43" s="83"/>
       <c r="J43" s="61"/>
-      <c r="K43" s="142"/>
-      <c r="L43" s="142"/>
-      <c r="M43" s="142"/>
-      <c r="N43" s="142"/>
+      <c r="K43" s="144"/>
+      <c r="L43" s="144"/>
+      <c r="M43" s="144"/>
+      <c r="N43" s="144"/>
       <c r="O43" s="42"/>
       <c r="P43" s="63"/>
-      <c r="Q43" s="142"/>
-      <c r="R43" s="142"/>
-      <c r="S43" s="142"/>
-      <c r="T43" s="142"/>
+      <c r="Q43" s="144"/>
+      <c r="R43" s="144"/>
+      <c r="S43" s="144"/>
+      <c r="T43" s="144"/>
       <c r="U43" s="42"/>
       <c r="V43" s="63"/>
-      <c r="W43" s="142"/>
-      <c r="X43" s="142"/>
-      <c r="Y43" s="142"/>
-      <c r="Z43" s="142"/>
+      <c r="W43" s="144"/>
+      <c r="X43" s="144"/>
+      <c r="Y43" s="144"/>
+      <c r="Z43" s="144"/>
       <c r="AA43" s="42"/>
       <c r="AB43" s="63"/>
-      <c r="AC43" s="142"/>
-      <c r="AD43" s="142"/>
-      <c r="AE43" s="142"/>
-      <c r="AF43" s="142"/>
+      <c r="AC43" s="144"/>
+      <c r="AD43" s="144"/>
+      <c r="AE43" s="144"/>
+      <c r="AF43" s="144"/>
       <c r="AG43" s="42"/>
       <c r="AH43" s="63"/>
-      <c r="AI43" s="142"/>
-      <c r="AJ43" s="142"/>
-      <c r="AK43" s="142"/>
-      <c r="AL43" s="142"/>
+      <c r="AI43" s="144"/>
+      <c r="AJ43" s="144"/>
+      <c r="AK43" s="144"/>
+      <c r="AL43" s="144"/>
       <c r="AM43" s="64"/>
       <c r="AN43" s="89"/>
-      <c r="AO43" s="140"/>
-      <c r="AP43" s="140"/>
-      <c r="AQ43" s="140"/>
-      <c r="AR43" s="140"/>
-      <c r="AS43" s="140"/>
-      <c r="AT43" s="140"/>
-      <c r="AU43" s="140"/>
+      <c r="AO43" s="142"/>
+      <c r="AP43" s="142"/>
+      <c r="AQ43" s="142"/>
+      <c r="AR43" s="142"/>
+      <c r="AS43" s="142"/>
+      <c r="AT43" s="142"/>
+      <c r="AU43" s="142"/>
       <c r="AV43" s="105"/>
     </row>
     <row r="44" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="80"/>
       <c r="B44" s="87"/>
-      <c r="C44" s="74"/>
+      <c r="C44" s="88"/>
       <c r="D44" s="88"/>
       <c r="E44" s="88"/>
       <c r="F44" s="74"/>
@@ -3922,59 +3925,59 @@
       <c r="H44" s="75"/>
       <c r="I44" s="83"/>
       <c r="J44" s="69"/>
-      <c r="K44" s="138" t="s">
+      <c r="K44" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="L44" s="137"/>
-      <c r="M44" s="136"/>
-      <c r="N44" s="137"/>
+      <c r="L44" s="139"/>
+      <c r="M44" s="138"/>
+      <c r="N44" s="139"/>
       <c r="O44" s="42"/>
       <c r="P44" s="63"/>
-      <c r="Q44" s="138" t="s">
+      <c r="Q44" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="R44" s="137"/>
-      <c r="S44" s="136"/>
-      <c r="T44" s="137"/>
+      <c r="R44" s="139"/>
+      <c r="S44" s="138"/>
+      <c r="T44" s="139"/>
       <c r="U44" s="42"/>
       <c r="V44" s="63"/>
-      <c r="W44" s="138" t="s">
+      <c r="W44" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="X44" s="137"/>
-      <c r="Y44" s="136"/>
-      <c r="Z44" s="137"/>
+      <c r="X44" s="139"/>
+      <c r="Y44" s="138"/>
+      <c r="Z44" s="139"/>
       <c r="AA44" s="42"/>
       <c r="AB44" s="63"/>
-      <c r="AC44" s="138" t="s">
+      <c r="AC44" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="AD44" s="137"/>
-      <c r="AE44" s="136"/>
-      <c r="AF44" s="137"/>
+      <c r="AD44" s="139"/>
+      <c r="AE44" s="138"/>
+      <c r="AF44" s="139"/>
       <c r="AG44" s="42"/>
       <c r="AH44" s="63"/>
-      <c r="AI44" s="138" t="s">
+      <c r="AI44" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="AJ44" s="137"/>
-      <c r="AK44" s="136"/>
-      <c r="AL44" s="137"/>
+      <c r="AJ44" s="139"/>
+      <c r="AK44" s="138"/>
+      <c r="AL44" s="139"/>
       <c r="AM44" s="42"/>
       <c r="AN44" s="89"/>
-      <c r="AO44" s="140"/>
-      <c r="AP44" s="140"/>
-      <c r="AQ44" s="140"/>
-      <c r="AR44" s="140"/>
-      <c r="AS44" s="140"/>
-      <c r="AT44" s="140"/>
-      <c r="AU44" s="140"/>
+      <c r="AO44" s="142"/>
+      <c r="AP44" s="142"/>
+      <c r="AQ44" s="142"/>
+      <c r="AR44" s="142"/>
+      <c r="AS44" s="142"/>
+      <c r="AT44" s="142"/>
+      <c r="AU44" s="142"/>
       <c r="AV44" s="105"/>
     </row>
     <row r="45" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="80"/>
       <c r="B45" s="87"/>
-      <c r="C45" s="74"/>
+      <c r="C45" s="88"/>
       <c r="D45" s="88"/>
       <c r="E45" s="88"/>
       <c r="F45" s="74"/>
@@ -3986,55 +3989,55 @@
         <v>32</v>
       </c>
       <c r="L45" s="63"/>
-      <c r="M45" s="136"/>
-      <c r="N45" s="137"/>
+      <c r="M45" s="138"/>
+      <c r="N45" s="139"/>
       <c r="O45" s="42"/>
       <c r="P45" s="63"/>
       <c r="Q45" s="66" t="s">
         <v>32</v>
       </c>
       <c r="R45" s="63"/>
-      <c r="S45" s="136"/>
-      <c r="T45" s="137"/>
+      <c r="S45" s="138"/>
+      <c r="T45" s="139"/>
       <c r="U45" s="42"/>
       <c r="V45" s="63"/>
       <c r="W45" s="66" t="s">
         <v>32</v>
       </c>
       <c r="X45" s="63"/>
-      <c r="Y45" s="136"/>
-      <c r="Z45" s="137"/>
+      <c r="Y45" s="138"/>
+      <c r="Z45" s="139"/>
       <c r="AA45" s="42"/>
       <c r="AB45" s="63"/>
       <c r="AC45" s="66" t="s">
         <v>32</v>
       </c>
       <c r="AD45" s="63"/>
-      <c r="AE45" s="136"/>
-      <c r="AF45" s="137"/>
+      <c r="AE45" s="138"/>
+      <c r="AF45" s="139"/>
       <c r="AG45" s="42"/>
       <c r="AH45" s="63"/>
       <c r="AI45" s="66" t="s">
         <v>32</v>
       </c>
       <c r="AJ45" s="63"/>
-      <c r="AK45" s="136"/>
-      <c r="AL45" s="137"/>
-      <c r="AM45" s="141"/>
+      <c r="AK45" s="138"/>
+      <c r="AL45" s="139"/>
+      <c r="AM45" s="143"/>
       <c r="AN45" s="89"/>
-      <c r="AO45" s="140"/>
-      <c r="AP45" s="140"/>
-      <c r="AQ45" s="140"/>
-      <c r="AR45" s="140"/>
-      <c r="AS45" s="140"/>
-      <c r="AT45" s="140"/>
-      <c r="AU45" s="140"/>
+      <c r="AO45" s="142"/>
+      <c r="AP45" s="142"/>
+      <c r="AQ45" s="142"/>
+      <c r="AR45" s="142"/>
+      <c r="AS45" s="142"/>
+      <c r="AT45" s="142"/>
+      <c r="AU45" s="142"/>
       <c r="AV45" s="105"/>
     </row>
     <row r="46" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="80"/>
       <c r="B46" s="87"/>
-      <c r="C46" s="74"/>
+      <c r="C46" s="88"/>
       <c r="D46" s="88"/>
       <c r="E46" s="88"/>
       <c r="F46" s="74"/>
@@ -4045,41 +4048,41 @@
       <c r="K46" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="L46" s="145"/>
-      <c r="M46" s="145"/>
-      <c r="N46" s="145"/>
+      <c r="L46" s="147"/>
+      <c r="M46" s="147"/>
+      <c r="N46" s="147"/>
       <c r="O46" s="39"/>
       <c r="P46" s="40"/>
       <c r="Q46" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="R46" s="143"/>
-      <c r="S46" s="144"/>
-      <c r="T46" s="144"/>
+      <c r="R46" s="145"/>
+      <c r="S46" s="146"/>
+      <c r="T46" s="146"/>
       <c r="U46" s="39"/>
       <c r="V46" s="40"/>
       <c r="W46" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="X46" s="145"/>
-      <c r="Y46" s="145"/>
-      <c r="Z46" s="145"/>
+      <c r="X46" s="147"/>
+      <c r="Y46" s="147"/>
+      <c r="Z46" s="147"/>
       <c r="AA46" s="39"/>
       <c r="AB46" s="40"/>
       <c r="AC46" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="AD46" s="143"/>
-      <c r="AE46" s="144"/>
-      <c r="AF46" s="144"/>
+      <c r="AD46" s="145"/>
+      <c r="AE46" s="146"/>
+      <c r="AF46" s="146"/>
       <c r="AG46" s="39"/>
       <c r="AH46" s="40"/>
       <c r="AI46" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="AJ46" s="143"/>
-      <c r="AK46" s="144"/>
-      <c r="AL46" s="144"/>
+      <c r="AJ46" s="145"/>
+      <c r="AK46" s="146"/>
+      <c r="AL46" s="146"/>
       <c r="AM46" s="39"/>
       <c r="AN46" s="106"/>
       <c r="AO46" s="106"/>
@@ -4094,7 +4097,7 @@
     <row r="47" spans="1:48" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="81"/>
       <c r="B47" s="128"/>
-      <c r="C47" s="129"/>
+      <c r="C47" s="89"/>
       <c r="D47" s="89"/>
       <c r="E47" s="96"/>
       <c r="F47" s="91"/>
@@ -4144,7 +4147,7 @@
     <row r="48" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="82"/>
       <c r="B48" s="131"/>
-      <c r="C48" s="132"/>
+      <c r="C48" s="90"/>
       <c r="D48" s="90"/>
       <c r="E48" s="97"/>
       <c r="F48" s="92"/>
@@ -4152,34 +4155,34 @@
       <c r="H48" s="94"/>
       <c r="I48" s="85"/>
       <c r="J48" s="65"/>
-      <c r="K48" s="142"/>
-      <c r="L48" s="142"/>
-      <c r="M48" s="142"/>
-      <c r="N48" s="142"/>
+      <c r="K48" s="144"/>
+      <c r="L48" s="144"/>
+      <c r="M48" s="144"/>
+      <c r="N48" s="144"/>
       <c r="O48" s="42"/>
       <c r="P48" s="63"/>
-      <c r="Q48" s="142"/>
-      <c r="R48" s="142"/>
-      <c r="S48" s="142"/>
-      <c r="T48" s="142"/>
+      <c r="Q48" s="144"/>
+      <c r="R48" s="144"/>
+      <c r="S48" s="144"/>
+      <c r="T48" s="144"/>
       <c r="U48" s="42"/>
       <c r="V48" s="63"/>
-      <c r="W48" s="142"/>
-      <c r="X48" s="142"/>
-      <c r="Y48" s="142"/>
-      <c r="Z48" s="142"/>
+      <c r="W48" s="144"/>
+      <c r="X48" s="144"/>
+      <c r="Y48" s="144"/>
+      <c r="Z48" s="144"/>
       <c r="AA48" s="42"/>
       <c r="AB48" s="63"/>
-      <c r="AC48" s="142"/>
-      <c r="AD48" s="142"/>
-      <c r="AE48" s="142"/>
-      <c r="AF48" s="142"/>
+      <c r="AC48" s="144"/>
+      <c r="AD48" s="144"/>
+      <c r="AE48" s="144"/>
+      <c r="AF48" s="144"/>
       <c r="AG48" s="42"/>
       <c r="AH48" s="63"/>
-      <c r="AI48" s="142"/>
-      <c r="AJ48" s="142"/>
-      <c r="AK48" s="142"/>
-      <c r="AL48" s="142"/>
+      <c r="AI48" s="144"/>
+      <c r="AJ48" s="144"/>
+      <c r="AK48" s="144"/>
+      <c r="AL48" s="144"/>
       <c r="AM48" s="64"/>
       <c r="AN48" s="106"/>
       <c r="AO48" s="106"/>
@@ -4194,7 +4197,7 @@
     <row r="49" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="80"/>
       <c r="B49" s="87"/>
-      <c r="C49" s="74"/>
+      <c r="C49" s="88"/>
       <c r="D49" s="88"/>
       <c r="E49" s="88"/>
       <c r="F49" s="74"/>
@@ -4202,34 +4205,34 @@
       <c r="H49" s="75"/>
       <c r="I49" s="83"/>
       <c r="J49" s="61"/>
-      <c r="K49" s="142"/>
-      <c r="L49" s="142"/>
-      <c r="M49" s="142"/>
-      <c r="N49" s="142"/>
+      <c r="K49" s="144"/>
+      <c r="L49" s="144"/>
+      <c r="M49" s="144"/>
+      <c r="N49" s="144"/>
       <c r="O49" s="42"/>
       <c r="P49" s="63"/>
-      <c r="Q49" s="142"/>
-      <c r="R49" s="142"/>
-      <c r="S49" s="142"/>
-      <c r="T49" s="142"/>
+      <c r="Q49" s="144"/>
+      <c r="R49" s="144"/>
+      <c r="S49" s="144"/>
+      <c r="T49" s="144"/>
       <c r="U49" s="42"/>
       <c r="V49" s="63"/>
-      <c r="W49" s="142"/>
-      <c r="X49" s="142"/>
-      <c r="Y49" s="142"/>
-      <c r="Z49" s="142"/>
+      <c r="W49" s="144"/>
+      <c r="X49" s="144"/>
+      <c r="Y49" s="144"/>
+      <c r="Z49" s="144"/>
       <c r="AA49" s="42"/>
       <c r="AB49" s="63"/>
-      <c r="AC49" s="142"/>
-      <c r="AD49" s="142"/>
-      <c r="AE49" s="142"/>
-      <c r="AF49" s="142"/>
+      <c r="AC49" s="144"/>
+      <c r="AD49" s="144"/>
+      <c r="AE49" s="144"/>
+      <c r="AF49" s="144"/>
       <c r="AG49" s="42"/>
       <c r="AH49" s="63"/>
-      <c r="AI49" s="142"/>
-      <c r="AJ49" s="142"/>
-      <c r="AK49" s="142"/>
-      <c r="AL49" s="142"/>
+      <c r="AI49" s="144"/>
+      <c r="AJ49" s="144"/>
+      <c r="AK49" s="144"/>
+      <c r="AL49" s="144"/>
       <c r="AM49" s="64"/>
       <c r="AN49" s="106"/>
       <c r="AO49" s="106"/>
@@ -4244,7 +4247,7 @@
     <row r="50" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="80"/>
       <c r="B50" s="87"/>
-      <c r="C50" s="74"/>
+      <c r="C50" s="88"/>
       <c r="D50" s="88"/>
       <c r="E50" s="88"/>
       <c r="F50" s="74"/>
@@ -4252,38 +4255,38 @@
       <c r="H50" s="75"/>
       <c r="I50" s="83"/>
       <c r="J50" s="65"/>
-      <c r="K50" s="142"/>
-      <c r="L50" s="142"/>
-      <c r="M50" s="142"/>
-      <c r="N50" s="142"/>
+      <c r="K50" s="144"/>
+      <c r="L50" s="144"/>
+      <c r="M50" s="144"/>
+      <c r="N50" s="144"/>
       <c r="O50" s="42"/>
       <c r="P50" s="63"/>
-      <c r="Q50" s="142"/>
-      <c r="R50" s="142"/>
-      <c r="S50" s="142"/>
-      <c r="T50" s="142"/>
+      <c r="Q50" s="144"/>
+      <c r="R50" s="144"/>
+      <c r="S50" s="144"/>
+      <c r="T50" s="144"/>
       <c r="U50" s="42"/>
       <c r="V50" s="63"/>
-      <c r="W50" s="142"/>
-      <c r="X50" s="142"/>
-      <c r="Y50" s="142"/>
-      <c r="Z50" s="142"/>
+      <c r="W50" s="144"/>
+      <c r="X50" s="144"/>
+      <c r="Y50" s="144"/>
+      <c r="Z50" s="144"/>
       <c r="AA50" s="42"/>
       <c r="AB50" s="63"/>
-      <c r="AC50" s="142"/>
-      <c r="AD50" s="142"/>
-      <c r="AE50" s="142"/>
-      <c r="AF50" s="142"/>
+      <c r="AC50" s="144"/>
+      <c r="AD50" s="144"/>
+      <c r="AE50" s="144"/>
+      <c r="AF50" s="144"/>
       <c r="AG50" s="42"/>
       <c r="AH50" s="63"/>
-      <c r="AI50" s="142"/>
-      <c r="AJ50" s="142"/>
-      <c r="AK50" s="142"/>
-      <c r="AL50" s="142"/>
+      <c r="AI50" s="144"/>
+      <c r="AJ50" s="144"/>
+      <c r="AK50" s="144"/>
+      <c r="AL50" s="144"/>
       <c r="AM50" s="64"/>
       <c r="AN50" s="113"/>
       <c r="AO50" s="114"/>
-      <c r="AP50" s="178"/>
+      <c r="AP50" s="136"/>
       <c r="AQ50" s="114"/>
       <c r="AR50" s="114"/>
       <c r="AS50" s="114"/>
@@ -4294,7 +4297,7 @@
     <row r="51" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="80"/>
       <c r="B51" s="87"/>
-      <c r="C51" s="74"/>
+      <c r="C51" s="88"/>
       <c r="D51" s="88"/>
       <c r="E51" s="88"/>
       <c r="F51" s="74"/>
@@ -4302,38 +4305,38 @@
       <c r="H51" s="75"/>
       <c r="I51" s="83"/>
       <c r="J51" s="65"/>
-      <c r="K51" s="142"/>
-      <c r="L51" s="142"/>
-      <c r="M51" s="142"/>
-      <c r="N51" s="142"/>
+      <c r="K51" s="144"/>
+      <c r="L51" s="144"/>
+      <c r="M51" s="144"/>
+      <c r="N51" s="144"/>
       <c r="O51" s="42"/>
       <c r="P51" s="63"/>
-      <c r="Q51" s="142"/>
-      <c r="R51" s="142"/>
-      <c r="S51" s="142"/>
-      <c r="T51" s="142"/>
+      <c r="Q51" s="144"/>
+      <c r="R51" s="144"/>
+      <c r="S51" s="144"/>
+      <c r="T51" s="144"/>
       <c r="U51" s="42"/>
       <c r="V51" s="63"/>
-      <c r="W51" s="142"/>
-      <c r="X51" s="142"/>
-      <c r="Y51" s="142"/>
-      <c r="Z51" s="142"/>
+      <c r="W51" s="144"/>
+      <c r="X51" s="144"/>
+      <c r="Y51" s="144"/>
+      <c r="Z51" s="144"/>
       <c r="AA51" s="42"/>
       <c r="AB51" s="63"/>
-      <c r="AC51" s="142"/>
-      <c r="AD51" s="142"/>
-      <c r="AE51" s="142"/>
-      <c r="AF51" s="142"/>
+      <c r="AC51" s="144"/>
+      <c r="AD51" s="144"/>
+      <c r="AE51" s="144"/>
+      <c r="AF51" s="144"/>
       <c r="AG51" s="42"/>
       <c r="AH51" s="63"/>
-      <c r="AI51" s="142"/>
-      <c r="AJ51" s="142"/>
-      <c r="AK51" s="142"/>
-      <c r="AL51" s="142"/>
+      <c r="AI51" s="144"/>
+      <c r="AJ51" s="144"/>
+      <c r="AK51" s="144"/>
+      <c r="AL51" s="144"/>
       <c r="AM51" s="64"/>
       <c r="AN51" s="113"/>
       <c r="AO51" s="114"/>
-      <c r="AP51" s="178"/>
+      <c r="AP51" s="136"/>
       <c r="AQ51" s="114"/>
       <c r="AR51" s="114"/>
       <c r="AS51" s="114"/>
@@ -4344,7 +4347,7 @@
     <row r="52" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="80"/>
       <c r="B52" s="87"/>
-      <c r="C52" s="74"/>
+      <c r="C52" s="88"/>
       <c r="D52" s="88"/>
       <c r="E52" s="88"/>
       <c r="F52" s="74"/>
@@ -4352,38 +4355,38 @@
       <c r="H52" s="75"/>
       <c r="I52" s="83"/>
       <c r="J52" s="65"/>
-      <c r="K52" s="142"/>
-      <c r="L52" s="142"/>
-      <c r="M52" s="142"/>
-      <c r="N52" s="142"/>
+      <c r="K52" s="144"/>
+      <c r="L52" s="144"/>
+      <c r="M52" s="144"/>
+      <c r="N52" s="144"/>
       <c r="O52" s="42"/>
       <c r="P52" s="63"/>
-      <c r="Q52" s="142"/>
-      <c r="R52" s="142"/>
-      <c r="S52" s="142"/>
-      <c r="T52" s="142"/>
+      <c r="Q52" s="144"/>
+      <c r="R52" s="144"/>
+      <c r="S52" s="144"/>
+      <c r="T52" s="144"/>
       <c r="U52" s="42"/>
       <c r="V52" s="63"/>
-      <c r="W52" s="142"/>
-      <c r="X52" s="142"/>
-      <c r="Y52" s="142"/>
-      <c r="Z52" s="142"/>
+      <c r="W52" s="144"/>
+      <c r="X52" s="144"/>
+      <c r="Y52" s="144"/>
+      <c r="Z52" s="144"/>
       <c r="AA52" s="42"/>
       <c r="AB52" s="63"/>
-      <c r="AC52" s="142"/>
-      <c r="AD52" s="142"/>
-      <c r="AE52" s="142"/>
-      <c r="AF52" s="142"/>
+      <c r="AC52" s="144"/>
+      <c r="AD52" s="144"/>
+      <c r="AE52" s="144"/>
+      <c r="AF52" s="144"/>
       <c r="AG52" s="42"/>
       <c r="AH52" s="63"/>
-      <c r="AI52" s="142"/>
-      <c r="AJ52" s="142"/>
-      <c r="AK52" s="142"/>
-      <c r="AL52" s="142"/>
+      <c r="AI52" s="144"/>
+      <c r="AJ52" s="144"/>
+      <c r="AK52" s="144"/>
+      <c r="AL52" s="144"/>
       <c r="AM52" s="64"/>
       <c r="AN52" s="113"/>
       <c r="AO52" s="114"/>
-      <c r="AP52" s="178"/>
+      <c r="AP52" s="136"/>
       <c r="AQ52" s="114"/>
       <c r="AR52" s="114"/>
       <c r="AS52" s="114"/>
@@ -4394,7 +4397,7 @@
     <row r="53" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="80"/>
       <c r="B53" s="87"/>
-      <c r="C53" s="74"/>
+      <c r="C53" s="88"/>
       <c r="D53" s="88"/>
       <c r="E53" s="88"/>
       <c r="F53" s="74"/>
@@ -4402,38 +4405,38 @@
       <c r="H53" s="75"/>
       <c r="I53" s="83"/>
       <c r="J53" s="61"/>
-      <c r="K53" s="142"/>
-      <c r="L53" s="142"/>
-      <c r="M53" s="142"/>
-      <c r="N53" s="142"/>
+      <c r="K53" s="144"/>
+      <c r="L53" s="144"/>
+      <c r="M53" s="144"/>
+      <c r="N53" s="144"/>
       <c r="O53" s="42"/>
       <c r="P53" s="63"/>
-      <c r="Q53" s="142"/>
-      <c r="R53" s="142"/>
-      <c r="S53" s="142"/>
-      <c r="T53" s="142"/>
+      <c r="Q53" s="144"/>
+      <c r="R53" s="144"/>
+      <c r="S53" s="144"/>
+      <c r="T53" s="144"/>
       <c r="U53" s="42"/>
       <c r="V53" s="63"/>
-      <c r="W53" s="142"/>
-      <c r="X53" s="142"/>
-      <c r="Y53" s="142"/>
-      <c r="Z53" s="142"/>
+      <c r="W53" s="144"/>
+      <c r="X53" s="144"/>
+      <c r="Y53" s="144"/>
+      <c r="Z53" s="144"/>
       <c r="AA53" s="42"/>
       <c r="AB53" s="63"/>
-      <c r="AC53" s="142"/>
-      <c r="AD53" s="142"/>
-      <c r="AE53" s="142"/>
-      <c r="AF53" s="142"/>
+      <c r="AC53" s="144"/>
+      <c r="AD53" s="144"/>
+      <c r="AE53" s="144"/>
+      <c r="AF53" s="144"/>
       <c r="AG53" s="42"/>
       <c r="AH53" s="63"/>
-      <c r="AI53" s="142"/>
-      <c r="AJ53" s="142"/>
-      <c r="AK53" s="142"/>
-      <c r="AL53" s="142"/>
+      <c r="AI53" s="144"/>
+      <c r="AJ53" s="144"/>
+      <c r="AK53" s="144"/>
+      <c r="AL53" s="144"/>
       <c r="AM53" s="63"/>
       <c r="AN53" s="116"/>
       <c r="AO53" s="110"/>
-      <c r="AP53" s="179"/>
+      <c r="AP53" s="137"/>
       <c r="AQ53" s="110"/>
       <c r="AR53" s="110"/>
       <c r="AS53" s="110"/>
@@ -4444,7 +4447,7 @@
     <row r="54" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="80"/>
       <c r="B54" s="87"/>
-      <c r="C54" s="74"/>
+      <c r="C54" s="88"/>
       <c r="D54" s="88"/>
       <c r="E54" s="88"/>
       <c r="F54" s="74"/>
@@ -4452,48 +4455,48 @@
       <c r="H54" s="75"/>
       <c r="I54" s="83"/>
       <c r="J54" s="69"/>
-      <c r="K54" s="138" t="s">
+      <c r="K54" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="L54" s="137"/>
-      <c r="M54" s="136"/>
-      <c r="N54" s="137"/>
+      <c r="L54" s="139"/>
+      <c r="M54" s="138"/>
+      <c r="N54" s="139"/>
       <c r="O54" s="42"/>
       <c r="P54" s="63"/>
-      <c r="Q54" s="138" t="s">
+      <c r="Q54" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="R54" s="137"/>
-      <c r="S54" s="136"/>
-      <c r="T54" s="137"/>
+      <c r="R54" s="139"/>
+      <c r="S54" s="138"/>
+      <c r="T54" s="139"/>
       <c r="U54" s="42"/>
       <c r="V54" s="63"/>
-      <c r="W54" s="138" t="s">
+      <c r="W54" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="X54" s="137"/>
-      <c r="Y54" s="136"/>
-      <c r="Z54" s="137"/>
+      <c r="X54" s="139"/>
+      <c r="Y54" s="138"/>
+      <c r="Z54" s="139"/>
       <c r="AA54" s="42"/>
       <c r="AB54" s="63"/>
-      <c r="AC54" s="138" t="s">
+      <c r="AC54" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="AD54" s="137"/>
-      <c r="AE54" s="136"/>
-      <c r="AF54" s="137"/>
+      <c r="AD54" s="139"/>
+      <c r="AE54" s="138"/>
+      <c r="AF54" s="139"/>
       <c r="AG54" s="42"/>
       <c r="AH54" s="63"/>
-      <c r="AI54" s="138" t="s">
+      <c r="AI54" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="AJ54" s="137"/>
-      <c r="AK54" s="136"/>
-      <c r="AL54" s="137"/>
+      <c r="AJ54" s="139"/>
+      <c r="AK54" s="138"/>
+      <c r="AL54" s="139"/>
       <c r="AM54" s="63"/>
       <c r="AN54" s="108"/>
       <c r="AO54" s="109"/>
-      <c r="AP54" s="179"/>
+      <c r="AP54" s="137"/>
       <c r="AQ54" s="109"/>
       <c r="AR54" s="110"/>
       <c r="AS54" s="110"/>
@@ -4504,7 +4507,7 @@
     <row r="55" spans="1:48" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="80"/>
       <c r="B55" s="87"/>
-      <c r="C55" s="74"/>
+      <c r="C55" s="88"/>
       <c r="D55" s="88"/>
       <c r="E55" s="88"/>
       <c r="F55" s="74"/>
@@ -4516,44 +4519,44 @@
         <v>32</v>
       </c>
       <c r="L55" s="72"/>
-      <c r="M55" s="176"/>
-      <c r="N55" s="177"/>
+      <c r="M55" s="178"/>
+      <c r="N55" s="179"/>
       <c r="O55" s="73"/>
       <c r="P55" s="72"/>
       <c r="Q55" s="71" t="s">
         <v>32</v>
       </c>
       <c r="R55" s="72"/>
-      <c r="S55" s="176"/>
-      <c r="T55" s="177"/>
+      <c r="S55" s="178"/>
+      <c r="T55" s="179"/>
       <c r="U55" s="73"/>
       <c r="V55" s="72"/>
       <c r="W55" s="71" t="s">
         <v>32</v>
       </c>
       <c r="X55" s="72"/>
-      <c r="Y55" s="176"/>
-      <c r="Z55" s="177"/>
+      <c r="Y55" s="178"/>
+      <c r="Z55" s="179"/>
       <c r="AA55" s="73"/>
       <c r="AB55" s="72"/>
       <c r="AC55" s="71" t="s">
         <v>32</v>
       </c>
       <c r="AD55" s="72"/>
-      <c r="AE55" s="176"/>
-      <c r="AF55" s="177"/>
+      <c r="AE55" s="178"/>
+      <c r="AF55" s="179"/>
       <c r="AG55" s="73"/>
       <c r="AH55" s="72"/>
       <c r="AI55" s="71" t="s">
         <v>32</v>
       </c>
       <c r="AJ55" s="72"/>
-      <c r="AK55" s="176"/>
-      <c r="AL55" s="177"/>
-      <c r="AM55" s="177"/>
+      <c r="AK55" s="178"/>
+      <c r="AL55" s="179"/>
+      <c r="AM55" s="179"/>
       <c r="AN55" s="108"/>
       <c r="AO55" s="109"/>
-      <c r="AP55" s="179"/>
+      <c r="AP55" s="137"/>
       <c r="AQ55" s="109"/>
       <c r="AR55" s="110"/>
       <c r="AS55" s="110"/>

</xml_diff>